<commit_message>
Updated germination data, added column for half dead
</commit_message>
<xml_diff>
--- a/data/germination_data.xlsx
+++ b/data/germination_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nolanmeier/git/morasoilinoculation/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B13E4E91-E12A-754D-B1B8-CD71FB014AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F4E325E-252E-AD41-BC46-3992FEE872DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
+    <workbookView xWindow="4420" yWindow="680" windowWidth="24980" windowHeight="17260" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="93">
   <si>
     <t>seed_species</t>
   </si>
@@ -320,6 +320,24 @@
   <si>
     <t>56_dead</t>
   </si>
+  <si>
+    <t>63_alive</t>
+  </si>
+  <si>
+    <t>63_dead</t>
+  </si>
+  <si>
+    <t>63_halfdead</t>
+  </si>
+  <si>
+    <t>doy63: previous measurements invalid, 4 alive germinants</t>
+  </si>
+  <si>
+    <t>doy63: previous measurements invalid, 5 alive</t>
+  </si>
+  <si>
+    <t>doy63: previous measurements invalid, 5 alive, 2 dead, one hald dead</t>
+  </si>
 </sst>
 </file>
 
@@ -406,9 +424,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:BF213" totalsRowShown="0">
-  <autoFilter ref="B2:BF213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
-  <tableColumns count="57">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:BI213" totalsRowShown="0">
+  <autoFilter ref="B2:BI213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="THPL"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <filters>
+        <filter val="PSME"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="2">
+      <filters>
+        <filter val="25"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <tableColumns count="60">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
     <tableColumn id="3" xr3:uid="{B695F4B4-8561-9D48-9FF3-12A40CB2B7C7}" name="inoculated_%"/>
@@ -466,6 +500,9 @@
     <tableColumn id="55" xr3:uid="{4D1FAACD-5D25-4B95-83A8-6720ABC03B67}" name="49_dead"/>
     <tableColumn id="56" xr3:uid="{06E2873B-5152-2F44-A074-B7A947E84C43}" name="56_alive"/>
     <tableColumn id="57" xr3:uid="{40925643-C0D0-6E4E-8D59-1183BA29DA5B}" name="56_dead"/>
+    <tableColumn id="58" xr3:uid="{7636AB78-1D8A-1F4F-92B2-B83E7667F173}" name="63_alive"/>
+    <tableColumn id="59" xr3:uid="{A34B5762-8865-9648-B94B-CC20AE08AC1C}" name="63_dead"/>
+    <tableColumn id="60" xr3:uid="{2DF71B88-B0E3-204B-8D60-D79B1E3CB444}" name="63_halfdead"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -788,7 +825,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:BF212"/>
+  <dimension ref="B2:BI213"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -796,7 +833,7 @@
     <col min="4" max="4" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -968,8 +1005,17 @@
       <c r="BF2" t="s">
         <v>86</v>
       </c>
+      <c r="BG2" t="s">
+        <v>87</v>
+      </c>
+      <c r="BH2" t="s">
+        <v>88</v>
+      </c>
+      <c r="BI2" t="s">
+        <v>89</v>
+      </c>
     </row>
-    <row r="3" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1108,8 +1154,14 @@
       <c r="BF3">
         <v>1</v>
       </c>
+      <c r="BG3">
+        <v>3</v>
+      </c>
+      <c r="BH3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1194,8 +1246,11 @@
       <c r="BE4">
         <v>9</v>
       </c>
+      <c r="BG4">
+        <v>9</v>
+      </c>
     </row>
-    <row r="5" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1334,8 +1389,14 @@
       <c r="BF5">
         <v>1</v>
       </c>
+      <c r="BG5">
+        <v>6</v>
+      </c>
+      <c r="BH5">
+        <v>1</v>
+      </c>
     </row>
-    <row r="6" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1420,8 +1481,11 @@
       <c r="BE6">
         <v>9</v>
       </c>
+      <c r="BG6">
+        <v>9</v>
+      </c>
     </row>
-    <row r="7" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -1527,8 +1591,14 @@
       <c r="BF7">
         <v>4</v>
       </c>
+      <c r="BG7">
+        <v>2</v>
+      </c>
+      <c r="BH7">
+        <v>4</v>
+      </c>
     </row>
-    <row r="8" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -1661,8 +1731,14 @@
       <c r="BF8">
         <v>1</v>
       </c>
+      <c r="BG8">
+        <v>6</v>
+      </c>
+      <c r="BH8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -1801,8 +1877,14 @@
       <c r="BF9">
         <v>1</v>
       </c>
+      <c r="BG9">
+        <v>6</v>
+      </c>
+      <c r="BH9">
+        <v>1</v>
+      </c>
     </row>
-    <row r="10" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -1890,8 +1972,11 @@
       <c r="BE10">
         <v>8</v>
       </c>
+      <c r="BG10">
+        <v>8</v>
+      </c>
     </row>
-    <row r="11" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -2024,8 +2109,14 @@
       <c r="BF11">
         <v>2</v>
       </c>
+      <c r="BG11">
+        <v>6</v>
+      </c>
+      <c r="BH11">
+        <v>2</v>
+      </c>
     </row>
-    <row r="12" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -2167,8 +2258,14 @@
       <c r="BF12">
         <v>4</v>
       </c>
+      <c r="BG12">
+        <v>5</v>
+      </c>
+      <c r="BH12">
+        <v>4</v>
+      </c>
     </row>
-    <row r="13" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -2280,8 +2377,17 @@
       <c r="BF13">
         <v>1</v>
       </c>
+      <c r="BG13">
+        <v>5</v>
+      </c>
+      <c r="BH13">
+        <v>1</v>
+      </c>
+      <c r="BI13">
+        <v>1</v>
+      </c>
     </row>
-    <row r="14" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -2387,8 +2493,11 @@
       <c r="BE14">
         <v>8</v>
       </c>
+      <c r="BG14">
+        <v>9</v>
+      </c>
     </row>
-    <row r="15" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -2507,8 +2616,14 @@
       <c r="BF15">
         <v>4</v>
       </c>
+      <c r="BG15">
+        <v>4</v>
+      </c>
+      <c r="BH15">
+        <v>4</v>
+      </c>
     </row>
-    <row r="16" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -2612,8 +2727,14 @@
       <c r="BF16">
         <v>1</v>
       </c>
+      <c r="BG16">
+        <v>8</v>
+      </c>
+      <c r="BH16">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -2741,8 +2862,14 @@
       <c r="BF17">
         <v>2</v>
       </c>
+      <c r="BG17">
+        <v>6</v>
+      </c>
+      <c r="BH17">
+        <v>2</v>
+      </c>
     </row>
-    <row r="18" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -2822,8 +2949,11 @@
       <c r="BE18">
         <v>10</v>
       </c>
+      <c r="BG18">
+        <v>10</v>
+      </c>
     </row>
-    <row r="19" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -2954,8 +3084,14 @@
       <c r="BF19">
         <v>4</v>
       </c>
+      <c r="BG19">
+        <v>2</v>
+      </c>
+      <c r="BH19">
+        <v>4</v>
+      </c>
     </row>
-    <row r="20" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -3059,8 +3195,14 @@
       <c r="BF20">
         <v>1</v>
       </c>
+      <c r="BG20">
+        <v>13</v>
+      </c>
+      <c r="BH20">
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -3169,8 +3311,14 @@
       <c r="BF21">
         <v>1</v>
       </c>
+      <c r="BG21">
+        <v>5</v>
+      </c>
+      <c r="BH21">
+        <v>1</v>
+      </c>
     </row>
-    <row r="22" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -3256,8 +3404,11 @@
       <c r="BE22">
         <v>8</v>
       </c>
+      <c r="BG22">
+        <v>8</v>
+      </c>
     </row>
-    <row r="23" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -3373,8 +3524,17 @@
       <c r="BF23">
         <v>1</v>
       </c>
+      <c r="BG23">
+        <v>8</v>
+      </c>
+      <c r="BH23">
+        <v>1</v>
+      </c>
+      <c r="BI23">
+        <v>1</v>
+      </c>
     </row>
-    <row r="24" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -3484,8 +3644,14 @@
       <c r="BF24">
         <v>4</v>
       </c>
+      <c r="BG24">
+        <v>8</v>
+      </c>
+      <c r="BH24">
+        <v>4</v>
+      </c>
     </row>
-    <row r="25" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -3568,8 +3734,11 @@
       <c r="BE25">
         <v>8</v>
       </c>
+      <c r="BG25">
+        <v>8</v>
+      </c>
     </row>
-    <row r="26" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -3730,8 +3899,17 @@
       <c r="BF26">
         <v>3</v>
       </c>
+      <c r="BG26">
+        <v>6</v>
+      </c>
+      <c r="BH26">
+        <v>1</v>
+      </c>
+      <c r="BI26">
+        <v>2</v>
+      </c>
     </row>
-    <row r="27" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -3823,8 +4001,14 @@
       <c r="BF27">
         <v>1</v>
       </c>
+      <c r="BG27">
+        <v>3</v>
+      </c>
+      <c r="BH27">
+        <v>1</v>
+      </c>
     </row>
-    <row r="28" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -3964,8 +4148,17 @@
       <c r="BF28">
         <v>2</v>
       </c>
+      <c r="BG28">
+        <v>7</v>
+      </c>
+      <c r="BH28">
+        <v>2</v>
+      </c>
+      <c r="BI28">
+        <v>1</v>
+      </c>
     </row>
-    <row r="29" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
         <v>3</v>
       </c>
@@ -3979,6 +4172,9 @@
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
+      <c r="F29" t="s">
+        <v>90</v>
+      </c>
       <c r="M29">
         <v>1</v>
       </c>
@@ -4072,8 +4268,17 @@
       <c r="BF29">
         <v>1</v>
       </c>
+      <c r="BG29">
+        <v>4</v>
+      </c>
+      <c r="BH29">
+        <v>0</v>
+      </c>
+      <c r="BI29">
+        <v>1</v>
+      </c>
     </row>
-    <row r="30" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -4162,8 +4367,11 @@
       <c r="BE30">
         <v>8</v>
       </c>
+      <c r="BG30">
+        <v>8</v>
+      </c>
     </row>
-    <row r="31" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -4300,8 +4508,14 @@
       <c r="BF31">
         <v>3</v>
       </c>
+      <c r="BG31">
+        <v>2</v>
+      </c>
+      <c r="BH31">
+        <v>3</v>
+      </c>
     </row>
-    <row r="32" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -4402,8 +4616,14 @@
       <c r="BF32">
         <v>1</v>
       </c>
+      <c r="BG32">
+        <v>9</v>
+      </c>
+      <c r="BH32">
+        <v>1</v>
+      </c>
     </row>
-    <row r="33" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -4498,8 +4718,14 @@
       <c r="BF33">
         <v>1</v>
       </c>
+      <c r="BG33">
+        <v>8</v>
+      </c>
+      <c r="BH33">
+        <v>1</v>
+      </c>
     </row>
-    <row r="34" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -4612,8 +4838,11 @@
       <c r="BE34">
         <v>6</v>
       </c>
+      <c r="BG34">
+        <v>6</v>
+      </c>
     </row>
-    <row r="35" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -4729,8 +4958,14 @@
       <c r="BF35">
         <v>2</v>
       </c>
+      <c r="BG35">
+        <v>6</v>
+      </c>
+      <c r="BH35">
+        <v>2</v>
+      </c>
     </row>
-    <row r="36" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -4834,8 +5069,14 @@
       <c r="BF36">
         <v>1</v>
       </c>
+      <c r="BG36">
+        <v>8</v>
+      </c>
+      <c r="BI36">
+        <v>1</v>
+      </c>
     </row>
-    <row r="37" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -4918,8 +5159,11 @@
       <c r="BE37">
         <v>8</v>
       </c>
+      <c r="BG37">
+        <v>8</v>
+      </c>
     </row>
-    <row r="38" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -5074,8 +5318,14 @@
       <c r="BF38">
         <v>3</v>
       </c>
+      <c r="BG38">
+        <v>5</v>
+      </c>
+      <c r="BH38">
+        <v>3</v>
+      </c>
     </row>
-    <row r="39" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -5212,8 +5462,14 @@
       <c r="BF39">
         <v>4</v>
       </c>
+      <c r="BG39">
+        <v>2</v>
+      </c>
+      <c r="BH39">
+        <v>4</v>
+      </c>
     </row>
-    <row r="40" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -5362,8 +5618,14 @@
       <c r="BF40">
         <v>6</v>
       </c>
+      <c r="BG40">
+        <v>4</v>
+      </c>
+      <c r="BH40">
+        <v>6</v>
+      </c>
     </row>
-    <row r="41" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -5479,8 +5741,14 @@
       <c r="BF41">
         <v>2</v>
       </c>
+      <c r="BG41">
+        <v>4</v>
+      </c>
+      <c r="BH41">
+        <v>2</v>
+      </c>
     </row>
-    <row r="42" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -5572,8 +5840,11 @@
       <c r="BE42">
         <v>7</v>
       </c>
+      <c r="BG42">
+        <v>7</v>
+      </c>
     </row>
-    <row r="43" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -5707,8 +5978,14 @@
       <c r="BF43">
         <v>6</v>
       </c>
+      <c r="BG43">
+        <v>3</v>
+      </c>
+      <c r="BH43">
+        <v>6</v>
+      </c>
     </row>
-    <row r="44" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -5785,8 +6062,11 @@
       <c r="BE44">
         <v>6</v>
       </c>
+      <c r="BG44">
+        <v>6</v>
+      </c>
     </row>
-    <row r="45" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -5947,8 +6227,17 @@
       <c r="BF45">
         <v>3</v>
       </c>
+      <c r="BG45">
+        <v>5</v>
+      </c>
+      <c r="BH45">
+        <v>3</v>
+      </c>
+      <c r="BI45">
+        <v>1</v>
+      </c>
     </row>
-    <row r="46" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -6037,8 +6326,11 @@
       <c r="BE46">
         <v>6</v>
       </c>
+      <c r="BG46">
+        <v>6</v>
+      </c>
     </row>
-    <row r="47" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -6130,8 +6422,14 @@
       <c r="BF47">
         <v>1</v>
       </c>
+      <c r="BG47">
+        <v>8</v>
+      </c>
+      <c r="BH47">
+        <v>1</v>
+      </c>
     </row>
-    <row r="48" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -6277,8 +6575,17 @@
       <c r="BF48">
         <v>5</v>
       </c>
+      <c r="BG48">
+        <v>5</v>
+      </c>
+      <c r="BH48">
+        <v>5</v>
+      </c>
+      <c r="BI48">
+        <v>1</v>
+      </c>
     </row>
-    <row r="49" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -6361,8 +6668,11 @@
       <c r="BE49">
         <v>8</v>
       </c>
+      <c r="BG49">
+        <v>8</v>
+      </c>
     </row>
-    <row r="50" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -6523,8 +6833,14 @@
       <c r="BF50">
         <v>1</v>
       </c>
+      <c r="BG50">
+        <v>7</v>
+      </c>
+      <c r="BH50">
+        <v>1</v>
+      </c>
     </row>
-    <row r="51" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -6658,8 +6974,17 @@
       <c r="BF51">
         <v>1</v>
       </c>
+      <c r="BG51">
+        <v>4</v>
+      </c>
+      <c r="BH51">
+        <v>1</v>
+      </c>
+      <c r="BI51">
+        <v>1</v>
+      </c>
     </row>
-    <row r="52" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -6742,8 +7067,11 @@
       <c r="BE52">
         <v>6</v>
       </c>
+      <c r="BG52">
+        <v>6</v>
+      </c>
     </row>
-    <row r="53" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -6868,8 +7196,14 @@
       <c r="BF53">
         <v>1</v>
       </c>
+      <c r="BG53">
+        <v>3</v>
+      </c>
+      <c r="BH53">
+        <v>1</v>
+      </c>
     </row>
-    <row r="54" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -6955,8 +7289,11 @@
       <c r="BE54">
         <v>5</v>
       </c>
+      <c r="BG54">
+        <v>5</v>
+      </c>
     </row>
-    <row r="55" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -7075,8 +7412,14 @@
       <c r="BF55">
         <v>4</v>
       </c>
+      <c r="BG55">
+        <v>2</v>
+      </c>
+      <c r="BH55">
+        <v>4</v>
+      </c>
     </row>
-    <row r="56" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -7153,8 +7496,11 @@
       <c r="BE56">
         <v>10</v>
       </c>
+      <c r="BG56">
+        <v>10</v>
+      </c>
     </row>
-    <row r="57" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -7237,8 +7583,11 @@
       <c r="BE57">
         <v>5</v>
       </c>
+      <c r="BG57">
+        <v>5</v>
+      </c>
     </row>
-    <row r="58" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -7327,8 +7676,11 @@
       <c r="BE58">
         <v>6</v>
       </c>
+      <c r="BG58">
+        <v>6</v>
+      </c>
     </row>
-    <row r="59" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -7408,8 +7760,11 @@
       <c r="BE59">
         <v>7</v>
       </c>
+      <c r="BG59">
+        <v>7</v>
+      </c>
     </row>
-    <row r="60" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -7528,8 +7883,14 @@
       <c r="BF60">
         <v>2</v>
       </c>
+      <c r="BG60">
+        <v>7</v>
+      </c>
+      <c r="BH60">
+        <v>2</v>
+      </c>
     </row>
-    <row r="61" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -7612,8 +7973,14 @@
       <c r="BE61">
         <v>7</v>
       </c>
+      <c r="BG61">
+        <v>7</v>
+      </c>
+      <c r="BI61">
+        <v>1</v>
+      </c>
     </row>
-    <row r="62" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -7762,8 +8129,14 @@
       <c r="BF62">
         <v>2</v>
       </c>
+      <c r="BG62">
+        <v>3</v>
+      </c>
+      <c r="BH62">
+        <v>2</v>
+      </c>
     </row>
-    <row r="63" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -7891,8 +8264,17 @@
       <c r="BF63">
         <v>3</v>
       </c>
+      <c r="BG63">
+        <v>4</v>
+      </c>
+      <c r="BH63">
+        <v>3</v>
+      </c>
+      <c r="BI63">
+        <v>1</v>
+      </c>
     </row>
-    <row r="64" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -7990,8 +8372,17 @@
       <c r="BF64">
         <v>2</v>
       </c>
+      <c r="BG64">
+        <v>6</v>
+      </c>
+      <c r="BH64">
+        <v>2</v>
+      </c>
+      <c r="BI64">
+        <v>1</v>
+      </c>
     </row>
-    <row r="65" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -8092,8 +8483,17 @@
       <c r="BF65">
         <v>1</v>
       </c>
+      <c r="BG65">
+        <v>5</v>
+      </c>
+      <c r="BH65">
+        <v>1</v>
+      </c>
+      <c r="BI65">
+        <v>1</v>
+      </c>
     </row>
-    <row r="66" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -8176,8 +8576,11 @@
       <c r="BE66">
         <v>4</v>
       </c>
+      <c r="BG66">
+        <v>4</v>
+      </c>
     </row>
-    <row r="67" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -8314,8 +8717,17 @@
       <c r="BF67">
         <v>7</v>
       </c>
+      <c r="BG67">
+        <v>3</v>
+      </c>
+      <c r="BH67">
+        <v>7</v>
+      </c>
+      <c r="BI67">
+        <v>1</v>
+      </c>
     </row>
-    <row r="68" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -8392,8 +8804,11 @@
       <c r="BE68">
         <v>11</v>
       </c>
+      <c r="BG68">
+        <v>11</v>
+      </c>
     </row>
-    <row r="69" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -8476,8 +8891,11 @@
       <c r="BE69">
         <v>9</v>
       </c>
+      <c r="BG69">
+        <v>9</v>
+      </c>
     </row>
-    <row r="70" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -8569,8 +8987,11 @@
       <c r="BE70">
         <v>7</v>
       </c>
+      <c r="BG70">
+        <v>7</v>
+      </c>
     </row>
-    <row r="71" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -8686,8 +9107,17 @@
       <c r="BF71">
         <v>3</v>
       </c>
+      <c r="BG71">
+        <v>7</v>
+      </c>
+      <c r="BH71">
+        <v>3</v>
+      </c>
+      <c r="BI71">
+        <v>1</v>
+      </c>
     </row>
-    <row r="72" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -8815,8 +9245,14 @@
       <c r="BF72">
         <v>1</v>
       </c>
+      <c r="BG72">
+        <v>6</v>
+      </c>
+      <c r="BH72">
+        <v>1</v>
+      </c>
     </row>
-    <row r="73" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -8899,8 +9335,11 @@
       <c r="BE73">
         <v>8</v>
       </c>
+      <c r="BG73">
+        <v>8</v>
+      </c>
     </row>
-    <row r="74" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -8992,8 +9431,11 @@
       <c r="BE74">
         <v>9</v>
       </c>
+      <c r="BG74">
+        <v>9</v>
+      </c>
     </row>
-    <row r="75" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="75" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -9106,8 +9548,14 @@
       <c r="BF75">
         <v>1</v>
       </c>
+      <c r="BG75">
+        <v>6</v>
+      </c>
+      <c r="BH75">
+        <v>1</v>
+      </c>
     </row>
-    <row r="76" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="76" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -9253,8 +9701,14 @@
       <c r="BF76">
         <v>1</v>
       </c>
+      <c r="BG76">
+        <v>7</v>
+      </c>
+      <c r="BH76">
+        <v>1</v>
+      </c>
     </row>
-    <row r="77" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -9352,8 +9806,14 @@
       <c r="BF77">
         <v>2</v>
       </c>
+      <c r="BG77">
+        <v>4</v>
+      </c>
+      <c r="BH77">
+        <v>2</v>
+      </c>
     </row>
-    <row r="78" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -9439,8 +9899,11 @@
       <c r="BE78">
         <v>7</v>
       </c>
+      <c r="BG78">
+        <v>7</v>
+      </c>
     </row>
-    <row r="79" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="79" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -9580,8 +10043,14 @@
       <c r="BF79">
         <v>6</v>
       </c>
+      <c r="BG79">
+        <v>2</v>
+      </c>
+      <c r="BH79">
+        <v>7</v>
+      </c>
     </row>
-    <row r="80" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="80" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -9691,8 +10160,14 @@
       <c r="BF80">
         <v>1</v>
       </c>
+      <c r="BG80">
+        <v>9</v>
+      </c>
+      <c r="BH80">
+        <v>1</v>
+      </c>
     </row>
-    <row r="81" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -9814,8 +10289,14 @@
       <c r="BF81">
         <v>2</v>
       </c>
+      <c r="BG81">
+        <v>4</v>
+      </c>
+      <c r="BH81">
+        <v>2</v>
+      </c>
     </row>
-    <row r="82" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -9952,8 +10433,17 @@
       <c r="BF82">
         <v>2</v>
       </c>
+      <c r="BG82">
+        <v>7</v>
+      </c>
+      <c r="BH82">
+        <v>2</v>
+      </c>
+      <c r="BI82">
+        <v>1</v>
+      </c>
     </row>
-    <row r="83" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -10093,8 +10583,14 @@
       <c r="BF83">
         <v>4</v>
       </c>
+      <c r="BG83">
+        <v>5</v>
+      </c>
+      <c r="BH83">
+        <v>4</v>
+      </c>
     </row>
-    <row r="84" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -10234,8 +10730,14 @@
       <c r="BF84">
         <v>2</v>
       </c>
+      <c r="BG84">
+        <v>7</v>
+      </c>
+      <c r="BH84">
+        <v>2</v>
+      </c>
     </row>
-    <row r="85" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -10372,8 +10874,14 @@
       <c r="BF85">
         <v>2</v>
       </c>
+      <c r="BG85">
+        <v>4</v>
+      </c>
+      <c r="BH85">
+        <v>2</v>
+      </c>
     </row>
-    <row r="86" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -10492,8 +11000,14 @@
       <c r="BF86">
         <v>1</v>
       </c>
+      <c r="BG86">
+        <v>8</v>
+      </c>
+      <c r="BH86">
+        <v>1</v>
+      </c>
     </row>
-    <row r="87" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -10636,8 +11150,14 @@
       <c r="BF87">
         <v>2</v>
       </c>
+      <c r="BG87">
+        <v>5</v>
+      </c>
+      <c r="BH87">
+        <v>2</v>
+      </c>
     </row>
-    <row r="88" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -10765,8 +11285,14 @@
       <c r="BF88">
         <v>3</v>
       </c>
+      <c r="BG88">
+        <v>6</v>
+      </c>
+      <c r="BH88">
+        <v>3</v>
+      </c>
     </row>
-    <row r="89" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B89" t="s">
         <v>3</v>
       </c>
@@ -10780,6 +11306,9 @@
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
+      <c r="F89" t="s">
+        <v>91</v>
+      </c>
       <c r="K89">
         <v>1</v>
       </c>
@@ -10873,8 +11402,11 @@
       <c r="BF89">
         <v>2</v>
       </c>
+      <c r="BG89">
+        <v>5</v>
+      </c>
     </row>
-    <row r="90" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -10960,8 +11492,11 @@
       <c r="BE90">
         <v>7</v>
       </c>
+      <c r="BG90">
+        <v>7</v>
+      </c>
     </row>
-    <row r="91" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -11098,8 +11633,17 @@
       <c r="BF91">
         <v>3</v>
       </c>
+      <c r="BG91">
+        <v>5</v>
+      </c>
+      <c r="BH91">
+        <v>3</v>
+      </c>
+      <c r="BI91">
+        <v>2</v>
+      </c>
     </row>
-    <row r="92" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="92" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B92" t="s">
         <v>1</v>
       </c>
@@ -11113,6 +11657,9 @@
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
+      <c r="F92" t="s">
+        <v>92</v>
+      </c>
       <c r="Q92">
         <v>0</v>
       </c>
@@ -11215,8 +11762,14 @@
       <c r="BF92">
         <v>3</v>
       </c>
+      <c r="BG92">
+        <v>5</v>
+      </c>
+      <c r="BH92">
+        <v>2</v>
+      </c>
     </row>
-    <row r="93" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -11308,8 +11861,14 @@
       <c r="BF93">
         <v>1</v>
       </c>
+      <c r="BG93">
+        <v>8</v>
+      </c>
+      <c r="BH93">
+        <v>1</v>
+      </c>
     </row>
-    <row r="94" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -11398,8 +11957,11 @@
       <c r="BE94">
         <v>7</v>
       </c>
+      <c r="BG94">
+        <v>7</v>
+      </c>
     </row>
-    <row r="95" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -11497,8 +12059,14 @@
       <c r="BF95">
         <v>1</v>
       </c>
+      <c r="BG95">
+        <v>7</v>
+      </c>
+      <c r="BH95">
+        <v>1</v>
+      </c>
     </row>
-    <row r="96" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -11620,8 +12188,14 @@
       <c r="BF96">
         <v>2</v>
       </c>
+      <c r="BG96">
+        <v>8</v>
+      </c>
+      <c r="BH96">
+        <v>2</v>
+      </c>
     </row>
-    <row r="97" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="97" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -11707,8 +12281,11 @@
       <c r="BE97">
         <v>7</v>
       </c>
+      <c r="BG97">
+        <v>7</v>
+      </c>
     </row>
-    <row r="98" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="98" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -11830,8 +12407,14 @@
       <c r="BF98">
         <v>2</v>
       </c>
+      <c r="BG98">
+        <v>5</v>
+      </c>
+      <c r="BH98">
+        <v>2</v>
+      </c>
     </row>
-    <row r="99" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="99" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -11911,8 +12494,11 @@
       <c r="BE99">
         <v>2</v>
       </c>
+      <c r="BG99">
+        <v>2</v>
+      </c>
     </row>
-    <row r="100" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="100" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -11995,8 +12581,11 @@
       <c r="BE100">
         <v>8</v>
       </c>
+      <c r="BG100">
+        <v>8</v>
+      </c>
     </row>
-    <row r="101" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="101" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -12106,8 +12695,14 @@
       <c r="BF101">
         <v>4</v>
       </c>
+      <c r="BG101">
+        <v>1</v>
+      </c>
+      <c r="BH101">
+        <v>4</v>
+      </c>
     </row>
-    <row r="102" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="102" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -12193,8 +12788,11 @@
       <c r="BE102">
         <v>7</v>
       </c>
+      <c r="BG102">
+        <v>7</v>
+      </c>
     </row>
-    <row r="103" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="103" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -12325,8 +12923,14 @@
       <c r="BF103">
         <v>4</v>
       </c>
+      <c r="BG103">
+        <v>2</v>
+      </c>
+      <c r="BH103">
+        <v>4</v>
+      </c>
     </row>
-    <row r="104" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="104" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -12430,8 +13034,17 @@
       <c r="BF104">
         <v>2</v>
       </c>
+      <c r="BG104">
+        <v>7</v>
+      </c>
+      <c r="BH104">
+        <v>2</v>
+      </c>
+      <c r="BI104">
+        <v>1</v>
+      </c>
     </row>
-    <row r="105" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="105" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -12547,8 +13160,14 @@
       <c r="BF105">
         <v>3</v>
       </c>
+      <c r="BG105">
+        <v>2</v>
+      </c>
+      <c r="BH105">
+        <v>3</v>
+      </c>
     </row>
-    <row r="106" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="106" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -12679,8 +13298,11 @@
       <c r="BE106">
         <v>7</v>
       </c>
+      <c r="BG106">
+        <v>7</v>
+      </c>
     </row>
-    <row r="107" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="107" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -12808,8 +13430,14 @@
       <c r="BF107">
         <v>1</v>
       </c>
+      <c r="BG107">
+        <v>4</v>
+      </c>
+      <c r="BH107">
+        <v>1</v>
+      </c>
     </row>
-    <row r="108" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="108" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -12901,8 +13529,17 @@
       <c r="BF108">
         <v>1</v>
       </c>
+      <c r="BG108">
+        <v>8</v>
+      </c>
+      <c r="BH108">
+        <v>1</v>
+      </c>
+      <c r="BI108">
+        <v>1</v>
+      </c>
     </row>
-    <row r="109" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="109" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -13018,8 +13655,17 @@
       <c r="BF109">
         <v>8</v>
       </c>
+      <c r="BG109">
+        <v>1</v>
+      </c>
+      <c r="BH109">
+        <v>8</v>
+      </c>
+      <c r="BI109">
+        <v>0</v>
+      </c>
     </row>
-    <row r="110" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="110" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -13147,8 +13793,17 @@
       <c r="BF110">
         <v>1</v>
       </c>
+      <c r="BG110">
+        <v>8</v>
+      </c>
+      <c r="BH110">
+        <v>0</v>
+      </c>
+      <c r="BI110">
+        <v>1</v>
+      </c>
     </row>
-    <row r="111" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="111" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -13249,8 +13904,14 @@
       <c r="BF111">
         <v>2</v>
       </c>
+      <c r="BG111">
+        <v>4</v>
+      </c>
+      <c r="BH111">
+        <v>2</v>
+      </c>
     </row>
-    <row r="112" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="112" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -13372,8 +14033,14 @@
       <c r="BF112">
         <v>2</v>
       </c>
+      <c r="BG112">
+        <v>6</v>
+      </c>
+      <c r="BH112">
+        <v>2</v>
+      </c>
     </row>
-    <row r="113" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="113" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -13510,8 +14177,14 @@
       <c r="BF113">
         <v>2</v>
       </c>
+      <c r="BG113">
+        <v>4</v>
+      </c>
+      <c r="BH113">
+        <v>2</v>
+      </c>
     </row>
-    <row r="114" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="114" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -13597,8 +14270,11 @@
       <c r="BE114">
         <v>8</v>
       </c>
+      <c r="BG114">
+        <v>8</v>
+      </c>
     </row>
-    <row r="115" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="115" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -13738,8 +14414,14 @@
       <c r="BF115">
         <v>3</v>
       </c>
+      <c r="BG115">
+        <v>1</v>
+      </c>
+      <c r="BH115">
+        <v>3</v>
+      </c>
     </row>
-    <row r="116" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="116" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -13843,8 +14525,17 @@
       <c r="BF116">
         <v>1</v>
       </c>
+      <c r="BG116">
+        <v>8</v>
+      </c>
+      <c r="BH116">
+        <v>1</v>
+      </c>
+      <c r="BI116">
+        <v>1</v>
+      </c>
     </row>
-    <row r="117" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="117" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -13960,8 +14651,17 @@
       <c r="BF117">
         <v>3</v>
       </c>
+      <c r="BG117">
+        <v>1</v>
+      </c>
+      <c r="BH117">
+        <v>3</v>
+      </c>
+      <c r="BI117">
+        <v>1</v>
+      </c>
     </row>
-    <row r="118" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="118" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -14051,8 +14751,11 @@
       <c r="BE118">
         <v>6</v>
       </c>
+      <c r="BG118">
+        <v>6</v>
+      </c>
     </row>
-    <row r="119" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="119" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -14132,8 +14835,11 @@
       <c r="BE119">
         <v>7</v>
       </c>
+      <c r="BG119">
+        <v>7</v>
+      </c>
     </row>
-    <row r="120" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="120" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -14216,8 +14922,11 @@
       <c r="BE120">
         <v>10</v>
       </c>
+      <c r="BG120">
+        <v>10</v>
+      </c>
     </row>
-    <row r="121" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="121" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -14303,8 +15012,11 @@
       <c r="BE121">
         <v>8</v>
       </c>
+      <c r="BG121">
+        <v>8</v>
+      </c>
     </row>
-    <row r="122" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="122" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -14393,8 +15105,11 @@
       <c r="BE122">
         <v>5</v>
       </c>
+      <c r="BG122">
+        <v>5</v>
+      </c>
     </row>
-    <row r="123" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="123" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -14513,8 +15228,14 @@
       <c r="BF123">
         <v>3</v>
       </c>
+      <c r="BG123">
+        <v>3</v>
+      </c>
+      <c r="BH123">
+        <v>3</v>
+      </c>
     </row>
-    <row r="124" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="124" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -14660,8 +15381,14 @@
       <c r="BF124">
         <v>3</v>
       </c>
+      <c r="BG124">
+        <v>6</v>
+      </c>
+      <c r="BH124">
+        <v>3</v>
+      </c>
     </row>
-    <row r="125" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="125" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -14807,8 +15534,14 @@
       <c r="BF125">
         <v>6</v>
       </c>
+      <c r="BG125">
+        <v>0</v>
+      </c>
+      <c r="BH125">
+        <v>6</v>
+      </c>
     </row>
-    <row r="126" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="126" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -14933,8 +15666,14 @@
       <c r="BF126">
         <v>1</v>
       </c>
+      <c r="BG126">
+        <v>5</v>
+      </c>
+      <c r="BH126">
+        <v>1</v>
+      </c>
     </row>
-    <row r="127" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="127" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -15056,8 +15795,14 @@
       <c r="BF127">
         <v>2</v>
       </c>
+      <c r="BG127">
+        <v>1</v>
+      </c>
+      <c r="BH127">
+        <v>2</v>
+      </c>
     </row>
-    <row r="128" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="128" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -15134,8 +15879,11 @@
       <c r="BE128">
         <v>7</v>
       </c>
+      <c r="BG128">
+        <v>7</v>
+      </c>
     </row>
-    <row r="129" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="129" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -15257,8 +16005,17 @@
       <c r="BF129">
         <v>3</v>
       </c>
+      <c r="BG129">
+        <v>2</v>
+      </c>
+      <c r="BH129">
+        <v>3</v>
+      </c>
+      <c r="BI129">
+        <v>1</v>
+      </c>
     </row>
-    <row r="130" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="130" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -15347,8 +16104,11 @@
       <c r="BE130">
         <v>7</v>
       </c>
+      <c r="BG130">
+        <v>8</v>
+      </c>
     </row>
-    <row r="131" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="131" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -15461,8 +16221,17 @@
       <c r="BF131">
         <v>2</v>
       </c>
+      <c r="BG131">
+        <v>7</v>
+      </c>
+      <c r="BH131">
+        <v>2</v>
+      </c>
+      <c r="BI131">
+        <v>1</v>
+      </c>
     </row>
-    <row r="132" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="132" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -15542,8 +16311,11 @@
       <c r="BE132">
         <v>6</v>
       </c>
+      <c r="BG132">
+        <v>6</v>
+      </c>
     </row>
-    <row r="133" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="133" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -15635,8 +16407,14 @@
       <c r="BF133">
         <v>1</v>
       </c>
+      <c r="BG133">
+        <v>6</v>
+      </c>
+      <c r="BH133">
+        <v>1</v>
+      </c>
     </row>
-    <row r="134" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="134" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -15728,8 +16506,11 @@
       <c r="BE134">
         <v>10</v>
       </c>
+      <c r="BG134">
+        <v>10</v>
+      </c>
     </row>
-    <row r="135" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="135" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -15821,8 +16602,17 @@
       <c r="BF135">
         <v>1</v>
       </c>
+      <c r="BG135">
+        <v>6</v>
+      </c>
+      <c r="BH135">
+        <v>1</v>
+      </c>
+      <c r="BI135">
+        <v>1</v>
+      </c>
     </row>
-    <row r="136" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="136" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -15926,8 +16716,14 @@
       <c r="BF136">
         <v>1</v>
       </c>
+      <c r="BG136">
+        <v>6</v>
+      </c>
+      <c r="BH136">
+        <v>1</v>
+      </c>
     </row>
-    <row r="137" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="137" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -16037,8 +16833,14 @@
       <c r="BF137">
         <v>2</v>
       </c>
+      <c r="BG137">
+        <v>3</v>
+      </c>
+      <c r="BH137">
+        <v>2</v>
+      </c>
     </row>
-    <row r="138" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="138" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -16166,8 +16968,14 @@
       <c r="BF138">
         <v>1</v>
       </c>
+      <c r="BG138">
+        <v>7</v>
+      </c>
+      <c r="BH138">
+        <v>1</v>
+      </c>
     </row>
-    <row r="139" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="139" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -16277,8 +17085,14 @@
       <c r="BF139">
         <v>1</v>
       </c>
+      <c r="BG139">
+        <v>5</v>
+      </c>
+      <c r="BH139">
+        <v>1</v>
+      </c>
     </row>
-    <row r="140" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="140" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -16355,8 +17169,11 @@
       <c r="BE140">
         <v>9</v>
       </c>
+      <c r="BG140">
+        <v>9</v>
+      </c>
     </row>
-    <row r="141" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="141" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -16505,8 +17322,14 @@
       <c r="BF141">
         <v>4</v>
       </c>
+      <c r="BG141">
+        <v>4</v>
+      </c>
+      <c r="BH141">
+        <v>4</v>
+      </c>
     </row>
-    <row r="142" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="142" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -16652,8 +17475,14 @@
       <c r="BF142">
         <v>2</v>
       </c>
+      <c r="BG142">
+        <v>6</v>
+      </c>
+      <c r="BH142">
+        <v>2</v>
+      </c>
     </row>
-    <row r="143" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="143" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -16745,8 +17574,14 @@
       <c r="BF143">
         <v>1</v>
       </c>
+      <c r="BG143">
+        <v>8</v>
+      </c>
+      <c r="BH143">
+        <v>1</v>
+      </c>
     </row>
-    <row r="144" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="144" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -16826,8 +17661,11 @@
       <c r="BE144">
         <v>7</v>
       </c>
+      <c r="BG144">
+        <v>7</v>
+      </c>
     </row>
-    <row r="145" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="145" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -16913,8 +17751,11 @@
       <c r="BE145">
         <v>7</v>
       </c>
+      <c r="BG145">
+        <v>7</v>
+      </c>
     </row>
-    <row r="146" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="146" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -17051,8 +17892,17 @@
       <c r="BF146">
         <v>2</v>
       </c>
+      <c r="BG146">
+        <v>8</v>
+      </c>
+      <c r="BH146">
+        <v>1</v>
+      </c>
+      <c r="BI146">
+        <v>1</v>
+      </c>
     </row>
-    <row r="147" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="147" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -17183,8 +18033,14 @@
       <c r="BF147">
         <v>1</v>
       </c>
+      <c r="BG147">
+        <v>2</v>
+      </c>
+      <c r="BH147">
+        <v>1</v>
+      </c>
     </row>
-    <row r="148" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="148" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -17267,8 +18123,11 @@
       <c r="BE148">
         <v>9</v>
       </c>
+      <c r="BG148">
+        <v>9</v>
+      </c>
     </row>
-    <row r="149" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="149" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -17390,8 +18249,14 @@
       <c r="BF149">
         <v>2</v>
       </c>
+      <c r="BG149">
+        <v>2</v>
+      </c>
+      <c r="BH149">
+        <v>2</v>
+      </c>
     </row>
-    <row r="150" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="150" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -17534,8 +18399,14 @@
       <c r="BF150">
         <v>1</v>
       </c>
+      <c r="BG150">
+        <v>8</v>
+      </c>
+      <c r="BH150">
+        <v>1</v>
+      </c>
     </row>
-    <row r="151" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="151" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -17630,8 +18501,14 @@
       <c r="BF151">
         <v>3</v>
       </c>
+      <c r="BG151">
+        <v>4</v>
+      </c>
+      <c r="BH151">
+        <v>3</v>
+      </c>
     </row>
-    <row r="152" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="152" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -17708,8 +18585,11 @@
       <c r="BE152">
         <v>9</v>
       </c>
+      <c r="BG152">
+        <v>9</v>
+      </c>
     </row>
-    <row r="153" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="153" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -17816,8 +18696,14 @@
       <c r="BF153">
         <v>1</v>
       </c>
+      <c r="BG153">
+        <v>5</v>
+      </c>
+      <c r="BH153">
+        <v>1</v>
+      </c>
     </row>
-    <row r="154" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="154" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -17969,8 +18855,17 @@
       <c r="BF154">
         <v>2</v>
       </c>
+      <c r="BG154">
+        <v>5</v>
+      </c>
+      <c r="BH154">
+        <v>2</v>
+      </c>
+      <c r="BI154">
+        <v>1</v>
+      </c>
     </row>
-    <row r="155" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="155" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -18089,8 +18984,14 @@
       <c r="BF155">
         <v>3</v>
       </c>
+      <c r="BG155">
+        <v>6</v>
+      </c>
+      <c r="BH155">
+        <v>3</v>
+      </c>
     </row>
-    <row r="156" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="156" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -18173,8 +19074,11 @@
       <c r="BE156">
         <v>6</v>
       </c>
+      <c r="BG156">
+        <v>6</v>
+      </c>
     </row>
-    <row r="157" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="157" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -18260,8 +19164,11 @@
       <c r="BE157">
         <v>5</v>
       </c>
+      <c r="BG157">
+        <v>5</v>
+      </c>
     </row>
-    <row r="158" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="158" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -18353,8 +19260,11 @@
       <c r="BE158">
         <v>7</v>
       </c>
+      <c r="BG158">
+        <v>7</v>
+      </c>
     </row>
-    <row r="159" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="159" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -18473,8 +19383,17 @@
       <c r="BF159">
         <v>3</v>
       </c>
+      <c r="BG159">
+        <v>3</v>
+      </c>
+      <c r="BH159">
+        <v>3</v>
+      </c>
+      <c r="BI159">
+        <v>1</v>
+      </c>
     </row>
-    <row r="160" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="160" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -18557,8 +19476,11 @@
       <c r="BE160">
         <v>9</v>
       </c>
+      <c r="BG160">
+        <v>9</v>
+      </c>
     </row>
-    <row r="161" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="161" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -18696,13 +19618,22 @@
         <v>4</v>
       </c>
       <c r="BE161">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BF161">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="BG161">
+        <v>2</v>
+      </c>
+      <c r="BH161">
+        <v>4</v>
+      </c>
+      <c r="BI161">
+        <v>1</v>
       </c>
     </row>
-    <row r="162" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="162" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -18788,8 +19719,11 @@
       <c r="BE162">
         <v>8</v>
       </c>
+      <c r="BG162">
+        <v>8</v>
+      </c>
     </row>
-    <row r="163" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="163" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -18905,8 +19839,14 @@
       <c r="BF163">
         <v>6</v>
       </c>
+      <c r="BG163">
+        <v>2</v>
+      </c>
+      <c r="BH163">
+        <v>6</v>
+      </c>
     </row>
-    <row r="164" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="164" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -18983,8 +19923,11 @@
       <c r="BE164">
         <v>9</v>
       </c>
+      <c r="BG164">
+        <v>9</v>
+      </c>
     </row>
-    <row r="165" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="165" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -19100,8 +20043,14 @@
       <c r="BF165">
         <v>2</v>
       </c>
+      <c r="BG165">
+        <v>4</v>
+      </c>
+      <c r="BH165">
+        <v>2</v>
+      </c>
     </row>
-    <row r="166" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="166" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -19229,8 +20178,11 @@
       <c r="BE166">
         <v>5</v>
       </c>
+      <c r="BG166">
+        <v>5</v>
+      </c>
     </row>
-    <row r="167" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="167" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -19334,8 +20286,14 @@
       <c r="BF167">
         <v>1</v>
       </c>
+      <c r="BG167">
+        <v>7</v>
+      </c>
+      <c r="BH167">
+        <v>1</v>
+      </c>
     </row>
-    <row r="168" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="168" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -19457,8 +20415,17 @@
       <c r="BF168">
         <v>1</v>
       </c>
+      <c r="BG168">
+        <v>9</v>
+      </c>
+      <c r="BH168">
+        <v>1</v>
+      </c>
+      <c r="BI168">
+        <v>1</v>
+      </c>
     </row>
-    <row r="169" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="169" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -19544,8 +20511,11 @@
       <c r="BE169">
         <v>6</v>
       </c>
+      <c r="BG169">
+        <v>6</v>
+      </c>
     </row>
-    <row r="170" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="170" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -19631,8 +20601,11 @@
       <c r="BE170">
         <v>8</v>
       </c>
+      <c r="BG170">
+        <v>8</v>
+      </c>
     </row>
-    <row r="171" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="171" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -19760,8 +20733,17 @@
       <c r="BF171">
         <v>3</v>
       </c>
+      <c r="BG171">
+        <v>5</v>
+      </c>
+      <c r="BH171">
+        <v>3</v>
+      </c>
+      <c r="BI171">
+        <v>2</v>
+      </c>
     </row>
-    <row r="172" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="172" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -19844,8 +20826,11 @@
       <c r="BE172">
         <v>8</v>
       </c>
+      <c r="BG172">
+        <v>8</v>
+      </c>
     </row>
-    <row r="173" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="173" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -19928,8 +20913,11 @@
       <c r="BE173">
         <v>6</v>
       </c>
+      <c r="BG173">
+        <v>6</v>
+      </c>
     </row>
-    <row r="174" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="174" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -20015,8 +21003,11 @@
       <c r="BE174">
         <v>9</v>
       </c>
+      <c r="BG174">
+        <v>9</v>
+      </c>
     </row>
-    <row r="175" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="175" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -20132,8 +21123,14 @@
       <c r="BF175">
         <v>2</v>
       </c>
+      <c r="BG175">
+        <v>7</v>
+      </c>
+      <c r="BH175">
+        <v>2</v>
+      </c>
     </row>
-    <row r="176" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="176" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -20210,8 +21207,11 @@
       <c r="BE176">
         <v>8</v>
       </c>
+      <c r="BG176">
+        <v>8</v>
+      </c>
     </row>
-    <row r="177" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="177" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -20294,8 +21294,11 @@
       <c r="BE177">
         <v>4</v>
       </c>
+      <c r="BG177">
+        <v>4</v>
+      </c>
     </row>
-    <row r="178" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="178" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -20384,8 +21387,11 @@
       <c r="BE178">
         <v>8</v>
       </c>
+      <c r="BG178">
+        <v>8</v>
+      </c>
     </row>
-    <row r="179" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="179" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -20504,8 +21510,14 @@
       <c r="BF179">
         <v>4</v>
       </c>
+      <c r="BG179">
+        <v>6</v>
+      </c>
+      <c r="BH179">
+        <v>4</v>
+      </c>
     </row>
-    <row r="180" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="180" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -20618,8 +21630,14 @@
       <c r="BF180">
         <v>2</v>
       </c>
+      <c r="BG180">
+        <v>7</v>
+      </c>
+      <c r="BH180">
+        <v>2</v>
+      </c>
     </row>
-    <row r="181" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="181" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -20726,8 +21744,17 @@
       <c r="BF181">
         <v>3</v>
       </c>
+      <c r="BG181">
+        <v>4</v>
+      </c>
+      <c r="BH181">
+        <v>3</v>
+      </c>
+      <c r="BI181">
+        <v>2</v>
+      </c>
     </row>
-    <row r="182" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="182" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -20813,8 +21840,11 @@
       <c r="BE182">
         <v>6</v>
       </c>
+      <c r="BG182">
+        <v>6</v>
+      </c>
     </row>
-    <row r="183" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="183" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -20947,8 +21977,17 @@
       <c r="BF183">
         <v>3</v>
       </c>
+      <c r="BG183">
+        <v>4</v>
+      </c>
+      <c r="BH183">
+        <v>3</v>
+      </c>
+      <c r="BI183">
+        <v>2</v>
+      </c>
     </row>
-    <row r="184" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="184" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -21030,8 +22069,11 @@
       <c r="BE184">
         <v>6</v>
       </c>
+      <c r="BG184">
+        <v>6</v>
+      </c>
     </row>
-    <row r="185" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="185" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -21137,8 +22179,17 @@
       <c r="BF185">
         <v>3</v>
       </c>
+      <c r="BG185">
+        <v>2</v>
+      </c>
+      <c r="BH185">
+        <v>0</v>
+      </c>
+      <c r="BI185">
+        <v>0</v>
+      </c>
     </row>
-    <row r="186" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="186" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -21250,8 +22301,14 @@
       <c r="BF186">
         <v>1</v>
       </c>
+      <c r="BG186">
+        <v>6</v>
+      </c>
+      <c r="BH186">
+        <v>1</v>
+      </c>
     </row>
-    <row r="187" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="187" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -21330,8 +22387,14 @@
       <c r="BE187">
         <v>7</v>
       </c>
+      <c r="BG187">
+        <v>7</v>
+      </c>
+      <c r="BI187">
+        <v>1</v>
+      </c>
     </row>
-    <row r="188" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="188" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B188" t="s">
         <v>4</v>
       </c>
@@ -21446,8 +22509,14 @@
       <c r="BF188">
         <v>4</v>
       </c>
+      <c r="BG188">
+        <v>6</v>
+      </c>
+      <c r="BH188">
+        <v>4</v>
+      </c>
     </row>
-    <row r="189" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="189" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -21586,8 +22655,14 @@
       <c r="BF189">
         <v>2</v>
       </c>
+      <c r="BG189">
+        <v>2</v>
+      </c>
+      <c r="BH189">
+        <v>2</v>
+      </c>
     </row>
-    <row r="190" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="190" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -21717,8 +22792,14 @@
       <c r="BF190">
         <v>2</v>
       </c>
+      <c r="BG190">
+        <v>3</v>
+      </c>
+      <c r="BH190">
+        <v>2</v>
+      </c>
     </row>
-    <row r="191" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="191" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -21848,8 +22929,17 @@
       <c r="BF191">
         <v>4</v>
       </c>
+      <c r="BG191">
+        <v>1</v>
+      </c>
+      <c r="BH191">
+        <v>4</v>
+      </c>
+      <c r="BI191">
+        <v>0</v>
+      </c>
     </row>
-    <row r="192" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="192" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -21964,8 +23054,14 @@
       <c r="BF192">
         <v>3</v>
       </c>
+      <c r="BG192">
+        <v>0</v>
+      </c>
+      <c r="BH192">
+        <v>3</v>
+      </c>
     </row>
-    <row r="193" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="193" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -22101,8 +23197,14 @@
       <c r="BF193">
         <v>3</v>
       </c>
+      <c r="BG193">
+        <v>3</v>
+      </c>
+      <c r="BH193">
+        <v>4</v>
+      </c>
     </row>
-    <row r="194" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="194" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B194" t="s">
         <v>4</v>
       </c>
@@ -22214,8 +23316,14 @@
       <c r="BF194">
         <v>1</v>
       </c>
+      <c r="BG194">
+        <v>4</v>
+      </c>
+      <c r="BH194">
+        <v>1</v>
+      </c>
     </row>
-    <row r="195" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="195" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -22351,8 +23459,14 @@
       <c r="BF195">
         <v>2</v>
       </c>
+      <c r="BG195">
+        <v>2</v>
+      </c>
+      <c r="BH195">
+        <v>2</v>
+      </c>
     </row>
-    <row r="196" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="196" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -22494,8 +23608,17 @@
       <c r="BF196">
         <v>6</v>
       </c>
+      <c r="BG196">
+        <v>2</v>
+      </c>
+      <c r="BH196">
+        <v>6</v>
+      </c>
+      <c r="BI196">
+        <v>1</v>
+      </c>
     </row>
-    <row r="197" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="197" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -22610,8 +23733,14 @@
       <c r="BF197">
         <v>3</v>
       </c>
+      <c r="BG197">
+        <v>2</v>
+      </c>
+      <c r="BH197">
+        <v>3</v>
+      </c>
     </row>
-    <row r="198" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="198" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -22699,8 +23828,14 @@
       <c r="BF198">
         <v>1</v>
       </c>
+      <c r="BG198">
+        <v>4</v>
+      </c>
+      <c r="BH198">
+        <v>1</v>
+      </c>
     </row>
-    <row r="199" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="199" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -22821,8 +23956,14 @@
       <c r="BF199">
         <v>1</v>
       </c>
+      <c r="BG199">
+        <v>5</v>
+      </c>
+      <c r="BI199">
+        <v>1</v>
+      </c>
     </row>
-    <row r="200" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="200" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B200" t="s">
         <v>4</v>
       </c>
@@ -22922,8 +24063,14 @@
       <c r="BF200">
         <v>1</v>
       </c>
+      <c r="BG200">
+        <v>6</v>
+      </c>
+      <c r="BH200">
+        <v>1</v>
+      </c>
     </row>
-    <row r="201" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="201" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -23050,8 +24197,17 @@
       <c r="BF201">
         <v>3</v>
       </c>
+      <c r="BG201">
+        <v>2</v>
+      </c>
+      <c r="BH201">
+        <v>3</v>
+      </c>
+      <c r="BI201">
+        <v>1</v>
+      </c>
     </row>
-    <row r="202" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="202" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -23187,8 +24343,14 @@
       <c r="BF202">
         <v>1</v>
       </c>
+      <c r="BG202">
+        <v>0</v>
+      </c>
+      <c r="BH202">
+        <v>1</v>
+      </c>
     </row>
-    <row r="203" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="203" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -23309,8 +24471,17 @@
       <c r="BF203">
         <v>2</v>
       </c>
+      <c r="BG203">
+        <v>2</v>
+      </c>
+      <c r="BH203">
+        <v>2</v>
+      </c>
+      <c r="BI203">
+        <v>1</v>
+      </c>
     </row>
-    <row r="204" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="204" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -23392,8 +24563,11 @@
       <c r="BE204">
         <v>5</v>
       </c>
+      <c r="BG204">
+        <v>5</v>
+      </c>
     </row>
-    <row r="205" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="205" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -23532,8 +24706,14 @@
       <c r="BF205">
         <v>1</v>
       </c>
+      <c r="BG205">
+        <v>9</v>
+      </c>
+      <c r="BH205">
+        <v>1</v>
+      </c>
     </row>
-    <row r="206" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="206" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B206" t="s">
         <v>4</v>
       </c>
@@ -23615,8 +24795,11 @@
       <c r="BE206">
         <v>6</v>
       </c>
+      <c r="BG206">
+        <v>6</v>
+      </c>
     </row>
-    <row r="207" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="207" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -23713,8 +24896,14 @@
       <c r="BF207">
         <v>1</v>
       </c>
+      <c r="BG207">
+        <v>3</v>
+      </c>
+      <c r="BH207">
+        <v>1</v>
+      </c>
     </row>
-    <row r="208" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="208" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -23844,8 +25033,14 @@
       <c r="BF208">
         <v>2</v>
       </c>
+      <c r="BG208">
+        <v>1</v>
+      </c>
+      <c r="BH208">
+        <v>2</v>
+      </c>
     </row>
-    <row r="209" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="209" spans="2:60" hidden="1" x14ac:dyDescent="0.2">
       <c r="B209" t="s">
         <v>3</v>
       </c>
@@ -23957,8 +25152,14 @@
       <c r="BF209">
         <v>2</v>
       </c>
+      <c r="BG209">
+        <v>3</v>
+      </c>
+      <c r="BH209">
+        <v>2</v>
+      </c>
     </row>
-    <row r="210" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="210" spans="2:60" hidden="1" x14ac:dyDescent="0.2">
       <c r="B210" t="s">
         <v>1</v>
       </c>
@@ -24094,8 +25295,14 @@
       <c r="BF210">
         <v>1</v>
       </c>
+      <c r="BG210">
+        <v>4</v>
+      </c>
+      <c r="BH210">
+        <v>1</v>
+      </c>
     </row>
-    <row r="211" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="211" spans="2:60" hidden="1" x14ac:dyDescent="0.2">
       <c r="B211" t="s">
         <v>4</v>
       </c>
@@ -24207,8 +25414,14 @@
       <c r="BF211">
         <v>2</v>
       </c>
+      <c r="BG211">
+        <v>3</v>
+      </c>
+      <c r="BH211">
+        <v>2</v>
+      </c>
     </row>
-    <row r="212" spans="2:58" x14ac:dyDescent="0.2">
+    <row r="212" spans="2:60" x14ac:dyDescent="0.2">
       <c r="B212" t="s">
         <v>4</v>
       </c>
@@ -24314,7 +25527,14 @@
       <c r="BF212">
         <v>1</v>
       </c>
+      <c r="BG212">
+        <v>4</v>
+      </c>
+      <c r="BH212">
+        <v>1</v>
+      </c>
     </row>
+    <row r="213" spans="2:60" hidden="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated analysis code to check death progress
</commit_message>
<xml_diff>
--- a/data/germination_data.xlsx
+++ b/data/germination_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nolanmeier/git/morasoilinoculation/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F4E325E-252E-AD41-BC46-3992FEE872DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910ABE2E-CC7C-C546-B14C-AE769A131FE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4420" yWindow="680" windowWidth="24980" windowHeight="17260" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="94">
   <si>
     <t>seed_species</t>
   </si>
@@ -164,9 +164,6 @@
   </si>
   <si>
     <t>doy296: mold on soil; doy303: no obvious signs of mold on soil; doy328: previously dead germinant is still quite green, so marking as alive this week</t>
-  </si>
-  <si>
-    <t>doy296: mold on soil; doy303: no obvious signs of mold on soil; doy310: germinant not dead but unhealthy; doy328: dead germinant appears to still be alive, very green</t>
   </si>
   <si>
     <t>doy328: could not find dead germinant, but assumed its there since all 5 look healthy</t>
@@ -338,6 +335,12 @@
   <si>
     <t>doy63: previous measurements invalid, 5 alive, 2 dead, one hald dead</t>
   </si>
+  <si>
+    <t>doy296: mold on soil; doy 358: green moss?;doy63: previous measurements invalid, 8 alive 1 dead</t>
+  </si>
+  <si>
+    <t>doy296: mold on soil; doy303: no obvious signs of mold on soil; doy310: germinant not dead but unhealthy; doy328: dead germinant appears to still be alive, very green; doy63:previous measurements invalid, 9 alive 1 half dead</t>
+  </si>
 </sst>
 </file>
 
@@ -365,7 +368,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -375,6 +378,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC0E6F5"/>
+        <bgColor rgb="FFC0E6F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFC0E6F5"/>
       </patternFill>
     </fill>
@@ -402,10 +417,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -425,23 +443,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:BI213" totalsRowShown="0">
-  <autoFilter ref="B2:BI213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="THPL"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="1">
-      <filters>
-        <filter val="PSME"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="2">
-      <filters>
-        <filter val="25"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B2:BI213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
   <tableColumns count="60">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
@@ -825,7 +827,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:BI213"/>
+  <dimension ref="B2:BI212"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -910,112 +912,112 @@
         <v>40</v>
       </c>
       <c r="AA2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB2" t="s">
         <v>44</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AC2" t="s">
         <v>45</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AD2" t="s">
         <v>46</v>
       </c>
-      <c r="AD2" t="s">
-        <v>47</v>
-      </c>
       <c r="AE2" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF2" t="s">
         <v>49</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AG2" t="s">
         <v>50</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AH2" t="s">
         <v>51</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AI2" t="s">
         <v>52</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="AJ2" t="s">
         <v>53</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AK2" t="s">
         <v>54</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AL2" t="s">
         <v>55</v>
       </c>
-      <c r="AL2" t="s">
+      <c r="AM2" t="s">
+        <v>57</v>
+      </c>
+      <c r="AN2" t="s">
         <v>56</v>
       </c>
-      <c r="AM2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>57</v>
-      </c>
       <c r="AO2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP2" t="s">
         <v>69</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="AQ2" t="s">
         <v>70</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AR2" t="s">
         <v>71</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="AS2" t="s">
         <v>72</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AT2" t="s">
         <v>73</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="AU2" t="s">
         <v>74</v>
       </c>
-      <c r="AU2" t="s">
+      <c r="AV2" t="s">
         <v>75</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="AW2" t="s">
         <v>76</v>
       </c>
-      <c r="AW2" t="s">
+      <c r="AX2" t="s">
         <v>77</v>
       </c>
-      <c r="AX2" t="s">
+      <c r="AY2" t="s">
         <v>78</v>
       </c>
-      <c r="AY2" t="s">
+      <c r="AZ2" t="s">
         <v>79</v>
       </c>
-      <c r="AZ2" t="s">
+      <c r="BA2" t="s">
         <v>80</v>
       </c>
-      <c r="BA2" t="s">
+      <c r="BB2" t="s">
         <v>81</v>
       </c>
-      <c r="BB2" t="s">
+      <c r="BC2" t="s">
         <v>82</v>
       </c>
-      <c r="BC2" t="s">
+      <c r="BD2" t="s">
         <v>83</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BE2" t="s">
         <v>84</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BF2" t="s">
         <v>85</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BG2" t="s">
         <v>86</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BH2" t="s">
         <v>87</v>
       </c>
-      <c r="BH2" t="s">
+      <c r="BI2" t="s">
         <v>88</v>
       </c>
-      <c r="BI2" t="s">
-        <v>89</v>
-      </c>
     </row>
-    <row r="3" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1161,7 +1163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1175,7 +1177,7 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -1250,7 +1252,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1396,7 +1398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1485,7 +1487,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -1598,7 +1600,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -1738,7 +1740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -1884,7 +1886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -1976,7 +1978,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -2116,7 +2118,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -2265,7 +2267,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -2387,7 +2389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -2497,7 +2499,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -2512,7 +2514,7 @@
         <v>2</v>
       </c>
       <c r="F15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M15">
         <v>2</v>
@@ -2623,7 +2625,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -2734,7 +2736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -2869,7 +2871,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -2953,7 +2955,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -2968,7 +2970,7 @@
         <v>2</v>
       </c>
       <c r="F19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Q19">
         <v>4</v>
@@ -3091,7 +3093,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -3202,7 +3204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -3318,7 +3320,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -3408,7 +3410,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -3534,7 +3536,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -3549,7 +3551,7 @@
         <v>2</v>
       </c>
       <c r="F24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M24">
         <v>1</v>
@@ -3651,7 +3653,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -3738,7 +3740,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -3903,13 +3905,13 @@
         <v>6</v>
       </c>
       <c r="BH26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BI26">
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -3924,7 +3926,7 @@
         <v>3</v>
       </c>
       <c r="F27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M27">
         <v>4</v>
@@ -4008,7 +4010,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -4158,127 +4160,127 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B29" t="s">
-        <v>3</v>
-      </c>
-      <c r="C29" t="s">
-        <v>1</v>
-      </c>
-      <c r="D29">
+    <row r="29" spans="2:61" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B29" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D29" s="3">
         <v>10</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="5">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="F29" t="s">
-        <v>90</v>
-      </c>
-      <c r="M29">
-        <v>1</v>
-      </c>
-      <c r="O29">
-        <v>2</v>
-      </c>
-      <c r="Q29">
-        <v>3</v>
-      </c>
-      <c r="S29">
-        <v>4</v>
-      </c>
-      <c r="U29">
-        <v>4</v>
-      </c>
-      <c r="W29">
-        <v>4</v>
-      </c>
-      <c r="Y29">
-        <v>4</v>
-      </c>
-      <c r="AA29">
-        <v>4</v>
-      </c>
-      <c r="AC29">
-        <v>4</v>
-      </c>
-      <c r="AE29">
-        <v>4</v>
-      </c>
-      <c r="AG29">
-        <v>4</v>
-      </c>
-      <c r="AI29">
-        <v>4</v>
-      </c>
-      <c r="AK29">
-        <v>4</v>
-      </c>
-      <c r="AM29">
-        <v>4</v>
-      </c>
-      <c r="AO29">
-        <v>4</v>
-      </c>
-      <c r="AQ29">
-        <v>3</v>
-      </c>
-      <c r="AR29">
-        <v>1</v>
-      </c>
-      <c r="AS29">
-        <v>3</v>
-      </c>
-      <c r="AT29">
-        <v>1</v>
-      </c>
-      <c r="AU29">
-        <v>3</v>
-      </c>
-      <c r="AV29">
-        <v>1</v>
-      </c>
-      <c r="AW29">
-        <v>3</v>
-      </c>
-      <c r="AX29">
-        <v>1</v>
-      </c>
-      <c r="AY29">
-        <v>3</v>
-      </c>
-      <c r="AZ29">
-        <v>1</v>
-      </c>
-      <c r="BA29">
-        <v>3</v>
-      </c>
-      <c r="BB29">
-        <v>1</v>
-      </c>
-      <c r="BC29">
-        <v>3</v>
-      </c>
-      <c r="BD29">
-        <v>1</v>
-      </c>
-      <c r="BE29">
-        <v>3</v>
-      </c>
-      <c r="BF29">
-        <v>1</v>
-      </c>
-      <c r="BG29">
-        <v>4</v>
-      </c>
-      <c r="BH29">
+      <c r="F29" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="M29" s="3">
+        <v>1</v>
+      </c>
+      <c r="O29" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q29" s="3">
+        <v>3</v>
+      </c>
+      <c r="S29" s="3">
+        <v>4</v>
+      </c>
+      <c r="U29" s="3">
+        <v>4</v>
+      </c>
+      <c r="W29" s="3">
+        <v>4</v>
+      </c>
+      <c r="Y29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AA29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AC29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AE29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AG29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AI29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AK29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AM29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AO29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AQ29" s="3">
+        <v>3</v>
+      </c>
+      <c r="AR29" s="3">
+        <v>1</v>
+      </c>
+      <c r="AS29" s="3">
+        <v>3</v>
+      </c>
+      <c r="AT29" s="3">
+        <v>1</v>
+      </c>
+      <c r="AU29" s="3">
+        <v>3</v>
+      </c>
+      <c r="AV29" s="3">
+        <v>1</v>
+      </c>
+      <c r="AW29" s="3">
+        <v>3</v>
+      </c>
+      <c r="AX29" s="3">
+        <v>1</v>
+      </c>
+      <c r="AY29" s="3">
+        <v>3</v>
+      </c>
+      <c r="AZ29" s="3">
+        <v>1</v>
+      </c>
+      <c r="BA29" s="3">
+        <v>3</v>
+      </c>
+      <c r="BB29" s="3">
+        <v>1</v>
+      </c>
+      <c r="BC29" s="3">
+        <v>3</v>
+      </c>
+      <c r="BD29" s="3">
+        <v>1</v>
+      </c>
+      <c r="BE29" s="3">
+        <v>3</v>
+      </c>
+      <c r="BF29" s="3">
+        <v>1</v>
+      </c>
+      <c r="BG29" s="3">
+        <v>4</v>
+      </c>
+      <c r="BH29" s="3">
         <v>0</v>
       </c>
-      <c r="BI29">
+      <c r="BI29" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -4371,7 +4373,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -4515,7 +4517,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -4623,7 +4625,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -4725,7 +4727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -4842,7 +4844,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -4857,7 +4859,7 @@
         <v>3</v>
       </c>
       <c r="F35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O35">
         <v>2</v>
@@ -4965,7 +4967,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -4980,7 +4982,7 @@
         <v>3</v>
       </c>
       <c r="F36" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="O36">
         <v>1</v>
@@ -5072,11 +5074,14 @@
       <c r="BG36">
         <v>8</v>
       </c>
+      <c r="BH36">
+        <v>1</v>
+      </c>
       <c r="BI36">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -5163,7 +5168,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -5325,7 +5330,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -5469,7 +5474,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -5484,7 +5489,7 @@
         <v>4</v>
       </c>
       <c r="F40" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M40">
         <v>1</v>
@@ -5625,7 +5630,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -5748,7 +5753,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -5844,7 +5849,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -5985,7 +5990,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -6066,7 +6071,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -6237,7 +6242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -6330,7 +6335,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -6345,7 +6350,7 @@
         <v>4</v>
       </c>
       <c r="F47" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O47">
         <v>1</v>
@@ -6429,7 +6434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -6444,7 +6449,7 @@
         <v>4</v>
       </c>
       <c r="F48" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M48">
         <v>1</v>
@@ -6585,7 +6590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -6672,7 +6677,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -6840,7 +6845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -6855,7 +6860,7 @@
         <v>5</v>
       </c>
       <c r="F51" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M51">
         <v>0</v>
@@ -6984,7 +6989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -7071,7 +7076,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -7203,7 +7208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -7293,7 +7298,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -7419,7 +7424,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -7500,7 +7505,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -7587,7 +7592,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -7680,7 +7685,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -7764,7 +7769,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="60" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -7890,7 +7895,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -7980,7 +7985,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -7995,7 +8000,7 @@
         <v>5</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K62">
         <v>2</v>
@@ -8136,7 +8141,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="63" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -8151,7 +8156,7 @@
         <v>6</v>
       </c>
       <c r="F63" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M63">
         <v>1</v>
@@ -8274,7 +8279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -8382,7 +8387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -8493,7 +8498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -8580,7 +8585,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -8727,7 +8732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -8808,7 +8813,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="69" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -8895,7 +8900,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="70" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -8991,7 +8996,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="71" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -9006,7 +9011,7 @@
         <v>6</v>
       </c>
       <c r="F71" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O71">
         <v>4</v>
@@ -9117,7 +9122,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -9132,7 +9137,7 @@
         <v>6</v>
       </c>
       <c r="F72" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O72">
         <v>2</v>
@@ -9252,7 +9257,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -9339,7 +9344,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="74" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -9435,7 +9440,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -9450,7 +9455,7 @@
         <v>7</v>
       </c>
       <c r="F75" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M75">
         <v>1</v>
@@ -9555,7 +9560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -9570,7 +9575,7 @@
         <v>7</v>
       </c>
       <c r="F76" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M76">
         <v>1</v>
@@ -9708,7 +9713,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -9813,7 +9818,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -9903,7 +9908,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="79" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -10050,7 +10055,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="80" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -10167,7 +10172,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -10296,7 +10301,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -10443,7 +10448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -10458,7 +10463,7 @@
         <v>7</v>
       </c>
       <c r="F83" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O83">
         <v>2</v>
@@ -10590,7 +10595,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="84" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -10605,7 +10610,7 @@
         <v>7</v>
       </c>
       <c r="F84" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O84">
         <v>2</v>
@@ -10737,7 +10742,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="85" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -10752,7 +10757,7 @@
         <v>7</v>
       </c>
       <c r="F85" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M85">
         <v>3</v>
@@ -10881,7 +10886,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="86" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -11007,7 +11012,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -11022,7 +11027,7 @@
         <v>8</v>
       </c>
       <c r="F87" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M87">
         <v>2</v>
@@ -11157,7 +11162,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="88" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -11172,7 +11177,7 @@
         <v>8</v>
       </c>
       <c r="F88" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M88">
         <v>0</v>
@@ -11292,121 +11297,121 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B89" t="s">
-        <v>3</v>
-      </c>
-      <c r="C89" t="s">
-        <v>1</v>
-      </c>
-      <c r="D89">
+    <row r="89" spans="2:61" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B89" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D89" s="3">
         <v>10</v>
       </c>
-      <c r="E89" s="2">
+      <c r="E89" s="5">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="F89" t="s">
-        <v>91</v>
-      </c>
-      <c r="K89">
-        <v>1</v>
-      </c>
-      <c r="M89">
-        <v>4</v>
-      </c>
-      <c r="O89">
-        <v>4</v>
-      </c>
-      <c r="Q89">
-        <v>5</v>
-      </c>
-      <c r="S89">
-        <v>5</v>
-      </c>
-      <c r="U89">
-        <v>5</v>
-      </c>
-      <c r="W89">
-        <v>5</v>
-      </c>
-      <c r="Y89">
-        <v>5</v>
-      </c>
-      <c r="AA89">
-        <v>5</v>
-      </c>
-      <c r="AC89">
-        <v>5</v>
-      </c>
-      <c r="AE89">
-        <v>5</v>
-      </c>
-      <c r="AG89">
-        <v>5</v>
-      </c>
-      <c r="AI89">
-        <v>5</v>
-      </c>
-      <c r="AK89">
-        <v>5</v>
-      </c>
-      <c r="AM89">
-        <v>5</v>
-      </c>
-      <c r="AO89">
-        <v>5</v>
-      </c>
-      <c r="AQ89">
-        <v>5</v>
-      </c>
-      <c r="AS89">
-        <v>4</v>
-      </c>
-      <c r="AT89">
-        <v>1</v>
-      </c>
-      <c r="AU89">
-        <v>4</v>
-      </c>
-      <c r="AV89">
-        <v>1</v>
-      </c>
-      <c r="AW89">
-        <v>3</v>
-      </c>
-      <c r="AX89">
-        <v>2</v>
-      </c>
-      <c r="AY89">
-        <v>3</v>
-      </c>
-      <c r="AZ89">
-        <v>2</v>
-      </c>
-      <c r="BA89">
-        <v>3</v>
-      </c>
-      <c r="BB89">
-        <v>2</v>
-      </c>
-      <c r="BC89">
-        <v>3</v>
-      </c>
-      <c r="BD89">
-        <v>2</v>
-      </c>
-      <c r="BE89">
-        <v>3</v>
-      </c>
-      <c r="BF89">
-        <v>2</v>
-      </c>
-      <c r="BG89">
+      <c r="F89" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="K89" s="3">
+        <v>1</v>
+      </c>
+      <c r="M89" s="3">
+        <v>4</v>
+      </c>
+      <c r="O89" s="3">
+        <v>4</v>
+      </c>
+      <c r="Q89" s="3">
+        <v>5</v>
+      </c>
+      <c r="S89" s="3">
+        <v>5</v>
+      </c>
+      <c r="U89" s="3">
+        <v>5</v>
+      </c>
+      <c r="W89" s="3">
+        <v>5</v>
+      </c>
+      <c r="Y89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AA89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AC89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AE89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AG89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AI89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AK89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AM89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AO89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AQ89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AS89" s="3">
+        <v>4</v>
+      </c>
+      <c r="AT89" s="3">
+        <v>1</v>
+      </c>
+      <c r="AU89" s="3">
+        <v>4</v>
+      </c>
+      <c r="AV89" s="3">
+        <v>1</v>
+      </c>
+      <c r="AW89" s="3">
+        <v>3</v>
+      </c>
+      <c r="AX89" s="3">
+        <v>2</v>
+      </c>
+      <c r="AY89" s="3">
+        <v>3</v>
+      </c>
+      <c r="AZ89" s="3">
+        <v>2</v>
+      </c>
+      <c r="BA89" s="3">
+        <v>3</v>
+      </c>
+      <c r="BB89" s="3">
+        <v>2</v>
+      </c>
+      <c r="BC89" s="3">
+        <v>3</v>
+      </c>
+      <c r="BD89" s="3">
+        <v>2</v>
+      </c>
+      <c r="BE89" s="3">
+        <v>3</v>
+      </c>
+      <c r="BF89" s="3">
+        <v>2</v>
+      </c>
+      <c r="BG89" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="90" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -11496,7 +11501,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="91" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -11643,133 +11648,136 @@
         <v>2</v>
       </c>
     </row>
-    <row r="92" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B92" t="s">
-        <v>1</v>
-      </c>
-      <c r="C92" t="s">
-        <v>3</v>
-      </c>
-      <c r="D92">
+    <row r="92" spans="2:61" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B92" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D92" s="3">
         <v>0</v>
       </c>
-      <c r="E92" s="1">
+      <c r="E92" s="4">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="F92" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q92">
+      <c r="F92" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q92" s="3">
         <v>0</v>
       </c>
-      <c r="S92">
-        <v>1</v>
-      </c>
-      <c r="U92">
-        <v>2</v>
-      </c>
-      <c r="W92">
-        <v>4</v>
-      </c>
-      <c r="Y92">
-        <v>4</v>
-      </c>
-      <c r="AA92">
-        <v>4</v>
-      </c>
-      <c r="AC92">
-        <v>5</v>
-      </c>
-      <c r="AE92">
-        <v>6</v>
-      </c>
-      <c r="AG92">
-        <v>5</v>
-      </c>
-      <c r="AH92">
-        <v>1</v>
-      </c>
-      <c r="AI92">
-        <v>5</v>
-      </c>
-      <c r="AJ92">
-        <v>2</v>
-      </c>
-      <c r="AK92">
-        <v>5</v>
-      </c>
-      <c r="AL92">
-        <v>2</v>
-      </c>
-      <c r="AM92">
-        <v>5</v>
-      </c>
-      <c r="AN92">
-        <v>2</v>
-      </c>
-      <c r="AO92">
-        <v>5</v>
-      </c>
-      <c r="AP92">
-        <v>2</v>
-      </c>
-      <c r="AQ92">
-        <v>5</v>
-      </c>
-      <c r="AR92">
-        <v>2</v>
-      </c>
-      <c r="AS92">
-        <v>5</v>
-      </c>
-      <c r="AT92">
-        <v>2</v>
-      </c>
-      <c r="AU92">
-        <v>5</v>
-      </c>
-      <c r="AV92">
-        <v>2</v>
-      </c>
-      <c r="AW92">
-        <v>5</v>
-      </c>
-      <c r="AX92">
-        <v>2</v>
-      </c>
-      <c r="AY92">
-        <v>5</v>
-      </c>
-      <c r="AZ92">
-        <v>2</v>
-      </c>
-      <c r="BA92">
-        <v>5</v>
-      </c>
-      <c r="BB92">
-        <v>2</v>
-      </c>
-      <c r="BC92">
-        <v>4</v>
-      </c>
-      <c r="BD92">
-        <v>3</v>
-      </c>
-      <c r="BE92">
-        <v>4</v>
-      </c>
-      <c r="BF92">
-        <v>3</v>
-      </c>
-      <c r="BG92">
-        <v>5</v>
-      </c>
-      <c r="BH92">
-        <v>2</v>
+      <c r="S92" s="3">
+        <v>1</v>
+      </c>
+      <c r="U92" s="3">
+        <v>2</v>
+      </c>
+      <c r="W92" s="3">
+        <v>4</v>
+      </c>
+      <c r="Y92" s="3">
+        <v>4</v>
+      </c>
+      <c r="AA92" s="3">
+        <v>4</v>
+      </c>
+      <c r="AC92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AE92" s="3">
+        <v>6</v>
+      </c>
+      <c r="AG92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AH92" s="3">
+        <v>1</v>
+      </c>
+      <c r="AI92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AJ92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AK92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AL92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AM92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AN92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AO92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AP92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AQ92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AR92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AS92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AT92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AU92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AV92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AW92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AX92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AY92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AZ92" s="3">
+        <v>2</v>
+      </c>
+      <c r="BA92" s="3">
+        <v>5</v>
+      </c>
+      <c r="BB92" s="3">
+        <v>2</v>
+      </c>
+      <c r="BC92" s="3">
+        <v>4</v>
+      </c>
+      <c r="BD92" s="3">
+        <v>3</v>
+      </c>
+      <c r="BE92" s="3">
+        <v>4</v>
+      </c>
+      <c r="BF92" s="3">
+        <v>3</v>
+      </c>
+      <c r="BG92" s="3">
+        <v>5</v>
+      </c>
+      <c r="BH92" s="3">
+        <v>2</v>
+      </c>
+      <c r="BI92" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="93" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -11868,7 +11876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -11961,7 +11969,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="95" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -11976,7 +11984,7 @@
         <v>8</v>
       </c>
       <c r="F95" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O95">
         <v>2</v>
@@ -12066,7 +12074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -12081,7 +12089,7 @@
         <v>8</v>
       </c>
       <c r="F96" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O96">
         <v>1</v>
@@ -12195,7 +12203,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="97" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -12285,7 +12293,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="98" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -12414,7 +12422,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="99" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -12498,7 +12506,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="100" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -12585,7 +12593,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="101" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -12600,7 +12608,7 @@
         <v>9</v>
       </c>
       <c r="F101" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M101">
         <v>1</v>
@@ -12702,7 +12710,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="102" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -12792,7 +12800,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="103" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -12807,7 +12815,7 @@
         <v>9</v>
       </c>
       <c r="F103" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Q103">
         <v>1</v>
@@ -12930,7 +12938,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="104" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -13044,7 +13052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -13167,7 +13175,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -13302,7 +13310,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="107" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -13437,7 +13445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -13539,7 +13547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -13665,7 +13673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -13680,7 +13688,7 @@
         <v>9</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>42</v>
+        <v>93</v>
       </c>
       <c r="K110">
         <v>4</v>
@@ -13794,7 +13802,7 @@
         <v>1</v>
       </c>
       <c r="BG110">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BH110">
         <v>0</v>
@@ -13803,7 +13811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -13911,7 +13919,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="112" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -14040,7 +14048,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="113" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -14184,7 +14192,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="114" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -14274,7 +14282,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="115" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -14289,7 +14297,7 @@
         <v>10</v>
       </c>
       <c r="F115" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="O115">
         <v>2</v>
@@ -14421,7 +14429,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="116" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -14535,7 +14543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -14661,7 +14669,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -14755,7 +14763,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -14839,7 +14847,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="120" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -14926,7 +14934,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="121" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -14941,7 +14949,7 @@
         <v>10</v>
       </c>
       <c r="F121" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M121">
         <v>3</v>
@@ -15016,7 +15024,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="122" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -15109,7 +15117,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="123" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -15235,7 +15243,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="124" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -15388,7 +15396,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="125" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -15403,7 +15411,7 @@
         <v>11</v>
       </c>
       <c r="F125" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="M125">
         <v>2</v>
@@ -15541,7 +15549,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="126" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -15673,7 +15681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -15802,7 +15810,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="128" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -15883,7 +15891,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="129" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -16015,7 +16023,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -16108,7 +16116,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="131" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -16123,7 +16131,7 @@
         <v>11</v>
       </c>
       <c r="F131" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Q131">
         <v>2</v>
@@ -16231,7 +16239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -16315,7 +16323,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="133" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -16414,7 +16422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -16510,7 +16518,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -16612,7 +16620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -16723,7 +16731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -16840,7 +16848,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="138" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -16975,7 +16983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -17092,7 +17100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -17173,7 +17181,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="141" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -17329,7 +17337,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="142" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -17482,7 +17490,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="143" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -17581,7 +17589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -17665,7 +17673,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="145" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -17755,7 +17763,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="146" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -17893,7 +17901,7 @@
         <v>2</v>
       </c>
       <c r="BG146">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BH146">
         <v>1</v>
@@ -17902,7 +17910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -17917,7 +17925,7 @@
         <v>13</v>
       </c>
       <c r="F147" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O147">
         <v>0</v>
@@ -18040,7 +18048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -18127,7 +18135,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="149" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -18256,7 +18264,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="150" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -18406,7 +18414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -18421,7 +18429,7 @@
         <v>13</v>
       </c>
       <c r="F151" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Q151">
         <v>1</v>
@@ -18508,7 +18516,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="152" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -18589,7 +18597,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="153" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -18703,7 +18711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -18718,7 +18726,7 @@
         <v>13</v>
       </c>
       <c r="F154" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K154">
         <v>0</v>
@@ -18865,7 +18873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -18991,7 +18999,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="156" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -19078,7 +19086,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="157" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -19093,7 +19101,7 @@
         <v>13</v>
       </c>
       <c r="F157" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M157">
         <v>3</v>
@@ -19168,7 +19176,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="158" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -19264,7 +19272,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="159" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -19393,7 +19401,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -19480,7 +19488,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="161" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -19633,7 +19641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -19723,7 +19731,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="163" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -19846,7 +19854,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -19927,7 +19935,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="165" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -20050,7 +20058,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="166" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -20182,7 +20190,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="167" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -20293,7 +20301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -20425,7 +20433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -20440,7 +20448,7 @@
         <v>14</v>
       </c>
       <c r="F169" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M169">
         <v>2</v>
@@ -20515,7 +20523,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="170" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -20605,7 +20613,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="171" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -20620,7 +20628,7 @@
         <v>15</v>
       </c>
       <c r="F171" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O171">
         <v>2</v>
@@ -20743,7 +20751,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="172" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -20830,7 +20838,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="173" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -20917,7 +20925,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="174" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -21007,7 +21015,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="175" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -21130,7 +21138,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="176" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -21211,7 +21219,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="177" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -21298,7 +21306,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="178" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -21313,7 +21321,7 @@
         <v>15</v>
       </c>
       <c r="F178" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K178">
         <v>1</v>
@@ -21391,7 +21399,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="179" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -21517,7 +21525,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="180" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -21637,7 +21645,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="181" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -21754,7 +21762,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="182" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -21844,7 +21852,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="183" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -21858,7 +21866,7 @@
         <v>1</v>
       </c>
       <c r="F183" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="O183">
         <v>0</v>
@@ -21987,7 +21995,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="184" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -22073,7 +22081,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="185" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -22183,13 +22191,13 @@
         <v>2</v>
       </c>
       <c r="BH185">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BI185">
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -22308,7 +22316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -22516,7 +22524,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="189" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -22530,7 +22538,7 @@
         <v>2</v>
       </c>
       <c r="F189" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O189">
         <v>0</v>
@@ -22662,7 +22670,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="190" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -22676,7 +22684,7 @@
         <v>2</v>
       </c>
       <c r="F190" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M190">
         <v>0</v>
@@ -22799,7 +22807,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="191" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -22813,7 +22821,7 @@
         <v>2</v>
       </c>
       <c r="F191" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K191">
         <v>1</v>
@@ -22939,7 +22947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -23061,7 +23069,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="193" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -23323,7 +23331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -23337,7 +23345,7 @@
         <v>3</v>
       </c>
       <c r="F195" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O195">
         <v>0</v>
@@ -23466,7 +23474,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="196" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -23480,7 +23488,7 @@
         <v>3</v>
       </c>
       <c r="F196" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K196">
         <v>1</v>
@@ -23618,7 +23626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -23740,7 +23748,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="198" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -23835,7 +23843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -23957,7 +23965,7 @@
         <v>1</v>
       </c>
       <c r="BG199">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BI199">
         <v>1</v>
@@ -24070,7 +24078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="201" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -24084,7 +24092,7 @@
         <v>4</v>
       </c>
       <c r="F201" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O201">
         <v>0</v>
@@ -24207,7 +24215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="202" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -24221,7 +24229,7 @@
         <v>4</v>
       </c>
       <c r="F202" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M202">
         <v>0</v>
@@ -24350,7 +24358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="203" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -24481,7 +24489,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -24567,7 +24575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="205" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -24799,7 +24807,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="207" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -24813,7 +24821,7 @@
         <v>5</v>
       </c>
       <c r="F207" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O207">
         <v>1</v>
@@ -24903,7 +24911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -25040,7 +25048,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="209" spans="2:60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="2:60" x14ac:dyDescent="0.2">
       <c r="B209" t="s">
         <v>3</v>
       </c>
@@ -25054,7 +25062,7 @@
         <v>5</v>
       </c>
       <c r="F209" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M209">
         <v>1</v>
@@ -25159,7 +25167,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="210" spans="2:60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="2:60" x14ac:dyDescent="0.2">
       <c r="B210" t="s">
         <v>1</v>
       </c>
@@ -25302,7 +25310,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="2:60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="2:60" x14ac:dyDescent="0.2">
       <c r="B211" t="s">
         <v>4</v>
       </c>
@@ -25534,7 +25542,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="213" spans="2:60" hidden="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data collection on DOY82
</commit_message>
<xml_diff>
--- a/data/germination_data.xlsx
+++ b/data/germination_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nolanmeier/git/morasoilinoculation/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\morasoilinoculation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35B518B6-F784-6E46-A671-AEAAF0E5F513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53C97945-385D-4472-87F9-657DD375223C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="680" windowWidth="24980" windowHeight="17140" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="109">
   <si>
     <t>seed_species</t>
   </si>
@@ -377,6 +377,18 @@
   <si>
     <t>doy84: previous measurements incorrect, 8 alive 2 dead</t>
   </si>
+  <si>
+    <t>92_alive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>92_dead</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>92_halfdead</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -386,20 +398,20 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Aptos Narrow"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -478,9 +490,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:BR213" totalsRowShown="0">
-  <autoFilter ref="B2:BR213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
-  <tableColumns count="69">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:BU213" totalsRowShown="0">
+  <autoFilter ref="B2:BU213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="THPL"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <filters>
+        <filter val="PSME"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="2">
+      <filters>
+        <filter val="10"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <tableColumns count="72">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
     <tableColumn id="3" xr3:uid="{B695F4B4-8561-9D48-9FF3-12A40CB2B7C7}" name="inoculated_%"/>
@@ -550,6 +578,9 @@
     <tableColumn id="67" xr3:uid="{02155F60-F988-E943-8188-ACB55B731A13}" name="84_alive"/>
     <tableColumn id="68" xr3:uid="{7EA6F4B1-CC4F-C14C-9A5F-BB2A24D1017C}" name="84_dead"/>
     <tableColumn id="69" xr3:uid="{E539BB2A-3A6F-0C41-ADC0-ACAC3BBD5EEA}" name="84_halfdead"/>
+    <tableColumn id="70" xr3:uid="{F8D28AA1-8516-4EF5-912B-6EAEB30196F4}" name="92_alive"/>
+    <tableColumn id="71" xr3:uid="{0913FB35-4E69-4D28-B94F-63FF36CE0B23}" name="92_dead"/>
+    <tableColumn id="72" xr3:uid="{5075C4B1-5989-4DD0-8B58-233633A09E9B}" name="92_halfdead"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -872,15 +903,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:BR212"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="B2:BU213"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" customWidth="1"/>
-    <col min="4" max="4" width="17.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.15234375" customWidth="1"/>
+    <col min="4" max="4" width="17.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -1088,8 +1119,17 @@
       <c r="BR2" t="s">
         <v>104</v>
       </c>
+      <c r="BS2" t="s">
+        <v>106</v>
+      </c>
+      <c r="BT2" t="s">
+        <v>107</v>
+      </c>
+      <c r="BU2" t="s">
+        <v>108</v>
+      </c>
     </row>
-    <row r="3" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1252,8 +1292,14 @@
       <c r="BQ3">
         <v>1</v>
       </c>
+      <c r="BS3">
+        <v>3</v>
+      </c>
+      <c r="BT3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1350,8 +1396,11 @@
       <c r="BP4">
         <v>9</v>
       </c>
+      <c r="BS4">
+        <v>9</v>
+      </c>
     </row>
-    <row r="5" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1514,8 +1563,14 @@
       <c r="BQ5">
         <v>2</v>
       </c>
+      <c r="BS5">
+        <v>5</v>
+      </c>
+      <c r="BT5">
+        <v>2</v>
+      </c>
     </row>
-    <row r="6" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1612,8 +1667,11 @@
       <c r="BP6">
         <v>9</v>
       </c>
+      <c r="BS6">
+        <v>9</v>
+      </c>
     </row>
-    <row r="7" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -1743,8 +1801,14 @@
       <c r="BQ7">
         <v>4</v>
       </c>
+      <c r="BS7">
+        <v>2</v>
+      </c>
+      <c r="BT7">
+        <v>4</v>
+      </c>
     </row>
-    <row r="8" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -1901,8 +1965,14 @@
       <c r="BQ8">
         <v>1</v>
       </c>
+      <c r="BS8">
+        <v>6</v>
+      </c>
+      <c r="BT8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2065,8 +2135,14 @@
       <c r="BQ9">
         <v>1</v>
       </c>
+      <c r="BS9">
+        <v>6</v>
+      </c>
+      <c r="BT9">
+        <v>1</v>
+      </c>
     </row>
-    <row r="10" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -2166,8 +2242,11 @@
       <c r="BP10">
         <v>8</v>
       </c>
+      <c r="BS10">
+        <v>8</v>
+      </c>
     </row>
-    <row r="11" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -2324,8 +2403,14 @@
       <c r="BQ11">
         <v>2</v>
       </c>
+      <c r="BS11">
+        <v>6</v>
+      </c>
+      <c r="BT11">
+        <v>2</v>
+      </c>
     </row>
-    <row r="12" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -2491,8 +2576,14 @@
       <c r="BQ12">
         <v>4</v>
       </c>
+      <c r="BS12">
+        <v>5</v>
+      </c>
+      <c r="BT12">
+        <v>4</v>
+      </c>
     </row>
-    <row r="13" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -2640,8 +2731,17 @@
       <c r="BR13">
         <v>1</v>
       </c>
+      <c r="BS13">
+        <v>5</v>
+      </c>
+      <c r="BT13">
+        <v>1</v>
+      </c>
+      <c r="BU13">
+        <v>1</v>
+      </c>
     </row>
-    <row r="14" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -2759,8 +2859,11 @@
       <c r="BP14">
         <v>9</v>
       </c>
+      <c r="BS14">
+        <v>9</v>
+      </c>
     </row>
-    <row r="15" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -2903,8 +3006,14 @@
       <c r="BQ15">
         <v>4</v>
       </c>
+      <c r="BS15">
+        <v>4</v>
+      </c>
+      <c r="BT15">
+        <v>4</v>
+      </c>
     </row>
-    <row r="16" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -3032,8 +3141,14 @@
       <c r="BQ16">
         <v>1</v>
       </c>
+      <c r="BS16">
+        <v>8</v>
+      </c>
+      <c r="BT16">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -3185,8 +3300,14 @@
       <c r="BQ17">
         <v>2</v>
       </c>
+      <c r="BS17">
+        <v>6</v>
+      </c>
+      <c r="BT17">
+        <v>2</v>
+      </c>
     </row>
-    <row r="18" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -3278,8 +3399,11 @@
       <c r="BP18">
         <v>10</v>
       </c>
+      <c r="BS18">
+        <v>10</v>
+      </c>
     </row>
-    <row r="19" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -3443,8 +3567,17 @@
       <c r="BR19">
         <v>1</v>
       </c>
+      <c r="BS19">
+        <v>2</v>
+      </c>
+      <c r="BT19">
+        <v>4</v>
+      </c>
+      <c r="BU19">
+        <v>1</v>
+      </c>
     </row>
-    <row r="20" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -3572,8 +3705,14 @@
       <c r="BQ20">
         <v>1</v>
       </c>
+      <c r="BS20">
+        <v>13</v>
+      </c>
+      <c r="BT20">
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -3706,8 +3845,14 @@
       <c r="BQ21">
         <v>1</v>
       </c>
+      <c r="BS21">
+        <v>5</v>
+      </c>
+      <c r="BT21">
+        <v>1</v>
+      </c>
     </row>
-    <row r="22" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -3805,8 +3950,11 @@
       <c r="BP22">
         <v>8</v>
       </c>
+      <c r="BS22">
+        <v>8</v>
+      </c>
     </row>
-    <row r="23" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -3958,8 +4106,17 @@
       <c r="BR23">
         <v>1</v>
       </c>
+      <c r="BS23">
+        <v>8</v>
+      </c>
+      <c r="BT23">
+        <v>1</v>
+      </c>
+      <c r="BU23">
+        <v>1</v>
+      </c>
     </row>
-    <row r="24" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -4093,8 +4250,14 @@
       <c r="BQ24">
         <v>4</v>
       </c>
+      <c r="BS24">
+        <v>8</v>
+      </c>
+      <c r="BT24">
+        <v>4</v>
+      </c>
     </row>
-    <row r="25" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -4189,8 +4352,11 @@
       <c r="BP25">
         <v>8</v>
       </c>
+      <c r="BS25">
+        <v>8</v>
+      </c>
     </row>
-    <row r="26" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -4387,8 +4553,17 @@
       <c r="BR26">
         <v>2</v>
       </c>
+      <c r="BS26">
+        <v>6</v>
+      </c>
+      <c r="BT26">
+        <v>3</v>
+      </c>
+      <c r="BU26">
+        <v>2</v>
+      </c>
     </row>
-    <row r="27" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -4513,8 +4688,17 @@
       <c r="BR27">
         <v>2</v>
       </c>
+      <c r="BS27">
+        <v>3</v>
+      </c>
+      <c r="BT27">
+        <v>2</v>
+      </c>
+      <c r="BU27">
+        <v>1</v>
+      </c>
     </row>
-    <row r="28" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -4690,8 +4874,17 @@
       <c r="BR28">
         <v>1</v>
       </c>
+      <c r="BS28">
+        <v>7</v>
+      </c>
+      <c r="BT28">
+        <v>2</v>
+      </c>
+      <c r="BU28">
+        <v>1</v>
+      </c>
     </row>
-    <row r="29" spans="2:70" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:73" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
         <v>3</v>
       </c>
@@ -4834,8 +5027,14 @@
       <c r="BQ29" s="3">
         <v>1</v>
       </c>
+      <c r="BS29" s="3">
+        <v>3</v>
+      </c>
+      <c r="BT29" s="3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="30" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -4936,8 +5135,11 @@
       <c r="BP30">
         <v>8</v>
       </c>
+      <c r="BS30">
+        <v>8</v>
+      </c>
     </row>
-    <row r="31" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -5098,8 +5300,14 @@
       <c r="BQ31">
         <v>3</v>
       </c>
+      <c r="BS31">
+        <v>2</v>
+      </c>
+      <c r="BT31">
+        <v>3</v>
+      </c>
     </row>
-    <row r="32" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -5224,8 +5432,14 @@
       <c r="BQ32">
         <v>1</v>
       </c>
+      <c r="BS32">
+        <v>9</v>
+      </c>
+      <c r="BT32">
+        <v>1</v>
+      </c>
     </row>
-    <row r="33" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -5344,8 +5558,14 @@
       <c r="BQ33">
         <v>1</v>
       </c>
+      <c r="BS33">
+        <v>8</v>
+      </c>
+      <c r="BT33">
+        <v>1</v>
+      </c>
     </row>
-    <row r="34" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -5470,8 +5690,11 @@
       <c r="BP34">
         <v>6</v>
       </c>
+      <c r="BS34">
+        <v>6</v>
+      </c>
     </row>
-    <row r="35" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -5611,8 +5834,14 @@
       <c r="BQ35">
         <v>2</v>
       </c>
+      <c r="BS35">
+        <v>6</v>
+      </c>
+      <c r="BT35">
+        <v>2</v>
+      </c>
     </row>
-    <row r="36" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -5752,8 +5981,14 @@
       <c r="BR36">
         <v>1</v>
       </c>
+      <c r="BS36">
+        <v>8</v>
+      </c>
+      <c r="BT36">
+        <v>2</v>
+      </c>
     </row>
-    <row r="37" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -5848,8 +6083,11 @@
       <c r="BP37">
         <v>9</v>
       </c>
+      <c r="BS37">
+        <v>9</v>
+      </c>
     </row>
-    <row r="38" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -6028,8 +6266,14 @@
       <c r="BQ38">
         <v>3</v>
       </c>
+      <c r="BS38">
+        <v>5</v>
+      </c>
+      <c r="BT38">
+        <v>3</v>
+      </c>
     </row>
-    <row r="39" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -6190,8 +6434,14 @@
       <c r="BQ39">
         <v>4</v>
       </c>
+      <c r="BS39">
+        <v>2</v>
+      </c>
+      <c r="BT39">
+        <v>4</v>
+      </c>
     </row>
-    <row r="40" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -6364,8 +6614,14 @@
       <c r="BQ40">
         <v>6</v>
       </c>
+      <c r="BS40">
+        <v>4</v>
+      </c>
+      <c r="BT40">
+        <v>6</v>
+      </c>
     </row>
-    <row r="41" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -6505,8 +6761,14 @@
       <c r="BQ41">
         <v>2</v>
       </c>
+      <c r="BS41">
+        <v>4</v>
+      </c>
+      <c r="BT41">
+        <v>2</v>
+      </c>
     </row>
-    <row r="42" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -6610,8 +6872,11 @@
       <c r="BP42">
         <v>7</v>
       </c>
+      <c r="BS42">
+        <v>7</v>
+      </c>
     </row>
-    <row r="43" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -6769,8 +7034,14 @@
       <c r="BQ43">
         <v>6</v>
       </c>
+      <c r="BS43">
+        <v>3</v>
+      </c>
+      <c r="BT43">
+        <v>6</v>
+      </c>
     </row>
-    <row r="44" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -6859,8 +7130,11 @@
       <c r="BP44">
         <v>6</v>
       </c>
+      <c r="BS44">
+        <v>6</v>
+      </c>
     </row>
-    <row r="45" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -7057,8 +7331,17 @@
       <c r="BR45">
         <v>1</v>
       </c>
+      <c r="BS45">
+        <v>5</v>
+      </c>
+      <c r="BT45">
+        <v>3</v>
+      </c>
+      <c r="BU45">
+        <v>1</v>
+      </c>
     </row>
-    <row r="46" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -7159,8 +7442,11 @@
       <c r="BP46">
         <v>6</v>
       </c>
+      <c r="BS46">
+        <v>6</v>
+      </c>
     </row>
-    <row r="47" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -7276,8 +7562,14 @@
       <c r="BQ47">
         <v>1</v>
       </c>
+      <c r="BS47">
+        <v>8</v>
+      </c>
+      <c r="BT47">
+        <v>1</v>
+      </c>
     </row>
-    <row r="48" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -7459,8 +7751,14 @@
       <c r="BR48">
         <v>1</v>
       </c>
+      <c r="BS48">
+        <v>5</v>
+      </c>
+      <c r="BT48">
+        <v>6</v>
+      </c>
     </row>
-    <row r="49" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -7555,8 +7853,11 @@
       <c r="BP49">
         <v>8</v>
       </c>
+      <c r="BS49">
+        <v>8</v>
+      </c>
     </row>
-    <row r="50" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -7741,8 +8042,14 @@
       <c r="BQ50">
         <v>1</v>
       </c>
+      <c r="BS50">
+        <v>7</v>
+      </c>
+      <c r="BT50">
+        <v>1</v>
+      </c>
     </row>
-    <row r="51" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -7912,8 +8219,14 @@
       <c r="BR51">
         <v>1</v>
       </c>
+      <c r="BS51">
+        <v>4</v>
+      </c>
+      <c r="BT51">
+        <v>2</v>
+      </c>
     </row>
-    <row r="52" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -8008,8 +8321,11 @@
       <c r="BP52">
         <v>6</v>
       </c>
+      <c r="BS52">
+        <v>6</v>
+      </c>
     </row>
-    <row r="53" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -8158,8 +8474,14 @@
       <c r="BQ53">
         <v>1</v>
       </c>
+      <c r="BS53">
+        <v>3</v>
+      </c>
+      <c r="BT53">
+        <v>1</v>
+      </c>
     </row>
-    <row r="54" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -8257,8 +8579,11 @@
       <c r="BP54">
         <v>5</v>
       </c>
+      <c r="BS54">
+        <v>5</v>
+      </c>
     </row>
-    <row r="55" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -8401,8 +8726,14 @@
       <c r="BQ55">
         <v>4</v>
       </c>
+      <c r="BS55">
+        <v>2</v>
+      </c>
+      <c r="BT55">
+        <v>4</v>
+      </c>
     </row>
-    <row r="56" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -8491,8 +8822,11 @@
       <c r="BP56">
         <v>10</v>
       </c>
+      <c r="BS56">
+        <v>10</v>
+      </c>
     </row>
-    <row r="57" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -8590,8 +8924,14 @@
       <c r="BR57">
         <v>1</v>
       </c>
+      <c r="BS57">
+        <v>6</v>
+      </c>
+      <c r="BT57">
+        <v>1</v>
+      </c>
     </row>
-    <row r="58" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -8692,8 +9032,11 @@
       <c r="BP58">
         <v>6</v>
       </c>
+      <c r="BS58">
+        <v>6</v>
+      </c>
     </row>
-    <row r="59" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -8785,8 +9128,11 @@
       <c r="BP59">
         <v>7</v>
       </c>
+      <c r="BS59">
+        <v>7</v>
+      </c>
     </row>
-    <row r="60" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -8929,8 +9275,14 @@
       <c r="BQ60">
         <v>2</v>
       </c>
+      <c r="BS60">
+        <v>7</v>
+      </c>
+      <c r="BT60">
+        <v>2</v>
+      </c>
     </row>
-    <row r="61" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -9031,8 +9383,11 @@
       <c r="BP61">
         <v>7</v>
       </c>
+      <c r="BS61">
+        <v>7</v>
+      </c>
     </row>
-    <row r="62" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -9205,8 +9560,14 @@
       <c r="BQ62">
         <v>2</v>
       </c>
+      <c r="BS62">
+        <v>3</v>
+      </c>
+      <c r="BT62">
+        <v>2</v>
+      </c>
     </row>
-    <row r="63" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -9370,8 +9731,17 @@
       <c r="BR63">
         <v>2</v>
       </c>
+      <c r="BS63">
+        <v>4</v>
+      </c>
+      <c r="BT63">
+        <v>3</v>
+      </c>
+      <c r="BU63">
+        <v>2</v>
+      </c>
     </row>
-    <row r="64" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -9505,8 +9875,17 @@
       <c r="BR64">
         <v>1</v>
       </c>
+      <c r="BS64">
+        <v>7</v>
+      </c>
+      <c r="BT64">
+        <v>2</v>
+      </c>
+      <c r="BU64">
+        <v>1</v>
+      </c>
     </row>
-    <row r="65" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -9643,8 +10022,14 @@
       <c r="BR65">
         <v>1</v>
       </c>
+      <c r="BS65">
+        <v>5</v>
+      </c>
+      <c r="BT65">
+        <v>1</v>
+      </c>
     </row>
-    <row r="66" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -9739,8 +10124,11 @@
       <c r="BP66">
         <v>5</v>
       </c>
+      <c r="BS66">
+        <v>5</v>
+      </c>
     </row>
-    <row r="67" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -9907,8 +10295,14 @@
       <c r="BQ67">
         <v>8</v>
       </c>
+      <c r="BS67">
+        <v>2</v>
+      </c>
+      <c r="BT67">
+        <v>8</v>
+      </c>
     </row>
-    <row r="68" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -9997,8 +10391,11 @@
       <c r="BP68">
         <v>11</v>
       </c>
+      <c r="BS68">
+        <v>11</v>
+      </c>
     </row>
-    <row r="69" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -10093,8 +10490,11 @@
       <c r="BP69">
         <v>9</v>
       </c>
+      <c r="BS69">
+        <v>9</v>
+      </c>
     </row>
-    <row r="70" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -10198,8 +10598,11 @@
       <c r="BP70">
         <v>7</v>
       </c>
+      <c r="BS70">
+        <v>7</v>
+      </c>
     </row>
-    <row r="71" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -10351,8 +10754,17 @@
       <c r="BR71">
         <v>1</v>
       </c>
+      <c r="BS71">
+        <v>7</v>
+      </c>
+      <c r="BT71">
+        <v>3</v>
+      </c>
+      <c r="BU71">
+        <v>1</v>
+      </c>
     </row>
-    <row r="72" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -10504,8 +10916,14 @@
       <c r="BQ72">
         <v>1</v>
       </c>
+      <c r="BS72">
+        <v>6</v>
+      </c>
+      <c r="BT72">
+        <v>1</v>
+      </c>
     </row>
-    <row r="73" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -10600,8 +11018,11 @@
       <c r="BP73">
         <v>9</v>
       </c>
+      <c r="BS73">
+        <v>9</v>
+      </c>
     </row>
-    <row r="74" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -10705,8 +11126,11 @@
       <c r="BP74">
         <v>9</v>
       </c>
+      <c r="BS74">
+        <v>9</v>
+      </c>
     </row>
-    <row r="75" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="75" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -10846,8 +11270,17 @@
       <c r="BR75">
         <v>1</v>
       </c>
+      <c r="BS75">
+        <v>7</v>
+      </c>
+      <c r="BT75">
+        <v>1</v>
+      </c>
+      <c r="BU75">
+        <v>1</v>
+      </c>
     </row>
-    <row r="76" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="76" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -11017,8 +11450,14 @@
       <c r="BQ76">
         <v>1</v>
       </c>
+      <c r="BS76">
+        <v>7</v>
+      </c>
+      <c r="BT76">
+        <v>1</v>
+      </c>
     </row>
-    <row r="77" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -11152,8 +11591,17 @@
       <c r="BR77">
         <v>1</v>
       </c>
+      <c r="BS77">
+        <v>4</v>
+      </c>
+      <c r="BT77">
+        <v>2</v>
+      </c>
+      <c r="BU77">
+        <v>1</v>
+      </c>
     </row>
-    <row r="78" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -11251,8 +11699,11 @@
       <c r="BP78">
         <v>7</v>
       </c>
+      <c r="BS78">
+        <v>7</v>
+      </c>
     </row>
-    <row r="79" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="79" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -11416,8 +11867,14 @@
       <c r="BQ79">
         <v>7</v>
       </c>
+      <c r="BS79">
+        <v>2</v>
+      </c>
+      <c r="BT79">
+        <v>7</v>
+      </c>
     </row>
-    <row r="80" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="80" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -11551,8 +12008,14 @@
       <c r="BQ80">
         <v>1</v>
       </c>
+      <c r="BS80">
+        <v>9</v>
+      </c>
+      <c r="BT80">
+        <v>1</v>
+      </c>
     </row>
-    <row r="81" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -11698,8 +12161,14 @@
       <c r="BQ81">
         <v>2</v>
       </c>
+      <c r="BS81">
+        <v>5</v>
+      </c>
+      <c r="BT81">
+        <v>2</v>
+      </c>
     </row>
-    <row r="82" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -11872,8 +12341,17 @@
       <c r="BR82">
         <v>1</v>
       </c>
+      <c r="BS82">
+        <v>6</v>
+      </c>
+      <c r="BT82">
+        <v>3</v>
+      </c>
+      <c r="BU82">
+        <v>1</v>
+      </c>
     </row>
-    <row r="83" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -12037,8 +12515,14 @@
       <c r="BQ83">
         <v>4</v>
       </c>
+      <c r="BS83">
+        <v>5</v>
+      </c>
+      <c r="BT83">
+        <v>4</v>
+      </c>
     </row>
-    <row r="84" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -12202,8 +12686,14 @@
       <c r="BQ84">
         <v>2</v>
       </c>
+      <c r="BS84">
+        <v>7</v>
+      </c>
+      <c r="BT84">
+        <v>2</v>
+      </c>
     </row>
-    <row r="85" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -12364,8 +12854,14 @@
       <c r="BQ85">
         <v>2</v>
       </c>
+      <c r="BS85">
+        <v>4</v>
+      </c>
+      <c r="BT85">
+        <v>2</v>
+      </c>
     </row>
-    <row r="86" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -12508,8 +13004,14 @@
       <c r="BQ86">
         <v>1</v>
       </c>
+      <c r="BS86">
+        <v>8</v>
+      </c>
+      <c r="BT86">
+        <v>1</v>
+      </c>
     </row>
-    <row r="87" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -12676,8 +13178,14 @@
       <c r="BQ87">
         <v>2</v>
       </c>
+      <c r="BS87">
+        <v>5</v>
+      </c>
+      <c r="BT87">
+        <v>2</v>
+      </c>
     </row>
-    <row r="88" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -12829,8 +13337,14 @@
       <c r="BQ88">
         <v>3</v>
       </c>
+      <c r="BS88">
+        <v>6</v>
+      </c>
+      <c r="BT88">
+        <v>3</v>
+      </c>
     </row>
-    <row r="89" spans="2:70" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:73" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="B89" s="3" t="s">
         <v>3</v>
       </c>
@@ -12958,8 +13472,14 @@
       <c r="BQ89" s="3">
         <v>2</v>
       </c>
+      <c r="BS89" s="3">
+        <v>3</v>
+      </c>
+      <c r="BT89" s="3">
+        <v>2</v>
+      </c>
     </row>
-    <row r="90" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -13057,8 +13577,11 @@
       <c r="BP90">
         <v>7</v>
       </c>
+      <c r="BS90">
+        <v>7</v>
+      </c>
     </row>
-    <row r="91" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -13231,8 +13754,17 @@
       <c r="BR91">
         <v>2</v>
       </c>
+      <c r="BS91">
+        <v>4</v>
+      </c>
+      <c r="BT91">
+        <v>4</v>
+      </c>
+      <c r="BU91">
+        <v>2</v>
+      </c>
     </row>
-    <row r="92" spans="2:70" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="2:73" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="B92" s="3" t="s">
         <v>1</v>
       </c>
@@ -13387,8 +13919,17 @@
       <c r="BR92" s="3">
         <v>1</v>
       </c>
+      <c r="BS92" s="3">
+        <v>5</v>
+      </c>
+      <c r="BT92" s="3">
+        <v>2</v>
+      </c>
+      <c r="BU92" s="3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="93" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -13504,8 +14045,14 @@
       <c r="BQ93">
         <v>1</v>
       </c>
+      <c r="BS93">
+        <v>8</v>
+      </c>
+      <c r="BT93">
+        <v>1</v>
+      </c>
     </row>
-    <row r="94" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -13606,8 +14153,11 @@
       <c r="BP94">
         <v>7</v>
       </c>
+      <c r="BS94">
+        <v>7</v>
+      </c>
     </row>
-    <row r="95" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -13729,8 +14279,14 @@
       <c r="BQ95">
         <v>1</v>
       </c>
+      <c r="BS95">
+        <v>7</v>
+      </c>
+      <c r="BT95">
+        <v>1</v>
+      </c>
     </row>
-    <row r="96" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -13876,8 +14432,14 @@
       <c r="BQ96">
         <v>2</v>
       </c>
+      <c r="BS96">
+        <v>8</v>
+      </c>
+      <c r="BT96">
+        <v>2</v>
+      </c>
     </row>
-    <row r="97" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="97" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -13975,8 +14537,11 @@
       <c r="BP97">
         <v>8</v>
       </c>
+      <c r="BS97">
+        <v>8</v>
+      </c>
     </row>
-    <row r="98" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="98" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -14122,8 +14687,14 @@
       <c r="BQ98">
         <v>2</v>
       </c>
+      <c r="BS98">
+        <v>5</v>
+      </c>
+      <c r="BT98">
+        <v>2</v>
+      </c>
     </row>
-    <row r="99" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="99" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -14224,8 +14795,14 @@
       <c r="BR99">
         <v>1</v>
       </c>
+      <c r="BS99">
+        <v>2</v>
+      </c>
+      <c r="BT99">
+        <v>1</v>
+      </c>
     </row>
-    <row r="100" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="100" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -14320,8 +14897,11 @@
       <c r="BP100">
         <v>8</v>
       </c>
+      <c r="BS100">
+        <v>8</v>
+      </c>
     </row>
-    <row r="101" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="101" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -14455,8 +15035,14 @@
       <c r="BQ101">
         <v>4</v>
       </c>
+      <c r="BS101">
+        <v>1</v>
+      </c>
+      <c r="BT101">
+        <v>4</v>
+      </c>
     </row>
-    <row r="102" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="102" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -14554,8 +15140,11 @@
       <c r="BP102">
         <v>7</v>
       </c>
+      <c r="BS102">
+        <v>7</v>
+      </c>
     </row>
-    <row r="103" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="103" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -14710,8 +15299,14 @@
       <c r="BQ103">
         <v>4</v>
       </c>
+      <c r="BS103">
+        <v>2</v>
+      </c>
+      <c r="BT103">
+        <v>4</v>
+      </c>
     </row>
-    <row r="104" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="104" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -14851,8 +15446,17 @@
       <c r="BR104">
         <v>1</v>
       </c>
+      <c r="BS104">
+        <v>7</v>
+      </c>
+      <c r="BT104">
+        <v>2</v>
+      </c>
+      <c r="BU104">
+        <v>1</v>
+      </c>
     </row>
-    <row r="105" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="105" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -14992,8 +15596,14 @@
       <c r="BQ105">
         <v>3</v>
       </c>
+      <c r="BS105">
+        <v>2</v>
+      </c>
+      <c r="BT105">
+        <v>3</v>
+      </c>
     </row>
-    <row r="106" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="106" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -15136,8 +15746,11 @@
       <c r="BP106">
         <v>7</v>
       </c>
+      <c r="BS106">
+        <v>7</v>
+      </c>
     </row>
-    <row r="107" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="107" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -15289,8 +15902,14 @@
       <c r="BQ107">
         <v>1</v>
       </c>
+      <c r="BS107">
+        <v>4</v>
+      </c>
+      <c r="BT107">
+        <v>1</v>
+      </c>
     </row>
-    <row r="108" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="108" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -15418,8 +16037,17 @@
       <c r="BR108">
         <v>1</v>
       </c>
+      <c r="BS108">
+        <v>7</v>
+      </c>
+      <c r="BT108">
+        <v>1</v>
+      </c>
+      <c r="BU108">
+        <v>2</v>
+      </c>
     </row>
-    <row r="109" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="109" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -15571,8 +16199,17 @@
       <c r="BR109">
         <v>0</v>
       </c>
+      <c r="BS109">
+        <v>0</v>
+      </c>
+      <c r="BT109">
+        <v>8</v>
+      </c>
+      <c r="BU109">
+        <v>1</v>
+      </c>
     </row>
-    <row r="110" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="110" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -15730,8 +16367,14 @@
       <c r="BQ110">
         <v>2</v>
       </c>
+      <c r="BS110">
+        <v>7</v>
+      </c>
+      <c r="BT110">
+        <v>2</v>
+      </c>
     </row>
-    <row r="111" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="111" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -15865,8 +16508,17 @@
       <c r="BR111">
         <v>2</v>
       </c>
+      <c r="BS111">
+        <v>4</v>
+      </c>
+      <c r="BT111">
+        <v>2</v>
+      </c>
+      <c r="BU111">
+        <v>2</v>
+      </c>
     </row>
-    <row r="112" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="112" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -16012,8 +16664,14 @@
       <c r="BQ112">
         <v>2</v>
       </c>
+      <c r="BS112">
+        <v>6</v>
+      </c>
+      <c r="BT112">
+        <v>2</v>
+      </c>
     </row>
-    <row r="113" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="113" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -16174,8 +16832,14 @@
       <c r="BQ113">
         <v>2</v>
       </c>
+      <c r="BS113">
+        <v>4</v>
+      </c>
+      <c r="BT113">
+        <v>2</v>
+      </c>
     </row>
-    <row r="114" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="114" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -16273,8 +16937,11 @@
       <c r="BP114">
         <v>8</v>
       </c>
+      <c r="BS114">
+        <v>8</v>
+      </c>
     </row>
-    <row r="115" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="115" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -16438,8 +17105,14 @@
       <c r="BQ115">
         <v>3</v>
       </c>
+      <c r="BS115">
+        <v>1</v>
+      </c>
+      <c r="BT115">
+        <v>3</v>
+      </c>
     </row>
-    <row r="116" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="116" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -16579,8 +17252,17 @@
       <c r="BR116">
         <v>1</v>
       </c>
+      <c r="BS116">
+        <v>7</v>
+      </c>
+      <c r="BT116">
+        <v>2</v>
+      </c>
+      <c r="BU116">
+        <v>1</v>
+      </c>
     </row>
-    <row r="117" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="117" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -16732,8 +17414,17 @@
       <c r="BR117">
         <v>1</v>
       </c>
+      <c r="BS117">
+        <v>1</v>
+      </c>
+      <c r="BT117">
+        <v>3</v>
+      </c>
+      <c r="BU117">
+        <v>1</v>
+      </c>
     </row>
-    <row r="118" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="118" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -16835,8 +17526,11 @@
       <c r="BP118">
         <v>6</v>
       </c>
+      <c r="BS118">
+        <v>6</v>
+      </c>
     </row>
-    <row r="119" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="119" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -16928,8 +17622,14 @@
       <c r="BP119">
         <v>7</v>
       </c>
+      <c r="BS119">
+        <v>6</v>
+      </c>
+      <c r="BU119">
+        <v>1</v>
+      </c>
     </row>
-    <row r="120" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="120" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -17024,8 +17724,11 @@
       <c r="BP120">
         <v>10</v>
       </c>
+      <c r="BS120">
+        <v>10</v>
+      </c>
     </row>
-    <row r="121" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="121" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -17123,8 +17826,11 @@
       <c r="BP121">
         <v>8</v>
       </c>
+      <c r="BS121">
+        <v>8</v>
+      </c>
     </row>
-    <row r="122" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="122" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -17225,8 +17931,11 @@
       <c r="BP122">
         <v>5</v>
       </c>
+      <c r="BS122">
+        <v>6</v>
+      </c>
     </row>
-    <row r="123" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="123" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -17369,8 +18078,14 @@
       <c r="BQ123">
         <v>3</v>
       </c>
+      <c r="BS123">
+        <v>3</v>
+      </c>
+      <c r="BT123">
+        <v>3</v>
+      </c>
     </row>
-    <row r="124" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="124" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -17540,8 +18255,14 @@
       <c r="BQ124">
         <v>3</v>
       </c>
+      <c r="BS124">
+        <v>6</v>
+      </c>
+      <c r="BT124">
+        <v>3</v>
+      </c>
     </row>
-    <row r="125" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="125" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -17711,8 +18432,14 @@
       <c r="BQ125">
         <v>6</v>
       </c>
+      <c r="BS125">
+        <v>0</v>
+      </c>
+      <c r="BT125">
+        <v>6</v>
+      </c>
     </row>
-    <row r="126" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="126" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -17861,8 +18588,14 @@
       <c r="BQ126">
         <v>1</v>
       </c>
+      <c r="BS126">
+        <v>5</v>
+      </c>
+      <c r="BT126">
+        <v>1</v>
+      </c>
     </row>
-    <row r="127" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="127" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -18008,8 +18741,14 @@
       <c r="BQ127">
         <v>2</v>
       </c>
+      <c r="BS127">
+        <v>1</v>
+      </c>
+      <c r="BT127">
+        <v>2</v>
+      </c>
     </row>
-    <row r="128" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="128" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -18098,8 +18837,11 @@
       <c r="BP128">
         <v>7</v>
       </c>
+      <c r="BS128">
+        <v>7</v>
+      </c>
     </row>
-    <row r="129" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="129" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -18257,8 +18999,17 @@
       <c r="BR129">
         <v>1</v>
       </c>
+      <c r="BS129">
+        <v>2</v>
+      </c>
+      <c r="BT129">
+        <v>3</v>
+      </c>
+      <c r="BU129">
+        <v>1</v>
+      </c>
     </row>
-    <row r="130" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="130" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -18359,8 +19110,11 @@
       <c r="BP130">
         <v>9</v>
       </c>
+      <c r="BS130">
+        <v>9</v>
+      </c>
     </row>
-    <row r="131" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="131" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -18509,8 +19263,17 @@
       <c r="BR131">
         <v>1</v>
       </c>
+      <c r="BS131">
+        <v>7</v>
+      </c>
+      <c r="BT131">
+        <v>2</v>
+      </c>
+      <c r="BU131">
+        <v>1</v>
+      </c>
     </row>
-    <row r="132" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="132" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -18602,8 +19365,11 @@
       <c r="BP132">
         <v>6</v>
       </c>
+      <c r="BS132">
+        <v>6</v>
+      </c>
     </row>
-    <row r="133" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="133" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -18719,8 +19485,11 @@
       <c r="BQ133">
         <v>1</v>
       </c>
+      <c r="BS133">
+        <v>6</v>
+      </c>
     </row>
-    <row r="134" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="134" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -18833,8 +19602,14 @@
       <c r="BQ134">
         <v>1</v>
       </c>
+      <c r="BS134">
+        <v>9</v>
+      </c>
+      <c r="BT134">
+        <v>1</v>
+      </c>
     </row>
-    <row r="135" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="135" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -18962,8 +19737,17 @@
       <c r="BR135">
         <v>1</v>
       </c>
+      <c r="BS135">
+        <v>3</v>
+      </c>
+      <c r="BT135">
+        <v>4</v>
+      </c>
+      <c r="BU135">
+        <v>1</v>
+      </c>
     </row>
-    <row r="136" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="136" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -19091,8 +19875,14 @@
       <c r="BQ136">
         <v>1</v>
       </c>
+      <c r="BS136">
+        <v>6</v>
+      </c>
+      <c r="BT136">
+        <v>1</v>
+      </c>
     </row>
-    <row r="137" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="137" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -19226,8 +20016,14 @@
       <c r="BQ137">
         <v>2</v>
       </c>
+      <c r="BS137">
+        <v>3</v>
+      </c>
+      <c r="BT137">
+        <v>2</v>
+      </c>
     </row>
-    <row r="138" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="138" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -19379,8 +20175,14 @@
       <c r="BQ138">
         <v>1</v>
       </c>
+      <c r="BS138">
+        <v>7</v>
+      </c>
+      <c r="BT138">
+        <v>1</v>
+      </c>
     </row>
-    <row r="139" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="139" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -19514,8 +20316,14 @@
       <c r="BQ139">
         <v>1</v>
       </c>
+      <c r="BS139">
+        <v>5</v>
+      </c>
+      <c r="BT139">
+        <v>1</v>
+      </c>
     </row>
-    <row r="140" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="140" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -19604,8 +20412,11 @@
       <c r="BP140">
         <v>9</v>
       </c>
+      <c r="BS140">
+        <v>9</v>
+      </c>
     </row>
-    <row r="141" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="141" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -19778,8 +20589,14 @@
       <c r="BQ141">
         <v>4</v>
       </c>
+      <c r="BS141">
+        <v>4</v>
+      </c>
+      <c r="BT141">
+        <v>4</v>
+      </c>
     </row>
-    <row r="142" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="142" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -19949,8 +20766,14 @@
       <c r="BQ142">
         <v>2</v>
       </c>
+      <c r="BS142">
+        <v>6</v>
+      </c>
+      <c r="BT142">
+        <v>2</v>
+      </c>
     </row>
-    <row r="143" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="143" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -20075,8 +20898,14 @@
       <c r="BR143">
         <v>2</v>
       </c>
+      <c r="BS143">
+        <v>8</v>
+      </c>
+      <c r="BT143">
+        <v>3</v>
+      </c>
     </row>
-    <row r="144" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="144" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -20168,8 +20997,11 @@
       <c r="BP144">
         <v>7</v>
       </c>
+      <c r="BS144">
+        <v>7</v>
+      </c>
     </row>
-    <row r="145" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="145" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -20267,8 +21099,11 @@
       <c r="BP145">
         <v>8</v>
       </c>
+      <c r="BS145">
+        <v>8</v>
+      </c>
     </row>
-    <row r="146" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="146" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -20441,8 +21276,17 @@
       <c r="BR146">
         <v>1</v>
       </c>
+      <c r="BS146">
+        <v>8</v>
+      </c>
+      <c r="BT146">
+        <v>1</v>
+      </c>
+      <c r="BU146">
+        <v>1</v>
+      </c>
     </row>
-    <row r="147" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="147" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -20606,8 +21450,17 @@
       <c r="BR147">
         <v>1</v>
       </c>
+      <c r="BS147">
+        <v>2</v>
+      </c>
+      <c r="BT147">
+        <v>1</v>
+      </c>
+      <c r="BU147">
+        <v>1</v>
+      </c>
     </row>
-    <row r="148" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="148" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -20702,8 +21555,11 @@
       <c r="BP148">
         <v>9</v>
       </c>
+      <c r="BS148">
+        <v>9</v>
+      </c>
     </row>
-    <row r="149" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="149" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -20858,8 +21714,17 @@
       <c r="BR149">
         <v>1</v>
       </c>
+      <c r="BS149">
+        <v>2</v>
+      </c>
+      <c r="BT149">
+        <v>2</v>
+      </c>
+      <c r="BU149">
+        <v>1</v>
+      </c>
     </row>
-    <row r="150" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="150" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -21026,8 +21891,14 @@
       <c r="BQ150">
         <v>1</v>
       </c>
+      <c r="BS150">
+        <v>8</v>
+      </c>
+      <c r="BT150">
+        <v>1</v>
+      </c>
     </row>
-    <row r="151" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="151" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -21155,8 +22026,17 @@
       <c r="BR151">
         <v>3</v>
       </c>
+      <c r="BS151">
+        <v>4</v>
+      </c>
+      <c r="BT151">
+        <v>3</v>
+      </c>
+      <c r="BU151">
+        <v>3</v>
+      </c>
     </row>
-    <row r="152" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="152" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -21245,8 +22125,11 @@
       <c r="BP152">
         <v>9</v>
       </c>
+      <c r="BS152">
+        <v>9</v>
+      </c>
     </row>
-    <row r="153" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="153" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -21377,8 +22260,14 @@
       <c r="BQ153">
         <v>1</v>
       </c>
+      <c r="BS153">
+        <v>5</v>
+      </c>
+      <c r="BT153">
+        <v>1</v>
+      </c>
     </row>
-    <row r="154" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="154" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -21566,8 +22455,17 @@
       <c r="BR154">
         <v>1</v>
       </c>
+      <c r="BS154">
+        <v>5</v>
+      </c>
+      <c r="BT154">
+        <v>2</v>
+      </c>
+      <c r="BU154">
+        <v>1</v>
+      </c>
     </row>
-    <row r="155" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="155" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -21710,8 +22608,14 @@
       <c r="BQ155">
         <v>3</v>
       </c>
+      <c r="BS155">
+        <v>6</v>
+      </c>
+      <c r="BT155">
+        <v>3</v>
+      </c>
     </row>
-    <row r="156" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="156" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -21806,8 +22710,11 @@
       <c r="BP156">
         <v>6</v>
       </c>
+      <c r="BS156">
+        <v>6</v>
+      </c>
     </row>
-    <row r="157" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="157" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -21905,8 +22812,11 @@
       <c r="BP157">
         <v>6</v>
       </c>
+      <c r="BS157">
+        <v>6</v>
+      </c>
     </row>
-    <row r="158" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="158" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -22016,8 +22926,14 @@
       <c r="BR158">
         <v>1</v>
       </c>
+      <c r="BS158">
+        <v>7</v>
+      </c>
+      <c r="BU158">
+        <v>1</v>
+      </c>
     </row>
-    <row r="159" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="159" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -22172,8 +23088,17 @@
       <c r="BR159">
         <v>1</v>
       </c>
+      <c r="BS159">
+        <v>2</v>
+      </c>
+      <c r="BT159">
+        <v>2</v>
+      </c>
+      <c r="BU159">
+        <v>1</v>
+      </c>
     </row>
-    <row r="160" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="160" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -22268,8 +23193,11 @@
       <c r="BP160">
         <v>9</v>
       </c>
+      <c r="BS160">
+        <v>9</v>
+      </c>
     </row>
-    <row r="161" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="161" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -22448,8 +23376,17 @@
       <c r="BR161">
         <v>1</v>
       </c>
+      <c r="BS161">
+        <v>1</v>
+      </c>
+      <c r="BT161">
+        <v>4</v>
+      </c>
+      <c r="BU161">
+        <v>2</v>
+      </c>
     </row>
-    <row r="162" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="162" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -22547,8 +23484,11 @@
       <c r="BP162">
         <v>8</v>
       </c>
+      <c r="BS162">
+        <v>8</v>
+      </c>
     </row>
-    <row r="163" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="163" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -22688,8 +23628,14 @@
       <c r="BQ163">
         <v>6</v>
       </c>
+      <c r="BS163">
+        <v>2</v>
+      </c>
+      <c r="BT163">
+        <v>6</v>
+      </c>
     </row>
-    <row r="164" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="164" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -22778,8 +23724,11 @@
       <c r="BP164">
         <v>9</v>
       </c>
+      <c r="BS164">
+        <v>9</v>
+      </c>
     </row>
-    <row r="165" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="165" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -22919,8 +23868,14 @@
       <c r="BQ165">
         <v>2</v>
       </c>
+      <c r="BS165">
+        <v>4</v>
+      </c>
+      <c r="BT165">
+        <v>2</v>
+      </c>
     </row>
-    <row r="166" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="166" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -23060,8 +24015,11 @@
       <c r="BP166">
         <v>5</v>
       </c>
+      <c r="BS166">
+        <v>5</v>
+      </c>
     </row>
-    <row r="167" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="167" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -23189,8 +24147,14 @@
       <c r="BQ167">
         <v>1</v>
       </c>
+      <c r="BS167">
+        <v>7</v>
+      </c>
+      <c r="BT167">
+        <v>1</v>
+      </c>
     </row>
-    <row r="168" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="168" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -23348,8 +24312,14 @@
       <c r="BR168">
         <v>1</v>
       </c>
+      <c r="BS168">
+        <v>9</v>
+      </c>
+      <c r="BT168">
+        <v>2</v>
+      </c>
     </row>
-    <row r="169" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="169" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -23447,8 +24417,11 @@
       <c r="BP169">
         <v>6</v>
       </c>
+      <c r="BS169">
+        <v>6</v>
+      </c>
     </row>
-    <row r="170" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="170" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -23552,8 +24525,14 @@
       <c r="BQ170">
         <v>1</v>
       </c>
+      <c r="BS170">
+        <v>8</v>
+      </c>
+      <c r="BT170">
+        <v>1</v>
+      </c>
     </row>
-    <row r="171" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="171" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -23717,8 +24696,17 @@
       <c r="BR171">
         <v>2</v>
       </c>
+      <c r="BS171">
+        <v>5</v>
+      </c>
+      <c r="BT171">
+        <v>3</v>
+      </c>
+      <c r="BU171">
+        <v>2</v>
+      </c>
     </row>
-    <row r="172" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="172" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -23813,8 +24801,11 @@
       <c r="BP172">
         <v>8</v>
       </c>
+      <c r="BS172">
+        <v>8</v>
+      </c>
     </row>
-    <row r="173" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="173" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -23918,8 +24909,14 @@
       <c r="BR173">
         <v>1</v>
       </c>
+      <c r="BS173">
+        <v>5</v>
+      </c>
+      <c r="BU173">
+        <v>2</v>
+      </c>
     </row>
-    <row r="174" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="174" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -24017,8 +25014,11 @@
       <c r="BP174">
         <v>9</v>
       </c>
+      <c r="BS174">
+        <v>9</v>
+      </c>
     </row>
-    <row r="175" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="175" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -24158,8 +25158,14 @@
       <c r="BQ175">
         <v>2</v>
       </c>
+      <c r="BS175">
+        <v>7</v>
+      </c>
+      <c r="BT175">
+        <v>2</v>
+      </c>
     </row>
-    <row r="176" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="176" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -24248,8 +25254,11 @@
       <c r="BP176">
         <v>8</v>
       </c>
+      <c r="BS176">
+        <v>8</v>
+      </c>
     </row>
-    <row r="177" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="177" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -24344,8 +25353,11 @@
       <c r="BP177">
         <v>5</v>
       </c>
+      <c r="BS177">
+        <v>5</v>
+      </c>
     </row>
-    <row r="178" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="178" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -24446,8 +25458,11 @@
       <c r="BP178">
         <v>8</v>
       </c>
+      <c r="BS178">
+        <v>8</v>
+      </c>
     </row>
-    <row r="179" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="179" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -24590,8 +25605,14 @@
       <c r="BQ179">
         <v>4</v>
       </c>
+      <c r="BS179">
+        <v>6</v>
+      </c>
+      <c r="BT179">
+        <v>4</v>
+      </c>
     </row>
-    <row r="180" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="180" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -24728,8 +25749,14 @@
       <c r="BQ180">
         <v>2</v>
       </c>
+      <c r="BS180">
+        <v>7</v>
+      </c>
+      <c r="BT180">
+        <v>2</v>
+      </c>
     </row>
-    <row r="181" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="181" spans="2:73" x14ac:dyDescent="0.35">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -24872,8 +25899,17 @@
       <c r="BR181">
         <v>2</v>
       </c>
+      <c r="BS181">
+        <v>3</v>
+      </c>
+      <c r="BT181">
+        <v>4</v>
+      </c>
+      <c r="BU181">
+        <v>2</v>
+      </c>
     </row>
-    <row r="182" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="182" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -24971,8 +26007,11 @@
       <c r="BP182">
         <v>6</v>
       </c>
+      <c r="BS182">
+        <v>6</v>
+      </c>
     </row>
-    <row r="183" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="183" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -25141,8 +26180,17 @@
       <c r="BR183">
         <v>1</v>
       </c>
+      <c r="BS183">
+        <v>3</v>
+      </c>
+      <c r="BT183">
+        <v>4</v>
+      </c>
+      <c r="BU183">
+        <v>1</v>
+      </c>
     </row>
-    <row r="184" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="184" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -25236,8 +26284,14 @@
       <c r="BP184">
         <v>6</v>
       </c>
+      <c r="BS184">
+        <v>5</v>
+      </c>
+      <c r="BU184">
+        <v>1</v>
+      </c>
     </row>
-    <row r="185" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="185" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -25382,8 +26436,17 @@
       <c r="BR185">
         <v>2</v>
       </c>
+      <c r="BS185">
+        <v>2</v>
+      </c>
+      <c r="BT185">
+        <v>3</v>
+      </c>
+      <c r="BU185">
+        <v>2</v>
+      </c>
     </row>
-    <row r="186" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="186" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -25519,8 +26582,14 @@
       <c r="BQ186">
         <v>1</v>
       </c>
+      <c r="BS186">
+        <v>6</v>
+      </c>
+      <c r="BT186">
+        <v>1</v>
+      </c>
     </row>
-    <row r="187" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="187" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -25623,8 +26692,14 @@
       <c r="BR187">
         <v>1</v>
       </c>
+      <c r="BS187">
+        <v>7</v>
+      </c>
+      <c r="BT187">
+        <v>1</v>
+      </c>
     </row>
-    <row r="188" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="188" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B188" t="s">
         <v>4</v>
       </c>
@@ -25766,8 +26841,14 @@
       <c r="BQ188">
         <v>2</v>
       </c>
+      <c r="BS188">
+        <v>8</v>
+      </c>
+      <c r="BT188">
+        <v>2</v>
+      </c>
     </row>
-    <row r="189" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="189" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -25930,8 +27011,14 @@
       <c r="BQ189">
         <v>2</v>
       </c>
+      <c r="BS189">
+        <v>2</v>
+      </c>
+      <c r="BT189">
+        <v>2</v>
+      </c>
     </row>
-    <row r="190" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="190" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -26085,8 +27172,14 @@
       <c r="BQ190">
         <v>2</v>
       </c>
+      <c r="BS190">
+        <v>3</v>
+      </c>
+      <c r="BT190">
+        <v>2</v>
+      </c>
     </row>
-    <row r="191" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="191" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -26246,8 +27339,14 @@
       <c r="BQ191">
         <v>4</v>
       </c>
+      <c r="BS191">
+        <v>1</v>
+      </c>
+      <c r="BT191">
+        <v>4</v>
+      </c>
     </row>
-    <row r="192" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="192" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -26386,8 +27485,14 @@
       <c r="BQ192">
         <v>3</v>
       </c>
+      <c r="BS192">
+        <v>0</v>
+      </c>
+      <c r="BT192">
+        <v>3</v>
+      </c>
     </row>
-    <row r="193" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="193" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -26547,8 +27652,14 @@
       <c r="BQ193">
         <v>4</v>
       </c>
+      <c r="BS193">
+        <v>3</v>
+      </c>
+      <c r="BT193">
+        <v>4</v>
+      </c>
     </row>
-    <row r="194" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="194" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B194" t="s">
         <v>4</v>
       </c>
@@ -26684,8 +27795,14 @@
       <c r="BQ194">
         <v>1</v>
       </c>
+      <c r="BS194">
+        <v>6</v>
+      </c>
+      <c r="BT194">
+        <v>1</v>
+      </c>
     </row>
-    <row r="195" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="195" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -26845,8 +27962,14 @@
       <c r="BQ195">
         <v>2</v>
       </c>
+      <c r="BS195">
+        <v>2</v>
+      </c>
+      <c r="BT195">
+        <v>2</v>
+      </c>
     </row>
-    <row r="196" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="196" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -27024,8 +28147,17 @@
       <c r="BR196">
         <v>1</v>
       </c>
+      <c r="BS196">
+        <v>2</v>
+      </c>
+      <c r="BT196">
+        <v>6</v>
+      </c>
+      <c r="BU196">
+        <v>1</v>
+      </c>
     </row>
-    <row r="197" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="197" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -27164,8 +28296,14 @@
       <c r="BQ197">
         <v>3</v>
       </c>
+      <c r="BS197">
+        <v>2</v>
+      </c>
+      <c r="BT197">
+        <v>3</v>
+      </c>
     </row>
-    <row r="198" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="198" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -27277,8 +28415,14 @@
       <c r="BQ198">
         <v>1</v>
       </c>
+      <c r="BS198">
+        <v>4</v>
+      </c>
+      <c r="BT198">
+        <v>1</v>
+      </c>
     </row>
-    <row r="199" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="199" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -27423,8 +28567,14 @@
       <c r="BR199">
         <v>1</v>
       </c>
+      <c r="BS199">
+        <v>6</v>
+      </c>
+      <c r="BU199">
+        <v>1</v>
+      </c>
     </row>
-    <row r="200" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="200" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B200" t="s">
         <v>4</v>
       </c>
@@ -27548,8 +28698,14 @@
       <c r="BQ200">
         <v>1</v>
       </c>
+      <c r="BS200">
+        <v>6</v>
+      </c>
+      <c r="BT200">
+        <v>1</v>
+      </c>
     </row>
-    <row r="201" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="201" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -27712,8 +28868,17 @@
       <c r="BR201">
         <v>1</v>
       </c>
+      <c r="BS201">
+        <v>1</v>
+      </c>
+      <c r="BT201">
+        <v>4</v>
+      </c>
+      <c r="BU201">
+        <v>1</v>
+      </c>
     </row>
-    <row r="202" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="202" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -27873,8 +29038,14 @@
       <c r="BQ202">
         <v>1</v>
       </c>
+      <c r="BS202">
+        <v>0</v>
+      </c>
+      <c r="BT202">
+        <v>1</v>
+      </c>
     </row>
-    <row r="203" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="203" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -28022,8 +29193,14 @@
       <c r="BQ203">
         <v>1</v>
       </c>
+      <c r="BS203">
+        <v>2</v>
+      </c>
+      <c r="BT203">
+        <v>1</v>
+      </c>
     </row>
-    <row r="204" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="204" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -28117,8 +29294,11 @@
       <c r="BP204">
         <v>5</v>
       </c>
+      <c r="BS204">
+        <v>5</v>
+      </c>
     </row>
-    <row r="205" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="205" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -28281,8 +29461,14 @@
       <c r="BQ205">
         <v>1</v>
       </c>
+      <c r="BS205">
+        <v>9</v>
+      </c>
+      <c r="BT205">
+        <v>1</v>
+      </c>
     </row>
-    <row r="206" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="206" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B206" t="s">
         <v>4</v>
       </c>
@@ -28376,8 +29562,11 @@
       <c r="BP206">
         <v>6</v>
       </c>
+      <c r="BS206">
+        <v>6</v>
+      </c>
     </row>
-    <row r="207" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="207" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -28498,8 +29687,14 @@
       <c r="BQ207">
         <v>1</v>
       </c>
+      <c r="BS207">
+        <v>2</v>
+      </c>
+      <c r="BT207">
+        <v>2</v>
+      </c>
     </row>
-    <row r="208" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="208" spans="2:73" hidden="1" x14ac:dyDescent="0.35">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -28653,8 +29848,14 @@
       <c r="BQ208">
         <v>2</v>
       </c>
+      <c r="BS208">
+        <v>1</v>
+      </c>
+      <c r="BT208">
+        <v>2</v>
+      </c>
     </row>
-    <row r="209" spans="2:69" x14ac:dyDescent="0.2">
+    <row r="209" spans="2:72" hidden="1" x14ac:dyDescent="0.35">
       <c r="B209" t="s">
         <v>3</v>
       </c>
@@ -28790,8 +29991,14 @@
       <c r="BQ209">
         <v>2</v>
       </c>
+      <c r="BS209">
+        <v>3</v>
+      </c>
+      <c r="BT209">
+        <v>2</v>
+      </c>
     </row>
-    <row r="210" spans="2:69" x14ac:dyDescent="0.2">
+    <row r="210" spans="2:72" hidden="1" x14ac:dyDescent="0.35">
       <c r="B210" t="s">
         <v>1</v>
       </c>
@@ -28951,8 +30158,14 @@
       <c r="BQ210">
         <v>1</v>
       </c>
+      <c r="BS210">
+        <v>4</v>
+      </c>
+      <c r="BT210">
+        <v>1</v>
+      </c>
     </row>
-    <row r="211" spans="2:69" x14ac:dyDescent="0.2">
+    <row r="211" spans="2:72" hidden="1" x14ac:dyDescent="0.35">
       <c r="B211" t="s">
         <v>4</v>
       </c>
@@ -29088,8 +30301,14 @@
       <c r="BQ211">
         <v>2</v>
       </c>
+      <c r="BS211">
+        <v>3</v>
+      </c>
+      <c r="BT211">
+        <v>2</v>
+      </c>
     </row>
-    <row r="212" spans="2:69" x14ac:dyDescent="0.2">
+    <row r="212" spans="2:72" hidden="1" x14ac:dyDescent="0.35">
       <c r="B212" t="s">
         <v>4</v>
       </c>
@@ -29219,7 +30438,14 @@
       <c r="BQ212">
         <v>1</v>
       </c>
+      <c r="BS212">
+        <v>4</v>
+      </c>
+      <c r="BT212">
+        <v>1</v>
+      </c>
     </row>
+    <row r="213" spans="2:72" hidden="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
DOY112 germinants data collection
</commit_message>
<xml_diff>
--- a/data/germination_data.xlsx
+++ b/data/germination_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\morasoilinoculation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D501B9B7-1EAD-4417-B47C-82FCDBA39A7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D69D0C-830E-44DE-AACE-2DB79A438926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="119">
   <si>
     <t>seed_species</t>
   </si>
@@ -413,6 +413,22 @@
     <t>105_halfdead</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>112_alive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>112_dead</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>112_halfdead</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>doy112: half dead came back to life</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -514,9 +530,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CA213" totalsRowShown="0">
-  <autoFilter ref="B2:CA213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
-  <tableColumns count="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CD213" totalsRowShown="0">
+  <autoFilter ref="B2:CD213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
+  <tableColumns count="81">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
     <tableColumn id="3" xr3:uid="{B695F4B4-8561-9D48-9FF3-12A40CB2B7C7}" name="inoculated_%"/>
@@ -595,6 +611,9 @@
     <tableColumn id="76" xr3:uid="{88CD0C83-90C2-4ABA-9CE0-5E955D579206}" name="105_alive"/>
     <tableColumn id="77" xr3:uid="{66ABC843-90F8-46FD-B593-D992CCBE49A0}" name="105_dead"/>
     <tableColumn id="78" xr3:uid="{D4012DFC-E5DE-4C56-95C7-D5E056AA0472}" name="105_halfdead"/>
+    <tableColumn id="79" xr3:uid="{B9D9BBC8-AB51-4EEE-A4FA-A8D68D32C92F}" name="112_alive"/>
+    <tableColumn id="80" xr3:uid="{323A31B7-B3A1-4C31-A41D-DD0B6BCD8E98}" name="112_dead"/>
+    <tableColumn id="81" xr3:uid="{CF820F6A-BC57-443F-A0F0-72AC59A5982D}" name="112_halfdead"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -917,7 +936,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:CA212"/>
+  <dimension ref="B2:CD212"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -925,7 +944,7 @@
     <col min="4" max="4" width="17.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -1160,8 +1179,17 @@
       <c r="CA2" t="s">
         <v>114</v>
       </c>
+      <c r="CB2" t="s">
+        <v>115</v>
+      </c>
+      <c r="CC2" t="s">
+        <v>116</v>
+      </c>
+      <c r="CD2" t="s">
+        <v>117</v>
+      </c>
     </row>
-    <row r="3" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1345,8 +1373,14 @@
       <c r="CA3">
         <v>1</v>
       </c>
+      <c r="CB3">
+        <v>2</v>
+      </c>
+      <c r="CC3">
+        <v>2</v>
+      </c>
     </row>
-    <row r="4" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1452,8 +1486,11 @@
       <c r="BY4">
         <v>9</v>
       </c>
+      <c r="CB4">
+        <v>9</v>
+      </c>
     </row>
-    <row r="5" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1637,8 +1674,14 @@
       <c r="CA5">
         <v>4</v>
       </c>
+      <c r="CB5">
+        <v>0</v>
+      </c>
+      <c r="CC5">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1744,8 +1787,11 @@
       <c r="BY6">
         <v>9</v>
       </c>
+      <c r="CB6">
+        <v>9</v>
+      </c>
     </row>
-    <row r="7" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -1893,8 +1939,14 @@
       <c r="BZ7">
         <v>4</v>
       </c>
+      <c r="CB7">
+        <v>2</v>
+      </c>
+      <c r="CC7">
+        <v>4</v>
+      </c>
     </row>
-    <row r="8" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -2069,8 +2121,14 @@
       <c r="BZ8">
         <v>1</v>
       </c>
+      <c r="CB8">
+        <v>6</v>
+      </c>
+      <c r="CC8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2251,8 +2309,14 @@
       <c r="BZ9">
         <v>1</v>
       </c>
+      <c r="CB9">
+        <v>6</v>
+      </c>
+      <c r="CC9">
+        <v>1</v>
+      </c>
     </row>
-    <row r="10" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -2361,8 +2425,14 @@
       <c r="BY10">
         <v>8</v>
       </c>
+      <c r="CB10">
+        <v>7</v>
+      </c>
+      <c r="CD10">
+        <v>1</v>
+      </c>
     </row>
-    <row r="11" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -2537,8 +2607,14 @@
       <c r="BZ11">
         <v>2</v>
       </c>
+      <c r="CB11">
+        <v>6</v>
+      </c>
+      <c r="CC11">
+        <v>2</v>
+      </c>
     </row>
-    <row r="12" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -2722,8 +2798,14 @@
       <c r="BZ12">
         <v>4</v>
       </c>
+      <c r="CB12">
+        <v>4</v>
+      </c>
+      <c r="CC12">
+        <v>5</v>
+      </c>
     </row>
-    <row r="13" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -2895,8 +2977,14 @@
       <c r="BZ13">
         <v>3</v>
       </c>
+      <c r="CB13">
+        <v>4</v>
+      </c>
+      <c r="CC13">
+        <v>3</v>
+      </c>
     </row>
-    <row r="14" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -3029,8 +3117,14 @@
       <c r="BZ14">
         <v>1</v>
       </c>
+      <c r="CB14">
+        <v>8</v>
+      </c>
+      <c r="CC14">
+        <v>1</v>
+      </c>
     </row>
-    <row r="15" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -3191,8 +3285,14 @@
       <c r="BZ15">
         <v>4</v>
       </c>
+      <c r="CB15">
+        <v>4</v>
+      </c>
+      <c r="CC15">
+        <v>4</v>
+      </c>
     </row>
-    <row r="16" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -3338,8 +3438,14 @@
       <c r="BZ16">
         <v>1</v>
       </c>
+      <c r="CB16">
+        <v>8</v>
+      </c>
+      <c r="CC16">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -3509,8 +3615,11 @@
       <c r="BZ17">
         <v>2</v>
       </c>
+      <c r="CB17">
+        <v>8</v>
+      </c>
     </row>
-    <row r="18" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -3611,8 +3720,11 @@
       <c r="BY18">
         <v>10</v>
       </c>
+      <c r="CB18">
+        <v>10</v>
+      </c>
     </row>
-    <row r="19" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -3797,8 +3909,14 @@
       <c r="BZ19">
         <v>6</v>
       </c>
+      <c r="CB19">
+        <v>1</v>
+      </c>
+      <c r="CC19">
+        <v>6</v>
+      </c>
     </row>
-    <row r="20" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -3944,8 +4062,14 @@
       <c r="BZ20">
         <v>1</v>
       </c>
+      <c r="CB20">
+        <v>13</v>
+      </c>
+      <c r="CC20">
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -4096,8 +4220,14 @@
       <c r="BZ21">
         <v>1</v>
       </c>
+      <c r="CB21">
+        <v>5</v>
+      </c>
+      <c r="CC21">
+        <v>1</v>
+      </c>
     </row>
-    <row r="22" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -4204,8 +4334,11 @@
       <c r="BY22">
         <v>8</v>
       </c>
+      <c r="CB22">
+        <v>8</v>
+      </c>
     </row>
-    <row r="23" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -4378,8 +4511,14 @@
       <c r="BZ23">
         <v>2</v>
       </c>
+      <c r="CB23">
+        <v>8</v>
+      </c>
+      <c r="CC23">
+        <v>2</v>
+      </c>
     </row>
-    <row r="24" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -4531,8 +4670,14 @@
       <c r="BZ24">
         <v>4</v>
       </c>
+      <c r="CB24">
+        <v>8</v>
+      </c>
+      <c r="CC24">
+        <v>4</v>
+      </c>
     </row>
-    <row r="25" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -4636,8 +4781,11 @@
       <c r="BY25">
         <v>8</v>
       </c>
+      <c r="CB25">
+        <v>8</v>
+      </c>
     </row>
-    <row r="26" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -4855,8 +5003,14 @@
       <c r="BZ26">
         <v>5</v>
       </c>
+      <c r="CB26">
+        <v>6</v>
+      </c>
+      <c r="CC26">
+        <v>5</v>
+      </c>
     </row>
-    <row r="27" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -5008,8 +5162,14 @@
       <c r="CA27">
         <v>1</v>
       </c>
+      <c r="CB27">
+        <v>4</v>
+      </c>
+      <c r="CC27">
+        <v>2</v>
+      </c>
     </row>
-    <row r="28" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -5206,8 +5366,14 @@
       <c r="BZ28">
         <v>3</v>
       </c>
+      <c r="CB28">
+        <v>7</v>
+      </c>
+      <c r="CC28">
+        <v>3</v>
+      </c>
     </row>
-    <row r="29" spans="2:79" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:82" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
         <v>3</v>
       </c>
@@ -5368,8 +5534,17 @@
       <c r="BZ29" s="3">
         <v>1</v>
       </c>
+      <c r="CB29" s="3">
+        <v>2</v>
+      </c>
+      <c r="CC29" s="3">
+        <v>1</v>
+      </c>
+      <c r="CD29" s="3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="30" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -5479,8 +5654,11 @@
       <c r="BY30">
         <v>8</v>
       </c>
+      <c r="CB30">
+        <v>8</v>
+      </c>
     </row>
-    <row r="31" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -5659,8 +5837,14 @@
       <c r="BZ31">
         <v>3</v>
       </c>
+      <c r="CB31">
+        <v>2</v>
+      </c>
+      <c r="CC31">
+        <v>3</v>
+      </c>
     </row>
-    <row r="32" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -5803,8 +5987,14 @@
       <c r="BZ32">
         <v>1</v>
       </c>
+      <c r="CB32">
+        <v>9</v>
+      </c>
+      <c r="CC32">
+        <v>1</v>
+      </c>
     </row>
-    <row r="33" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -5941,8 +6131,14 @@
       <c r="BZ33">
         <v>1</v>
       </c>
+      <c r="CB33">
+        <v>8</v>
+      </c>
+      <c r="CC33">
+        <v>1</v>
+      </c>
     </row>
-    <row r="34" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -6076,8 +6272,11 @@
       <c r="BY34">
         <v>6</v>
       </c>
+      <c r="CB34">
+        <v>6</v>
+      </c>
     </row>
-    <row r="35" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -6235,8 +6434,14 @@
       <c r="BZ35">
         <v>2</v>
       </c>
+      <c r="CB35">
+        <v>3</v>
+      </c>
+      <c r="CC35">
+        <v>5</v>
+      </c>
     </row>
-    <row r="36" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -6394,8 +6599,14 @@
       <c r="BZ36">
         <v>2</v>
       </c>
+      <c r="CB36">
+        <v>8</v>
+      </c>
+      <c r="CC36">
+        <v>2</v>
+      </c>
     </row>
-    <row r="37" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -6499,8 +6710,14 @@
       <c r="BY37">
         <v>9</v>
       </c>
+      <c r="CB37">
+        <v>8</v>
+      </c>
+      <c r="CD37">
+        <v>1</v>
+      </c>
     </row>
-    <row r="38" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -6697,8 +6914,14 @@
       <c r="BZ38">
         <v>3</v>
       </c>
+      <c r="CB38">
+        <v>5</v>
+      </c>
+      <c r="CC38">
+        <v>3</v>
+      </c>
     </row>
-    <row r="39" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -6877,8 +7100,14 @@
       <c r="BZ39">
         <v>4</v>
       </c>
+      <c r="CB39">
+        <v>2</v>
+      </c>
+      <c r="CC39">
+        <v>4</v>
+      </c>
     </row>
-    <row r="40" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -7069,8 +7298,14 @@
       <c r="BZ40">
         <v>6</v>
       </c>
+      <c r="CB40">
+        <v>4</v>
+      </c>
+      <c r="CC40">
+        <v>6</v>
+      </c>
     </row>
-    <row r="41" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -7228,8 +7463,14 @@
       <c r="BZ41">
         <v>2</v>
       </c>
+      <c r="CB41">
+        <v>4</v>
+      </c>
+      <c r="CC41">
+        <v>2</v>
+      </c>
     </row>
-    <row r="42" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -7342,8 +7583,11 @@
       <c r="BY42">
         <v>7</v>
       </c>
+      <c r="CB42">
+        <v>7</v>
+      </c>
     </row>
-    <row r="43" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -7522,8 +7766,17 @@
       <c r="CA43">
         <v>1</v>
       </c>
+      <c r="CB43">
+        <v>2</v>
+      </c>
+      <c r="CC43">
+        <v>6</v>
+      </c>
+      <c r="CD43">
+        <v>1</v>
+      </c>
     </row>
-    <row r="44" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -7621,8 +7874,11 @@
       <c r="BY44">
         <v>6</v>
       </c>
+      <c r="CB44">
+        <v>6</v>
+      </c>
     </row>
-    <row r="45" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -7846,8 +8102,17 @@
       <c r="CA45">
         <v>1</v>
       </c>
+      <c r="CB45">
+        <v>5</v>
+      </c>
+      <c r="CC45">
+        <v>3</v>
+      </c>
+      <c r="CD45">
+        <v>1</v>
+      </c>
     </row>
-    <row r="46" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -7957,8 +8222,11 @@
       <c r="BY46">
         <v>6</v>
       </c>
+      <c r="CB46">
+        <v>6</v>
+      </c>
     </row>
-    <row r="47" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -8092,8 +8360,14 @@
       <c r="BZ47">
         <v>9</v>
       </c>
+      <c r="CB47">
+        <v>0</v>
+      </c>
+      <c r="CC47">
+        <v>9</v>
+      </c>
     </row>
-    <row r="48" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -8293,8 +8567,14 @@
       <c r="BZ48">
         <v>6</v>
       </c>
+      <c r="CB48">
+        <v>5</v>
+      </c>
+      <c r="CC48">
+        <v>6</v>
+      </c>
     </row>
-    <row r="49" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -8401,8 +8681,14 @@
       <c r="CA49">
         <v>1</v>
       </c>
+      <c r="CB49">
+        <v>7</v>
+      </c>
+      <c r="CD49">
+        <v>1</v>
+      </c>
     </row>
-    <row r="50" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -8605,8 +8891,14 @@
       <c r="BZ50">
         <v>1</v>
       </c>
+      <c r="CB50">
+        <v>7</v>
+      </c>
+      <c r="CC50">
+        <v>1</v>
+      </c>
     </row>
-    <row r="51" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -8794,8 +9086,14 @@
       <c r="BZ51">
         <v>2</v>
       </c>
+      <c r="CB51">
+        <v>4</v>
+      </c>
+      <c r="CC51">
+        <v>2</v>
+      </c>
     </row>
-    <row r="52" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -8899,8 +9197,11 @@
       <c r="BY52">
         <v>6</v>
       </c>
+      <c r="CB52">
+        <v>6</v>
+      </c>
     </row>
-    <row r="53" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -9067,8 +9368,14 @@
       <c r="BZ53">
         <v>1</v>
       </c>
+      <c r="CB53">
+        <v>3</v>
+      </c>
+      <c r="CC53">
+        <v>1</v>
+      </c>
     </row>
-    <row r="54" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -9175,8 +9482,11 @@
       <c r="BY54">
         <v>5</v>
       </c>
+      <c r="CB54">
+        <v>5</v>
+      </c>
     </row>
-    <row r="55" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -9337,8 +9647,14 @@
       <c r="BZ55">
         <v>4</v>
       </c>
+      <c r="CB55">
+        <v>2</v>
+      </c>
+      <c r="CC55">
+        <v>4</v>
+      </c>
     </row>
-    <row r="56" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -9442,8 +9758,14 @@
       <c r="CA56">
         <v>1</v>
       </c>
+      <c r="CB56">
+        <v>9</v>
+      </c>
+      <c r="CD56">
+        <v>1</v>
+      </c>
     </row>
-    <row r="57" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -9559,8 +9881,14 @@
       <c r="BZ57">
         <v>1</v>
       </c>
+      <c r="CB57">
+        <v>6</v>
+      </c>
+      <c r="CC57">
+        <v>1</v>
+      </c>
     </row>
-    <row r="58" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -9670,8 +9998,11 @@
       <c r="BY58">
         <v>6</v>
       </c>
+      <c r="CB58">
+        <v>6</v>
+      </c>
     </row>
-    <row r="59" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -9772,8 +10103,11 @@
       <c r="BY59">
         <v>7</v>
       </c>
+      <c r="CB59">
+        <v>7</v>
+      </c>
     </row>
-    <row r="60" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -9934,8 +10268,14 @@
       <c r="BZ60">
         <v>2</v>
       </c>
+      <c r="CB60">
+        <v>7</v>
+      </c>
+      <c r="CC60">
+        <v>2</v>
+      </c>
     </row>
-    <row r="61" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -10045,8 +10385,14 @@
       <c r="BY61">
         <v>7</v>
       </c>
+      <c r="CB61">
+        <v>6</v>
+      </c>
+      <c r="CD61">
+        <v>1</v>
+      </c>
     </row>
-    <row r="62" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -10237,8 +10583,14 @@
       <c r="BZ62">
         <v>2</v>
       </c>
+      <c r="CB62">
+        <v>3</v>
+      </c>
+      <c r="CC62">
+        <v>2</v>
+      </c>
     </row>
-    <row r="63" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -10423,8 +10775,14 @@
       <c r="BZ63">
         <v>5</v>
       </c>
+      <c r="CB63">
+        <v>4</v>
+      </c>
+      <c r="CC63">
+        <v>5</v>
+      </c>
     </row>
-    <row r="64" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -10579,8 +10937,14 @@
       <c r="BZ64">
         <v>3</v>
       </c>
+      <c r="CB64">
+        <v>7</v>
+      </c>
+      <c r="CC64">
+        <v>3</v>
+      </c>
     </row>
-    <row r="65" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -10738,8 +11102,14 @@
       <c r="BZ65">
         <v>2</v>
       </c>
+      <c r="CB65">
+        <v>4</v>
+      </c>
+      <c r="CC65">
+        <v>2</v>
+      </c>
     </row>
-    <row r="66" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -10753,6 +11123,9 @@
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
+      <c r="F66" t="s">
+        <v>118</v>
+      </c>
       <c r="M66">
         <v>1</v>
       </c>
@@ -10846,8 +11219,11 @@
       <c r="CA66">
         <v>1</v>
       </c>
+      <c r="CB66">
+        <v>5</v>
+      </c>
     </row>
-    <row r="67" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -11032,8 +11408,14 @@
       <c r="BZ67">
         <v>8</v>
       </c>
+      <c r="CB67">
+        <v>2</v>
+      </c>
+      <c r="CC67">
+        <v>8</v>
+      </c>
     </row>
-    <row r="68" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -11131,8 +11513,11 @@
       <c r="BY68">
         <v>11</v>
       </c>
+      <c r="CB68">
+        <v>11</v>
+      </c>
     </row>
-    <row r="69" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -11236,8 +11621,11 @@
       <c r="BY69">
         <v>9</v>
       </c>
+      <c r="CB69">
+        <v>9</v>
+      </c>
     </row>
-    <row r="70" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -11350,8 +11738,11 @@
       <c r="BY70">
         <v>8</v>
       </c>
+      <c r="CB70">
+        <v>8</v>
+      </c>
     </row>
-    <row r="71" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -11530,8 +11921,14 @@
       <c r="CA71">
         <v>1</v>
       </c>
+      <c r="CB71">
+        <v>6</v>
+      </c>
+      <c r="CC71">
+        <v>4</v>
+      </c>
     </row>
-    <row r="72" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -11701,8 +12098,14 @@
       <c r="BZ72">
         <v>1</v>
       </c>
+      <c r="CB72">
+        <v>6</v>
+      </c>
+      <c r="CC72">
+        <v>1</v>
+      </c>
     </row>
-    <row r="73" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -11806,8 +12209,11 @@
       <c r="BY73">
         <v>10</v>
       </c>
+      <c r="CB73">
+        <v>10</v>
+      </c>
     </row>
-    <row r="74" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -11920,8 +12326,11 @@
       <c r="BY74">
         <v>9</v>
       </c>
+      <c r="CB74">
+        <v>9</v>
+      </c>
     </row>
-    <row r="75" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -12082,8 +12491,17 @@
       <c r="BZ75">
         <v>2</v>
       </c>
+      <c r="CB75">
+        <v>6</v>
+      </c>
+      <c r="CC75">
+        <v>2</v>
+      </c>
+      <c r="CD75">
+        <v>1</v>
+      </c>
     </row>
-    <row r="76" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -12271,8 +12689,14 @@
       <c r="BZ76">
         <v>1</v>
       </c>
+      <c r="CB76">
+        <v>7</v>
+      </c>
+      <c r="CC76">
+        <v>1</v>
+      </c>
     </row>
-    <row r="77" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -12416,19 +12840,25 @@
         <v>1</v>
       </c>
       <c r="BV77">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BW77">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BY77">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BZ77">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="CB77">
+        <v>4</v>
+      </c>
+      <c r="CC77">
+        <v>3</v>
       </c>
     </row>
-    <row r="78" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -12535,8 +12965,11 @@
       <c r="BY78">
         <v>7</v>
       </c>
+      <c r="CB78">
+        <v>7</v>
+      </c>
     </row>
-    <row r="79" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -12718,8 +13151,14 @@
       <c r="BZ79">
         <v>7</v>
       </c>
+      <c r="CB79">
+        <v>2</v>
+      </c>
+      <c r="CC79">
+        <v>7</v>
+      </c>
     </row>
-    <row r="80" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -12871,8 +13310,14 @@
       <c r="BZ80">
         <v>1</v>
       </c>
+      <c r="CB80">
+        <v>9</v>
+      </c>
+      <c r="CC80">
+        <v>1</v>
+      </c>
     </row>
-    <row r="81" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -13036,8 +13481,14 @@
       <c r="BZ81">
         <v>2</v>
       </c>
+      <c r="CB81">
+        <v>5</v>
+      </c>
+      <c r="CC81">
+        <v>2</v>
+      </c>
     </row>
-    <row r="82" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -13237,8 +13688,14 @@
       <c r="CA82">
         <v>1</v>
       </c>
+      <c r="CB82">
+        <v>6</v>
+      </c>
+      <c r="CC82">
+        <v>4</v>
+      </c>
     </row>
-    <row r="83" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -13420,8 +13877,14 @@
       <c r="BZ83">
         <v>4</v>
       </c>
+      <c r="CB83">
+        <v>5</v>
+      </c>
+      <c r="CC83">
+        <v>4</v>
+      </c>
     </row>
-    <row r="84" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -13603,8 +14066,14 @@
       <c r="BZ84">
         <v>2</v>
       </c>
+      <c r="CB84">
+        <v>7</v>
+      </c>
+      <c r="CC84">
+        <v>2</v>
+      </c>
     </row>
-    <row r="85" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -13786,8 +14255,14 @@
       <c r="CA85">
         <v>1</v>
       </c>
+      <c r="CB85">
+        <v>3</v>
+      </c>
+      <c r="CC85">
+        <v>3</v>
+      </c>
     </row>
-    <row r="86" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -13948,8 +14423,14 @@
       <c r="BZ86">
         <v>1</v>
       </c>
+      <c r="CB86">
+        <v>8</v>
+      </c>
+      <c r="CC86">
+        <v>1</v>
+      </c>
     </row>
-    <row r="87" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -14134,8 +14615,14 @@
       <c r="BZ87">
         <v>2</v>
       </c>
+      <c r="CB87">
+        <v>5</v>
+      </c>
+      <c r="CC87">
+        <v>2</v>
+      </c>
     </row>
-    <row r="88" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -14305,8 +14792,14 @@
       <c r="BZ88">
         <v>3</v>
       </c>
+      <c r="CB88">
+        <v>6</v>
+      </c>
+      <c r="CC88">
+        <v>3</v>
+      </c>
     </row>
-    <row r="89" spans="2:79" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:81" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B89" s="3" t="s">
         <v>3</v>
       </c>
@@ -14452,8 +14945,14 @@
       <c r="BZ89" s="3">
         <v>2</v>
       </c>
+      <c r="CB89" s="3">
+        <v>3</v>
+      </c>
+      <c r="CC89" s="3">
+        <v>2</v>
+      </c>
     </row>
-    <row r="90" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -14560,8 +15059,11 @@
       <c r="BY90">
         <v>8</v>
       </c>
+      <c r="CB90">
+        <v>8</v>
+      </c>
     </row>
-    <row r="91" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -14755,8 +15257,14 @@
       <c r="BZ91">
         <v>2</v>
       </c>
+      <c r="CB91">
+        <v>4</v>
+      </c>
+      <c r="CC91">
+        <v>2</v>
+      </c>
     </row>
-    <row r="92" spans="2:79" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:81" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B92" s="3" t="s">
         <v>1</v>
       </c>
@@ -14932,8 +15440,14 @@
       <c r="BZ92" s="3">
         <v>3</v>
       </c>
+      <c r="CB92" s="3">
+        <v>5</v>
+      </c>
+      <c r="CC92" s="3">
+        <v>3</v>
+      </c>
     </row>
-    <row r="93" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -15067,8 +15581,14 @@
       <c r="BZ93">
         <v>1</v>
       </c>
+      <c r="CB93">
+        <v>8</v>
+      </c>
+      <c r="CC93">
+        <v>1</v>
+      </c>
     </row>
-    <row r="94" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -15178,8 +15698,11 @@
       <c r="BY94">
         <v>7</v>
       </c>
+      <c r="CB94">
+        <v>7</v>
+      </c>
     </row>
-    <row r="95" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -15319,8 +15842,14 @@
       <c r="BZ95">
         <v>3</v>
       </c>
+      <c r="CB95">
+        <v>5</v>
+      </c>
+      <c r="CC95">
+        <v>3</v>
+      </c>
     </row>
-    <row r="96" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -15484,8 +16013,14 @@
       <c r="BZ96">
         <v>2</v>
       </c>
+      <c r="CB96">
+        <v>8</v>
+      </c>
+      <c r="CC96">
+        <v>2</v>
+      </c>
     </row>
-    <row r="97" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -15592,8 +16127,11 @@
       <c r="BY97">
         <v>8</v>
       </c>
+      <c r="CB97">
+        <v>8</v>
+      </c>
     </row>
-    <row r="98" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -15757,8 +16295,14 @@
       <c r="BZ98">
         <v>2</v>
       </c>
+      <c r="CB98">
+        <v>5</v>
+      </c>
+      <c r="CC98">
+        <v>2</v>
+      </c>
     </row>
-    <row r="99" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -15877,8 +16421,14 @@
       <c r="BZ99">
         <v>1</v>
       </c>
+      <c r="CB99">
+        <v>2</v>
+      </c>
+      <c r="CC99">
+        <v>1</v>
+      </c>
     </row>
-    <row r="100" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -15982,8 +16532,14 @@
       <c r="BY100">
         <v>8</v>
       </c>
+      <c r="CB100">
+        <v>7</v>
+      </c>
+      <c r="CD100">
+        <v>1</v>
+      </c>
     </row>
-    <row r="101" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -16135,8 +16691,14 @@
       <c r="BZ101">
         <v>4</v>
       </c>
+      <c r="CB101">
+        <v>1</v>
+      </c>
+      <c r="CC101">
+        <v>4</v>
+      </c>
     </row>
-    <row r="102" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -16243,8 +16805,11 @@
       <c r="BY102">
         <v>7</v>
       </c>
+      <c r="CB102">
+        <v>7</v>
+      </c>
     </row>
-    <row r="103" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -16417,8 +16982,14 @@
       <c r="BZ103">
         <v>4</v>
       </c>
+      <c r="CB103">
+        <v>2</v>
+      </c>
+      <c r="CC103">
+        <v>4</v>
+      </c>
     </row>
-    <row r="104" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -16582,8 +17153,14 @@
       <c r="BZ104">
         <v>3</v>
       </c>
+      <c r="CB104">
+        <v>7</v>
+      </c>
+      <c r="CC104">
+        <v>3</v>
+      </c>
     </row>
-    <row r="105" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -16741,8 +17318,14 @@
       <c r="BZ105">
         <v>3</v>
       </c>
+      <c r="CB105">
+        <v>3</v>
+      </c>
+      <c r="CC105">
+        <v>3</v>
+      </c>
     </row>
-    <row r="106" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -16894,8 +17477,11 @@
       <c r="BY106">
         <v>8</v>
       </c>
+      <c r="CB106">
+        <v>8</v>
+      </c>
     </row>
-    <row r="107" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -17065,8 +17651,14 @@
       <c r="BZ107">
         <v>1</v>
       </c>
+      <c r="CB107">
+        <v>4</v>
+      </c>
+      <c r="CC107">
+        <v>1</v>
+      </c>
     </row>
-    <row r="108" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -17221,8 +17813,17 @@
       <c r="CA108">
         <v>1</v>
       </c>
+      <c r="CB108">
+        <v>6</v>
+      </c>
+      <c r="CC108">
+        <v>3</v>
+      </c>
+      <c r="CD108">
+        <v>1</v>
+      </c>
     </row>
-    <row r="109" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -17398,8 +17999,14 @@
       <c r="BZ109">
         <v>9</v>
       </c>
+      <c r="CB109">
+        <v>0</v>
+      </c>
+      <c r="CC109">
+        <v>9</v>
+      </c>
     </row>
-    <row r="110" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -17578,8 +18185,14 @@
       <c r="CA110">
         <v>1</v>
       </c>
+      <c r="CB110">
+        <v>6</v>
+      </c>
+      <c r="CC110">
+        <v>3</v>
+      </c>
     </row>
-    <row r="111" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -17737,8 +18350,14 @@
       <c r="BZ111">
         <v>4</v>
       </c>
+      <c r="CB111">
+        <v>4</v>
+      </c>
+      <c r="CC111">
+        <v>4</v>
+      </c>
     </row>
-    <row r="112" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -17902,8 +18521,14 @@
       <c r="BZ112">
         <v>2</v>
       </c>
+      <c r="CB112">
+        <v>6</v>
+      </c>
+      <c r="CC112">
+        <v>2</v>
+      </c>
     </row>
-    <row r="113" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -18082,8 +18707,14 @@
       <c r="BZ113">
         <v>2</v>
       </c>
+      <c r="CB113">
+        <v>4</v>
+      </c>
+      <c r="CC113">
+        <v>2</v>
+      </c>
     </row>
-    <row r="114" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -18190,8 +18821,11 @@
       <c r="BY114">
         <v>8</v>
       </c>
+      <c r="CB114">
+        <v>8</v>
+      </c>
     </row>
-    <row r="115" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -18373,8 +19007,14 @@
       <c r="BZ115">
         <v>3</v>
       </c>
+      <c r="CB115">
+        <v>1</v>
+      </c>
+      <c r="CC115">
+        <v>3</v>
+      </c>
     </row>
-    <row r="116" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -18538,8 +19178,14 @@
       <c r="BZ116">
         <v>2</v>
       </c>
+      <c r="CB116">
+        <v>6</v>
+      </c>
+      <c r="CC116">
+        <v>2</v>
+      </c>
     </row>
-    <row r="117" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -18712,8 +19358,14 @@
       <c r="BZ117">
         <v>4</v>
       </c>
+      <c r="CB117">
+        <v>1</v>
+      </c>
+      <c r="CC117">
+        <v>4</v>
+      </c>
     </row>
-    <row r="118" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -18824,8 +19476,11 @@
       <c r="BY118">
         <v>6</v>
       </c>
+      <c r="CB118">
+        <v>6</v>
+      </c>
     </row>
-    <row r="119" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -18935,8 +19590,14 @@
       <c r="CA119">
         <v>1</v>
       </c>
+      <c r="CB119">
+        <v>6</v>
+      </c>
+      <c r="CD119">
+        <v>1</v>
+      </c>
     </row>
-    <row r="120" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -19040,8 +19701,11 @@
       <c r="BY120">
         <v>10</v>
       </c>
+      <c r="CB120">
+        <v>10</v>
+      </c>
     </row>
-    <row r="121" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -19148,8 +19812,11 @@
       <c r="BY121">
         <v>8</v>
       </c>
+      <c r="CB121">
+        <v>8</v>
+      </c>
     </row>
-    <row r="122" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -19259,8 +19926,11 @@
       <c r="BY122">
         <v>6</v>
       </c>
+      <c r="CB122">
+        <v>6</v>
+      </c>
     </row>
-    <row r="123" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -19421,8 +20091,14 @@
       <c r="BZ123">
         <v>3</v>
       </c>
+      <c r="CB123">
+        <v>3</v>
+      </c>
+      <c r="CC123">
+        <v>3</v>
+      </c>
     </row>
-    <row r="124" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -19613,8 +20289,14 @@
       <c r="BZ124">
         <v>4</v>
       </c>
+      <c r="CB124">
+        <v>5</v>
+      </c>
+      <c r="CC124">
+        <v>4</v>
+      </c>
     </row>
-    <row r="125" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -19802,8 +20484,14 @@
       <c r="BZ125">
         <v>6</v>
       </c>
+      <c r="CB125">
+        <v>0</v>
+      </c>
+      <c r="CC125">
+        <v>6</v>
+      </c>
     </row>
-    <row r="126" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -19970,8 +20658,14 @@
       <c r="BZ126">
         <v>1</v>
       </c>
+      <c r="CB126">
+        <v>5</v>
+      </c>
+      <c r="CC126">
+        <v>1</v>
+      </c>
     </row>
-    <row r="127" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -20135,8 +20829,14 @@
       <c r="BZ127">
         <v>2</v>
       </c>
+      <c r="CB127">
+        <v>1</v>
+      </c>
+      <c r="CC127">
+        <v>2</v>
+      </c>
     </row>
-    <row r="128" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -20234,8 +20934,11 @@
       <c r="BY128">
         <v>7</v>
       </c>
+      <c r="CB128">
+        <v>7</v>
+      </c>
     </row>
-    <row r="129" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="129" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -20414,8 +21117,14 @@
       <c r="BZ129">
         <v>4</v>
       </c>
+      <c r="CB129">
+        <v>2</v>
+      </c>
+      <c r="CC129">
+        <v>4</v>
+      </c>
     </row>
-    <row r="130" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="130" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -20525,8 +21234,14 @@
       <c r="BY130">
         <v>10</v>
       </c>
+      <c r="CB130">
+        <v>6</v>
+      </c>
+      <c r="CC130">
+        <v>4</v>
+      </c>
     </row>
-    <row r="131" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="131" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -20699,8 +21414,17 @@
       <c r="CA131">
         <v>1</v>
       </c>
+      <c r="CB131">
+        <v>6</v>
+      </c>
+      <c r="CC131">
+        <v>3</v>
+      </c>
+      <c r="CD131">
+        <v>1</v>
+      </c>
     </row>
-    <row r="132" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="132" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -20801,8 +21525,14 @@
       <c r="BY132">
         <v>6</v>
       </c>
+      <c r="CB132">
+        <v>5</v>
+      </c>
+      <c r="CC132">
+        <v>1</v>
+      </c>
     </row>
-    <row r="133" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="133" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -20936,8 +21666,14 @@
       <c r="BZ133">
         <v>1</v>
       </c>
+      <c r="CB133">
+        <v>6</v>
+      </c>
+      <c r="CC133">
+        <v>1</v>
+      </c>
     </row>
-    <row r="134" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="134" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -21065,8 +21801,17 @@
       <c r="BY134">
         <v>9</v>
       </c>
+      <c r="BZ134">
+        <v>1</v>
+      </c>
+      <c r="CB134">
+        <v>9</v>
+      </c>
+      <c r="CC134">
+        <v>1</v>
+      </c>
     </row>
-    <row r="135" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="135" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -21221,8 +21966,14 @@
       <c r="CA135">
         <v>1</v>
       </c>
+      <c r="CB135">
+        <v>3</v>
+      </c>
+      <c r="CC135">
+        <v>5</v>
+      </c>
     </row>
-    <row r="136" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="136" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -21368,8 +22119,14 @@
       <c r="BZ136">
         <v>1</v>
       </c>
+      <c r="CB136">
+        <v>6</v>
+      </c>
+      <c r="CC136">
+        <v>1</v>
+      </c>
     </row>
-    <row r="137" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="137" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -21524,8 +22281,14 @@
       <c r="CA137">
         <v>1</v>
       </c>
+      <c r="CB137">
+        <v>3</v>
+      </c>
+      <c r="CC137">
+        <v>2</v>
+      </c>
     </row>
-    <row r="138" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="138" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -21695,8 +22458,14 @@
       <c r="BZ138">
         <v>1</v>
       </c>
+      <c r="CB138">
+        <v>7</v>
+      </c>
+      <c r="CC138">
+        <v>1</v>
+      </c>
     </row>
-    <row r="139" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="139" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -21851,8 +22620,14 @@
       <c r="CA139">
         <v>1</v>
       </c>
+      <c r="CB139">
+        <v>4</v>
+      </c>
+      <c r="CC139">
+        <v>1</v>
+      </c>
     </row>
-    <row r="140" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="140" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -21956,8 +22731,14 @@
       <c r="BZ140">
         <v>6</v>
       </c>
+      <c r="CB140">
+        <v>2</v>
+      </c>
+      <c r="CC140">
+        <v>7</v>
+      </c>
     </row>
-    <row r="141" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="141" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -22148,8 +22929,14 @@
       <c r="BZ141">
         <v>4</v>
       </c>
+      <c r="CB141">
+        <v>4</v>
+      </c>
+      <c r="CC141">
+        <v>4</v>
+      </c>
     </row>
-    <row r="142" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="142" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -22337,8 +23124,14 @@
       <c r="BZ142">
         <v>2</v>
       </c>
+      <c r="CB142">
+        <v>3</v>
+      </c>
+      <c r="CC142">
+        <v>5</v>
+      </c>
     </row>
-    <row r="143" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="143" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -22481,8 +23274,14 @@
       <c r="BZ143">
         <v>3</v>
       </c>
+      <c r="CB143">
+        <v>8</v>
+      </c>
+      <c r="CC143">
+        <v>3</v>
+      </c>
     </row>
-    <row r="144" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="144" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -22583,8 +23382,14 @@
       <c r="BY144">
         <v>7</v>
       </c>
+      <c r="CB144">
+        <v>5</v>
+      </c>
+      <c r="CC144">
+        <v>2</v>
+      </c>
     </row>
-    <row r="145" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="145" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -22691,8 +23496,14 @@
       <c r="BY145">
         <v>8</v>
       </c>
+      <c r="CB145">
+        <v>7</v>
+      </c>
+      <c r="CC145">
+        <v>1</v>
+      </c>
     </row>
-    <row r="146" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="146" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -22886,8 +23697,14 @@
       <c r="BZ146">
         <v>2</v>
       </c>
+      <c r="CB146">
+        <v>8</v>
+      </c>
+      <c r="CC146">
+        <v>2</v>
+      </c>
     </row>
-    <row r="147" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="147" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -23072,8 +23889,14 @@
       <c r="BZ147">
         <v>3</v>
       </c>
+      <c r="CB147">
+        <v>1</v>
+      </c>
+      <c r="CC147">
+        <v>3</v>
+      </c>
     </row>
-    <row r="148" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="148" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -23177,8 +24000,11 @@
       <c r="BY148">
         <v>9</v>
       </c>
+      <c r="CB148">
+        <v>9</v>
+      </c>
     </row>
-    <row r="149" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="149" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -23360,8 +24186,17 @@
       <c r="CA149">
         <v>2</v>
       </c>
+      <c r="CB149">
+        <v>1</v>
+      </c>
+      <c r="CC149">
+        <v>2</v>
+      </c>
+      <c r="CD149">
+        <v>2</v>
+      </c>
     </row>
-    <row r="150" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="150" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -23546,8 +24381,14 @@
       <c r="BZ150">
         <v>1</v>
       </c>
+      <c r="CB150">
+        <v>8</v>
+      </c>
+      <c r="CC150">
+        <v>1</v>
+      </c>
     </row>
-    <row r="151" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="151" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -23702,8 +24543,14 @@
       <c r="CA151">
         <v>3</v>
       </c>
+      <c r="CB151">
+        <v>4</v>
+      </c>
+      <c r="CC151">
+        <v>6</v>
+      </c>
     </row>
-    <row r="152" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="152" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -23801,8 +24648,11 @@
       <c r="BY152">
         <v>9</v>
       </c>
+      <c r="CB152">
+        <v>9</v>
+      </c>
     </row>
-    <row r="153" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="153" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -23951,8 +24801,14 @@
       <c r="BZ153">
         <v>1</v>
       </c>
+      <c r="CB153">
+        <v>5</v>
+      </c>
+      <c r="CC153">
+        <v>1</v>
+      </c>
     </row>
-    <row r="154" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="154" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -24161,8 +25017,17 @@
       <c r="BZ154">
         <v>3</v>
       </c>
+      <c r="CB154">
+        <v>4</v>
+      </c>
+      <c r="CC154">
+        <v>3</v>
+      </c>
+      <c r="CD154">
+        <v>1</v>
+      </c>
     </row>
-    <row r="155" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="155" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -24323,8 +25188,14 @@
       <c r="BZ155">
         <v>3</v>
       </c>
+      <c r="CB155">
+        <v>6</v>
+      </c>
+      <c r="CC155">
+        <v>3</v>
+      </c>
     </row>
-    <row r="156" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="156" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -24428,8 +25299,11 @@
       <c r="BY156">
         <v>6</v>
       </c>
+      <c r="CB156">
+        <v>6</v>
+      </c>
     </row>
-    <row r="157" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="157" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -24536,8 +25410,11 @@
       <c r="BY157">
         <v>6</v>
       </c>
+      <c r="CB157">
+        <v>6</v>
+      </c>
     </row>
-    <row r="158" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="158" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -24665,8 +25542,14 @@
       <c r="BZ158">
         <v>2</v>
       </c>
+      <c r="CB158">
+        <v>6</v>
+      </c>
+      <c r="CC158">
+        <v>2</v>
+      </c>
     </row>
-    <row r="159" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="159" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -24842,8 +25725,14 @@
       <c r="BZ159">
         <v>3</v>
       </c>
+      <c r="CB159">
+        <v>2</v>
+      </c>
+      <c r="CC159">
+        <v>3</v>
+      </c>
     </row>
-    <row r="160" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="160" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -24947,8 +25836,11 @@
       <c r="BY160">
         <v>9</v>
       </c>
+      <c r="CB160">
+        <v>9</v>
+      </c>
     </row>
-    <row r="161" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="161" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -25148,8 +26040,14 @@
       <c r="BZ161">
         <v>6</v>
       </c>
+      <c r="CB161">
+        <v>1</v>
+      </c>
+      <c r="CC161">
+        <v>6</v>
+      </c>
     </row>
-    <row r="162" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="162" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -25256,8 +26154,11 @@
       <c r="BY162">
         <v>8</v>
       </c>
+      <c r="CB162">
+        <v>8</v>
+      </c>
     </row>
-    <row r="163" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="163" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -25418,8 +26319,14 @@
       <c r="CA163">
         <v>2</v>
       </c>
+      <c r="CB163">
+        <v>1</v>
+      </c>
+      <c r="CC163">
+        <v>7</v>
+      </c>
     </row>
-    <row r="164" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="164" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -25517,8 +26424,11 @@
       <c r="BY164">
         <v>9</v>
       </c>
+      <c r="CB164">
+        <v>9</v>
+      </c>
     </row>
-    <row r="165" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="165" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -25676,8 +26586,14 @@
       <c r="BZ165">
         <v>2</v>
       </c>
+      <c r="CB165">
+        <v>4</v>
+      </c>
+      <c r="CC165">
+        <v>2</v>
+      </c>
     </row>
-    <row r="166" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="166" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -25826,8 +26742,11 @@
       <c r="BY166">
         <v>5</v>
       </c>
+      <c r="CB166">
+        <v>6</v>
+      </c>
     </row>
-    <row r="167" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="167" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -25973,8 +26892,14 @@
       <c r="BZ167">
         <v>1</v>
       </c>
+      <c r="CB167">
+        <v>7</v>
+      </c>
+      <c r="CC167">
+        <v>1</v>
+      </c>
     </row>
-    <row r="168" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="168" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -26150,8 +27075,14 @@
       <c r="BZ168">
         <v>2</v>
       </c>
+      <c r="CB168">
+        <v>9</v>
+      </c>
+      <c r="CC168">
+        <v>2</v>
+      </c>
     </row>
-    <row r="169" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="169" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -26258,8 +27189,11 @@
       <c r="BY169">
         <v>6</v>
       </c>
+      <c r="CB169">
+        <v>6</v>
+      </c>
     </row>
-    <row r="170" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="170" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -26381,8 +27315,17 @@
       <c r="BZ170">
         <v>1</v>
       </c>
+      <c r="CB170">
+        <v>7</v>
+      </c>
+      <c r="CC170">
+        <v>1</v>
+      </c>
+      <c r="CD170">
+        <v>1</v>
+      </c>
     </row>
-    <row r="171" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="171" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -26570,8 +27513,14 @@
       <c r="CA171">
         <v>1</v>
       </c>
+      <c r="CB171">
+        <v>4</v>
+      </c>
+      <c r="CC171">
+        <v>6</v>
+      </c>
     </row>
-    <row r="172" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="172" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -26678,8 +27627,14 @@
       <c r="CA172">
         <v>1</v>
       </c>
+      <c r="CB172">
+        <v>7</v>
+      </c>
+      <c r="CD172">
+        <v>1</v>
+      </c>
     </row>
-    <row r="173" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="173" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -26804,8 +27759,14 @@
       <c r="BZ173">
         <v>2</v>
       </c>
+      <c r="CB173">
+        <v>6</v>
+      </c>
+      <c r="CC173">
+        <v>2</v>
+      </c>
     </row>
-    <row r="174" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="174" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -26912,8 +27873,11 @@
       <c r="BY174">
         <v>9</v>
       </c>
+      <c r="CB174">
+        <v>9</v>
+      </c>
     </row>
-    <row r="175" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="175" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -27074,8 +28038,14 @@
       <c r="CA175">
         <v>2</v>
       </c>
+      <c r="CB175">
+        <v>5</v>
+      </c>
+      <c r="CC175">
+        <v>4</v>
+      </c>
     </row>
-    <row r="176" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="176" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -27173,8 +28143,14 @@
       <c r="BY176">
         <v>8</v>
       </c>
+      <c r="CB176">
+        <v>7</v>
+      </c>
+      <c r="CD176">
+        <v>1</v>
+      </c>
     </row>
-    <row r="177" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="177" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -27281,8 +28257,14 @@
       <c r="CA177">
         <v>1</v>
       </c>
+      <c r="CB177">
+        <v>4</v>
+      </c>
+      <c r="CC177">
+        <v>1</v>
+      </c>
     </row>
-    <row r="178" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="178" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -27392,8 +28374,14 @@
       <c r="BY178">
         <v>8</v>
       </c>
+      <c r="CB178">
+        <v>6</v>
+      </c>
+      <c r="CD178">
+        <v>2</v>
+      </c>
     </row>
-    <row r="179" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="179" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -27554,8 +28542,14 @@
       <c r="BZ179">
         <v>5</v>
       </c>
+      <c r="CB179">
+        <v>5</v>
+      </c>
+      <c r="CC179">
+        <v>5</v>
+      </c>
     </row>
-    <row r="180" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="180" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -27710,8 +28704,17 @@
       <c r="BZ180">
         <v>2</v>
       </c>
+      <c r="CB180">
+        <v>5</v>
+      </c>
+      <c r="CC180">
+        <v>2</v>
+      </c>
+      <c r="CD180">
+        <v>2</v>
+      </c>
     </row>
-    <row r="181" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="181" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -27875,8 +28878,14 @@
       <c r="BZ181">
         <v>8</v>
       </c>
+      <c r="CC181">
+        <v>8</v>
+      </c>
+      <c r="CD181">
+        <v>1</v>
+      </c>
     </row>
-    <row r="182" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="182" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -27983,8 +28992,11 @@
       <c r="BY182">
         <v>6</v>
       </c>
+      <c r="CB182">
+        <v>6</v>
+      </c>
     </row>
-    <row r="183" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="183" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -28180,8 +29192,14 @@
       <c r="CA183">
         <v>1</v>
       </c>
+      <c r="CB183">
+        <v>3</v>
+      </c>
+      <c r="CC183">
+        <v>2</v>
+      </c>
     </row>
-    <row r="184" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="184" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -28293,8 +29311,14 @@
       <c r="BZ184">
         <v>1</v>
       </c>
+      <c r="CB184">
+        <v>5</v>
+      </c>
+      <c r="CC184">
+        <v>1</v>
+      </c>
     </row>
-    <row r="185" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="185" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -28460,8 +29484,14 @@
       <c r="CA185">
         <v>2</v>
       </c>
+      <c r="CB185">
+        <v>0</v>
+      </c>
+      <c r="CC185">
+        <v>7</v>
+      </c>
     </row>
-    <row r="186" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="186" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -28615,8 +29645,14 @@
       <c r="BZ186">
         <v>1</v>
       </c>
+      <c r="CB186">
+        <v>6</v>
+      </c>
+      <c r="CC186">
+        <v>1</v>
+      </c>
     </row>
-    <row r="187" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="187" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -28737,8 +29773,14 @@
       <c r="BZ187">
         <v>1</v>
       </c>
+      <c r="CB187">
+        <v>7</v>
+      </c>
+      <c r="CC187">
+        <v>1</v>
+      </c>
     </row>
-    <row r="188" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="188" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B188" t="s">
         <v>4</v>
       </c>
@@ -28901,8 +29943,17 @@
       <c r="CA188">
         <v>1</v>
       </c>
+      <c r="CB188">
+        <v>6</v>
+      </c>
+      <c r="CC188">
+        <v>3</v>
+      </c>
+      <c r="CD188">
+        <v>1</v>
+      </c>
     </row>
-    <row r="189" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="189" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -29080,8 +30131,11 @@
       <c r="BY189">
         <v>2</v>
       </c>
+      <c r="CB189">
+        <v>2</v>
+      </c>
     </row>
-    <row r="190" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="190" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -29253,8 +30307,14 @@
       <c r="BZ190">
         <v>2</v>
       </c>
+      <c r="CB190">
+        <v>3</v>
+      </c>
+      <c r="CC190">
+        <v>2</v>
+      </c>
     </row>
-    <row r="191" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="191" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -29432,8 +30492,14 @@
       <c r="CA191">
         <v>1</v>
       </c>
+      <c r="CB191">
+        <v>0</v>
+      </c>
+      <c r="CC191">
+        <v>5</v>
+      </c>
     </row>
-    <row r="192" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="192" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -29590,8 +30656,14 @@
       <c r="BZ192">
         <v>3</v>
       </c>
+      <c r="CB192">
+        <v>0</v>
+      </c>
+      <c r="CC192">
+        <v>3</v>
+      </c>
     </row>
-    <row r="193" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="193" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -29769,8 +30841,14 @@
       <c r="BZ193">
         <v>4</v>
       </c>
+      <c r="CB193">
+        <v>3</v>
+      </c>
+      <c r="CC193">
+        <v>4</v>
+      </c>
     </row>
-    <row r="194" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="194" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B194" t="s">
         <v>4</v>
       </c>
@@ -29924,8 +31002,14 @@
       <c r="BZ194">
         <v>1</v>
       </c>
+      <c r="CB194">
+        <v>6</v>
+      </c>
+      <c r="CC194">
+        <v>1</v>
+      </c>
     </row>
-    <row r="195" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="195" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -30100,8 +31184,11 @@
       <c r="BY195">
         <v>2</v>
       </c>
+      <c r="CB195">
+        <v>2</v>
+      </c>
     </row>
-    <row r="196" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="196" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -30306,8 +31393,14 @@
       <c r="CA196">
         <v>1</v>
       </c>
+      <c r="CB196">
+        <v>2</v>
+      </c>
+      <c r="CC196">
+        <v>7</v>
+      </c>
     </row>
-    <row r="197" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="197" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -30467,8 +31560,14 @@
       <c r="CA197">
         <v>1</v>
       </c>
+      <c r="CB197">
+        <v>0</v>
+      </c>
+      <c r="CC197">
+        <v>4</v>
+      </c>
     </row>
-    <row r="198" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="198" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -30601,8 +31700,17 @@
       <c r="CA198">
         <v>1</v>
       </c>
+      <c r="CB198">
+        <v>3</v>
+      </c>
+      <c r="CC198">
+        <v>1</v>
+      </c>
+      <c r="CD198">
+        <v>1</v>
+      </c>
     </row>
-    <row r="199" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="199" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -30759,8 +31867,11 @@
       <c r="BY199">
         <v>6</v>
       </c>
+      <c r="CB199">
+        <v>6</v>
+      </c>
     </row>
-    <row r="200" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="200" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B200" t="s">
         <v>4</v>
       </c>
@@ -30902,8 +32013,14 @@
       <c r="BZ200">
         <v>1</v>
       </c>
+      <c r="CB200">
+        <v>6</v>
+      </c>
+      <c r="CC200">
+        <v>1</v>
+      </c>
     </row>
-    <row r="201" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="201" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -31087,8 +32204,14 @@
       <c r="BZ201">
         <v>5</v>
       </c>
+      <c r="CB201">
+        <v>1</v>
+      </c>
+      <c r="CC201">
+        <v>5</v>
+      </c>
     </row>
-    <row r="202" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="202" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -31266,8 +32389,14 @@
       <c r="BZ202">
         <v>1</v>
       </c>
+      <c r="CB202">
+        <v>0</v>
+      </c>
+      <c r="CC202">
+        <v>1</v>
+      </c>
     </row>
-    <row r="203" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="203" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -31436,8 +32565,17 @@
       <c r="CA203">
         <v>1</v>
       </c>
+      <c r="CB203">
+        <v>0</v>
+      </c>
+      <c r="CC203">
+        <v>2</v>
+      </c>
+      <c r="CD203">
+        <v>1</v>
+      </c>
     </row>
-    <row r="204" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="204" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -31540,8 +32678,11 @@
       <c r="BY204">
         <v>6</v>
       </c>
+      <c r="CB204">
+        <v>6</v>
+      </c>
     </row>
-    <row r="205" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="205" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -31722,8 +32863,14 @@
       <c r="BZ205">
         <v>1</v>
       </c>
+      <c r="CB205">
+        <v>9</v>
+      </c>
+      <c r="CC205">
+        <v>1</v>
+      </c>
     </row>
-    <row r="206" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="206" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B206" t="s">
         <v>4</v>
       </c>
@@ -31826,8 +32973,11 @@
       <c r="BY206">
         <v>6</v>
       </c>
+      <c r="CB206">
+        <v>6</v>
+      </c>
     </row>
-    <row r="207" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="207" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -31966,8 +33116,14 @@
       <c r="BZ207">
         <v>2</v>
       </c>
+      <c r="CB207">
+        <v>2</v>
+      </c>
+      <c r="CC207">
+        <v>2</v>
+      </c>
     </row>
-    <row r="208" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="208" spans="2:82" x14ac:dyDescent="0.35">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -32139,8 +33295,14 @@
       <c r="BZ208">
         <v>2</v>
       </c>
+      <c r="CB208">
+        <v>1</v>
+      </c>
+      <c r="CC208">
+        <v>2</v>
+      </c>
     </row>
-    <row r="209" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="209" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B209" t="s">
         <v>3</v>
       </c>
@@ -32297,8 +33459,14 @@
       <c r="CA209">
         <v>2</v>
       </c>
+      <c r="CB209">
+        <v>0</v>
+      </c>
+      <c r="CC209">
+        <v>5</v>
+      </c>
     </row>
-    <row r="210" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="210" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B210" t="s">
         <v>1</v>
       </c>
@@ -32476,8 +33644,14 @@
       <c r="BZ210">
         <v>1</v>
       </c>
+      <c r="CB210">
+        <v>4</v>
+      </c>
+      <c r="CC210">
+        <v>1</v>
+      </c>
     </row>
-    <row r="211" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="211" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B211" t="s">
         <v>4</v>
       </c>
@@ -32631,8 +33805,14 @@
       <c r="BZ211">
         <v>2</v>
       </c>
+      <c r="CB211">
+        <v>3</v>
+      </c>
+      <c r="CC211">
+        <v>2</v>
+      </c>
     </row>
-    <row r="212" spans="2:79" x14ac:dyDescent="0.35">
+    <row r="212" spans="2:81" x14ac:dyDescent="0.35">
       <c r="B212" t="s">
         <v>4</v>
       </c>
@@ -32778,6 +33958,12 @@
         <v>4</v>
       </c>
       <c r="BZ212">
+        <v>1</v>
+      </c>
+      <c r="CB212">
+        <v>5</v>
+      </c>
+      <c r="CC212">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
DOY 126 germinants data collection
</commit_message>
<xml_diff>
--- a/data/germination_data.xlsx
+++ b/data/germination_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\morasoilinoculation\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temporal Ecology Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D69D0C-830E-44DE-AACE-2DB79A438926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{99947861-4AC3-4972-A06A-0496258833AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="122">
   <si>
     <t>seed_species</t>
   </si>
@@ -429,29 +429,38 @@
     <t>doy112: half dead came back to life</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>126_alive</t>
+  </si>
+  <si>
+    <t>126_dead</t>
+  </si>
+  <si>
+    <t>126_halfdead</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -517,7 +526,9 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{6FF63B51-7338-4191-A71A-C86BE581743C}"/>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -530,9 +541,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CD213" totalsRowShown="0">
-  <autoFilter ref="B2:CD213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
-  <tableColumns count="81">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CG213" totalsRowShown="0">
+  <autoFilter ref="B2:CG213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
+  <tableColumns count="84">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
     <tableColumn id="3" xr3:uid="{B695F4B4-8561-9D48-9FF3-12A40CB2B7C7}" name="inoculated_%"/>
@@ -614,6 +625,9 @@
     <tableColumn id="79" xr3:uid="{B9D9BBC8-AB51-4EEE-A4FA-A8D68D32C92F}" name="112_alive"/>
     <tableColumn id="80" xr3:uid="{323A31B7-B3A1-4C31-A41D-DD0B6BCD8E98}" name="112_dead"/>
     <tableColumn id="81" xr3:uid="{CF820F6A-BC57-443F-A0F0-72AC59A5982D}" name="112_halfdead"/>
+    <tableColumn id="82" xr3:uid="{CE3EC9BD-EB21-4BAC-886C-89B8FF48600F}" name="126_alive"/>
+    <tableColumn id="83" xr3:uid="{DA9CFA23-EC52-4220-82CD-9B249E55FE19}" name="126_dead"/>
+    <tableColumn id="84" xr3:uid="{4EC5F6FC-B356-46C6-B57F-3AAEE58C6498}" name="126_halfdead"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -936,15 +950,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:CD212"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B2:CG212"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="14.15234375" customWidth="1"/>
-    <col min="4" max="4" width="17.84375" customWidth="1"/>
+    <col min="3" max="3" width="14.09765625" customWidth="1"/>
+    <col min="4" max="4" width="17.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -1188,8 +1202,17 @@
       <c r="CD2" t="s">
         <v>117</v>
       </c>
+      <c r="CE2" t="s">
+        <v>119</v>
+      </c>
+      <c r="CF2" t="s">
+        <v>120</v>
+      </c>
+      <c r="CG2" t="s">
+        <v>121</v>
+      </c>
     </row>
-    <row r="3" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1379,8 +1402,14 @@
       <c r="CC3">
         <v>2</v>
       </c>
+      <c r="CE3">
+        <v>2</v>
+      </c>
+      <c r="CF3">
+        <v>2</v>
+      </c>
     </row>
-    <row r="4" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1489,8 +1518,14 @@
       <c r="CB4">
         <v>9</v>
       </c>
+      <c r="CE4">
+        <v>6</v>
+      </c>
+      <c r="CG4">
+        <v>3</v>
+      </c>
     </row>
-    <row r="5" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1680,8 +1715,14 @@
       <c r="CC5">
         <v>7</v>
       </c>
+      <c r="CE5">
+        <v>0</v>
+      </c>
+      <c r="CF5">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1790,8 +1831,11 @@
       <c r="CB6">
         <v>9</v>
       </c>
+      <c r="CE6">
+        <v>9</v>
+      </c>
     </row>
-    <row r="7" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -1945,8 +1989,14 @@
       <c r="CC7">
         <v>4</v>
       </c>
+      <c r="CE7">
+        <v>2</v>
+      </c>
+      <c r="CF7">
+        <v>4</v>
+      </c>
     </row>
-    <row r="8" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -2127,8 +2177,14 @@
       <c r="CC8">
         <v>1</v>
       </c>
+      <c r="CE8">
+        <v>6</v>
+      </c>
+      <c r="CF8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2315,8 +2371,14 @@
       <c r="CC9">
         <v>1</v>
       </c>
+      <c r="CE9">
+        <v>6</v>
+      </c>
+      <c r="CF9">
+        <v>1</v>
+      </c>
     </row>
-    <row r="10" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -2431,8 +2493,17 @@
       <c r="CD10">
         <v>1</v>
       </c>
+      <c r="CE10">
+        <v>6</v>
+      </c>
+      <c r="CF10">
+        <v>1</v>
+      </c>
+      <c r="CG10">
+        <v>1</v>
+      </c>
     </row>
-    <row r="11" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -2613,8 +2684,17 @@
       <c r="CC11">
         <v>2</v>
       </c>
+      <c r="CE11">
+        <v>0</v>
+      </c>
+      <c r="CF11">
+        <v>7</v>
+      </c>
+      <c r="CG11">
+        <v>1</v>
+      </c>
     </row>
-    <row r="12" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -2804,8 +2884,14 @@
       <c r="CC12">
         <v>5</v>
       </c>
+      <c r="CE12">
+        <v>4</v>
+      </c>
+      <c r="CF12">
+        <v>5</v>
+      </c>
     </row>
-    <row r="13" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -2983,8 +3069,14 @@
       <c r="CC13">
         <v>3</v>
       </c>
+      <c r="CE13">
+        <v>3</v>
+      </c>
+      <c r="CF13">
+        <v>4</v>
+      </c>
     </row>
-    <row r="14" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -3123,8 +3215,14 @@
       <c r="CC14">
         <v>1</v>
       </c>
+      <c r="CE14">
+        <v>8</v>
+      </c>
+      <c r="CF14">
+        <v>1</v>
+      </c>
     </row>
-    <row r="15" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -3291,8 +3389,14 @@
       <c r="CC15">
         <v>4</v>
       </c>
+      <c r="CE15">
+        <v>4</v>
+      </c>
+      <c r="CF15">
+        <v>4</v>
+      </c>
     </row>
-    <row r="16" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -3444,8 +3548,14 @@
       <c r="CC16">
         <v>1</v>
       </c>
+      <c r="CE16">
+        <v>8</v>
+      </c>
+      <c r="CF16">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -3618,8 +3728,14 @@
       <c r="CB17">
         <v>8</v>
       </c>
+      <c r="CE17">
+        <v>0</v>
+      </c>
+      <c r="CF17">
+        <v>8</v>
+      </c>
     </row>
-    <row r="18" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -3723,8 +3839,14 @@
       <c r="CB18">
         <v>10</v>
       </c>
+      <c r="CE18">
+        <v>9</v>
+      </c>
+      <c r="CG18">
+        <v>1</v>
+      </c>
     </row>
-    <row r="19" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -3915,8 +4037,14 @@
       <c r="CC19">
         <v>6</v>
       </c>
+      <c r="CE19">
+        <v>1</v>
+      </c>
+      <c r="CF19">
+        <v>6</v>
+      </c>
     </row>
-    <row r="20" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -4068,8 +4196,14 @@
       <c r="CC20">
         <v>1</v>
       </c>
+      <c r="CE20">
+        <v>13</v>
+      </c>
+      <c r="CF20">
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -4226,8 +4360,14 @@
       <c r="CC21">
         <v>1</v>
       </c>
+      <c r="CE21">
+        <v>4</v>
+      </c>
+      <c r="CF21">
+        <v>2</v>
+      </c>
     </row>
-    <row r="22" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -4337,8 +4477,14 @@
       <c r="CB22">
         <v>8</v>
       </c>
+      <c r="CE22">
+        <v>7</v>
+      </c>
+      <c r="CG22">
+        <v>1</v>
+      </c>
     </row>
-    <row r="23" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -4517,8 +4663,17 @@
       <c r="CC23">
         <v>2</v>
       </c>
+      <c r="CE23">
+        <v>0</v>
+      </c>
+      <c r="CF23">
+        <v>7</v>
+      </c>
+      <c r="CG23">
+        <v>3</v>
+      </c>
     </row>
-    <row r="24" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -4676,8 +4831,14 @@
       <c r="CC24">
         <v>4</v>
       </c>
+      <c r="CE24">
+        <v>8</v>
+      </c>
+      <c r="CF24">
+        <v>4</v>
+      </c>
     </row>
-    <row r="25" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -4784,8 +4945,11 @@
       <c r="CB25">
         <v>8</v>
       </c>
+      <c r="CE25">
+        <v>8</v>
+      </c>
     </row>
-    <row r="26" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -5009,8 +5173,17 @@
       <c r="CC26">
         <v>5</v>
       </c>
+      <c r="CE26">
+        <v>5</v>
+      </c>
+      <c r="CF26">
+        <v>5</v>
+      </c>
+      <c r="CG26">
+        <v>1</v>
+      </c>
     </row>
-    <row r="27" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -5168,8 +5341,17 @@
       <c r="CC27">
         <v>2</v>
       </c>
+      <c r="CE27">
+        <v>2</v>
+      </c>
+      <c r="CF27">
+        <v>2</v>
+      </c>
+      <c r="CG27">
+        <v>2</v>
+      </c>
     </row>
-    <row r="28" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -5372,8 +5554,14 @@
       <c r="CC28">
         <v>3</v>
       </c>
+      <c r="CE28">
+        <v>7</v>
+      </c>
+      <c r="CF28">
+        <v>3</v>
+      </c>
     </row>
-    <row r="29" spans="2:82" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:85" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>3</v>
       </c>
@@ -5543,8 +5731,17 @@
       <c r="CD29" s="3">
         <v>1</v>
       </c>
+      <c r="CE29" s="3">
+        <v>0</v>
+      </c>
+      <c r="CF29" s="3">
+        <v>3</v>
+      </c>
+      <c r="CG29" s="3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="30" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -5657,8 +5854,11 @@
       <c r="CB30">
         <v>8</v>
       </c>
+      <c r="CE30">
+        <v>8</v>
+      </c>
     </row>
-    <row r="31" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -5843,8 +6043,17 @@
       <c r="CC31">
         <v>3</v>
       </c>
+      <c r="CE31">
+        <v>1</v>
+      </c>
+      <c r="CF31">
+        <v>3</v>
+      </c>
+      <c r="CG31">
+        <v>1</v>
+      </c>
     </row>
-    <row r="32" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -5993,8 +6202,14 @@
       <c r="CC32">
         <v>1</v>
       </c>
+      <c r="CE32">
+        <v>9</v>
+      </c>
+      <c r="CF32">
+        <v>1</v>
+      </c>
     </row>
-    <row r="33" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -6137,8 +6352,14 @@
       <c r="CC33">
         <v>1</v>
       </c>
+      <c r="CE33">
+        <v>7</v>
+      </c>
+      <c r="CF33">
+        <v>2</v>
+      </c>
     </row>
-    <row r="34" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -6275,8 +6496,11 @@
       <c r="CB34">
         <v>6</v>
       </c>
+      <c r="CE34">
+        <v>6</v>
+      </c>
     </row>
-    <row r="35" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -6440,8 +6664,17 @@
       <c r="CC35">
         <v>5</v>
       </c>
+      <c r="CE35">
+        <v>0</v>
+      </c>
+      <c r="CF35">
+        <v>7</v>
+      </c>
+      <c r="CG35">
+        <v>1</v>
+      </c>
     </row>
-    <row r="36" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -6605,8 +6838,14 @@
       <c r="CC36">
         <v>2</v>
       </c>
+      <c r="CE36">
+        <v>8</v>
+      </c>
+      <c r="CF36">
+        <v>2</v>
+      </c>
     </row>
-    <row r="37" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -6716,8 +6955,17 @@
       <c r="CD37">
         <v>1</v>
       </c>
+      <c r="CE37">
+        <v>4</v>
+      </c>
+      <c r="CF37">
+        <v>1</v>
+      </c>
+      <c r="CG37">
+        <v>4</v>
+      </c>
     </row>
-    <row r="38" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -6920,8 +7168,17 @@
       <c r="CC38">
         <v>3</v>
       </c>
+      <c r="CE38">
+        <v>3</v>
+      </c>
+      <c r="CF38">
+        <v>3</v>
+      </c>
+      <c r="CG38">
+        <v>2</v>
+      </c>
     </row>
-    <row r="39" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -7106,8 +7363,14 @@
       <c r="CC39">
         <v>4</v>
       </c>
+      <c r="CE39">
+        <v>2</v>
+      </c>
+      <c r="CF39">
+        <v>4</v>
+      </c>
     </row>
-    <row r="40" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -7304,8 +7567,17 @@
       <c r="CC40">
         <v>6</v>
       </c>
+      <c r="CE40">
+        <v>3</v>
+      </c>
+      <c r="CF40">
+        <v>6</v>
+      </c>
+      <c r="CG40">
+        <v>1</v>
+      </c>
     </row>
-    <row r="41" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -7469,8 +7741,17 @@
       <c r="CC41">
         <v>2</v>
       </c>
+      <c r="CE41">
+        <v>0</v>
+      </c>
+      <c r="CF41">
+        <v>4</v>
+      </c>
+      <c r="CG41">
+        <v>2</v>
+      </c>
     </row>
-    <row r="42" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -7586,8 +7867,14 @@
       <c r="CB42">
         <v>7</v>
       </c>
+      <c r="CE42">
+        <v>5</v>
+      </c>
+      <c r="CG42">
+        <v>2</v>
+      </c>
     </row>
-    <row r="43" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -7775,8 +8062,17 @@
       <c r="CD43">
         <v>1</v>
       </c>
+      <c r="CE43">
+        <v>1</v>
+      </c>
+      <c r="CF43">
+        <v>7</v>
+      </c>
+      <c r="CG43">
+        <v>1</v>
+      </c>
     </row>
-    <row r="44" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -7877,8 +8173,14 @@
       <c r="CB44">
         <v>6</v>
       </c>
+      <c r="CE44">
+        <v>5</v>
+      </c>
+      <c r="CG44">
+        <v>1</v>
+      </c>
     </row>
-    <row r="45" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -8111,8 +8413,17 @@
       <c r="CD45">
         <v>1</v>
       </c>
+      <c r="CE45">
+        <v>0</v>
+      </c>
+      <c r="CF45">
+        <v>6</v>
+      </c>
+      <c r="CG45">
+        <v>3</v>
+      </c>
     </row>
-    <row r="46" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -8225,8 +8536,11 @@
       <c r="CB46">
         <v>6</v>
       </c>
+      <c r="CE46">
+        <v>6</v>
+      </c>
     </row>
-    <row r="47" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -8366,8 +8680,14 @@
       <c r="CC47">
         <v>9</v>
       </c>
+      <c r="CE47">
+        <v>0</v>
+      </c>
+      <c r="CF47">
+        <v>9</v>
+      </c>
     </row>
-    <row r="48" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -8573,8 +8893,17 @@
       <c r="CC48">
         <v>6</v>
       </c>
+      <c r="CE48">
+        <v>1</v>
+      </c>
+      <c r="CF48">
+        <v>9</v>
+      </c>
+      <c r="CG48">
+        <v>1</v>
+      </c>
     </row>
-    <row r="49" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -8687,8 +9016,14 @@
       <c r="CD49">
         <v>1</v>
       </c>
+      <c r="CE49">
+        <v>6</v>
+      </c>
+      <c r="CF49">
+        <v>2</v>
+      </c>
     </row>
-    <row r="50" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -8897,8 +9232,14 @@
       <c r="CC50">
         <v>1</v>
       </c>
+      <c r="CE50">
+        <v>7</v>
+      </c>
+      <c r="CF50">
+        <v>1</v>
+      </c>
     </row>
-    <row r="51" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -9092,8 +9433,17 @@
       <c r="CC51">
         <v>2</v>
       </c>
+      <c r="CE51">
+        <v>2</v>
+      </c>
+      <c r="CF51">
+        <v>2</v>
+      </c>
+      <c r="CG51">
+        <v>2</v>
+      </c>
     </row>
-    <row r="52" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -9200,8 +9550,11 @@
       <c r="CB52">
         <v>6</v>
       </c>
+      <c r="CE52">
+        <v>6</v>
+      </c>
     </row>
-    <row r="53" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -9374,8 +9727,14 @@
       <c r="CC53">
         <v>1</v>
       </c>
+      <c r="CE53">
+        <v>2</v>
+      </c>
+      <c r="CF53">
+        <v>2</v>
+      </c>
     </row>
-    <row r="54" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -9485,8 +9844,14 @@
       <c r="CB54">
         <v>5</v>
       </c>
+      <c r="CE54">
+        <v>4</v>
+      </c>
+      <c r="CG54">
+        <v>1</v>
+      </c>
     </row>
-    <row r="55" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -9653,8 +10018,17 @@
       <c r="CC55">
         <v>4</v>
       </c>
+      <c r="CE55">
+        <v>0</v>
+      </c>
+      <c r="CF55">
+        <v>4</v>
+      </c>
+      <c r="CG55">
+        <v>2</v>
+      </c>
     </row>
-    <row r="56" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -9764,8 +10138,14 @@
       <c r="CD56">
         <v>1</v>
       </c>
+      <c r="CE56">
+        <v>9</v>
+      </c>
+      <c r="CG56">
+        <v>1</v>
+      </c>
     </row>
-    <row r="57" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -9887,8 +10267,14 @@
       <c r="CC57">
         <v>1</v>
       </c>
+      <c r="CE57">
+        <v>6</v>
+      </c>
+      <c r="CF57">
+        <v>1</v>
+      </c>
     </row>
-    <row r="58" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -10001,8 +10387,11 @@
       <c r="CB58">
         <v>6</v>
       </c>
+      <c r="CE58">
+        <v>6</v>
+      </c>
     </row>
-    <row r="59" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -10106,8 +10495,17 @@
       <c r="CB59">
         <v>7</v>
       </c>
+      <c r="CE59">
+        <v>0</v>
+      </c>
+      <c r="CF59">
+        <v>6</v>
+      </c>
+      <c r="CG59">
+        <v>1</v>
+      </c>
     </row>
-    <row r="60" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -10274,8 +10672,14 @@
       <c r="CC60">
         <v>2</v>
       </c>
+      <c r="CE60">
+        <v>7</v>
+      </c>
+      <c r="CF60">
+        <v>2</v>
+      </c>
     </row>
-    <row r="61" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -10391,8 +10795,14 @@
       <c r="CD61">
         <v>1</v>
       </c>
+      <c r="CE61">
+        <v>6</v>
+      </c>
+      <c r="CF61">
+        <v>1</v>
+      </c>
     </row>
-    <row r="62" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -10589,8 +10999,14 @@
       <c r="CC62">
         <v>2</v>
       </c>
+      <c r="CE62">
+        <v>3</v>
+      </c>
+      <c r="CF62">
+        <v>2</v>
+      </c>
     </row>
-    <row r="63" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -10781,8 +11197,17 @@
       <c r="CC63">
         <v>5</v>
       </c>
+      <c r="CE63">
+        <v>2</v>
+      </c>
+      <c r="CF63">
+        <v>5</v>
+      </c>
+      <c r="CG63">
+        <v>2</v>
+      </c>
     </row>
-    <row r="64" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -10943,8 +11368,17 @@
       <c r="CC64">
         <v>3</v>
       </c>
+      <c r="CE64">
+        <v>6</v>
+      </c>
+      <c r="CF64">
+        <v>3</v>
+      </c>
+      <c r="CG64">
+        <v>1</v>
+      </c>
     </row>
-    <row r="65" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -11108,8 +11542,17 @@
       <c r="CC65">
         <v>2</v>
       </c>
+      <c r="CE65">
+        <v>0</v>
+      </c>
+      <c r="CF65">
+        <v>5</v>
+      </c>
+      <c r="CG65">
+        <v>1</v>
+      </c>
     </row>
-    <row r="66" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -11222,8 +11665,14 @@
       <c r="CB66">
         <v>5</v>
       </c>
+      <c r="CE66">
+        <v>4</v>
+      </c>
+      <c r="CG66">
+        <v>1</v>
+      </c>
     </row>
-    <row r="67" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -11414,8 +11863,17 @@
       <c r="CC67">
         <v>8</v>
       </c>
+      <c r="CE67">
+        <v>0</v>
+      </c>
+      <c r="CF67">
+        <v>8</v>
+      </c>
+      <c r="CG67">
+        <v>2</v>
+      </c>
     </row>
-    <row r="68" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -11516,8 +11974,14 @@
       <c r="CB68">
         <v>11</v>
       </c>
+      <c r="CE68">
+        <v>9</v>
+      </c>
+      <c r="CG68">
+        <v>2</v>
+      </c>
     </row>
-    <row r="69" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -11624,8 +12088,11 @@
       <c r="CB69">
         <v>9</v>
       </c>
+      <c r="CE69">
+        <v>9</v>
+      </c>
     </row>
-    <row r="70" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -11741,8 +12208,11 @@
       <c r="CB70">
         <v>8</v>
       </c>
+      <c r="CE70">
+        <v>8</v>
+      </c>
     </row>
-    <row r="71" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -11927,8 +12397,17 @@
       <c r="CC71">
         <v>4</v>
       </c>
+      <c r="CE71">
+        <v>0</v>
+      </c>
+      <c r="CF71">
+        <v>9</v>
+      </c>
+      <c r="CG71">
+        <v>1</v>
+      </c>
     </row>
-    <row r="72" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -12104,8 +12583,14 @@
       <c r="CC72">
         <v>1</v>
       </c>
+      <c r="CE72">
+        <v>6</v>
+      </c>
+      <c r="CF72">
+        <v>1</v>
+      </c>
     </row>
-    <row r="73" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -12212,8 +12697,11 @@
       <c r="CB73">
         <v>10</v>
       </c>
+      <c r="CE73">
+        <v>10</v>
+      </c>
     </row>
-    <row r="74" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -12329,8 +12817,11 @@
       <c r="CB74">
         <v>9</v>
       </c>
+      <c r="CE74">
+        <v>9</v>
+      </c>
     </row>
-    <row r="75" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -12500,8 +12991,17 @@
       <c r="CD75">
         <v>1</v>
       </c>
+      <c r="CE75">
+        <v>4</v>
+      </c>
+      <c r="CF75">
+        <v>3</v>
+      </c>
+      <c r="CG75">
+        <v>2</v>
+      </c>
     </row>
-    <row r="76" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -12695,8 +13195,14 @@
       <c r="CC76">
         <v>1</v>
       </c>
+      <c r="CE76">
+        <v>7</v>
+      </c>
+      <c r="CF76">
+        <v>1</v>
+      </c>
     </row>
-    <row r="77" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -12857,8 +13363,14 @@
       <c r="CC77">
         <v>3</v>
       </c>
+      <c r="CE77">
+        <v>0</v>
+      </c>
+      <c r="CF77">
+        <v>7</v>
+      </c>
     </row>
-    <row r="78" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -12968,8 +13480,14 @@
       <c r="CB78">
         <v>7</v>
       </c>
+      <c r="CE78">
+        <v>4</v>
+      </c>
+      <c r="CG78">
+        <v>3</v>
+      </c>
     </row>
-    <row r="79" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -13157,8 +13675,14 @@
       <c r="CC79">
         <v>7</v>
       </c>
+      <c r="CE79">
+        <v>2</v>
+      </c>
+      <c r="CF79">
+        <v>7</v>
+      </c>
     </row>
-    <row r="80" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -13316,8 +13840,17 @@
       <c r="CC80">
         <v>1</v>
       </c>
+      <c r="CE80">
+        <v>7</v>
+      </c>
+      <c r="CF80">
+        <v>1</v>
+      </c>
+      <c r="CG80">
+        <v>2</v>
+      </c>
     </row>
-    <row r="81" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -13487,8 +14020,14 @@
       <c r="CC81">
         <v>2</v>
       </c>
+      <c r="CE81">
+        <v>5</v>
+      </c>
+      <c r="CF81">
+        <v>2</v>
+      </c>
     </row>
-    <row r="82" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -13694,8 +14233,17 @@
       <c r="CC82">
         <v>4</v>
       </c>
+      <c r="CE82">
+        <v>5</v>
+      </c>
+      <c r="CF82">
+        <v>4</v>
+      </c>
+      <c r="CG82">
+        <v>1</v>
+      </c>
     </row>
-    <row r="83" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -13883,8 +14431,17 @@
       <c r="CC83">
         <v>4</v>
       </c>
+      <c r="CE83">
+        <v>0</v>
+      </c>
+      <c r="CF83">
+        <v>8</v>
+      </c>
+      <c r="CG83">
+        <v>1</v>
+      </c>
     </row>
-    <row r="84" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -14072,8 +14629,17 @@
       <c r="CC84">
         <v>2</v>
       </c>
+      <c r="CE84">
+        <v>0</v>
+      </c>
+      <c r="CF84">
+        <v>8</v>
+      </c>
+      <c r="CG84">
+        <v>1</v>
+      </c>
     </row>
-    <row r="85" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -14261,8 +14827,17 @@
       <c r="CC85">
         <v>3</v>
       </c>
+      <c r="CE85">
+        <v>1</v>
+      </c>
+      <c r="CF85">
+        <v>3</v>
+      </c>
+      <c r="CG85">
+        <v>2</v>
+      </c>
     </row>
-    <row r="86" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -14429,8 +15004,14 @@
       <c r="CC86">
         <v>1</v>
       </c>
+      <c r="CE86">
+        <v>8</v>
+      </c>
+      <c r="CF86">
+        <v>1</v>
+      </c>
     </row>
-    <row r="87" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -14621,8 +15202,14 @@
       <c r="CC87">
         <v>2</v>
       </c>
+      <c r="CE87">
+        <v>5</v>
+      </c>
+      <c r="CF87">
+        <v>2</v>
+      </c>
     </row>
-    <row r="88" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -14798,8 +15385,17 @@
       <c r="CC88">
         <v>3</v>
       </c>
+      <c r="CE88">
+        <v>4</v>
+      </c>
+      <c r="CF88">
+        <v>3</v>
+      </c>
+      <c r="CG88">
+        <v>2</v>
+      </c>
     </row>
-    <row r="89" spans="2:81" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:85" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>3</v>
       </c>
@@ -14951,8 +15547,17 @@
       <c r="CC89" s="3">
         <v>2</v>
       </c>
+      <c r="CE89" s="3">
+        <v>1</v>
+      </c>
+      <c r="CF89" s="3">
+        <v>3</v>
+      </c>
+      <c r="CG89" s="3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="90" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -15062,8 +15667,14 @@
       <c r="CB90">
         <v>8</v>
       </c>
+      <c r="CE90">
+        <v>6</v>
+      </c>
+      <c r="CG90">
+        <v>2</v>
+      </c>
     </row>
-    <row r="91" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -15263,8 +15874,14 @@
       <c r="CC91">
         <v>2</v>
       </c>
+      <c r="CE91">
+        <v>3</v>
+      </c>
+      <c r="CF91">
+        <v>3</v>
+      </c>
     </row>
-    <row r="92" spans="2:81" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:85" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>1</v>
       </c>
@@ -15446,8 +16063,14 @@
       <c r="CC92" s="3">
         <v>3</v>
       </c>
+      <c r="CE92" s="3">
+        <v>5</v>
+      </c>
+      <c r="CF92" s="3">
+        <v>3</v>
+      </c>
     </row>
-    <row r="93" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -15587,8 +16210,14 @@
       <c r="CC93">
         <v>1</v>
       </c>
+      <c r="CE93">
+        <v>7</v>
+      </c>
+      <c r="CF93">
+        <v>2</v>
+      </c>
     </row>
-    <row r="94" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -15701,8 +16330,11 @@
       <c r="CB94">
         <v>7</v>
       </c>
+      <c r="CE94">
+        <v>7</v>
+      </c>
     </row>
-    <row r="95" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -15848,8 +16480,17 @@
       <c r="CC95">
         <v>3</v>
       </c>
+      <c r="CE95">
+        <v>0</v>
+      </c>
+      <c r="CF95">
+        <v>6</v>
+      </c>
+      <c r="CG95">
+        <v>2</v>
+      </c>
     </row>
-    <row r="96" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -16019,8 +16660,17 @@
       <c r="CC96">
         <v>2</v>
       </c>
+      <c r="CE96">
+        <v>7</v>
+      </c>
+      <c r="CF96">
+        <v>2</v>
+      </c>
+      <c r="CG96">
+        <v>1</v>
+      </c>
     </row>
-    <row r="97" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -16130,8 +16780,17 @@
       <c r="CB97">
         <v>8</v>
       </c>
+      <c r="CE97">
+        <v>6</v>
+      </c>
+      <c r="CF97">
+        <v>1</v>
+      </c>
+      <c r="CG97">
+        <v>1</v>
+      </c>
     </row>
-    <row r="98" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -16301,8 +16960,14 @@
       <c r="CC98">
         <v>2</v>
       </c>
+      <c r="CE98">
+        <v>5</v>
+      </c>
+      <c r="CF98">
+        <v>2</v>
+      </c>
     </row>
-    <row r="99" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -16427,8 +17092,14 @@
       <c r="CC99">
         <v>1</v>
       </c>
+      <c r="CE99">
+        <v>2</v>
+      </c>
+      <c r="CF99">
+        <v>1</v>
+      </c>
     </row>
-    <row r="100" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -16538,8 +17209,14 @@
       <c r="CD100">
         <v>1</v>
       </c>
+      <c r="CE100">
+        <v>6</v>
+      </c>
+      <c r="CG100">
+        <v>2</v>
+      </c>
     </row>
-    <row r="101" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -16697,8 +17374,14 @@
       <c r="CC101">
         <v>4</v>
       </c>
+      <c r="CE101">
+        <v>1</v>
+      </c>
+      <c r="CF101">
+        <v>4</v>
+      </c>
     </row>
-    <row r="102" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -16808,8 +17491,11 @@
       <c r="CB102">
         <v>7</v>
       </c>
+      <c r="CE102">
+        <v>7</v>
+      </c>
     </row>
-    <row r="103" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -16988,8 +17674,14 @@
       <c r="CC103">
         <v>4</v>
       </c>
+      <c r="CE103">
+        <v>0</v>
+      </c>
+      <c r="CF103">
+        <v>6</v>
+      </c>
     </row>
-    <row r="104" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -17159,8 +17851,17 @@
       <c r="CC104">
         <v>3</v>
       </c>
+      <c r="CE104">
+        <v>6</v>
+      </c>
+      <c r="CF104">
+        <v>3</v>
+      </c>
+      <c r="CG104">
+        <v>1</v>
+      </c>
     </row>
-    <row r="105" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -17324,8 +18025,17 @@
       <c r="CC105">
         <v>3</v>
       </c>
+      <c r="CE105">
+        <v>1</v>
+      </c>
+      <c r="CF105">
+        <v>3</v>
+      </c>
+      <c r="CG105">
+        <v>2</v>
+      </c>
     </row>
-    <row r="106" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -17480,8 +18190,17 @@
       <c r="CB106">
         <v>8</v>
       </c>
+      <c r="CE106">
+        <v>2</v>
+      </c>
+      <c r="CF106">
+        <v>5</v>
+      </c>
+      <c r="CG106">
+        <v>1</v>
+      </c>
     </row>
-    <row r="107" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -17657,8 +18376,17 @@
       <c r="CC107">
         <v>1</v>
       </c>
+      <c r="CE107">
+        <v>0</v>
+      </c>
+      <c r="CF107">
+        <v>4</v>
+      </c>
+      <c r="CG107">
+        <v>1</v>
+      </c>
     </row>
-    <row r="108" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -17822,8 +18550,14 @@
       <c r="CD108">
         <v>1</v>
       </c>
+      <c r="CE108">
+        <v>6</v>
+      </c>
+      <c r="CF108">
+        <v>4</v>
+      </c>
     </row>
-    <row r="109" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -18005,8 +18739,14 @@
       <c r="CC109">
         <v>9</v>
       </c>
+      <c r="CE109">
+        <v>0</v>
+      </c>
+      <c r="CF109">
+        <v>9</v>
+      </c>
     </row>
-    <row r="110" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -18191,8 +18931,14 @@
       <c r="CC110">
         <v>3</v>
       </c>
+      <c r="CE110">
+        <v>6</v>
+      </c>
+      <c r="CF110">
+        <v>3</v>
+      </c>
     </row>
-    <row r="111" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -18356,8 +19102,17 @@
       <c r="CC111">
         <v>4</v>
       </c>
+      <c r="CE111">
+        <v>3</v>
+      </c>
+      <c r="CF111">
+        <v>3</v>
+      </c>
+      <c r="CG111">
+        <v>2</v>
+      </c>
     </row>
-    <row r="112" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -18527,8 +19282,17 @@
       <c r="CC112">
         <v>2</v>
       </c>
+      <c r="CE112">
+        <v>4</v>
+      </c>
+      <c r="CF112">
+        <v>2</v>
+      </c>
+      <c r="CG112">
+        <v>2</v>
+      </c>
     </row>
-    <row r="113" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -18713,8 +19477,14 @@
       <c r="CC113">
         <v>2</v>
       </c>
+      <c r="CE113">
+        <v>4</v>
+      </c>
+      <c r="CF113">
+        <v>2</v>
+      </c>
     </row>
-    <row r="114" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -18824,8 +19594,14 @@
       <c r="CB114">
         <v>8</v>
       </c>
+      <c r="CE114">
+        <v>2</v>
+      </c>
+      <c r="CG114">
+        <v>6</v>
+      </c>
     </row>
-    <row r="115" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -19013,8 +19789,14 @@
       <c r="CC115">
         <v>3</v>
       </c>
+      <c r="CE115">
+        <v>0</v>
+      </c>
+      <c r="CF115">
+        <v>4</v>
+      </c>
     </row>
-    <row r="116" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -19184,8 +19966,14 @@
       <c r="CC116">
         <v>2</v>
       </c>
+      <c r="CE116">
+        <v>5</v>
+      </c>
+      <c r="CF116">
+        <v>3</v>
+      </c>
     </row>
-    <row r="117" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -19364,8 +20152,14 @@
       <c r="CC117">
         <v>4</v>
       </c>
+      <c r="CE117">
+        <v>1</v>
+      </c>
+      <c r="CF117">
+        <v>4</v>
+      </c>
     </row>
-    <row r="118" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -19479,8 +20273,17 @@
       <c r="CB118">
         <v>6</v>
       </c>
+      <c r="CE118">
+        <v>2</v>
+      </c>
+      <c r="CF118">
+        <v>2</v>
+      </c>
+      <c r="CG118">
+        <v>2</v>
+      </c>
     </row>
-    <row r="119" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -19596,8 +20399,17 @@
       <c r="CD119">
         <v>1</v>
       </c>
+      <c r="CE119">
+        <v>0</v>
+      </c>
+      <c r="CF119">
+        <v>3</v>
+      </c>
+      <c r="CG119">
+        <v>4</v>
+      </c>
     </row>
-    <row r="120" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -19704,8 +20516,17 @@
       <c r="CB120">
         <v>10</v>
       </c>
+      <c r="CE120">
+        <v>4</v>
+      </c>
+      <c r="CF120">
+        <v>4</v>
+      </c>
+      <c r="CG120">
+        <v>2</v>
+      </c>
     </row>
-    <row r="121" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -19815,8 +20636,11 @@
       <c r="CB121">
         <v>8</v>
       </c>
+      <c r="CE121">
+        <v>8</v>
+      </c>
     </row>
-    <row r="122" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -19929,8 +20753,14 @@
       <c r="CB122">
         <v>6</v>
       </c>
+      <c r="CE122">
+        <v>5</v>
+      </c>
+      <c r="CG122">
+        <v>1</v>
+      </c>
     </row>
-    <row r="123" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -20097,8 +20927,14 @@
       <c r="CC123">
         <v>3</v>
       </c>
+      <c r="CE123">
+        <v>3</v>
+      </c>
+      <c r="CF123">
+        <v>3</v>
+      </c>
     </row>
-    <row r="124" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -20295,8 +21131,17 @@
       <c r="CC124">
         <v>4</v>
       </c>
+      <c r="CE124">
+        <v>4</v>
+      </c>
+      <c r="CF124">
+        <v>4</v>
+      </c>
+      <c r="CG124">
+        <v>1</v>
+      </c>
     </row>
-    <row r="125" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -20490,8 +21335,14 @@
       <c r="CC125">
         <v>6</v>
       </c>
+      <c r="CE125">
+        <v>0</v>
+      </c>
+      <c r="CF125">
+        <v>6</v>
+      </c>
     </row>
-    <row r="126" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -20664,8 +21515,14 @@
       <c r="CC126">
         <v>1</v>
       </c>
+      <c r="CE126">
+        <v>3</v>
+      </c>
+      <c r="CF126">
+        <v>3</v>
+      </c>
     </row>
-    <row r="127" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -20835,8 +21692,14 @@
       <c r="CC127">
         <v>2</v>
       </c>
+      <c r="CE127">
+        <v>0</v>
+      </c>
+      <c r="CF127">
+        <v>3</v>
+      </c>
     </row>
-    <row r="128" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -20937,8 +21800,14 @@
       <c r="CB128">
         <v>7</v>
       </c>
+      <c r="CE128">
+        <v>3</v>
+      </c>
+      <c r="CF128">
+        <v>4</v>
+      </c>
     </row>
-    <row r="129" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="129" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -21123,8 +21992,14 @@
       <c r="CC129">
         <v>4</v>
       </c>
+      <c r="CE129">
+        <v>1</v>
+      </c>
+      <c r="CF129">
+        <v>5</v>
+      </c>
     </row>
-    <row r="130" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="130" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -21240,8 +22115,17 @@
       <c r="CC130">
         <v>4</v>
       </c>
+      <c r="CE130">
+        <v>0</v>
+      </c>
+      <c r="CF130">
+        <v>8</v>
+      </c>
+      <c r="CG130">
+        <v>2</v>
+      </c>
     </row>
-    <row r="131" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="131" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -21423,8 +22307,17 @@
       <c r="CD131">
         <v>1</v>
       </c>
+      <c r="CE131">
+        <v>1</v>
+      </c>
+      <c r="CF131">
+        <v>4</v>
+      </c>
+      <c r="CG131">
+        <v>5</v>
+      </c>
     </row>
-    <row r="132" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="132" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -21531,8 +22424,17 @@
       <c r="CC132">
         <v>1</v>
       </c>
+      <c r="CE132">
+        <v>3</v>
+      </c>
+      <c r="CF132">
+        <v>2</v>
+      </c>
+      <c r="CG132">
+        <v>1</v>
+      </c>
     </row>
-    <row r="133" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="133" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -21672,8 +22574,17 @@
       <c r="CC133">
         <v>1</v>
       </c>
+      <c r="CE133">
+        <v>1</v>
+      </c>
+      <c r="CF133">
+        <v>1</v>
+      </c>
+      <c r="CG133">
+        <v>5</v>
+      </c>
     </row>
-    <row r="134" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="134" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -21810,8 +22721,17 @@
       <c r="CC134">
         <v>1</v>
       </c>
+      <c r="CE134">
+        <v>6</v>
+      </c>
+      <c r="CF134">
+        <v>1</v>
+      </c>
+      <c r="CG134">
+        <v>3</v>
+      </c>
     </row>
-    <row r="135" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="135" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -21972,8 +22892,17 @@
       <c r="CC135">
         <v>5</v>
       </c>
+      <c r="CE135">
+        <v>2</v>
+      </c>
+      <c r="CF135">
+        <v>5</v>
+      </c>
+      <c r="CG135">
+        <v>1</v>
+      </c>
     </row>
-    <row r="136" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="136" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -22125,8 +23054,17 @@
       <c r="CC136">
         <v>1</v>
       </c>
+      <c r="CE136">
+        <v>5</v>
+      </c>
+      <c r="CF136">
+        <v>1</v>
+      </c>
+      <c r="CG136">
+        <v>1</v>
+      </c>
     </row>
-    <row r="137" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="137" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -22287,8 +23225,14 @@
       <c r="CC137">
         <v>2</v>
       </c>
+      <c r="CE137">
+        <v>3</v>
+      </c>
+      <c r="CF137">
+        <v>2</v>
+      </c>
     </row>
-    <row r="138" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="138" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -22464,8 +23408,17 @@
       <c r="CC138">
         <v>1</v>
       </c>
+      <c r="CE138">
+        <v>0</v>
+      </c>
+      <c r="CF138">
+        <v>3</v>
+      </c>
+      <c r="CG138">
+        <v>4</v>
+      </c>
     </row>
-    <row r="139" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="139" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -22626,8 +23579,14 @@
       <c r="CC139">
         <v>1</v>
       </c>
+      <c r="CE139">
+        <v>0</v>
+      </c>
+      <c r="CF139">
+        <v>5</v>
+      </c>
     </row>
-    <row r="140" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="140" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -22737,8 +23696,17 @@
       <c r="CC140">
         <v>7</v>
       </c>
+      <c r="CE140">
+        <v>0</v>
+      </c>
+      <c r="CF140">
+        <v>7</v>
+      </c>
+      <c r="CG140">
+        <v>2</v>
+      </c>
     </row>
-    <row r="141" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="141" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -22935,8 +23903,14 @@
       <c r="CC141">
         <v>4</v>
       </c>
+      <c r="CE141">
+        <v>4</v>
+      </c>
+      <c r="CF141">
+        <v>4</v>
+      </c>
     </row>
-    <row r="142" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="142" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -23130,8 +24104,14 @@
       <c r="CC142">
         <v>5</v>
       </c>
+      <c r="CE142">
+        <v>1</v>
+      </c>
+      <c r="CF142">
+        <v>7</v>
+      </c>
     </row>
-    <row r="143" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="143" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -23280,8 +24260,17 @@
       <c r="CC143">
         <v>3</v>
       </c>
+      <c r="CE143">
+        <v>3</v>
+      </c>
+      <c r="CF143">
+        <v>3</v>
+      </c>
+      <c r="CG143">
+        <v>5</v>
+      </c>
     </row>
-    <row r="144" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="144" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -23388,8 +24377,14 @@
       <c r="CC144">
         <v>2</v>
       </c>
+      <c r="CE144">
+        <v>0</v>
+      </c>
+      <c r="CF144">
+        <v>7</v>
+      </c>
     </row>
-    <row r="145" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="145" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -23502,8 +24497,14 @@
       <c r="CC145">
         <v>1</v>
       </c>
+      <c r="CE145">
+        <v>3</v>
+      </c>
+      <c r="CF145">
+        <v>5</v>
+      </c>
     </row>
-    <row r="146" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="146" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -23703,8 +24704,17 @@
       <c r="CC146">
         <v>2</v>
       </c>
+      <c r="CE146">
+        <v>5</v>
+      </c>
+      <c r="CF146">
+        <v>2</v>
+      </c>
+      <c r="CG146">
+        <v>3</v>
+      </c>
     </row>
-    <row r="147" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="147" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -23895,8 +24905,17 @@
       <c r="CC147">
         <v>3</v>
       </c>
+      <c r="CE147">
+        <v>1</v>
+      </c>
+      <c r="CF147">
+        <v>2</v>
+      </c>
+      <c r="CG147">
+        <v>1</v>
+      </c>
     </row>
-    <row r="148" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="148" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -24003,8 +25022,14 @@
       <c r="CB148">
         <v>9</v>
       </c>
+      <c r="CE148">
+        <v>8</v>
+      </c>
+      <c r="CG148">
+        <v>1</v>
+      </c>
     </row>
-    <row r="149" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="149" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -24195,8 +25220,17 @@
       <c r="CD149">
         <v>2</v>
       </c>
+      <c r="CE149">
+        <v>1</v>
+      </c>
+      <c r="CF149">
+        <v>2</v>
+      </c>
+      <c r="CG149">
+        <v>2</v>
+      </c>
     </row>
-    <row r="150" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="150" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -24387,8 +25421,14 @@
       <c r="CC150">
         <v>1</v>
       </c>
+      <c r="CE150">
+        <v>8</v>
+      </c>
+      <c r="CF150">
+        <v>1</v>
+      </c>
     </row>
-    <row r="151" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="151" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -24549,8 +25589,17 @@
       <c r="CC151">
         <v>6</v>
       </c>
+      <c r="CE151">
+        <v>0</v>
+      </c>
+      <c r="CF151">
+        <v>6</v>
+      </c>
+      <c r="CG151">
+        <v>4</v>
+      </c>
     </row>
-    <row r="152" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="152" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -24651,8 +25700,11 @@
       <c r="CB152">
         <v>9</v>
       </c>
+      <c r="CE152">
+        <v>9</v>
+      </c>
     </row>
-    <row r="153" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="153" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -24807,8 +25859,17 @@
       <c r="CC153">
         <v>1</v>
       </c>
+      <c r="CE153">
+        <v>3</v>
+      </c>
+      <c r="CF153">
+        <v>1</v>
+      </c>
+      <c r="CG153">
+        <v>2</v>
+      </c>
     </row>
-    <row r="154" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="154" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -25026,8 +26087,17 @@
       <c r="CD154">
         <v>1</v>
       </c>
+      <c r="CE154">
+        <v>3</v>
+      </c>
+      <c r="CF154">
+        <v>3</v>
+      </c>
+      <c r="CG154">
+        <v>2</v>
+      </c>
     </row>
-    <row r="155" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="155" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -25194,8 +26264,17 @@
       <c r="CC155">
         <v>3</v>
       </c>
+      <c r="CE155">
+        <v>4</v>
+      </c>
+      <c r="CF155">
+        <v>4</v>
+      </c>
+      <c r="CG155">
+        <v>1</v>
+      </c>
     </row>
-    <row r="156" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="156" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -25302,8 +26381,14 @@
       <c r="CB156">
         <v>6</v>
       </c>
+      <c r="CE156">
+        <v>4</v>
+      </c>
+      <c r="CF156">
+        <v>2</v>
+      </c>
     </row>
-    <row r="157" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="157" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -25413,8 +26498,11 @@
       <c r="CB157">
         <v>6</v>
       </c>
+      <c r="CE157">
+        <v>6</v>
+      </c>
     </row>
-    <row r="158" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="158" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -25548,8 +26636,17 @@
       <c r="CC158">
         <v>2</v>
       </c>
+      <c r="CE158">
+        <v>4</v>
+      </c>
+      <c r="CF158">
+        <v>2</v>
+      </c>
+      <c r="CG158">
+        <v>2</v>
+      </c>
     </row>
-    <row r="159" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="159" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -25731,8 +26828,17 @@
       <c r="CC159">
         <v>3</v>
       </c>
+      <c r="CE159">
+        <v>0</v>
+      </c>
+      <c r="CF159">
+        <v>3</v>
+      </c>
+      <c r="CG159">
+        <v>2</v>
+      </c>
     </row>
-    <row r="160" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="160" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -25839,8 +26945,14 @@
       <c r="CB160">
         <v>9</v>
       </c>
+      <c r="CE160">
+        <v>8</v>
+      </c>
+      <c r="CG160">
+        <v>1</v>
+      </c>
     </row>
-    <row r="161" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="161" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -26046,8 +27158,14 @@
       <c r="CC161">
         <v>6</v>
       </c>
+      <c r="CE161">
+        <v>1</v>
+      </c>
+      <c r="CF161">
+        <v>6</v>
+      </c>
     </row>
-    <row r="162" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="162" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -26157,8 +27275,11 @@
       <c r="CB162">
         <v>8</v>
       </c>
+      <c r="CE162">
+        <v>8</v>
+      </c>
     </row>
-    <row r="163" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="163" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -26325,8 +27446,14 @@
       <c r="CC163">
         <v>7</v>
       </c>
+      <c r="CE163">
+        <v>0</v>
+      </c>
+      <c r="CF163">
+        <v>8</v>
+      </c>
     </row>
-    <row r="164" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="164" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -26427,8 +27554,17 @@
       <c r="CB164">
         <v>9</v>
       </c>
+      <c r="CE164">
+        <v>5</v>
+      </c>
+      <c r="CF164">
+        <v>2</v>
+      </c>
+      <c r="CG164">
+        <v>2</v>
+      </c>
     </row>
-    <row r="165" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="165" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -26592,8 +27728,17 @@
       <c r="CC165">
         <v>2</v>
       </c>
+      <c r="CE165">
+        <v>0</v>
+      </c>
+      <c r="CF165">
+        <v>2</v>
+      </c>
+      <c r="CG165">
+        <v>4</v>
+      </c>
     </row>
-    <row r="166" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="166" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -26745,8 +27890,14 @@
       <c r="CB166">
         <v>6</v>
       </c>
+      <c r="CE166">
+        <v>1</v>
+      </c>
+      <c r="CG166">
+        <v>5</v>
+      </c>
     </row>
-    <row r="167" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="167" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -26898,8 +28049,17 @@
       <c r="CC167">
         <v>1</v>
       </c>
+      <c r="CE167">
+        <v>0</v>
+      </c>
+      <c r="CF167">
+        <v>7</v>
+      </c>
+      <c r="CG167">
+        <v>1</v>
+      </c>
     </row>
-    <row r="168" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="168" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -27081,8 +28241,17 @@
       <c r="CC168">
         <v>2</v>
       </c>
+      <c r="CE168">
+        <v>1</v>
+      </c>
+      <c r="CF168">
+        <v>7</v>
+      </c>
+      <c r="CG168">
+        <v>3</v>
+      </c>
     </row>
-    <row r="169" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="169" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -27192,8 +28361,11 @@
       <c r="CB169">
         <v>6</v>
       </c>
+      <c r="CE169">
+        <v>6</v>
+      </c>
     </row>
-    <row r="170" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="170" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -27324,8 +28496,17 @@
       <c r="CD170">
         <v>1</v>
       </c>
+      <c r="CE170">
+        <v>7</v>
+      </c>
+      <c r="CF170">
+        <v>1</v>
+      </c>
+      <c r="CG170">
+        <v>1</v>
+      </c>
     </row>
-    <row r="171" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="171" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -27519,8 +28700,14 @@
       <c r="CC171">
         <v>6</v>
       </c>
+      <c r="CE171">
+        <v>4</v>
+      </c>
+      <c r="CF171">
+        <v>6</v>
+      </c>
     </row>
-    <row r="172" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="172" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -27633,8 +28820,17 @@
       <c r="CD172">
         <v>1</v>
       </c>
+      <c r="CE172">
+        <v>6</v>
+      </c>
+      <c r="CF172">
+        <v>1</v>
+      </c>
+      <c r="CG172">
+        <v>1</v>
+      </c>
     </row>
-    <row r="173" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="173" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -27765,8 +28961,14 @@
       <c r="CC173">
         <v>2</v>
       </c>
+      <c r="CE173">
+        <v>6</v>
+      </c>
+      <c r="CF173">
+        <v>2</v>
+      </c>
     </row>
-    <row r="174" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="174" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -27876,8 +29078,14 @@
       <c r="CB174">
         <v>9</v>
       </c>
+      <c r="CE174">
+        <v>8</v>
+      </c>
+      <c r="CG174">
+        <v>1</v>
+      </c>
     </row>
-    <row r="175" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="175" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -28044,8 +29252,14 @@
       <c r="CC175">
         <v>4</v>
       </c>
+      <c r="CE175">
+        <v>1</v>
+      </c>
+      <c r="CF175">
+        <v>8</v>
+      </c>
     </row>
-    <row r="176" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="176" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -28149,8 +29363,17 @@
       <c r="CD176">
         <v>1</v>
       </c>
+      <c r="CE176">
+        <v>0</v>
+      </c>
+      <c r="CF176">
+        <v>4</v>
+      </c>
+      <c r="CG176">
+        <v>4</v>
+      </c>
     </row>
-    <row r="177" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="177" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -28263,8 +29486,17 @@
       <c r="CC177">
         <v>1</v>
       </c>
+      <c r="CE177">
+        <v>0</v>
+      </c>
+      <c r="CF177">
+        <v>2</v>
+      </c>
+      <c r="CG177">
+        <v>3</v>
+      </c>
     </row>
-    <row r="178" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="178" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -28380,8 +29612,17 @@
       <c r="CD178">
         <v>2</v>
       </c>
+      <c r="CE178">
+        <v>2</v>
+      </c>
+      <c r="CF178">
+        <v>2</v>
+      </c>
+      <c r="CG178">
+        <v>4</v>
+      </c>
     </row>
-    <row r="179" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="179" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -28548,8 +29789,17 @@
       <c r="CC179">
         <v>5</v>
       </c>
+      <c r="CE179">
+        <v>0</v>
+      </c>
+      <c r="CF179">
+        <v>8</v>
+      </c>
+      <c r="CG179">
+        <v>2</v>
+      </c>
     </row>
-    <row r="180" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="180" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -28713,8 +29963,17 @@
       <c r="CD180">
         <v>2</v>
       </c>
+      <c r="CE180">
+        <v>1</v>
+      </c>
+      <c r="CF180">
+        <v>7</v>
+      </c>
+      <c r="CG180">
+        <v>1</v>
+      </c>
     </row>
-    <row r="181" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="181" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -28884,8 +30143,14 @@
       <c r="CD181">
         <v>1</v>
       </c>
+      <c r="CE181">
+        <v>0</v>
+      </c>
+      <c r="CF181">
+        <v>9</v>
+      </c>
     </row>
-    <row r="182" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="182" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -28995,8 +30260,14 @@
       <c r="CB182">
         <v>6</v>
       </c>
+      <c r="CE182">
+        <v>2</v>
+      </c>
+      <c r="CG182">
+        <v>4</v>
+      </c>
     </row>
-    <row r="183" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="183" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -29198,8 +30469,14 @@
       <c r="CC183">
         <v>2</v>
       </c>
+      <c r="CE183">
+        <v>3</v>
+      </c>
+      <c r="CF183">
+        <v>2</v>
+      </c>
     </row>
-    <row r="184" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="184" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -29317,8 +30594,14 @@
       <c r="CC184">
         <v>1</v>
       </c>
+      <c r="CE184">
+        <v>4</v>
+      </c>
+      <c r="CF184">
+        <v>2</v>
+      </c>
     </row>
-    <row r="185" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="185" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -29490,8 +30773,14 @@
       <c r="CC185">
         <v>7</v>
       </c>
+      <c r="CE185">
+        <v>0</v>
+      </c>
+      <c r="CF185">
+        <v>7</v>
+      </c>
     </row>
-    <row r="186" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="186" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -29651,8 +30940,14 @@
       <c r="CC186">
         <v>1</v>
       </c>
+      <c r="CE186">
+        <v>6</v>
+      </c>
+      <c r="CF186">
+        <v>1</v>
+      </c>
     </row>
-    <row r="187" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="187" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -29779,8 +31074,14 @@
       <c r="CC187">
         <v>1</v>
       </c>
+      <c r="CE187">
+        <v>5</v>
+      </c>
+      <c r="CG187">
+        <v>2</v>
+      </c>
     </row>
-    <row r="188" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="188" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B188" t="s">
         <v>4</v>
       </c>
@@ -29952,8 +31253,17 @@
       <c r="CD188">
         <v>1</v>
       </c>
+      <c r="CE188">
+        <v>6</v>
+      </c>
+      <c r="CF188">
+        <v>3</v>
+      </c>
+      <c r="CG188">
+        <v>1</v>
+      </c>
     </row>
-    <row r="189" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="189" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -30134,8 +31444,11 @@
       <c r="CB189">
         <v>2</v>
       </c>
+      <c r="CE189">
+        <v>2</v>
+      </c>
     </row>
-    <row r="190" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="190" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -30313,8 +31626,17 @@
       <c r="CC190">
         <v>2</v>
       </c>
+      <c r="CE190">
+        <v>0</v>
+      </c>
+      <c r="CF190">
+        <v>4</v>
+      </c>
+      <c r="CG190">
+        <v>1</v>
+      </c>
     </row>
-    <row r="191" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="191" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -30498,8 +31820,14 @@
       <c r="CC191">
         <v>5</v>
       </c>
+      <c r="CE191">
+        <v>0</v>
+      </c>
+      <c r="CF191">
+        <v>5</v>
+      </c>
     </row>
-    <row r="192" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="192" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -30662,8 +31990,14 @@
       <c r="CC192">
         <v>3</v>
       </c>
+      <c r="CE192">
+        <v>0</v>
+      </c>
+      <c r="CF192">
+        <v>3</v>
+      </c>
     </row>
-    <row r="193" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="193" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -30847,8 +32181,14 @@
       <c r="CC193">
         <v>4</v>
       </c>
+      <c r="CE193">
+        <v>3</v>
+      </c>
+      <c r="CF193">
+        <v>4</v>
+      </c>
     </row>
-    <row r="194" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="194" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B194" t="s">
         <v>4</v>
       </c>
@@ -31008,8 +32348,14 @@
       <c r="CC194">
         <v>1</v>
       </c>
+      <c r="CE194">
+        <v>6</v>
+      </c>
+      <c r="CF194">
+        <v>1</v>
+      </c>
     </row>
-    <row r="195" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="195" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -31187,8 +32533,11 @@
       <c r="CB195">
         <v>2</v>
       </c>
+      <c r="CE195">
+        <v>2</v>
+      </c>
     </row>
-    <row r="196" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="196" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -31399,8 +32748,14 @@
       <c r="CC196">
         <v>7</v>
       </c>
+      <c r="CE196">
+        <v>0</v>
+      </c>
+      <c r="CF196">
+        <v>9</v>
+      </c>
     </row>
-    <row r="197" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="197" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -31566,8 +32921,14 @@
       <c r="CC197">
         <v>4</v>
       </c>
+      <c r="CE197">
+        <v>0</v>
+      </c>
+      <c r="CF197">
+        <v>4</v>
+      </c>
     </row>
-    <row r="198" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="198" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -31709,8 +33070,17 @@
       <c r="CD198">
         <v>1</v>
       </c>
+      <c r="CE198">
+        <v>3</v>
+      </c>
+      <c r="CF198">
+        <v>1</v>
+      </c>
+      <c r="CG198">
+        <v>1</v>
+      </c>
     </row>
-    <row r="199" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="199" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -31870,8 +33240,14 @@
       <c r="CB199">
         <v>6</v>
       </c>
+      <c r="CE199">
+        <v>5</v>
+      </c>
+      <c r="CG199">
+        <v>1</v>
+      </c>
     </row>
-    <row r="200" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="200" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
         <v>4</v>
       </c>
@@ -32019,8 +33395,17 @@
       <c r="CC200">
         <v>1</v>
       </c>
+      <c r="CE200">
+        <v>1</v>
+      </c>
+      <c r="CF200">
+        <v>2</v>
+      </c>
+      <c r="CG200">
+        <v>4</v>
+      </c>
     </row>
-    <row r="201" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="201" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -32210,8 +33595,17 @@
       <c r="CC201">
         <v>5</v>
       </c>
+      <c r="CE201">
+        <v>0</v>
+      </c>
+      <c r="CF201">
+        <v>5</v>
+      </c>
+      <c r="CG201">
+        <v>1</v>
+      </c>
     </row>
-    <row r="202" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="202" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -32395,8 +33789,14 @@
       <c r="CC202">
         <v>1</v>
       </c>
+      <c r="CE202">
+        <v>0</v>
+      </c>
+      <c r="CF202">
+        <v>1</v>
+      </c>
     </row>
-    <row r="203" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="203" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -32574,8 +33974,14 @@
       <c r="CD203">
         <v>1</v>
       </c>
+      <c r="CE203">
+        <v>0</v>
+      </c>
+      <c r="CF203">
+        <v>3</v>
+      </c>
     </row>
-    <row r="204" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="204" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -32681,8 +34087,11 @@
       <c r="CB204">
         <v>6</v>
       </c>
+      <c r="CE204">
+        <v>6</v>
+      </c>
     </row>
-    <row r="205" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="205" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -32869,8 +34278,17 @@
       <c r="CC205">
         <v>1</v>
       </c>
+      <c r="CE205">
+        <v>8</v>
+      </c>
+      <c r="CF205">
+        <v>1</v>
+      </c>
+      <c r="CG205">
+        <v>1</v>
+      </c>
     </row>
-    <row r="206" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="206" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B206" t="s">
         <v>4</v>
       </c>
@@ -32976,8 +34394,11 @@
       <c r="CB206">
         <v>6</v>
       </c>
+      <c r="CE206">
+        <v>6</v>
+      </c>
     </row>
-    <row r="207" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="207" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -33122,8 +34543,14 @@
       <c r="CC207">
         <v>2</v>
       </c>
+      <c r="CE207">
+        <v>2</v>
+      </c>
+      <c r="CF207">
+        <v>2</v>
+      </c>
     </row>
-    <row r="208" spans="2:82" x14ac:dyDescent="0.35">
+    <row r="208" spans="2:85" x14ac:dyDescent="0.3">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -33301,8 +34728,14 @@
       <c r="CC208">
         <v>2</v>
       </c>
+      <c r="CE208">
+        <v>0</v>
+      </c>
+      <c r="CF208">
+        <v>3</v>
+      </c>
     </row>
-    <row r="209" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="209" spans="2:84" x14ac:dyDescent="0.3">
       <c r="B209" t="s">
         <v>3</v>
       </c>
@@ -33465,8 +34898,14 @@
       <c r="CC209">
         <v>5</v>
       </c>
+      <c r="CE209">
+        <v>0</v>
+      </c>
+      <c r="CF209">
+        <v>5</v>
+      </c>
     </row>
-    <row r="210" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="210" spans="2:84" x14ac:dyDescent="0.3">
       <c r="B210" t="s">
         <v>1</v>
       </c>
@@ -33650,8 +35089,14 @@
       <c r="CC210">
         <v>1</v>
       </c>
+      <c r="CE210">
+        <v>4</v>
+      </c>
+      <c r="CF210">
+        <v>1</v>
+      </c>
     </row>
-    <row r="211" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="211" spans="2:84" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
         <v>4</v>
       </c>
@@ -33811,8 +35256,14 @@
       <c r="CC211">
         <v>2</v>
       </c>
+      <c r="CE211">
+        <v>3</v>
+      </c>
+      <c r="CF211">
+        <v>2</v>
+      </c>
     </row>
-    <row r="212" spans="2:81" x14ac:dyDescent="0.35">
+    <row r="212" spans="2:84" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
         <v>4</v>
       </c>
@@ -33964,6 +35415,12 @@
         <v>5</v>
       </c>
       <c r="CC212">
+        <v>1</v>
+      </c>
+      <c r="CE212">
+        <v>5</v>
+      </c>
+      <c r="CF212">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
DOY 140 germinants data collection
</commit_message>
<xml_diff>
--- a/data/germination_data.xlsx
+++ b/data/germination_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temporal Ecology Lab\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ailun\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{99947861-4AC3-4972-A06A-0496258833AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6D83FF4-006A-4F8F-BDE1-C297DAD05134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="125">
   <si>
     <t>seed_species</t>
   </si>
@@ -438,6 +438,15 @@
   <si>
     <t>126_halfdead</t>
   </si>
+  <si>
+    <t>140_alive</t>
+  </si>
+  <si>
+    <t>140_dead</t>
+  </si>
+  <si>
+    <t>140_halfdead</t>
+  </si>
 </sst>
 </file>
 
@@ -541,9 +550,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CG213" totalsRowShown="0">
-  <autoFilter ref="B2:CG213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
-  <tableColumns count="84">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CJ213" totalsRowShown="0">
+  <autoFilter ref="B2:CJ213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="25"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <tableColumns count="87">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
     <tableColumn id="3" xr3:uid="{B695F4B4-8561-9D48-9FF3-12A40CB2B7C7}" name="inoculated_%"/>
@@ -628,6 +643,9 @@
     <tableColumn id="82" xr3:uid="{CE3EC9BD-EB21-4BAC-886C-89B8FF48600F}" name="126_alive"/>
     <tableColumn id="83" xr3:uid="{DA9CFA23-EC52-4220-82CD-9B249E55FE19}" name="126_dead"/>
     <tableColumn id="84" xr3:uid="{4EC5F6FC-B356-46C6-B57F-3AAEE58C6498}" name="126_halfdead"/>
+    <tableColumn id="85" xr3:uid="{563B32CE-FAA2-4820-A00E-BA719FBA6A1E}" name="140_alive"/>
+    <tableColumn id="86" xr3:uid="{12BABDCE-FBD8-4A85-BAA6-7981A89F386D}" name="140_dead"/>
+    <tableColumn id="87" xr3:uid="{644BBFBD-A683-4B49-8F95-95C2D3663641}" name="140_halfdead"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -950,7 +968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:CG212"/>
+  <dimension ref="B2:CJ213"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -958,7 +976,7 @@
     <col min="4" max="4" width="17.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -1211,8 +1229,17 @@
       <c r="CG2" t="s">
         <v>121</v>
       </c>
+      <c r="CH2" t="s">
+        <v>122</v>
+      </c>
+      <c r="CI2" t="s">
+        <v>123</v>
+      </c>
+      <c r="CJ2" t="s">
+        <v>124</v>
+      </c>
     </row>
-    <row r="3" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1408,8 +1435,14 @@
       <c r="CF3">
         <v>2</v>
       </c>
+      <c r="CH3">
+        <v>2</v>
+      </c>
+      <c r="CI3">
+        <v>2</v>
+      </c>
     </row>
-    <row r="4" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1524,8 +1557,11 @@
       <c r="CG4">
         <v>3</v>
       </c>
+      <c r="CH4">
+        <v>9</v>
+      </c>
     </row>
-    <row r="5" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1721,8 +1757,14 @@
       <c r="CF5">
         <v>7</v>
       </c>
+      <c r="CH5">
+        <v>0</v>
+      </c>
+      <c r="CI5">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1834,8 +1876,11 @@
       <c r="CE6">
         <v>9</v>
       </c>
+      <c r="CH6">
+        <v>9</v>
+      </c>
     </row>
-    <row r="7" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -1995,8 +2040,14 @@
       <c r="CF7">
         <v>4</v>
       </c>
+      <c r="CH7">
+        <v>2</v>
+      </c>
+      <c r="CI7">
+        <v>4</v>
+      </c>
     </row>
-    <row r="8" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -2183,8 +2234,14 @@
       <c r="CF8">
         <v>1</v>
       </c>
+      <c r="CH8">
+        <v>6</v>
+      </c>
+      <c r="CI8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2377,8 +2434,14 @@
       <c r="CF9">
         <v>1</v>
       </c>
+      <c r="CH9">
+        <v>6</v>
+      </c>
+      <c r="CI9">
+        <v>1</v>
+      </c>
     </row>
-    <row r="10" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -2502,8 +2565,17 @@
       <c r="CG10">
         <v>1</v>
       </c>
+      <c r="CH10">
+        <v>6</v>
+      </c>
+      <c r="CI10">
+        <v>1</v>
+      </c>
+      <c r="CJ10">
+        <v>1</v>
+      </c>
     </row>
-    <row r="11" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -2693,8 +2765,17 @@
       <c r="CG11">
         <v>1</v>
       </c>
+      <c r="CH11">
+        <v>0</v>
+      </c>
+      <c r="CI11">
+        <v>7</v>
+      </c>
+      <c r="CJ11">
+        <v>1</v>
+      </c>
     </row>
-    <row r="12" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -2890,8 +2971,14 @@
       <c r="CF12">
         <v>5</v>
       </c>
+      <c r="CH12">
+        <v>4</v>
+      </c>
+      <c r="CI12">
+        <v>5</v>
+      </c>
     </row>
-    <row r="13" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -3075,8 +3162,17 @@
       <c r="CF13">
         <v>4</v>
       </c>
+      <c r="CH13">
+        <v>1</v>
+      </c>
+      <c r="CI13">
+        <v>4</v>
+      </c>
+      <c r="CJ13">
+        <v>2</v>
+      </c>
     </row>
-    <row r="14" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -3221,8 +3317,14 @@
       <c r="CF14">
         <v>1</v>
       </c>
+      <c r="CH14">
+        <v>8</v>
+      </c>
+      <c r="CI14">
+        <v>1</v>
+      </c>
     </row>
-    <row r="15" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -3395,8 +3497,17 @@
       <c r="CF15">
         <v>4</v>
       </c>
+      <c r="CH15">
+        <v>0</v>
+      </c>
+      <c r="CI15">
+        <v>4</v>
+      </c>
+      <c r="CJ15">
+        <v>4</v>
+      </c>
     </row>
-    <row r="16" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -3554,8 +3665,14 @@
       <c r="CF16">
         <v>1</v>
       </c>
+      <c r="CH16">
+        <v>8</v>
+      </c>
+      <c r="CI16">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -3734,8 +3851,14 @@
       <c r="CF17">
         <v>8</v>
       </c>
+      <c r="CH17">
+        <v>0</v>
+      </c>
+      <c r="CI17">
+        <v>8</v>
+      </c>
     </row>
-    <row r="18" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -3845,8 +3968,11 @@
       <c r="CG18">
         <v>1</v>
       </c>
+      <c r="CH18">
+        <v>10</v>
+      </c>
     </row>
-    <row r="19" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -4043,8 +4169,14 @@
       <c r="CF19">
         <v>6</v>
       </c>
+      <c r="CH19">
+        <v>0</v>
+      </c>
+      <c r="CI19">
+        <v>7</v>
+      </c>
     </row>
-    <row r="20" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -4202,8 +4334,14 @@
       <c r="CF20">
         <v>1</v>
       </c>
+      <c r="CH20">
+        <v>13</v>
+      </c>
+      <c r="CI20">
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -4366,8 +4504,14 @@
       <c r="CF21">
         <v>2</v>
       </c>
+      <c r="CH21">
+        <v>0</v>
+      </c>
+      <c r="CI21">
+        <v>6</v>
+      </c>
     </row>
-    <row r="22" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -4483,8 +4627,11 @@
       <c r="CG22">
         <v>1</v>
       </c>
+      <c r="CH22">
+        <v>8</v>
+      </c>
     </row>
-    <row r="23" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -4672,8 +4819,17 @@
       <c r="CG23">
         <v>3</v>
       </c>
+      <c r="CH23">
+        <v>0</v>
+      </c>
+      <c r="CI23">
+        <v>7</v>
+      </c>
+      <c r="CJ23">
+        <v>3</v>
+      </c>
     </row>
-    <row r="24" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -4837,8 +4993,14 @@
       <c r="CF24">
         <v>4</v>
       </c>
+      <c r="CH24">
+        <v>8</v>
+      </c>
+      <c r="CI24">
+        <v>4</v>
+      </c>
     </row>
-    <row r="25" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -4948,8 +5110,17 @@
       <c r="CE25">
         <v>8</v>
       </c>
+      <c r="CH25">
+        <v>1</v>
+      </c>
+      <c r="CI25">
+        <v>6</v>
+      </c>
+      <c r="CJ25">
+        <v>1</v>
+      </c>
     </row>
-    <row r="26" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -5182,8 +5353,17 @@
       <c r="CG26">
         <v>1</v>
       </c>
+      <c r="CH26">
+        <v>1</v>
+      </c>
+      <c r="CI26">
+        <v>7</v>
+      </c>
+      <c r="CJ26">
+        <v>3</v>
+      </c>
     </row>
-    <row r="27" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -5350,8 +5530,17 @@
       <c r="CG27">
         <v>2</v>
       </c>
+      <c r="CH27">
+        <v>2</v>
+      </c>
+      <c r="CI27">
+        <v>3</v>
+      </c>
+      <c r="CJ27">
+        <v>1</v>
+      </c>
     </row>
-    <row r="28" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -5560,8 +5749,14 @@
       <c r="CF28">
         <v>3</v>
       </c>
+      <c r="CH28">
+        <v>7</v>
+      </c>
+      <c r="CI28">
+        <v>3</v>
+      </c>
     </row>
-    <row r="29" spans="2:85" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:88" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>3</v>
       </c>
@@ -5740,8 +5935,14 @@
       <c r="CG29" s="3">
         <v>1</v>
       </c>
+      <c r="CH29" s="3">
+        <v>0</v>
+      </c>
+      <c r="CI29" s="3">
+        <v>4</v>
+      </c>
     </row>
-    <row r="30" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -5857,8 +6058,11 @@
       <c r="CE30">
         <v>8</v>
       </c>
+      <c r="CH30">
+        <v>8</v>
+      </c>
     </row>
-    <row r="31" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -6052,8 +6256,17 @@
       <c r="CG31">
         <v>1</v>
       </c>
+      <c r="CH31">
+        <v>0</v>
+      </c>
+      <c r="CI31">
+        <v>3</v>
+      </c>
+      <c r="CJ31">
+        <v>2</v>
+      </c>
     </row>
-    <row r="32" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -6208,8 +6421,14 @@
       <c r="CF32">
         <v>1</v>
       </c>
+      <c r="CH32">
+        <v>9</v>
+      </c>
+      <c r="CI32">
+        <v>1</v>
+      </c>
     </row>
-    <row r="33" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -6358,8 +6577,17 @@
       <c r="CF33">
         <v>2</v>
       </c>
+      <c r="CH33">
+        <v>0</v>
+      </c>
+      <c r="CI33">
+        <v>7</v>
+      </c>
+      <c r="CJ33">
+        <v>2</v>
+      </c>
     </row>
-    <row r="34" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -6499,8 +6727,17 @@
       <c r="CE34">
         <v>6</v>
       </c>
+      <c r="CH34">
+        <v>2</v>
+      </c>
+      <c r="CI34">
+        <v>1</v>
+      </c>
+      <c r="CJ34">
+        <v>3</v>
+      </c>
     </row>
-    <row r="35" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -6673,8 +6910,17 @@
       <c r="CG35">
         <v>1</v>
       </c>
+      <c r="CH35">
+        <v>0</v>
+      </c>
+      <c r="CI35">
+        <v>7</v>
+      </c>
+      <c r="CJ35">
+        <v>1</v>
+      </c>
     </row>
-    <row r="36" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -6844,8 +7090,14 @@
       <c r="CF36">
         <v>2</v>
       </c>
+      <c r="CH36">
+        <v>8</v>
+      </c>
+      <c r="CI36">
+        <v>2</v>
+      </c>
     </row>
-    <row r="37" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -6964,8 +7216,14 @@
       <c r="CG37">
         <v>4</v>
       </c>
+      <c r="CH37">
+        <v>1</v>
+      </c>
+      <c r="CI37">
+        <v>8</v>
+      </c>
     </row>
-    <row r="38" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -7177,8 +7435,14 @@
       <c r="CG38">
         <v>2</v>
       </c>
+      <c r="CH38">
+        <v>2</v>
+      </c>
+      <c r="CI38">
+        <v>4</v>
+      </c>
     </row>
-    <row r="39" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -7369,8 +7633,14 @@
       <c r="CF39">
         <v>4</v>
       </c>
+      <c r="CH39">
+        <v>2</v>
+      </c>
+      <c r="CI39">
+        <v>4</v>
+      </c>
     </row>
-    <row r="40" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -7576,8 +7846,17 @@
       <c r="CG40">
         <v>1</v>
       </c>
+      <c r="CH40">
+        <v>2</v>
+      </c>
+      <c r="CI40">
+        <v>6</v>
+      </c>
+      <c r="CJ40">
+        <v>2</v>
+      </c>
     </row>
-    <row r="41" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -7750,8 +8029,14 @@
       <c r="CG41">
         <v>2</v>
       </c>
+      <c r="CH41">
+        <v>0</v>
+      </c>
+      <c r="CI41">
+        <v>6</v>
+      </c>
     </row>
-    <row r="42" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -7873,8 +8158,14 @@
       <c r="CG42">
         <v>2</v>
       </c>
+      <c r="CH42">
+        <v>5</v>
+      </c>
+      <c r="CJ42">
+        <v>2</v>
+      </c>
     </row>
-    <row r="43" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -8071,8 +8362,17 @@
       <c r="CG43">
         <v>1</v>
       </c>
+      <c r="CH43">
+        <v>0</v>
+      </c>
+      <c r="CI43">
+        <v>7</v>
+      </c>
+      <c r="CJ43">
+        <v>2</v>
+      </c>
     </row>
-    <row r="44" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -8179,8 +8479,14 @@
       <c r="CG44">
         <v>1</v>
       </c>
+      <c r="CH44">
+        <v>3</v>
+      </c>
+      <c r="CJ44">
+        <v>3</v>
+      </c>
     </row>
-    <row r="45" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -8422,8 +8728,14 @@
       <c r="CG45">
         <v>3</v>
       </c>
+      <c r="CH45">
+        <v>0</v>
+      </c>
+      <c r="CI45">
+        <v>9</v>
+      </c>
     </row>
-    <row r="46" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -8539,8 +8851,14 @@
       <c r="CE46">
         <v>6</v>
       </c>
+      <c r="CH46">
+        <v>3</v>
+      </c>
+      <c r="CJ46">
+        <v>3</v>
+      </c>
     </row>
-    <row r="47" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -8686,8 +9004,14 @@
       <c r="CF47">
         <v>9</v>
       </c>
+      <c r="CH47">
+        <v>0</v>
+      </c>
+      <c r="CI47">
+        <v>9</v>
+      </c>
     </row>
-    <row r="48" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -8902,8 +9226,14 @@
       <c r="CG48">
         <v>1</v>
       </c>
+      <c r="CH48">
+        <v>1</v>
+      </c>
+      <c r="CI48">
+        <v>10</v>
+      </c>
     </row>
-    <row r="49" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -9022,8 +9352,17 @@
       <c r="CF49">
         <v>2</v>
       </c>
+      <c r="CH49">
+        <v>4</v>
+      </c>
+      <c r="CI49">
+        <v>3</v>
+      </c>
+      <c r="CJ49">
+        <v>1</v>
+      </c>
     </row>
-    <row r="50" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -9238,8 +9577,14 @@
       <c r="CF50">
         <v>1</v>
       </c>
+      <c r="CH50">
+        <v>6</v>
+      </c>
+      <c r="CI50">
+        <v>2</v>
+      </c>
     </row>
-    <row r="51" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -9442,8 +9787,17 @@
       <c r="CG51">
         <v>2</v>
       </c>
+      <c r="CH51">
+        <v>1</v>
+      </c>
+      <c r="CI51">
+        <v>3</v>
+      </c>
+      <c r="CJ51">
+        <v>2</v>
+      </c>
     </row>
-    <row r="52" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -9553,8 +9907,11 @@
       <c r="CE52">
         <v>6</v>
       </c>
+      <c r="CH52">
+        <v>6</v>
+      </c>
     </row>
-    <row r="53" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -9733,8 +10090,14 @@
       <c r="CF53">
         <v>2</v>
       </c>
+      <c r="CH53">
+        <v>0</v>
+      </c>
+      <c r="CI53">
+        <v>4</v>
+      </c>
     </row>
-    <row r="54" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -9850,8 +10213,11 @@
       <c r="CG54">
         <v>1</v>
       </c>
+      <c r="CH54">
+        <v>5</v>
+      </c>
     </row>
-    <row r="55" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -10027,8 +10393,17 @@
       <c r="CG55">
         <v>2</v>
       </c>
+      <c r="CH55">
+        <v>0</v>
+      </c>
+      <c r="CI55">
+        <v>4</v>
+      </c>
+      <c r="CJ55">
+        <v>2</v>
+      </c>
     </row>
-    <row r="56" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -10144,8 +10519,11 @@
       <c r="CG56">
         <v>1</v>
       </c>
+      <c r="CH56">
+        <v>10</v>
+      </c>
     </row>
-    <row r="57" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -10273,8 +10651,14 @@
       <c r="CF57">
         <v>1</v>
       </c>
+      <c r="CH57">
+        <v>6</v>
+      </c>
+      <c r="CI57">
+        <v>1</v>
+      </c>
     </row>
-    <row r="58" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -10390,8 +10774,17 @@
       <c r="CE58">
         <v>6</v>
       </c>
+      <c r="CH58">
+        <v>3</v>
+      </c>
+      <c r="CI58">
+        <v>2</v>
+      </c>
+      <c r="CJ58">
+        <v>1</v>
+      </c>
     </row>
-    <row r="59" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -10504,8 +10897,17 @@
       <c r="CG59">
         <v>1</v>
       </c>
+      <c r="CH59">
+        <v>0</v>
+      </c>
+      <c r="CI59">
+        <v>6</v>
+      </c>
+      <c r="CJ59">
+        <v>1</v>
+      </c>
     </row>
-    <row r="60" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -10678,8 +11080,14 @@
       <c r="CF60">
         <v>2</v>
       </c>
+      <c r="CH60">
+        <v>7</v>
+      </c>
+      <c r="CI60">
+        <v>2</v>
+      </c>
     </row>
-    <row r="61" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -10801,8 +11209,17 @@
       <c r="CF61">
         <v>1</v>
       </c>
+      <c r="CH61">
+        <v>4</v>
+      </c>
+      <c r="CI61">
+        <v>1</v>
+      </c>
+      <c r="CJ61">
+        <v>2</v>
+      </c>
     </row>
-    <row r="62" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -11005,8 +11422,14 @@
       <c r="CF62">
         <v>2</v>
       </c>
+      <c r="CH62">
+        <v>3</v>
+      </c>
+      <c r="CI62">
+        <v>2</v>
+      </c>
     </row>
-    <row r="63" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -11206,8 +11629,17 @@
       <c r="CG63">
         <v>2</v>
       </c>
+      <c r="CH63">
+        <v>0</v>
+      </c>
+      <c r="CI63">
+        <v>7</v>
+      </c>
+      <c r="CJ63">
+        <v>2</v>
+      </c>
     </row>
-    <row r="64" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -11377,8 +11809,17 @@
       <c r="CG64">
         <v>1</v>
       </c>
+      <c r="CH64">
+        <v>6</v>
+      </c>
+      <c r="CI64">
+        <v>3</v>
+      </c>
+      <c r="CJ64">
+        <v>1</v>
+      </c>
     </row>
-    <row r="65" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -11551,8 +11992,17 @@
       <c r="CG65">
         <v>1</v>
       </c>
+      <c r="CH65">
+        <v>0</v>
+      </c>
+      <c r="CI65">
+        <v>5</v>
+      </c>
+      <c r="CJ65">
+        <v>1</v>
+      </c>
     </row>
-    <row r="66" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -11671,8 +12121,14 @@
       <c r="CG66">
         <v>1</v>
       </c>
+      <c r="CH66">
+        <v>4</v>
+      </c>
+      <c r="CJ66">
+        <v>1</v>
+      </c>
     </row>
-    <row r="67" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -11872,8 +12328,17 @@
       <c r="CG67">
         <v>2</v>
       </c>
+      <c r="CH67">
+        <v>0</v>
+      </c>
+      <c r="CI67">
+        <v>9</v>
+      </c>
+      <c r="CJ67">
+        <v>1</v>
+      </c>
     </row>
-    <row r="68" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -11980,8 +12445,11 @@
       <c r="CG68">
         <v>2</v>
       </c>
+      <c r="CH68">
+        <v>11</v>
+      </c>
     </row>
-    <row r="69" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -12091,8 +12559,17 @@
       <c r="CE69">
         <v>9</v>
       </c>
+      <c r="CH69">
+        <v>2</v>
+      </c>
+      <c r="CI69">
+        <v>5</v>
+      </c>
+      <c r="CJ69">
+        <v>2</v>
+      </c>
     </row>
-    <row r="70" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -12211,8 +12688,11 @@
       <c r="CE70">
         <v>8</v>
       </c>
+      <c r="CH70">
+        <v>8</v>
+      </c>
     </row>
-    <row r="71" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -12406,8 +12886,17 @@
       <c r="CG71">
         <v>1</v>
       </c>
+      <c r="CH71">
+        <v>0</v>
+      </c>
+      <c r="CI71">
+        <v>9</v>
+      </c>
+      <c r="CJ71">
+        <v>1</v>
+      </c>
     </row>
-    <row r="72" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -12589,8 +13078,14 @@
       <c r="CF72">
         <v>1</v>
       </c>
+      <c r="CH72">
+        <v>6</v>
+      </c>
+      <c r="CI72">
+        <v>1</v>
+      </c>
     </row>
-    <row r="73" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -12700,8 +13195,17 @@
       <c r="CE73">
         <v>10</v>
       </c>
+      <c r="CH73">
+        <v>3</v>
+      </c>
+      <c r="CI73">
+        <v>4</v>
+      </c>
+      <c r="CJ73">
+        <v>3</v>
+      </c>
     </row>
-    <row r="74" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -12820,8 +13324,11 @@
       <c r="CE74">
         <v>9</v>
       </c>
+      <c r="CH74">
+        <v>9</v>
+      </c>
     </row>
-    <row r="75" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -13000,8 +13507,17 @@
       <c r="CG75">
         <v>2</v>
       </c>
+      <c r="CH75">
+        <v>1</v>
+      </c>
+      <c r="CI75">
+        <v>5</v>
+      </c>
+      <c r="CJ75">
+        <v>3</v>
+      </c>
     </row>
-    <row r="76" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -13201,8 +13717,14 @@
       <c r="CF76">
         <v>1</v>
       </c>
+      <c r="CH76">
+        <v>7</v>
+      </c>
+      <c r="CI76">
+        <v>1</v>
+      </c>
     </row>
-    <row r="77" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -13369,8 +13891,14 @@
       <c r="CF77">
         <v>7</v>
       </c>
+      <c r="CH77">
+        <v>0</v>
+      </c>
+      <c r="CI77">
+        <v>7</v>
+      </c>
     </row>
-    <row r="78" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -13486,8 +14014,14 @@
       <c r="CG78">
         <v>3</v>
       </c>
+      <c r="CH78">
+        <v>4</v>
+      </c>
+      <c r="CJ78">
+        <v>3</v>
+      </c>
     </row>
-    <row r="79" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -13681,8 +14215,17 @@
       <c r="CF79">
         <v>7</v>
       </c>
+      <c r="CH79">
+        <v>1</v>
+      </c>
+      <c r="CI79">
+        <v>7</v>
+      </c>
+      <c r="CJ79">
+        <v>1</v>
+      </c>
     </row>
-    <row r="80" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -13849,8 +14392,14 @@
       <c r="CG80">
         <v>2</v>
       </c>
+      <c r="CH80">
+        <v>9</v>
+      </c>
+      <c r="CI80">
+        <v>1</v>
+      </c>
     </row>
-    <row r="81" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -14026,8 +14575,17 @@
       <c r="CF81">
         <v>2</v>
       </c>
+      <c r="CH81">
+        <v>0</v>
+      </c>
+      <c r="CI81">
+        <v>6</v>
+      </c>
+      <c r="CJ81">
+        <v>1</v>
+      </c>
     </row>
-    <row r="82" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -14242,8 +14800,17 @@
       <c r="CG82">
         <v>1</v>
       </c>
+      <c r="CH82">
+        <v>0</v>
+      </c>
+      <c r="CI82">
+        <v>8</v>
+      </c>
+      <c r="CJ82">
+        <v>2</v>
+      </c>
     </row>
-    <row r="83" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -14440,8 +15007,17 @@
       <c r="CG83">
         <v>1</v>
       </c>
+      <c r="CH83">
+        <v>0</v>
+      </c>
+      <c r="CI83">
+        <v>8</v>
+      </c>
+      <c r="CJ83">
+        <v>1</v>
+      </c>
     </row>
-    <row r="84" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -14630,16 +15206,19 @@
         <v>2</v>
       </c>
       <c r="CE84">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="CF84">
-        <v>8</v>
-      </c>
-      <c r="CG84">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="CH84">
+        <v>7</v>
+      </c>
+      <c r="CI84">
+        <v>2</v>
       </c>
     </row>
-    <row r="85" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -14836,8 +15415,17 @@
       <c r="CG85">
         <v>2</v>
       </c>
+      <c r="CH85">
+        <v>0</v>
+      </c>
+      <c r="CI85">
+        <v>5</v>
+      </c>
+      <c r="CJ85">
+        <v>1</v>
+      </c>
     </row>
-    <row r="86" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -15010,8 +15598,17 @@
       <c r="CF86">
         <v>1</v>
       </c>
+      <c r="CH86">
+        <v>2</v>
+      </c>
+      <c r="CI86">
+        <v>4</v>
+      </c>
+      <c r="CJ86">
+        <v>3</v>
+      </c>
     </row>
-    <row r="87" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -15208,8 +15805,17 @@
       <c r="CF87">
         <v>2</v>
       </c>
+      <c r="CH87">
+        <v>4</v>
+      </c>
+      <c r="CI87">
+        <v>2</v>
+      </c>
+      <c r="CJ87">
+        <v>1</v>
+      </c>
     </row>
-    <row r="88" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -15394,8 +16000,14 @@
       <c r="CG88">
         <v>2</v>
       </c>
+      <c r="CH88">
+        <v>6</v>
+      </c>
+      <c r="CI88">
+        <v>3</v>
+      </c>
     </row>
-    <row r="89" spans="2:85" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:88" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>3</v>
       </c>
@@ -15556,8 +16168,17 @@
       <c r="CG89" s="3">
         <v>1</v>
       </c>
+      <c r="CH89" s="3">
+        <v>0</v>
+      </c>
+      <c r="CI89" s="3">
+        <v>4</v>
+      </c>
+      <c r="CJ89" s="3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="90" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -15673,8 +16294,11 @@
       <c r="CG90">
         <v>2</v>
       </c>
+      <c r="CH90">
+        <v>8</v>
+      </c>
     </row>
-    <row r="91" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -15880,8 +16504,17 @@
       <c r="CF91">
         <v>3</v>
       </c>
+      <c r="CH91">
+        <v>1</v>
+      </c>
+      <c r="CI91">
+        <v>3</v>
+      </c>
+      <c r="CJ91">
+        <v>2</v>
+      </c>
     </row>
-    <row r="92" spans="2:85" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:88" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>1</v>
       </c>
@@ -16069,8 +16702,14 @@
       <c r="CF92" s="3">
         <v>3</v>
       </c>
+      <c r="CH92" s="3">
+        <v>5</v>
+      </c>
+      <c r="CI92" s="3">
+        <v>3</v>
+      </c>
     </row>
-    <row r="93" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -16216,8 +16855,17 @@
       <c r="CF93">
         <v>2</v>
       </c>
+      <c r="CH93">
+        <v>0</v>
+      </c>
+      <c r="CI93">
+        <v>8</v>
+      </c>
+      <c r="CJ93">
+        <v>1</v>
+      </c>
     </row>
-    <row r="94" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -16333,8 +16981,17 @@
       <c r="CE94">
         <v>7</v>
       </c>
+      <c r="CH94">
+        <v>1</v>
+      </c>
+      <c r="CI94">
+        <v>2</v>
+      </c>
+      <c r="CJ94">
+        <v>4</v>
+      </c>
     </row>
-    <row r="95" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -16489,8 +17146,17 @@
       <c r="CG95">
         <v>2</v>
       </c>
+      <c r="CH95">
+        <v>0</v>
+      </c>
+      <c r="CI95">
+        <v>6</v>
+      </c>
+      <c r="CJ95">
+        <v>2</v>
+      </c>
     </row>
-    <row r="96" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -16669,8 +17335,14 @@
       <c r="CG96">
         <v>1</v>
       </c>
+      <c r="CH96">
+        <v>5</v>
+      </c>
+      <c r="CI96">
+        <v>5</v>
+      </c>
     </row>
-    <row r="97" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -16789,8 +17461,17 @@
       <c r="CG97">
         <v>1</v>
       </c>
+      <c r="CH97">
+        <v>2</v>
+      </c>
+      <c r="CI97">
+        <v>3</v>
+      </c>
+      <c r="CJ97">
+        <v>3</v>
+      </c>
     </row>
-    <row r="98" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -16966,8 +17647,17 @@
       <c r="CF98">
         <v>2</v>
       </c>
+      <c r="CH98">
+        <v>4</v>
+      </c>
+      <c r="CI98">
+        <v>2</v>
+      </c>
+      <c r="CJ98">
+        <v>1</v>
+      </c>
     </row>
-    <row r="99" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -17098,8 +17788,14 @@
       <c r="CF99">
         <v>1</v>
       </c>
+      <c r="CH99">
+        <v>2</v>
+      </c>
+      <c r="CI99">
+        <v>1</v>
+      </c>
     </row>
-    <row r="100" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -17215,8 +17911,11 @@
       <c r="CG100">
         <v>2</v>
       </c>
+      <c r="CH100">
+        <v>8</v>
+      </c>
     </row>
-    <row r="101" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -17380,8 +18079,14 @@
       <c r="CF101">
         <v>4</v>
       </c>
+      <c r="CH101">
+        <v>1</v>
+      </c>
+      <c r="CI101">
+        <v>4</v>
+      </c>
     </row>
-    <row r="102" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -17494,8 +18199,17 @@
       <c r="CE102">
         <v>7</v>
       </c>
+      <c r="CH102">
+        <v>4</v>
+      </c>
+      <c r="CI102">
+        <v>1</v>
+      </c>
+      <c r="CJ102">
+        <v>2</v>
+      </c>
     </row>
-    <row r="103" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -17680,8 +18394,14 @@
       <c r="CF103">
         <v>6</v>
       </c>
+      <c r="CH103">
+        <v>0</v>
+      </c>
+      <c r="CI103">
+        <v>6</v>
+      </c>
     </row>
-    <row r="104" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -17860,8 +18580,17 @@
       <c r="CG104">
         <v>1</v>
       </c>
+      <c r="CH104">
+        <v>4</v>
+      </c>
+      <c r="CI104">
+        <v>3</v>
+      </c>
+      <c r="CJ104">
+        <v>3</v>
+      </c>
     </row>
-    <row r="105" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -18034,8 +18763,17 @@
       <c r="CG105">
         <v>2</v>
       </c>
+      <c r="CH105">
+        <v>0</v>
+      </c>
+      <c r="CI105">
+        <v>5</v>
+      </c>
+      <c r="CJ105">
+        <v>1</v>
+      </c>
     </row>
-    <row r="106" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -18199,8 +18937,14 @@
       <c r="CG106">
         <v>1</v>
       </c>
+      <c r="CH106">
+        <v>1</v>
+      </c>
+      <c r="CI106">
+        <v>7</v>
+      </c>
     </row>
-    <row r="107" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -18385,8 +19129,17 @@
       <c r="CG107">
         <v>1</v>
       </c>
+      <c r="CH107">
+        <v>0</v>
+      </c>
+      <c r="CI107">
+        <v>4</v>
+      </c>
+      <c r="CJ107">
+        <v>1</v>
+      </c>
     </row>
-    <row r="108" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -18556,8 +19309,17 @@
       <c r="CF108">
         <v>4</v>
       </c>
+      <c r="CH108">
+        <v>2</v>
+      </c>
+      <c r="CI108">
+        <v>4</v>
+      </c>
+      <c r="CJ108">
+        <v>4</v>
+      </c>
     </row>
-    <row r="109" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -18745,8 +19507,14 @@
       <c r="CF109">
         <v>9</v>
       </c>
+      <c r="CH109">
+        <v>0</v>
+      </c>
+      <c r="CI109">
+        <v>9</v>
+      </c>
     </row>
-    <row r="110" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -18937,8 +19705,14 @@
       <c r="CF110">
         <v>3</v>
       </c>
+      <c r="CH110">
+        <v>6</v>
+      </c>
+      <c r="CI110">
+        <v>3</v>
+      </c>
     </row>
-    <row r="111" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -19111,8 +19885,17 @@
       <c r="CG111">
         <v>2</v>
       </c>
+      <c r="CH111">
+        <v>3</v>
+      </c>
+      <c r="CI111">
+        <v>3</v>
+      </c>
+      <c r="CJ111">
+        <v>2</v>
+      </c>
     </row>
-    <row r="112" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -19291,8 +20074,17 @@
       <c r="CG112">
         <v>2</v>
       </c>
+      <c r="CH112">
+        <v>4</v>
+      </c>
+      <c r="CI112">
+        <v>2</v>
+      </c>
+      <c r="CJ112">
+        <v>2</v>
+      </c>
     </row>
-    <row r="113" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -19483,8 +20275,14 @@
       <c r="CF113">
         <v>2</v>
       </c>
+      <c r="CH113">
+        <v>4</v>
+      </c>
+      <c r="CI113">
+        <v>2</v>
+      </c>
     </row>
-    <row r="114" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -19600,8 +20398,14 @@
       <c r="CG114">
         <v>6</v>
       </c>
+      <c r="CH114">
+        <v>0</v>
+      </c>
+      <c r="CI114">
+        <v>8</v>
+      </c>
     </row>
-    <row r="115" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -19795,8 +20599,14 @@
       <c r="CF115">
         <v>4</v>
       </c>
+      <c r="CH115">
+        <v>0</v>
+      </c>
+      <c r="CI115">
+        <v>4</v>
+      </c>
     </row>
-    <row r="116" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -19972,8 +20782,17 @@
       <c r="CF116">
         <v>3</v>
       </c>
+      <c r="CH116">
+        <v>0</v>
+      </c>
+      <c r="CI116">
+        <v>7</v>
+      </c>
+      <c r="CJ116">
+        <v>1</v>
+      </c>
     </row>
-    <row r="117" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -20158,8 +20977,14 @@
       <c r="CF117">
         <v>4</v>
       </c>
+      <c r="CH117">
+        <v>0</v>
+      </c>
+      <c r="CI117">
+        <v>5</v>
+      </c>
     </row>
-    <row r="118" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -20282,8 +21107,17 @@
       <c r="CG118">
         <v>2</v>
       </c>
+      <c r="CH118">
+        <v>0</v>
+      </c>
+      <c r="CI118">
+        <v>4</v>
+      </c>
+      <c r="CJ118">
+        <v>2</v>
+      </c>
     </row>
-    <row r="119" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -20408,8 +21242,17 @@
       <c r="CG119">
         <v>4</v>
       </c>
+      <c r="CH119">
+        <v>0</v>
+      </c>
+      <c r="CI119">
+        <v>4</v>
+      </c>
+      <c r="CJ119">
+        <v>3</v>
+      </c>
     </row>
-    <row r="120" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -20525,8 +21368,17 @@
       <c r="CG120">
         <v>2</v>
       </c>
+      <c r="CH120">
+        <v>0</v>
+      </c>
+      <c r="CI120">
+        <v>9</v>
+      </c>
+      <c r="CJ120">
+        <v>1</v>
+      </c>
     </row>
-    <row r="121" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -20639,8 +21491,17 @@
       <c r="CE121">
         <v>8</v>
       </c>
+      <c r="CH121">
+        <v>2</v>
+      </c>
+      <c r="CI121">
+        <v>3</v>
+      </c>
+      <c r="CJ121">
+        <v>3</v>
+      </c>
     </row>
-    <row r="122" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -20759,8 +21620,14 @@
       <c r="CG122">
         <v>1</v>
       </c>
+      <c r="CH122">
+        <v>5</v>
+      </c>
+      <c r="CJ122">
+        <v>1</v>
+      </c>
     </row>
-    <row r="123" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -20933,8 +21800,14 @@
       <c r="CF123">
         <v>3</v>
       </c>
+      <c r="CH123">
+        <v>3</v>
+      </c>
+      <c r="CI123">
+        <v>3</v>
+      </c>
     </row>
-    <row r="124" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -21135,13 +22008,22 @@
         <v>4</v>
       </c>
       <c r="CF124">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="CG124">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="CH124">
+        <v>4</v>
+      </c>
+      <c r="CI124">
+        <v>3</v>
+      </c>
+      <c r="CJ124">
+        <v>2</v>
       </c>
     </row>
-    <row r="125" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -21341,8 +22223,14 @@
       <c r="CF125">
         <v>6</v>
       </c>
+      <c r="CH125">
+        <v>0</v>
+      </c>
+      <c r="CI125">
+        <v>6</v>
+      </c>
     </row>
-    <row r="126" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -21521,8 +22409,17 @@
       <c r="CF126">
         <v>3</v>
       </c>
+      <c r="CH126">
+        <v>0</v>
+      </c>
+      <c r="CI126">
+        <v>5</v>
+      </c>
+      <c r="CJ126">
+        <v>1</v>
+      </c>
     </row>
-    <row r="127" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -21698,8 +22595,14 @@
       <c r="CF127">
         <v>3</v>
       </c>
+      <c r="CH127">
+        <v>0</v>
+      </c>
+      <c r="CI127">
+        <v>3</v>
+      </c>
     </row>
-    <row r="128" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -21806,8 +22709,14 @@
       <c r="CF128">
         <v>4</v>
       </c>
+      <c r="CH128">
+        <v>0</v>
+      </c>
+      <c r="CI128">
+        <v>7</v>
+      </c>
     </row>
-    <row r="129" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -21998,8 +22907,14 @@
       <c r="CF129">
         <v>5</v>
       </c>
+      <c r="CH129">
+        <v>0</v>
+      </c>
+      <c r="CI129">
+        <v>6</v>
+      </c>
     </row>
-    <row r="130" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -22124,8 +23039,17 @@
       <c r="CG130">
         <v>2</v>
       </c>
+      <c r="CH130">
+        <v>0</v>
+      </c>
+      <c r="CI130">
+        <v>9</v>
+      </c>
+      <c r="CJ130">
+        <v>1</v>
+      </c>
     </row>
-    <row r="131" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -22316,8 +23240,17 @@
       <c r="CG131">
         <v>5</v>
       </c>
+      <c r="CH131">
+        <v>0</v>
+      </c>
+      <c r="CI131">
+        <v>7</v>
+      </c>
+      <c r="CJ131">
+        <v>3</v>
+      </c>
     </row>
-    <row r="132" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -22433,8 +23366,14 @@
       <c r="CG132">
         <v>1</v>
       </c>
+      <c r="CH132">
+        <v>0</v>
+      </c>
+      <c r="CI132">
+        <v>6</v>
+      </c>
     </row>
-    <row r="133" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -22583,8 +23522,14 @@
       <c r="CG133">
         <v>5</v>
       </c>
+      <c r="CH133">
+        <v>0</v>
+      </c>
+      <c r="CI133">
+        <v>7</v>
+      </c>
     </row>
-    <row r="134" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -22730,8 +23675,17 @@
       <c r="CG134">
         <v>3</v>
       </c>
+      <c r="CH134">
+        <v>3</v>
+      </c>
+      <c r="CI134">
+        <v>4</v>
+      </c>
+      <c r="CJ134">
+        <v>3</v>
+      </c>
     </row>
-    <row r="135" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -22901,8 +23855,14 @@
       <c r="CG135">
         <v>1</v>
       </c>
+      <c r="CH135">
+        <v>1</v>
+      </c>
+      <c r="CI135">
+        <v>7</v>
+      </c>
     </row>
-    <row r="136" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -23063,8 +24023,17 @@
       <c r="CG136">
         <v>1</v>
       </c>
+      <c r="CH136">
+        <v>3</v>
+      </c>
+      <c r="CI136">
+        <v>1</v>
+      </c>
+      <c r="CJ136">
+        <v>3</v>
+      </c>
     </row>
-    <row r="137" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -23231,8 +24200,14 @@
       <c r="CF137">
         <v>2</v>
       </c>
+      <c r="CH137">
+        <v>3</v>
+      </c>
+      <c r="CI137">
+        <v>2</v>
+      </c>
     </row>
-    <row r="138" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -23417,8 +24392,14 @@
       <c r="CG138">
         <v>4</v>
       </c>
+      <c r="CH138">
+        <v>0</v>
+      </c>
+      <c r="CI138">
+        <v>7</v>
+      </c>
     </row>
-    <row r="139" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -23585,8 +24566,14 @@
       <c r="CF139">
         <v>5</v>
       </c>
+      <c r="CH139">
+        <v>0</v>
+      </c>
+      <c r="CI139">
+        <v>5</v>
+      </c>
     </row>
-    <row r="140" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -23705,8 +24692,17 @@
       <c r="CG140">
         <v>2</v>
       </c>
+      <c r="CH140">
+        <v>0</v>
+      </c>
+      <c r="CI140">
+        <v>8</v>
+      </c>
+      <c r="CJ140">
+        <v>1</v>
+      </c>
     </row>
-    <row r="141" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -23909,8 +24905,14 @@
       <c r="CF141">
         <v>4</v>
       </c>
+      <c r="CH141">
+        <v>0</v>
+      </c>
+      <c r="CI141">
+        <v>8</v>
+      </c>
     </row>
-    <row r="142" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -24110,8 +25112,17 @@
       <c r="CF142">
         <v>7</v>
       </c>
+      <c r="CH142">
+        <v>0</v>
+      </c>
+      <c r="CI142">
+        <v>7</v>
+      </c>
+      <c r="CJ142">
+        <v>1</v>
+      </c>
     </row>
-    <row r="143" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -24269,8 +25280,17 @@
       <c r="CG143">
         <v>5</v>
       </c>
+      <c r="CH143">
+        <v>0</v>
+      </c>
+      <c r="CI143">
+        <v>9</v>
+      </c>
+      <c r="CJ143">
+        <v>2</v>
+      </c>
     </row>
-    <row r="144" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -24383,8 +25403,14 @@
       <c r="CF144">
         <v>7</v>
       </c>
+      <c r="CH144">
+        <v>0</v>
+      </c>
+      <c r="CI144">
+        <v>7</v>
+      </c>
     </row>
-    <row r="145" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -24503,8 +25529,17 @@
       <c r="CF145">
         <v>5</v>
       </c>
+      <c r="CH145">
+        <v>0</v>
+      </c>
+      <c r="CI145">
+        <v>5</v>
+      </c>
+      <c r="CJ145">
+        <v>3</v>
+      </c>
     </row>
-    <row r="146" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -24713,8 +25748,17 @@
       <c r="CG146">
         <v>3</v>
       </c>
+      <c r="CH146">
+        <v>3</v>
+      </c>
+      <c r="CI146">
+        <v>6</v>
+      </c>
+      <c r="CJ146">
+        <v>1</v>
+      </c>
     </row>
-    <row r="147" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -24914,8 +25958,17 @@
       <c r="CG147">
         <v>1</v>
       </c>
+      <c r="CH147">
+        <v>1</v>
+      </c>
+      <c r="CI147">
+        <v>2</v>
+      </c>
+      <c r="CJ147">
+        <v>1</v>
+      </c>
     </row>
-    <row r="148" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -25028,8 +26081,11 @@
       <c r="CG148">
         <v>1</v>
       </c>
+      <c r="CH148">
+        <v>9</v>
+      </c>
     </row>
-    <row r="149" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -25229,8 +26285,17 @@
       <c r="CG149">
         <v>2</v>
       </c>
+      <c r="CH149">
+        <v>1</v>
+      </c>
+      <c r="CI149">
+        <v>2</v>
+      </c>
+      <c r="CJ149">
+        <v>2</v>
+      </c>
     </row>
-    <row r="150" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -25427,8 +26492,14 @@
       <c r="CF150">
         <v>1</v>
       </c>
+      <c r="CH150">
+        <v>8</v>
+      </c>
+      <c r="CI150">
+        <v>1</v>
+      </c>
     </row>
-    <row r="151" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -25598,8 +26669,17 @@
       <c r="CG151">
         <v>4</v>
       </c>
+      <c r="CH151">
+        <v>0</v>
+      </c>
+      <c r="CI151">
+        <v>8</v>
+      </c>
+      <c r="CJ151">
+        <v>2</v>
+      </c>
     </row>
-    <row r="152" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -25703,8 +26783,17 @@
       <c r="CE152">
         <v>9</v>
       </c>
+      <c r="CH152">
+        <v>5</v>
+      </c>
+      <c r="CI152">
+        <v>1</v>
+      </c>
+      <c r="CJ152">
+        <v>3</v>
+      </c>
     </row>
-    <row r="153" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -25868,8 +26957,14 @@
       <c r="CG153">
         <v>2</v>
       </c>
+      <c r="CH153">
+        <v>0</v>
+      </c>
+      <c r="CI153">
+        <v>6</v>
+      </c>
     </row>
-    <row r="154" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -26096,8 +27191,17 @@
       <c r="CG154">
         <v>2</v>
       </c>
+      <c r="CH154">
+        <v>0</v>
+      </c>
+      <c r="CI154">
+        <v>5</v>
+      </c>
+      <c r="CJ154">
+        <v>3</v>
+      </c>
     </row>
-    <row r="155" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -26273,8 +27377,17 @@
       <c r="CG155">
         <v>1</v>
       </c>
+      <c r="CH155">
+        <v>0</v>
+      </c>
+      <c r="CI155">
+        <v>5</v>
+      </c>
+      <c r="CJ155">
+        <v>4</v>
+      </c>
     </row>
-    <row r="156" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="156" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -26387,8 +27500,14 @@
       <c r="CF156">
         <v>2</v>
       </c>
+      <c r="CH156">
+        <v>1</v>
+      </c>
+      <c r="CI156">
+        <v>5</v>
+      </c>
     </row>
-    <row r="157" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="157" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -26501,8 +27620,17 @@
       <c r="CE157">
         <v>6</v>
       </c>
+      <c r="CH157">
+        <v>0</v>
+      </c>
+      <c r="CI157">
+        <v>4</v>
+      </c>
+      <c r="CJ157">
+        <v>2</v>
+      </c>
     </row>
-    <row r="158" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="158" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -26645,8 +27773,14 @@
       <c r="CG158">
         <v>2</v>
       </c>
+      <c r="CH158">
+        <v>6</v>
+      </c>
+      <c r="CI158">
+        <v>2</v>
+      </c>
     </row>
-    <row r="159" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -26837,8 +27971,17 @@
       <c r="CG159">
         <v>2</v>
       </c>
+      <c r="CH159">
+        <v>0</v>
+      </c>
+      <c r="CI159">
+        <v>4</v>
+      </c>
+      <c r="CJ159">
+        <v>1</v>
+      </c>
     </row>
-    <row r="160" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -26951,8 +28094,11 @@
       <c r="CG160">
         <v>1</v>
       </c>
+      <c r="CH160">
+        <v>9</v>
+      </c>
     </row>
-    <row r="161" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -27164,8 +28310,14 @@
       <c r="CF161">
         <v>6</v>
       </c>
+      <c r="CH161">
+        <v>1</v>
+      </c>
+      <c r="CI161">
+        <v>6</v>
+      </c>
     </row>
-    <row r="162" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -27278,8 +28430,11 @@
       <c r="CE162">
         <v>8</v>
       </c>
+      <c r="CH162">
+        <v>8</v>
+      </c>
     </row>
-    <row r="163" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="163" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -27452,8 +28607,14 @@
       <c r="CF163">
         <v>8</v>
       </c>
+      <c r="CH163">
+        <v>0</v>
+      </c>
+      <c r="CI163">
+        <v>8</v>
+      </c>
     </row>
-    <row r="164" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="164" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -27563,8 +28724,17 @@
       <c r="CG164">
         <v>2</v>
       </c>
+      <c r="CH164">
+        <v>2</v>
+      </c>
+      <c r="CI164">
+        <v>6</v>
+      </c>
+      <c r="CJ164">
+        <v>1</v>
+      </c>
     </row>
-    <row r="165" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -27737,8 +28907,14 @@
       <c r="CG165">
         <v>4</v>
       </c>
+      <c r="CH165">
+        <v>0</v>
+      </c>
+      <c r="CI165">
+        <v>6</v>
+      </c>
     </row>
-    <row r="166" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="166" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -27896,8 +29072,14 @@
       <c r="CG166">
         <v>5</v>
       </c>
+      <c r="CH166">
+        <v>0</v>
+      </c>
+      <c r="CI166">
+        <v>6</v>
+      </c>
     </row>
-    <row r="167" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -28058,8 +29240,14 @@
       <c r="CG167">
         <v>1</v>
       </c>
+      <c r="CH167">
+        <v>0</v>
+      </c>
+      <c r="CI167">
+        <v>8</v>
+      </c>
     </row>
-    <row r="168" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -28250,8 +29438,17 @@
       <c r="CG168">
         <v>3</v>
       </c>
+      <c r="CH168">
+        <v>0</v>
+      </c>
+      <c r="CI168">
+        <v>8</v>
+      </c>
+      <c r="CJ168">
+        <v>3</v>
+      </c>
     </row>
-    <row r="169" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -28364,8 +29561,17 @@
       <c r="CE169">
         <v>6</v>
       </c>
+      <c r="CH169">
+        <v>1</v>
+      </c>
+      <c r="CI169">
+        <v>3</v>
+      </c>
+      <c r="CJ169">
+        <v>2</v>
+      </c>
     </row>
-    <row r="170" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -28505,8 +29711,17 @@
       <c r="CG170">
         <v>1</v>
       </c>
+      <c r="CH170">
+        <v>7</v>
+      </c>
+      <c r="CI170">
+        <v>1</v>
+      </c>
+      <c r="CJ170">
+        <v>1</v>
+      </c>
     </row>
-    <row r="171" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="171" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -28706,8 +29921,17 @@
       <c r="CF171">
         <v>6</v>
       </c>
+      <c r="CH171">
+        <v>2</v>
+      </c>
+      <c r="CI171">
+        <v>7</v>
+      </c>
+      <c r="CJ171">
+        <v>1</v>
+      </c>
     </row>
-    <row r="172" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -28823,14 +30047,17 @@
       <c r="CE172">
         <v>6</v>
       </c>
-      <c r="CF172">
-        <v>1</v>
-      </c>
       <c r="CG172">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="CH172">
+        <v>6</v>
+      </c>
+      <c r="CJ172">
+        <v>2</v>
       </c>
     </row>
-    <row r="173" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -28967,8 +30194,14 @@
       <c r="CF173">
         <v>2</v>
       </c>
+      <c r="CH173">
+        <v>6</v>
+      </c>
+      <c r="CI173">
+        <v>2</v>
+      </c>
     </row>
-    <row r="174" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -29084,8 +30317,17 @@
       <c r="CG174">
         <v>1</v>
       </c>
+      <c r="CH174">
+        <v>6</v>
+      </c>
+      <c r="CI174">
+        <v>2</v>
+      </c>
+      <c r="CJ174">
+        <v>1</v>
+      </c>
     </row>
-    <row r="175" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -29258,8 +30500,17 @@
       <c r="CF175">
         <v>8</v>
       </c>
+      <c r="CH175">
+        <v>0</v>
+      </c>
+      <c r="CI175">
+        <v>8</v>
+      </c>
+      <c r="CJ175">
+        <v>1</v>
+      </c>
     </row>
-    <row r="176" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="176" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -29372,8 +30623,14 @@
       <c r="CG176">
         <v>4</v>
       </c>
+      <c r="CH176">
+        <v>0</v>
+      </c>
+      <c r="CI176">
+        <v>8</v>
+      </c>
     </row>
-    <row r="177" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -29495,8 +30752,14 @@
       <c r="CG177">
         <v>3</v>
       </c>
+      <c r="CH177">
+        <v>0</v>
+      </c>
+      <c r="CI177">
+        <v>5</v>
+      </c>
     </row>
-    <row r="178" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -29621,8 +30884,17 @@
       <c r="CG178">
         <v>4</v>
       </c>
+      <c r="CH178">
+        <v>0</v>
+      </c>
+      <c r="CI178">
+        <v>7</v>
+      </c>
+      <c r="CJ178">
+        <v>1</v>
+      </c>
     </row>
-    <row r="179" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -29798,8 +31070,17 @@
       <c r="CG179">
         <v>2</v>
       </c>
+      <c r="CH179">
+        <v>0</v>
+      </c>
+      <c r="CI179">
+        <v>8</v>
+      </c>
+      <c r="CJ179">
+        <v>2</v>
+      </c>
     </row>
-    <row r="180" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -29972,8 +31253,17 @@
       <c r="CG180">
         <v>1</v>
       </c>
+      <c r="CH180">
+        <v>0</v>
+      </c>
+      <c r="CI180">
+        <v>8</v>
+      </c>
+      <c r="CJ180">
+        <v>1</v>
+      </c>
     </row>
-    <row r="181" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -30149,8 +31439,14 @@
       <c r="CF181">
         <v>9</v>
       </c>
+      <c r="CH181">
+        <v>0</v>
+      </c>
+      <c r="CI181">
+        <v>9</v>
+      </c>
     </row>
-    <row r="182" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -30266,8 +31562,17 @@
       <c r="CG182">
         <v>4</v>
       </c>
+      <c r="CH182">
+        <v>2</v>
+      </c>
+      <c r="CI182">
+        <v>2</v>
+      </c>
+      <c r="CJ182">
+        <v>2</v>
+      </c>
     </row>
-    <row r="183" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -30475,8 +31780,14 @@
       <c r="CF183">
         <v>2</v>
       </c>
+      <c r="CH183">
+        <v>3</v>
+      </c>
+      <c r="CI183">
+        <v>2</v>
+      </c>
     </row>
-    <row r="184" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -30600,8 +31911,17 @@
       <c r="CF184">
         <v>2</v>
       </c>
+      <c r="CH184">
+        <v>1</v>
+      </c>
+      <c r="CI184">
+        <v>2</v>
+      </c>
+      <c r="CJ184">
+        <v>3</v>
+      </c>
     </row>
-    <row r="185" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -30779,8 +32099,14 @@
       <c r="CF185">
         <v>7</v>
       </c>
+      <c r="CH185">
+        <v>0</v>
+      </c>
+      <c r="CI185">
+        <v>7</v>
+      </c>
     </row>
-    <row r="186" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -30946,8 +32272,14 @@
       <c r="CF186">
         <v>1</v>
       </c>
+      <c r="CH186">
+        <v>6</v>
+      </c>
+      <c r="CI186">
+        <v>1</v>
+      </c>
     </row>
-    <row r="187" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -31080,8 +32412,14 @@
       <c r="CG187">
         <v>2</v>
       </c>
+      <c r="CH187">
+        <v>6</v>
+      </c>
+      <c r="CJ187">
+        <v>1</v>
+      </c>
     </row>
-    <row r="188" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B188" t="s">
         <v>4</v>
       </c>
@@ -31262,8 +32600,14 @@
       <c r="CG188">
         <v>1</v>
       </c>
+      <c r="CH188">
+        <v>6</v>
+      </c>
+      <c r="CI188">
+        <v>4</v>
+      </c>
     </row>
-    <row r="189" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -31447,8 +32791,14 @@
       <c r="CE189">
         <v>2</v>
       </c>
+      <c r="CH189">
+        <v>0</v>
+      </c>
+      <c r="CJ189">
+        <v>2</v>
+      </c>
     </row>
-    <row r="190" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="190" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -31635,8 +32985,14 @@
       <c r="CG190">
         <v>1</v>
       </c>
+      <c r="CH190">
+        <v>0</v>
+      </c>
+      <c r="CI190">
+        <v>5</v>
+      </c>
     </row>
-    <row r="191" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="191" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -31826,8 +33182,14 @@
       <c r="CF191">
         <v>5</v>
       </c>
+      <c r="CH191">
+        <v>0</v>
+      </c>
+      <c r="CI191">
+        <v>5</v>
+      </c>
     </row>
-    <row r="192" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="192" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -31996,8 +33358,14 @@
       <c r="CF192">
         <v>3</v>
       </c>
+      <c r="CH192">
+        <v>0</v>
+      </c>
+      <c r="CI192">
+        <v>3</v>
+      </c>
     </row>
-    <row r="193" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="193" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -32187,8 +33555,14 @@
       <c r="CF193">
         <v>4</v>
       </c>
+      <c r="CH193">
+        <v>3</v>
+      </c>
+      <c r="CI193">
+        <v>4</v>
+      </c>
     </row>
-    <row r="194" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="194" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B194" t="s">
         <v>4</v>
       </c>
@@ -32354,8 +33728,14 @@
       <c r="CF194">
         <v>1</v>
       </c>
+      <c r="CH194">
+        <v>6</v>
+      </c>
+      <c r="CI194">
+        <v>1</v>
+      </c>
     </row>
-    <row r="195" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="195" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -32536,8 +33916,14 @@
       <c r="CE195">
         <v>2</v>
       </c>
+      <c r="CH195">
+        <v>1</v>
+      </c>
+      <c r="CI195">
+        <v>1</v>
+      </c>
     </row>
-    <row r="196" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="196" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -32754,8 +34140,14 @@
       <c r="CF196">
         <v>9</v>
       </c>
+      <c r="CH196">
+        <v>0</v>
+      </c>
+      <c r="CI196">
+        <v>9</v>
+      </c>
     </row>
-    <row r="197" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="197" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -32927,8 +34319,14 @@
       <c r="CF197">
         <v>4</v>
       </c>
+      <c r="CH197">
+        <v>0</v>
+      </c>
+      <c r="CI197">
+        <v>4</v>
+      </c>
     </row>
-    <row r="198" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="198" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -33079,8 +34477,17 @@
       <c r="CG198">
         <v>1</v>
       </c>
+      <c r="CH198">
+        <v>0</v>
+      </c>
+      <c r="CI198">
+        <v>4</v>
+      </c>
+      <c r="CJ198">
+        <v>1</v>
+      </c>
     </row>
-    <row r="199" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="199" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -33246,8 +34653,14 @@
       <c r="CG199">
         <v>1</v>
       </c>
+      <c r="CH199">
+        <v>5</v>
+      </c>
+      <c r="CJ199">
+        <v>1</v>
+      </c>
     </row>
-    <row r="200" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="200" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
         <v>4</v>
       </c>
@@ -33404,8 +34817,17 @@
       <c r="CG200">
         <v>4</v>
       </c>
+      <c r="CH200">
+        <v>0</v>
+      </c>
+      <c r="CI200">
+        <v>6</v>
+      </c>
+      <c r="CJ200">
+        <v>1</v>
+      </c>
     </row>
-    <row r="201" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="201" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -33604,8 +35026,14 @@
       <c r="CG201">
         <v>1</v>
       </c>
+      <c r="CH201">
+        <v>1</v>
+      </c>
+      <c r="CI201">
+        <v>5</v>
+      </c>
     </row>
-    <row r="202" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="202" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -33795,8 +35223,14 @@
       <c r="CF202">
         <v>1</v>
       </c>
+      <c r="CH202">
+        <v>0</v>
+      </c>
+      <c r="CI202">
+        <v>1</v>
+      </c>
     </row>
-    <row r="203" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="203" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -33980,8 +35414,14 @@
       <c r="CF203">
         <v>3</v>
       </c>
+      <c r="CH203">
+        <v>0</v>
+      </c>
+      <c r="CI203">
+        <v>3</v>
+      </c>
     </row>
-    <row r="204" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="204" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -34090,8 +35530,11 @@
       <c r="CE204">
         <v>6</v>
       </c>
+      <c r="CH204">
+        <v>6</v>
+      </c>
     </row>
-    <row r="205" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="205" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -34287,8 +35730,17 @@
       <c r="CG205">
         <v>1</v>
       </c>
+      <c r="CH205">
+        <v>8</v>
+      </c>
+      <c r="CI205">
+        <v>1</v>
+      </c>
+      <c r="CJ205">
+        <v>1</v>
+      </c>
     </row>
-    <row r="206" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="206" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B206" t="s">
         <v>4</v>
       </c>
@@ -34397,8 +35849,14 @@
       <c r="CE206">
         <v>6</v>
       </c>
+      <c r="CH206">
+        <v>0</v>
+      </c>
+      <c r="CI206">
+        <v>6</v>
+      </c>
     </row>
-    <row r="207" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="207" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -34549,8 +36007,17 @@
       <c r="CF207">
         <v>2</v>
       </c>
+      <c r="CH207">
+        <v>1</v>
+      </c>
+      <c r="CI207">
+        <v>2</v>
+      </c>
+      <c r="CJ207">
+        <v>1</v>
+      </c>
     </row>
-    <row r="208" spans="2:85" x14ac:dyDescent="0.3">
+    <row r="208" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -34734,8 +36201,14 @@
       <c r="CF208">
         <v>3</v>
       </c>
+      <c r="CH208">
+        <v>0</v>
+      </c>
+      <c r="CI208">
+        <v>3</v>
+      </c>
     </row>
-    <row r="209" spans="2:84" x14ac:dyDescent="0.3">
+    <row r="209" spans="2:87" x14ac:dyDescent="0.3">
       <c r="B209" t="s">
         <v>3</v>
       </c>
@@ -34904,8 +36377,14 @@
       <c r="CF209">
         <v>5</v>
       </c>
+      <c r="CH209">
+        <v>0</v>
+      </c>
+      <c r="CI209">
+        <v>5</v>
+      </c>
     </row>
-    <row r="210" spans="2:84" x14ac:dyDescent="0.3">
+    <row r="210" spans="2:87" x14ac:dyDescent="0.3">
       <c r="B210" t="s">
         <v>1</v>
       </c>
@@ -35095,8 +36574,14 @@
       <c r="CF210">
         <v>1</v>
       </c>
+      <c r="CH210">
+        <v>4</v>
+      </c>
+      <c r="CI210">
+        <v>1</v>
+      </c>
     </row>
-    <row r="211" spans="2:84" x14ac:dyDescent="0.3">
+    <row r="211" spans="2:87" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
         <v>4</v>
       </c>
@@ -35262,8 +36747,14 @@
       <c r="CF211">
         <v>2</v>
       </c>
+      <c r="CH211">
+        <v>3</v>
+      </c>
+      <c r="CI211">
+        <v>2</v>
+      </c>
     </row>
-    <row r="212" spans="2:84" x14ac:dyDescent="0.3">
+    <row r="212" spans="2:87" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
         <v>4</v>
       </c>
@@ -35423,7 +36914,14 @@
       <c r="CF212">
         <v>1</v>
       </c>
+      <c r="CH212">
+        <v>5</v>
+      </c>
+      <c r="CI212">
+        <v>1</v>
+      </c>
     </row>
+    <row r="213" spans="2:87" hidden="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
DOY 154 germinants data collection
</commit_message>
<xml_diff>
--- a/data/germination_data.xlsx
+++ b/data/germination_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ailun\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temporal Ecology Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6D83FF4-006A-4F8F-BDE1-C297DAD05134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D7BFCE4-6EB9-4777-BFCA-89E73DC8D008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="128">
   <si>
     <t>seed_species</t>
   </si>
@@ -447,6 +447,15 @@
   <si>
     <t>140_halfdead</t>
   </si>
+  <si>
+    <t>154_alive</t>
+  </si>
+  <si>
+    <t>154_dead</t>
+  </si>
+  <si>
+    <t>154_halfdead</t>
+  </si>
 </sst>
 </file>
 
@@ -550,15 +559,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CJ213" totalsRowShown="0">
-  <autoFilter ref="B2:CJ213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="25"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
-  <tableColumns count="87">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CM213" totalsRowShown="0">
+  <autoFilter ref="B2:CM213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
+  <tableColumns count="90">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
     <tableColumn id="3" xr3:uid="{B695F4B4-8561-9D48-9FF3-12A40CB2B7C7}" name="inoculated_%"/>
@@ -646,6 +649,9 @@
     <tableColumn id="85" xr3:uid="{563B32CE-FAA2-4820-A00E-BA719FBA6A1E}" name="140_alive"/>
     <tableColumn id="86" xr3:uid="{12BABDCE-FBD8-4A85-BAA6-7981A89F386D}" name="140_dead"/>
     <tableColumn id="87" xr3:uid="{644BBFBD-A683-4B49-8F95-95C2D3663641}" name="140_halfdead"/>
+    <tableColumn id="88" xr3:uid="{5C77EBFE-EDC9-455C-A405-C2A7DA5D973E}" name="154_alive"/>
+    <tableColumn id="89" xr3:uid="{1762B7C6-1B6C-4691-AC50-45E17B49E79D}" name="154_dead"/>
+    <tableColumn id="90" xr3:uid="{E94F12E3-B02B-47BA-8281-4BD0C9F47EA5}" name="154_halfdead"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -968,7 +974,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:CJ213"/>
+  <dimension ref="B2:CM212"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -976,7 +982,7 @@
     <col min="4" max="4" width="17.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -1238,8 +1244,17 @@
       <c r="CJ2" t="s">
         <v>124</v>
       </c>
+      <c r="CK2" t="s">
+        <v>125</v>
+      </c>
+      <c r="CL2" t="s">
+        <v>126</v>
+      </c>
+      <c r="CM2" t="s">
+        <v>127</v>
+      </c>
     </row>
-    <row r="3" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1441,8 +1456,14 @@
       <c r="CI3">
         <v>2</v>
       </c>
+      <c r="CK3">
+        <v>1</v>
+      </c>
+      <c r="CL3">
+        <v>3</v>
+      </c>
     </row>
-    <row r="4" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1560,8 +1581,11 @@
       <c r="CH4">
         <v>9</v>
       </c>
+      <c r="CK4">
+        <v>9</v>
+      </c>
     </row>
-    <row r="5" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1763,8 +1787,14 @@
       <c r="CI5">
         <v>7</v>
       </c>
+      <c r="CK5">
+        <v>0</v>
+      </c>
+      <c r="CL5">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1879,8 +1909,11 @@
       <c r="CH6">
         <v>9</v>
       </c>
+      <c r="CK6">
+        <v>9</v>
+      </c>
     </row>
-    <row r="7" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -2046,8 +2079,14 @@
       <c r="CI7">
         <v>4</v>
       </c>
+      <c r="CK7">
+        <v>1</v>
+      </c>
+      <c r="CL7">
+        <v>5</v>
+      </c>
     </row>
-    <row r="8" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -2240,8 +2279,14 @@
       <c r="CI8">
         <v>1</v>
       </c>
+      <c r="CK8">
+        <v>6</v>
+      </c>
+      <c r="CL8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2440,8 +2485,14 @@
       <c r="CI9">
         <v>1</v>
       </c>
+      <c r="CK9">
+        <v>6</v>
+      </c>
+      <c r="CL9">
+        <v>1</v>
+      </c>
     </row>
-    <row r="10" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -2574,8 +2625,14 @@
       <c r="CJ10">
         <v>1</v>
       </c>
+      <c r="CK10">
+        <v>6</v>
+      </c>
+      <c r="CL10">
+        <v>2</v>
+      </c>
     </row>
-    <row r="11" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -2774,8 +2831,14 @@
       <c r="CJ11">
         <v>1</v>
       </c>
+      <c r="CK11">
+        <v>0</v>
+      </c>
+      <c r="CL11">
+        <v>8</v>
+      </c>
     </row>
-    <row r="12" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -2977,8 +3040,14 @@
       <c r="CI12">
         <v>5</v>
       </c>
+      <c r="CK12">
+        <v>5</v>
+      </c>
+      <c r="CL12">
+        <v>5</v>
+      </c>
     </row>
-    <row r="13" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -3171,8 +3240,14 @@
       <c r="CJ13">
         <v>2</v>
       </c>
+      <c r="CK13">
+        <v>0</v>
+      </c>
+      <c r="CL13">
+        <v>7</v>
+      </c>
     </row>
-    <row r="14" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -3323,8 +3398,14 @@
       <c r="CI14">
         <v>1</v>
       </c>
+      <c r="CK14">
+        <v>8</v>
+      </c>
+      <c r="CL14">
+        <v>1</v>
+      </c>
     </row>
-    <row r="15" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -3506,8 +3587,14 @@
       <c r="CJ15">
         <v>4</v>
       </c>
+      <c r="CK15">
+        <v>0</v>
+      </c>
+      <c r="CL15">
+        <v>8</v>
+      </c>
     </row>
-    <row r="16" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -3671,8 +3758,14 @@
       <c r="CI16">
         <v>1</v>
       </c>
+      <c r="CK16">
+        <v>8</v>
+      </c>
+      <c r="CL16">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -3857,8 +3950,14 @@
       <c r="CI17">
         <v>8</v>
       </c>
+      <c r="CK17">
+        <v>0</v>
+      </c>
+      <c r="CL17">
+        <v>8</v>
+      </c>
     </row>
-    <row r="18" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -3971,8 +4070,11 @@
       <c r="CH18">
         <v>10</v>
       </c>
+      <c r="CK18">
+        <v>10</v>
+      </c>
     </row>
-    <row r="19" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -4175,8 +4277,14 @@
       <c r="CI19">
         <v>7</v>
       </c>
+      <c r="CK19">
+        <v>0</v>
+      </c>
+      <c r="CL19">
+        <v>7</v>
+      </c>
     </row>
-    <row r="20" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -4340,8 +4448,14 @@
       <c r="CI20">
         <v>1</v>
       </c>
+      <c r="CK20">
+        <v>13</v>
+      </c>
+      <c r="CL20">
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -4510,8 +4624,14 @@
       <c r="CI21">
         <v>6</v>
       </c>
+      <c r="CK21">
+        <v>0</v>
+      </c>
+      <c r="CL21">
+        <v>6</v>
+      </c>
     </row>
-    <row r="22" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -4630,8 +4750,17 @@
       <c r="CH22">
         <v>8</v>
       </c>
+      <c r="CK22">
+        <v>6</v>
+      </c>
+      <c r="CL22">
+        <v>1</v>
+      </c>
+      <c r="CM22">
+        <v>1</v>
+      </c>
     </row>
-    <row r="23" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -4828,8 +4957,14 @@
       <c r="CJ23">
         <v>3</v>
       </c>
+      <c r="CK23">
+        <v>0</v>
+      </c>
+      <c r="CL23">
+        <v>10</v>
+      </c>
     </row>
-    <row r="24" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -4999,8 +5134,14 @@
       <c r="CI24">
         <v>4</v>
       </c>
+      <c r="CK24">
+        <v>8</v>
+      </c>
+      <c r="CL24">
+        <v>4</v>
+      </c>
     </row>
-    <row r="25" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -5119,8 +5260,14 @@
       <c r="CJ25">
         <v>1</v>
       </c>
+      <c r="CK25">
+        <v>0</v>
+      </c>
+      <c r="CL25">
+        <v>8</v>
+      </c>
     </row>
-    <row r="26" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -5362,8 +5509,17 @@
       <c r="CJ26">
         <v>3</v>
       </c>
+      <c r="CK26">
+        <v>1</v>
+      </c>
+      <c r="CL26">
+        <v>9</v>
+      </c>
+      <c r="CM26">
+        <v>1</v>
+      </c>
     </row>
-    <row r="27" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -5539,8 +5695,14 @@
       <c r="CJ27">
         <v>1</v>
       </c>
+      <c r="CK27">
+        <v>2</v>
+      </c>
+      <c r="CL27">
+        <v>4</v>
+      </c>
     </row>
-    <row r="28" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -5755,8 +5917,14 @@
       <c r="CI28">
         <v>3</v>
       </c>
+      <c r="CK28">
+        <v>6</v>
+      </c>
+      <c r="CL28">
+        <v>4</v>
+      </c>
     </row>
-    <row r="29" spans="2:88" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:91" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>3</v>
       </c>
@@ -5941,8 +6109,14 @@
       <c r="CI29" s="3">
         <v>4</v>
       </c>
+      <c r="CK29" s="3">
+        <v>0</v>
+      </c>
+      <c r="CL29" s="3">
+        <v>4</v>
+      </c>
     </row>
-    <row r="30" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -6061,8 +6235,11 @@
       <c r="CH30">
         <v>8</v>
       </c>
+      <c r="CK30">
+        <v>8</v>
+      </c>
     </row>
-    <row r="31" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -6265,8 +6442,14 @@
       <c r="CJ31">
         <v>2</v>
       </c>
+      <c r="CK31">
+        <v>0</v>
+      </c>
+      <c r="CL31">
+        <v>5</v>
+      </c>
     </row>
-    <row r="32" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -6427,8 +6610,14 @@
       <c r="CI32">
         <v>1</v>
       </c>
+      <c r="CK32">
+        <v>9</v>
+      </c>
+      <c r="CL32">
+        <v>1</v>
+      </c>
     </row>
-    <row r="33" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -6586,8 +6775,14 @@
       <c r="CJ33">
         <v>2</v>
       </c>
+      <c r="CK33">
+        <v>0</v>
+      </c>
+      <c r="CL33">
+        <v>9</v>
+      </c>
     </row>
-    <row r="34" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -6736,8 +6931,14 @@
       <c r="CJ34">
         <v>3</v>
       </c>
+      <c r="CK34">
+        <v>1</v>
+      </c>
+      <c r="CL34">
+        <v>5</v>
+      </c>
     </row>
-    <row r="35" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -6919,8 +7120,14 @@
       <c r="CJ35">
         <v>1</v>
       </c>
+      <c r="CK35">
+        <v>0</v>
+      </c>
+      <c r="CL35">
+        <v>8</v>
+      </c>
     </row>
-    <row r="36" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -7096,8 +7303,14 @@
       <c r="CI36">
         <v>2</v>
       </c>
+      <c r="CK36">
+        <v>8</v>
+      </c>
+      <c r="CL36">
+        <v>2</v>
+      </c>
     </row>
-    <row r="37" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -7220,10 +7433,16 @@
         <v>1</v>
       </c>
       <c r="CI37">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="CK37">
+        <v>1</v>
+      </c>
+      <c r="CL37">
+        <v>5</v>
       </c>
     </row>
-    <row r="38" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -7441,8 +7660,14 @@
       <c r="CI38">
         <v>4</v>
       </c>
+      <c r="CK38">
+        <v>2</v>
+      </c>
+      <c r="CL38">
+        <v>4</v>
+      </c>
     </row>
-    <row r="39" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -7639,8 +7864,14 @@
       <c r="CI39">
         <v>4</v>
       </c>
+      <c r="CK39">
+        <v>2</v>
+      </c>
+      <c r="CL39">
+        <v>4</v>
+      </c>
     </row>
-    <row r="40" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -7855,8 +8086,14 @@
       <c r="CJ40">
         <v>2</v>
       </c>
+      <c r="CK40">
+        <v>2</v>
+      </c>
+      <c r="CL40">
+        <v>8</v>
+      </c>
     </row>
-    <row r="41" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -8035,8 +8272,14 @@
       <c r="CI41">
         <v>6</v>
       </c>
+      <c r="CK41">
+        <v>0</v>
+      </c>
+      <c r="CL41">
+        <v>6</v>
+      </c>
     </row>
-    <row r="42" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -8164,8 +8407,11 @@
       <c r="CJ42">
         <v>2</v>
       </c>
+      <c r="CK42">
+        <v>7</v>
+      </c>
     </row>
-    <row r="43" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -8371,8 +8617,14 @@
       <c r="CJ43">
         <v>2</v>
       </c>
+      <c r="CK43">
+        <v>0</v>
+      </c>
+      <c r="CL43">
+        <v>9</v>
+      </c>
     </row>
-    <row r="44" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -8485,8 +8737,14 @@
       <c r="CJ44">
         <v>3</v>
       </c>
+      <c r="CK44">
+        <v>2</v>
+      </c>
+      <c r="CM44">
+        <v>4</v>
+      </c>
     </row>
-    <row r="45" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -8734,8 +8992,14 @@
       <c r="CI45">
         <v>9</v>
       </c>
+      <c r="CK45">
+        <v>0</v>
+      </c>
+      <c r="CL45">
+        <v>9</v>
+      </c>
     </row>
-    <row r="46" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -8857,8 +9121,14 @@
       <c r="CJ46">
         <v>3</v>
       </c>
+      <c r="CK46">
+        <v>1</v>
+      </c>
+      <c r="CL46">
+        <v>5</v>
+      </c>
     </row>
-    <row r="47" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -9010,8 +9280,14 @@
       <c r="CI47">
         <v>9</v>
       </c>
+      <c r="CK47">
+        <v>0</v>
+      </c>
+      <c r="CL47">
+        <v>9</v>
+      </c>
     </row>
-    <row r="48" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -9232,8 +9508,14 @@
       <c r="CI48">
         <v>10</v>
       </c>
+      <c r="CK48">
+        <v>1</v>
+      </c>
+      <c r="CL48">
+        <v>10</v>
+      </c>
     </row>
-    <row r="49" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -9361,8 +9643,14 @@
       <c r="CJ49">
         <v>1</v>
       </c>
+      <c r="CK49">
+        <v>1</v>
+      </c>
+      <c r="CL49">
+        <v>6</v>
+      </c>
     </row>
-    <row r="50" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -9583,8 +9871,17 @@
       <c r="CI50">
         <v>2</v>
       </c>
+      <c r="CK50">
+        <v>4</v>
+      </c>
+      <c r="CL50">
+        <v>3</v>
+      </c>
+      <c r="CM50">
+        <v>1</v>
+      </c>
     </row>
-    <row r="51" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -9796,8 +10093,14 @@
       <c r="CJ51">
         <v>2</v>
       </c>
+      <c r="CK51">
+        <v>1</v>
+      </c>
+      <c r="CL51">
+        <v>5</v>
+      </c>
     </row>
-    <row r="52" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -9910,8 +10213,14 @@
       <c r="CH52">
         <v>6</v>
       </c>
+      <c r="CK52">
+        <v>5</v>
+      </c>
+      <c r="CM52">
+        <v>1</v>
+      </c>
     </row>
-    <row r="53" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -10096,8 +10405,14 @@
       <c r="CI53">
         <v>4</v>
       </c>
+      <c r="CK53">
+        <v>0</v>
+      </c>
+      <c r="CL53">
+        <v>4</v>
+      </c>
     </row>
-    <row r="54" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -10216,8 +10531,11 @@
       <c r="CH54">
         <v>5</v>
       </c>
+      <c r="CK54">
+        <v>6</v>
+      </c>
     </row>
-    <row r="55" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -10402,8 +10720,17 @@
       <c r="CJ55">
         <v>2</v>
       </c>
+      <c r="CK55">
+        <v>0</v>
+      </c>
+      <c r="CL55">
+        <v>4</v>
+      </c>
+      <c r="CM55">
+        <v>2</v>
+      </c>
     </row>
-    <row r="56" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -10522,8 +10849,11 @@
       <c r="CH56">
         <v>10</v>
       </c>
+      <c r="CK56">
+        <v>10</v>
+      </c>
     </row>
-    <row r="57" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -10657,8 +10987,14 @@
       <c r="CI57">
         <v>1</v>
       </c>
+      <c r="CK57">
+        <v>6</v>
+      </c>
+      <c r="CL57">
+        <v>1</v>
+      </c>
     </row>
-    <row r="58" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -10783,8 +11119,14 @@
       <c r="CJ58">
         <v>1</v>
       </c>
+      <c r="CK58">
+        <v>2</v>
+      </c>
+      <c r="CL58">
+        <v>4</v>
+      </c>
     </row>
-    <row r="59" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -10906,8 +11248,14 @@
       <c r="CJ59">
         <v>1</v>
       </c>
+      <c r="CK59">
+        <v>0</v>
+      </c>
+      <c r="CL59">
+        <v>7</v>
+      </c>
     </row>
-    <row r="60" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -11086,8 +11434,14 @@
       <c r="CI60">
         <v>2</v>
       </c>
+      <c r="CK60">
+        <v>7</v>
+      </c>
+      <c r="CL60">
+        <v>2</v>
+      </c>
     </row>
-    <row r="61" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -11218,8 +11572,14 @@
       <c r="CJ61">
         <v>2</v>
       </c>
+      <c r="CK61">
+        <v>3</v>
+      </c>
+      <c r="CL61">
+        <v>4</v>
+      </c>
     </row>
-    <row r="62" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -11428,8 +11788,14 @@
       <c r="CI62">
         <v>2</v>
       </c>
+      <c r="CK62">
+        <v>3</v>
+      </c>
+      <c r="CL62">
+        <v>2</v>
+      </c>
     </row>
-    <row r="63" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -11638,8 +12004,14 @@
       <c r="CJ63">
         <v>2</v>
       </c>
+      <c r="CK63">
+        <v>0</v>
+      </c>
+      <c r="CL63">
+        <v>9</v>
+      </c>
     </row>
-    <row r="64" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -11818,8 +12190,17 @@
       <c r="CJ64">
         <v>1</v>
       </c>
+      <c r="CK64">
+        <v>6</v>
+      </c>
+      <c r="CL64">
+        <v>3</v>
+      </c>
+      <c r="CM64">
+        <v>1</v>
+      </c>
     </row>
-    <row r="65" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -12001,8 +12382,14 @@
       <c r="CJ65">
         <v>1</v>
       </c>
+      <c r="CK65">
+        <v>0</v>
+      </c>
+      <c r="CL65">
+        <v>6</v>
+      </c>
     </row>
-    <row r="66" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -12127,8 +12514,11 @@
       <c r="CJ66">
         <v>1</v>
       </c>
+      <c r="CK66">
+        <v>5</v>
+      </c>
     </row>
-    <row r="67" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -12337,8 +12727,17 @@
       <c r="CJ67">
         <v>1</v>
       </c>
+      <c r="CK67">
+        <v>0</v>
+      </c>
+      <c r="CL67">
+        <v>9</v>
+      </c>
+      <c r="CM67">
+        <v>1</v>
+      </c>
     </row>
-    <row r="68" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -12448,8 +12847,11 @@
       <c r="CH68">
         <v>11</v>
       </c>
+      <c r="CK68">
+        <v>11</v>
+      </c>
     </row>
-    <row r="69" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -12568,8 +12970,17 @@
       <c r="CJ69">
         <v>2</v>
       </c>
+      <c r="CK69">
+        <v>0</v>
+      </c>
+      <c r="CL69">
+        <v>8</v>
+      </c>
+      <c r="CM69">
+        <v>1</v>
+      </c>
     </row>
-    <row r="70" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -12691,8 +13102,17 @@
       <c r="CH70">
         <v>8</v>
       </c>
+      <c r="CK70">
+        <v>2</v>
+      </c>
+      <c r="CL70">
+        <v>4</v>
+      </c>
+      <c r="CM70">
+        <v>2</v>
+      </c>
     </row>
-    <row r="71" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -12895,8 +13315,14 @@
       <c r="CJ71">
         <v>1</v>
       </c>
+      <c r="CK71">
+        <v>0</v>
+      </c>
+      <c r="CL71">
+        <v>10</v>
+      </c>
     </row>
-    <row r="72" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -13084,8 +13510,14 @@
       <c r="CI72">
         <v>1</v>
       </c>
+      <c r="CK72">
+        <v>6</v>
+      </c>
+      <c r="CL72">
+        <v>1</v>
+      </c>
     </row>
-    <row r="73" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -13204,8 +13636,14 @@
       <c r="CJ73">
         <v>3</v>
       </c>
+      <c r="CK73">
+        <v>2</v>
+      </c>
+      <c r="CL73">
+        <v>8</v>
+      </c>
     </row>
-    <row r="74" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -13327,8 +13765,11 @@
       <c r="CH74">
         <v>9</v>
       </c>
+      <c r="CK74">
+        <v>9</v>
+      </c>
     </row>
-    <row r="75" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -13516,8 +13957,14 @@
       <c r="CJ75">
         <v>3</v>
       </c>
+      <c r="CK75">
+        <v>1</v>
+      </c>
+      <c r="CL75">
+        <v>8</v>
+      </c>
     </row>
-    <row r="76" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -13723,8 +14170,17 @@
       <c r="CI76">
         <v>1</v>
       </c>
+      <c r="CK76">
+        <v>6</v>
+      </c>
+      <c r="CL76">
+        <v>1</v>
+      </c>
+      <c r="CM76">
+        <v>1</v>
+      </c>
     </row>
-    <row r="77" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -13897,8 +14353,14 @@
       <c r="CI77">
         <v>7</v>
       </c>
+      <c r="CK77">
+        <v>0</v>
+      </c>
+      <c r="CL77">
+        <v>7</v>
+      </c>
     </row>
-    <row r="78" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -14015,13 +14477,16 @@
         <v>3</v>
       </c>
       <c r="CH78">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="CJ78">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="CK78">
+        <v>7</v>
       </c>
     </row>
-    <row r="79" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -14224,8 +14689,17 @@
       <c r="CJ79">
         <v>1</v>
       </c>
+      <c r="CK79">
+        <v>1</v>
+      </c>
+      <c r="CL79">
+        <v>7</v>
+      </c>
+      <c r="CM79">
+        <v>1</v>
+      </c>
     </row>
-    <row r="80" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -14398,8 +14872,14 @@
       <c r="CI80">
         <v>1</v>
       </c>
+      <c r="CK80">
+        <v>9</v>
+      </c>
+      <c r="CL80">
+        <v>1</v>
+      </c>
     </row>
-    <row r="81" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -14584,8 +15064,14 @@
       <c r="CJ81">
         <v>1</v>
       </c>
+      <c r="CK81">
+        <v>0</v>
+      </c>
+      <c r="CL81">
+        <v>7</v>
+      </c>
     </row>
-    <row r="82" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -14809,8 +15295,14 @@
       <c r="CJ82">
         <v>2</v>
       </c>
+      <c r="CK82">
+        <v>0</v>
+      </c>
+      <c r="CL82">
+        <v>10</v>
+      </c>
     </row>
-    <row r="83" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -15016,8 +15508,14 @@
       <c r="CJ83">
         <v>1</v>
       </c>
+      <c r="CK83">
+        <v>0</v>
+      </c>
+      <c r="CL83">
+        <v>9</v>
+      </c>
     </row>
-    <row r="84" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -15217,8 +15715,14 @@
       <c r="CI84">
         <v>2</v>
       </c>
+      <c r="CK84">
+        <v>7</v>
+      </c>
+      <c r="CL84">
+        <v>2</v>
+      </c>
     </row>
-    <row r="85" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -15424,8 +15928,14 @@
       <c r="CJ85">
         <v>1</v>
       </c>
+      <c r="CK85">
+        <v>0</v>
+      </c>
+      <c r="CL85">
+        <v>6</v>
+      </c>
     </row>
-    <row r="86" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -15607,8 +16117,17 @@
       <c r="CJ86">
         <v>3</v>
       </c>
+      <c r="CK86">
+        <v>2</v>
+      </c>
+      <c r="CL86">
+        <v>6</v>
+      </c>
+      <c r="CM86">
+        <v>1</v>
+      </c>
     </row>
-    <row r="87" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -15814,8 +16333,17 @@
       <c r="CJ87">
         <v>1</v>
       </c>
+      <c r="CK87">
+        <v>0</v>
+      </c>
+      <c r="CL87">
+        <v>6</v>
+      </c>
+      <c r="CM87">
+        <v>1</v>
+      </c>
     </row>
-    <row r="88" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -16006,8 +16534,14 @@
       <c r="CI88">
         <v>3</v>
       </c>
+      <c r="CK88">
+        <v>6</v>
+      </c>
+      <c r="CL88">
+        <v>3</v>
+      </c>
     </row>
-    <row r="89" spans="2:88" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:91" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>3</v>
       </c>
@@ -16177,8 +16711,14 @@
       <c r="CJ89" s="3">
         <v>1</v>
       </c>
+      <c r="CK89" s="3">
+        <v>0</v>
+      </c>
+      <c r="CL89" s="3">
+        <v>5</v>
+      </c>
     </row>
-    <row r="90" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -16297,8 +16837,14 @@
       <c r="CH90">
         <v>8</v>
       </c>
+      <c r="CK90">
+        <v>7</v>
+      </c>
+      <c r="CM90">
+        <v>1</v>
+      </c>
     </row>
-    <row r="91" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -16513,8 +17059,14 @@
       <c r="CJ91">
         <v>2</v>
       </c>
+      <c r="CK91">
+        <v>1</v>
+      </c>
+      <c r="CL91">
+        <v>5</v>
+      </c>
     </row>
-    <row r="92" spans="2:88" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:91" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>1</v>
       </c>
@@ -16708,8 +17260,14 @@
       <c r="CI92" s="3">
         <v>3</v>
       </c>
+      <c r="CK92" s="3">
+        <v>5</v>
+      </c>
+      <c r="CL92" s="3">
+        <v>3</v>
+      </c>
     </row>
-    <row r="93" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -16864,8 +17422,14 @@
       <c r="CJ93">
         <v>1</v>
       </c>
+      <c r="CK93">
+        <v>0</v>
+      </c>
+      <c r="CL93">
+        <v>9</v>
+      </c>
     </row>
-    <row r="94" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -16990,8 +17554,14 @@
       <c r="CJ94">
         <v>4</v>
       </c>
+      <c r="CK94">
+        <v>0</v>
+      </c>
+      <c r="CL94">
+        <v>7</v>
+      </c>
     </row>
-    <row r="95" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -17155,8 +17725,14 @@
       <c r="CJ95">
         <v>2</v>
       </c>
+      <c r="CK95">
+        <v>0</v>
+      </c>
+      <c r="CL95">
+        <v>8</v>
+      </c>
     </row>
-    <row r="96" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -17341,8 +17917,17 @@
       <c r="CI96">
         <v>5</v>
       </c>
+      <c r="CK96">
+        <v>4</v>
+      </c>
+      <c r="CL96">
+        <v>5</v>
+      </c>
+      <c r="CM96">
+        <v>1</v>
+      </c>
     </row>
-    <row r="97" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -17470,8 +18055,14 @@
       <c r="CJ97">
         <v>3</v>
       </c>
+      <c r="CK97">
+        <v>1</v>
+      </c>
+      <c r="CL97">
+        <v>7</v>
+      </c>
     </row>
-    <row r="98" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -17656,8 +18247,14 @@
       <c r="CJ98">
         <v>1</v>
       </c>
+      <c r="CK98">
+        <v>1</v>
+      </c>
+      <c r="CL98">
+        <v>6</v>
+      </c>
     </row>
-    <row r="99" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -17794,8 +18391,14 @@
       <c r="CI99">
         <v>1</v>
       </c>
+      <c r="CK99">
+        <v>2</v>
+      </c>
+      <c r="CL99">
+        <v>1</v>
+      </c>
     </row>
-    <row r="100" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -17914,8 +18517,11 @@
       <c r="CH100">
         <v>8</v>
       </c>
+      <c r="CK100">
+        <v>8</v>
+      </c>
     </row>
-    <row r="101" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -18085,8 +18691,14 @@
       <c r="CI101">
         <v>4</v>
       </c>
+      <c r="CK101">
+        <v>1</v>
+      </c>
+      <c r="CL101">
+        <v>4</v>
+      </c>
     </row>
-    <row r="102" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -18208,8 +18820,17 @@
       <c r="CJ102">
         <v>2</v>
       </c>
+      <c r="CK102">
+        <v>3</v>
+      </c>
+      <c r="CL102">
+        <v>3</v>
+      </c>
+      <c r="CM102">
+        <v>1</v>
+      </c>
     </row>
-    <row r="103" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -18400,8 +19021,14 @@
       <c r="CI103">
         <v>6</v>
       </c>
+      <c r="CK103">
+        <v>0</v>
+      </c>
+      <c r="CL103">
+        <v>6</v>
+      </c>
     </row>
-    <row r="104" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -18589,8 +19216,14 @@
       <c r="CJ104">
         <v>3</v>
       </c>
+      <c r="CK104">
+        <v>2</v>
+      </c>
+      <c r="CL104">
+        <v>8</v>
+      </c>
     </row>
-    <row r="105" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -18772,8 +19405,14 @@
       <c r="CJ105">
         <v>1</v>
       </c>
+      <c r="CK105">
+        <v>0</v>
+      </c>
+      <c r="CL105">
+        <v>6</v>
+      </c>
     </row>
-    <row r="106" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -18943,8 +19582,17 @@
       <c r="CI106">
         <v>7</v>
       </c>
+      <c r="CK106">
+        <v>0</v>
+      </c>
+      <c r="CL106">
+        <v>7</v>
+      </c>
+      <c r="CM106">
+        <v>1</v>
+      </c>
     </row>
-    <row r="107" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -19138,8 +19786,14 @@
       <c r="CJ107">
         <v>1</v>
       </c>
+      <c r="CK107">
+        <v>0</v>
+      </c>
+      <c r="CL107">
+        <v>5</v>
+      </c>
     </row>
-    <row r="108" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -19318,8 +19972,14 @@
       <c r="CJ108">
         <v>4</v>
       </c>
+      <c r="CK108">
+        <v>0</v>
+      </c>
+      <c r="CL108">
+        <v>10</v>
+      </c>
     </row>
-    <row r="109" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -19513,8 +20173,14 @@
       <c r="CI109">
         <v>9</v>
       </c>
+      <c r="CK109">
+        <v>0</v>
+      </c>
+      <c r="CL109">
+        <v>9</v>
+      </c>
     </row>
-    <row r="110" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -19711,8 +20377,14 @@
       <c r="CI110">
         <v>3</v>
       </c>
+      <c r="CK110">
+        <v>6</v>
+      </c>
+      <c r="CL110">
+        <v>3</v>
+      </c>
     </row>
-    <row r="111" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -19894,8 +20566,14 @@
       <c r="CJ111">
         <v>2</v>
       </c>
+      <c r="CK111">
+        <v>5</v>
+      </c>
+      <c r="CL111">
+        <v>3</v>
+      </c>
     </row>
-    <row r="112" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -20083,8 +20761,17 @@
       <c r="CJ112">
         <v>2</v>
       </c>
+      <c r="CK112">
+        <v>5</v>
+      </c>
+      <c r="CL112">
+        <v>2</v>
+      </c>
+      <c r="CM112">
+        <v>1</v>
+      </c>
     </row>
-    <row r="113" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -20281,8 +20968,14 @@
       <c r="CI113">
         <v>2</v>
       </c>
+      <c r="CK113">
+        <v>4</v>
+      </c>
+      <c r="CL113">
+        <v>2</v>
+      </c>
     </row>
-    <row r="114" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -20404,8 +21097,14 @@
       <c r="CI114">
         <v>8</v>
       </c>
+      <c r="CK114">
+        <v>0</v>
+      </c>
+      <c r="CL114">
+        <v>8</v>
+      </c>
     </row>
-    <row r="115" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -20605,8 +21304,14 @@
       <c r="CI115">
         <v>4</v>
       </c>
+      <c r="CK115">
+        <v>0</v>
+      </c>
+      <c r="CL115">
+        <v>4</v>
+      </c>
     </row>
-    <row r="116" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -20791,8 +21496,14 @@
       <c r="CJ116">
         <v>1</v>
       </c>
+      <c r="CK116">
+        <v>0</v>
+      </c>
+      <c r="CL116">
+        <v>8</v>
+      </c>
     </row>
-    <row r="117" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -20983,8 +21694,14 @@
       <c r="CI117">
         <v>5</v>
       </c>
+      <c r="CK117">
+        <v>0</v>
+      </c>
+      <c r="CL117">
+        <v>5</v>
+      </c>
     </row>
-    <row r="118" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -21116,8 +21833,14 @@
       <c r="CJ118">
         <v>2</v>
       </c>
+      <c r="CK118">
+        <v>0</v>
+      </c>
+      <c r="CL118">
+        <v>6</v>
+      </c>
     </row>
-    <row r="119" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -21251,8 +21974,14 @@
       <c r="CJ119">
         <v>3</v>
       </c>
+      <c r="CK119">
+        <v>0</v>
+      </c>
+      <c r="CL119">
+        <v>7</v>
+      </c>
     </row>
-    <row r="120" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -21377,8 +22106,14 @@
       <c r="CJ120">
         <v>1</v>
       </c>
+      <c r="CK120">
+        <v>0</v>
+      </c>
+      <c r="CL120">
+        <v>10</v>
+      </c>
     </row>
-    <row r="121" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -21500,8 +22235,17 @@
       <c r="CJ121">
         <v>3</v>
       </c>
+      <c r="CK121">
+        <v>0</v>
+      </c>
+      <c r="CL121">
+        <v>6</v>
+      </c>
+      <c r="CM121">
+        <v>2</v>
+      </c>
     </row>
-    <row r="122" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -21626,8 +22370,17 @@
       <c r="CJ122">
         <v>1</v>
       </c>
+      <c r="CK122">
+        <v>1</v>
+      </c>
+      <c r="CL122">
+        <v>4</v>
+      </c>
+      <c r="CM122">
+        <v>1</v>
+      </c>
     </row>
-    <row r="123" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -21806,8 +22559,14 @@
       <c r="CI123">
         <v>3</v>
       </c>
+      <c r="CK123">
+        <v>3</v>
+      </c>
+      <c r="CL123">
+        <v>3</v>
+      </c>
     </row>
-    <row r="124" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -22022,8 +22781,17 @@
       <c r="CJ124">
         <v>2</v>
       </c>
+      <c r="CK124">
+        <v>2</v>
+      </c>
+      <c r="CL124">
+        <v>6</v>
+      </c>
+      <c r="CM124">
+        <v>1</v>
+      </c>
     </row>
-    <row r="125" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -22229,8 +22997,14 @@
       <c r="CI125">
         <v>6</v>
       </c>
+      <c r="CK125">
+        <v>0</v>
+      </c>
+      <c r="CL125">
+        <v>6</v>
+      </c>
     </row>
-    <row r="126" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -22418,8 +23192,14 @@
       <c r="CJ126">
         <v>1</v>
       </c>
+      <c r="CK126">
+        <v>0</v>
+      </c>
+      <c r="CL126">
+        <v>6</v>
+      </c>
     </row>
-    <row r="127" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -22601,8 +23381,14 @@
       <c r="CI127">
         <v>3</v>
       </c>
+      <c r="CK127">
+        <v>0</v>
+      </c>
+      <c r="CL127">
+        <v>3</v>
+      </c>
     </row>
-    <row r="128" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -22715,8 +23501,14 @@
       <c r="CI128">
         <v>7</v>
       </c>
+      <c r="CK128">
+        <v>0</v>
+      </c>
+      <c r="CL128">
+        <v>7</v>
+      </c>
     </row>
-    <row r="129" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -22913,8 +23705,14 @@
       <c r="CI129">
         <v>6</v>
       </c>
+      <c r="CK129">
+        <v>0</v>
+      </c>
+      <c r="CL129">
+        <v>6</v>
+      </c>
     </row>
-    <row r="130" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -23048,8 +23846,14 @@
       <c r="CJ130">
         <v>1</v>
       </c>
+      <c r="CK130">
+        <v>0</v>
+      </c>
+      <c r="CL130">
+        <v>10</v>
+      </c>
     </row>
-    <row r="131" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -23249,8 +24053,14 @@
       <c r="CJ131">
         <v>3</v>
       </c>
+      <c r="CK131">
+        <v>0</v>
+      </c>
+      <c r="CL131">
+        <v>10</v>
+      </c>
     </row>
-    <row r="132" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -23372,8 +24182,14 @@
       <c r="CI132">
         <v>6</v>
       </c>
+      <c r="CK132">
+        <v>0</v>
+      </c>
+      <c r="CL132">
+        <v>6</v>
+      </c>
     </row>
-    <row r="133" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -23528,8 +24344,14 @@
       <c r="CI133">
         <v>7</v>
       </c>
+      <c r="CK133">
+        <v>0</v>
+      </c>
+      <c r="CL133">
+        <v>7</v>
+      </c>
     </row>
-    <row r="134" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -23684,8 +24506,14 @@
       <c r="CJ134">
         <v>3</v>
       </c>
+      <c r="CK134">
+        <v>2</v>
+      </c>
+      <c r="CL134">
+        <v>8</v>
+      </c>
     </row>
-    <row r="135" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -23861,8 +24689,14 @@
       <c r="CI135">
         <v>7</v>
       </c>
+      <c r="CK135">
+        <v>1</v>
+      </c>
+      <c r="CL135">
+        <v>7</v>
+      </c>
     </row>
-    <row r="136" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -24032,8 +24866,14 @@
       <c r="CJ136">
         <v>3</v>
       </c>
+      <c r="CK136">
+        <v>0</v>
+      </c>
+      <c r="CL136">
+        <v>7</v>
+      </c>
     </row>
-    <row r="137" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -24206,8 +25046,14 @@
       <c r="CI137">
         <v>2</v>
       </c>
+      <c r="CK137">
+        <v>3</v>
+      </c>
+      <c r="CL137">
+        <v>2</v>
+      </c>
     </row>
-    <row r="138" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -24398,8 +25244,14 @@
       <c r="CI138">
         <v>7</v>
       </c>
+      <c r="CK138">
+        <v>0</v>
+      </c>
+      <c r="CL138">
+        <v>7</v>
+      </c>
     </row>
-    <row r="139" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -24572,8 +25424,14 @@
       <c r="CI139">
         <v>5</v>
       </c>
+      <c r="CK139">
+        <v>0</v>
+      </c>
+      <c r="CL139">
+        <v>5</v>
+      </c>
     </row>
-    <row r="140" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -24701,8 +25559,14 @@
       <c r="CJ140">
         <v>1</v>
       </c>
+      <c r="CK140">
+        <v>0</v>
+      </c>
+      <c r="CL140">
+        <v>9</v>
+      </c>
     </row>
-    <row r="141" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -24911,8 +25775,14 @@
       <c r="CI141">
         <v>8</v>
       </c>
+      <c r="CK141">
+        <v>0</v>
+      </c>
+      <c r="CL141">
+        <v>8</v>
+      </c>
     </row>
-    <row r="142" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -25121,8 +25991,14 @@
       <c r="CJ142">
         <v>1</v>
       </c>
+      <c r="CK142">
+        <v>0</v>
+      </c>
+      <c r="CL142">
+        <v>8</v>
+      </c>
     </row>
-    <row r="143" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -25289,8 +26165,14 @@
       <c r="CJ143">
         <v>2</v>
       </c>
+      <c r="CK143">
+        <v>0</v>
+      </c>
+      <c r="CL143">
+        <v>11</v>
+      </c>
     </row>
-    <row r="144" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -25409,8 +26291,14 @@
       <c r="CI144">
         <v>7</v>
       </c>
+      <c r="CK144">
+        <v>0</v>
+      </c>
+      <c r="CL144">
+        <v>7</v>
+      </c>
     </row>
-    <row r="145" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -25538,8 +26426,14 @@
       <c r="CJ145">
         <v>3</v>
       </c>
+      <c r="CK145">
+        <v>0</v>
+      </c>
+      <c r="CL145">
+        <v>5</v>
+      </c>
     </row>
-    <row r="146" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -25757,8 +26651,14 @@
       <c r="CJ146">
         <v>1</v>
       </c>
+      <c r="CK146">
+        <v>3</v>
+      </c>
+      <c r="CL146">
+        <v>7</v>
+      </c>
     </row>
-    <row r="147" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -25967,8 +26867,14 @@
       <c r="CJ147">
         <v>1</v>
       </c>
+      <c r="CK147">
+        <v>2</v>
+      </c>
+      <c r="CL147">
+        <v>1</v>
+      </c>
     </row>
-    <row r="148" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -26084,8 +26990,11 @@
       <c r="CH148">
         <v>9</v>
       </c>
+      <c r="CK148">
+        <v>9</v>
+      </c>
     </row>
-    <row r="149" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -26294,8 +27203,17 @@
       <c r="CJ149">
         <v>2</v>
       </c>
+      <c r="CK149">
+        <v>1</v>
+      </c>
+      <c r="CL149">
+        <v>2</v>
+      </c>
+      <c r="CM149">
+        <v>2</v>
+      </c>
     </row>
-    <row r="150" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -26498,8 +27416,14 @@
       <c r="CI150">
         <v>1</v>
       </c>
+      <c r="CK150">
+        <v>8</v>
+      </c>
+      <c r="CL150">
+        <v>1</v>
+      </c>
     </row>
-    <row r="151" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -26678,8 +27602,14 @@
       <c r="CJ151">
         <v>2</v>
       </c>
+      <c r="CK151">
+        <v>0</v>
+      </c>
+      <c r="CL151">
+        <v>10</v>
+      </c>
     </row>
-    <row r="152" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -26792,8 +27722,17 @@
       <c r="CJ152">
         <v>3</v>
       </c>
+      <c r="CK152">
+        <v>0</v>
+      </c>
+      <c r="CL152">
+        <v>5</v>
+      </c>
+      <c r="CM152">
+        <v>4</v>
+      </c>
     </row>
-    <row r="153" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -26961,10 +27900,16 @@
         <v>0</v>
       </c>
       <c r="CI153">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="CK153">
+        <v>0</v>
+      </c>
+      <c r="CL153">
+        <v>7</v>
       </c>
     </row>
-    <row r="154" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -27200,8 +28145,14 @@
       <c r="CJ154">
         <v>3</v>
       </c>
+      <c r="CK154">
+        <v>0</v>
+      </c>
+      <c r="CL154">
+        <v>8</v>
+      </c>
     </row>
-    <row r="155" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -27386,8 +28337,14 @@
       <c r="CJ155">
         <v>4</v>
       </c>
+      <c r="CK155">
+        <v>0</v>
+      </c>
+      <c r="CL155">
+        <v>9</v>
+      </c>
     </row>
-    <row r="156" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -27506,8 +28463,14 @@
       <c r="CI156">
         <v>5</v>
       </c>
+      <c r="CK156">
+        <v>1</v>
+      </c>
+      <c r="CL156">
+        <v>5</v>
+      </c>
     </row>
-    <row r="157" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -27629,8 +28592,14 @@
       <c r="CJ157">
         <v>2</v>
       </c>
+      <c r="CK157">
+        <v>0</v>
+      </c>
+      <c r="CL157">
+        <v>6</v>
+      </c>
     </row>
-    <row r="158" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -27779,8 +28748,17 @@
       <c r="CI158">
         <v>2</v>
       </c>
+      <c r="CK158">
+        <v>4</v>
+      </c>
+      <c r="CL158">
+        <v>2</v>
+      </c>
+      <c r="CM158">
+        <v>2</v>
+      </c>
     </row>
-    <row r="159" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -27980,8 +28958,14 @@
       <c r="CJ159">
         <v>1</v>
       </c>
+      <c r="CK159">
+        <v>0</v>
+      </c>
+      <c r="CL159">
+        <v>5</v>
+      </c>
     </row>
-    <row r="160" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -28097,8 +29081,11 @@
       <c r="CH160">
         <v>9</v>
       </c>
+      <c r="CK160">
+        <v>9</v>
+      </c>
     </row>
-    <row r="161" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -28316,8 +29303,14 @@
       <c r="CI161">
         <v>6</v>
       </c>
+      <c r="CK161">
+        <v>1</v>
+      </c>
+      <c r="CL161">
+        <v>6</v>
+      </c>
     </row>
-    <row r="162" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -28433,8 +29426,14 @@
       <c r="CH162">
         <v>8</v>
       </c>
+      <c r="CK162">
+        <v>7</v>
+      </c>
+      <c r="CM162">
+        <v>1</v>
+      </c>
     </row>
-    <row r="163" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -28613,8 +29612,14 @@
       <c r="CI163">
         <v>8</v>
       </c>
+      <c r="CK163">
+        <v>0</v>
+      </c>
+      <c r="CL163">
+        <v>8</v>
+      </c>
     </row>
-    <row r="164" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -28733,8 +29738,17 @@
       <c r="CJ164">
         <v>1</v>
       </c>
+      <c r="CK164">
+        <v>1</v>
+      </c>
+      <c r="CL164">
+        <v>7</v>
+      </c>
+      <c r="CM164">
+        <v>1</v>
+      </c>
     </row>
-    <row r="165" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -28913,8 +29927,14 @@
       <c r="CI165">
         <v>6</v>
       </c>
+      <c r="CK165">
+        <v>0</v>
+      </c>
+      <c r="CL165">
+        <v>6</v>
+      </c>
     </row>
-    <row r="166" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -29078,8 +30098,14 @@
       <c r="CI166">
         <v>6</v>
       </c>
+      <c r="CK166">
+        <v>0</v>
+      </c>
+      <c r="CL166">
+        <v>6</v>
+      </c>
     </row>
-    <row r="167" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -29246,8 +30272,14 @@
       <c r="CI167">
         <v>8</v>
       </c>
+      <c r="CK167">
+        <v>0</v>
+      </c>
+      <c r="CL167">
+        <v>8</v>
+      </c>
     </row>
-    <row r="168" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -29447,8 +30479,14 @@
       <c r="CJ168">
         <v>3</v>
       </c>
+      <c r="CK168">
+        <v>0</v>
+      </c>
+      <c r="CL168">
+        <v>11</v>
+      </c>
     </row>
-    <row r="169" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -29570,8 +30608,14 @@
       <c r="CJ169">
         <v>2</v>
       </c>
+      <c r="CK169">
+        <v>0</v>
+      </c>
+      <c r="CL169">
+        <v>6</v>
+      </c>
     </row>
-    <row r="170" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -29712,16 +30756,16 @@
         <v>1</v>
       </c>
       <c r="CH170">
-        <v>7</v>
-      </c>
-      <c r="CI170">
-        <v>1</v>
-      </c>
-      <c r="CJ170">
+        <v>8</v>
+      </c>
+      <c r="CK170">
+        <v>7</v>
+      </c>
+      <c r="CM170">
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -29930,8 +30974,14 @@
       <c r="CJ171">
         <v>1</v>
       </c>
+      <c r="CK171">
+        <v>2</v>
+      </c>
+      <c r="CL171">
+        <v>8</v>
+      </c>
     </row>
-    <row r="172" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -30056,8 +31106,14 @@
       <c r="CJ172">
         <v>2</v>
       </c>
+      <c r="CK172">
+        <v>7</v>
+      </c>
+      <c r="CM172">
+        <v>1</v>
+      </c>
     </row>
-    <row r="173" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -30200,8 +31256,14 @@
       <c r="CI173">
         <v>2</v>
       </c>
+      <c r="CK173">
+        <v>6</v>
+      </c>
+      <c r="CL173">
+        <v>2</v>
+      </c>
     </row>
-    <row r="174" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -30326,8 +31388,14 @@
       <c r="CJ174">
         <v>1</v>
       </c>
+      <c r="CK174">
+        <v>6</v>
+      </c>
+      <c r="CL174">
+        <v>3</v>
+      </c>
     </row>
-    <row r="175" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -30509,8 +31577,17 @@
       <c r="CJ175">
         <v>1</v>
       </c>
+      <c r="CK175">
+        <v>0</v>
+      </c>
+      <c r="CL175">
+        <v>8</v>
+      </c>
+      <c r="CM175">
+        <v>1</v>
+      </c>
     </row>
-    <row r="176" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -30629,8 +31706,14 @@
       <c r="CI176">
         <v>8</v>
       </c>
+      <c r="CK176">
+        <v>0</v>
+      </c>
+      <c r="CL176">
+        <v>8</v>
+      </c>
     </row>
-    <row r="177" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -30758,8 +31841,14 @@
       <c r="CI177">
         <v>5</v>
       </c>
+      <c r="CK177">
+        <v>0</v>
+      </c>
+      <c r="CL177">
+        <v>5</v>
+      </c>
     </row>
-    <row r="178" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -30893,8 +31982,14 @@
       <c r="CJ178">
         <v>1</v>
       </c>
+      <c r="CK178">
+        <v>0</v>
+      </c>
+      <c r="CL178">
+        <v>8</v>
+      </c>
     </row>
-    <row r="179" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -31079,8 +32174,14 @@
       <c r="CJ179">
         <v>2</v>
       </c>
+      <c r="CK179">
+        <v>0</v>
+      </c>
+      <c r="CL179">
+        <v>10</v>
+      </c>
     </row>
-    <row r="180" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -31262,8 +32363,14 @@
       <c r="CJ180">
         <v>1</v>
       </c>
+      <c r="CK180">
+        <v>0</v>
+      </c>
+      <c r="CL180">
+        <v>9</v>
+      </c>
     </row>
-    <row r="181" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -31445,8 +32552,14 @@
       <c r="CI181">
         <v>9</v>
       </c>
+      <c r="CK181">
+        <v>0</v>
+      </c>
+      <c r="CL181">
+        <v>9</v>
+      </c>
     </row>
-    <row r="182" spans="2:88" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -31571,8 +32684,14 @@
       <c r="CJ182">
         <v>2</v>
       </c>
+      <c r="CK182">
+        <v>2</v>
+      </c>
+      <c r="CL182">
+        <v>4</v>
+      </c>
     </row>
-    <row r="183" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -31786,8 +32905,14 @@
       <c r="CI183">
         <v>2</v>
       </c>
+      <c r="CK183">
+        <v>3</v>
+      </c>
+      <c r="CL183">
+        <v>2</v>
+      </c>
     </row>
-    <row r="184" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -31920,8 +33045,14 @@
       <c r="CJ184">
         <v>3</v>
       </c>
+      <c r="CK184">
+        <v>0</v>
+      </c>
+      <c r="CL184">
+        <v>6</v>
+      </c>
     </row>
-    <row r="185" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -32105,8 +33236,14 @@
       <c r="CI185">
         <v>7</v>
       </c>
+      <c r="CK185">
+        <v>0</v>
+      </c>
+      <c r="CL185">
+        <v>7</v>
+      </c>
     </row>
-    <row r="186" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -32278,8 +33415,14 @@
       <c r="CI186">
         <v>1</v>
       </c>
+      <c r="CK186">
+        <v>6</v>
+      </c>
+      <c r="CL186">
+        <v>1</v>
+      </c>
     </row>
-    <row r="187" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -32418,8 +33561,14 @@
       <c r="CJ187">
         <v>1</v>
       </c>
+      <c r="CK187">
+        <v>6</v>
+      </c>
+      <c r="CM187">
+        <v>1</v>
+      </c>
     </row>
-    <row r="188" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B188" t="s">
         <v>4</v>
       </c>
@@ -32606,8 +33755,14 @@
       <c r="CI188">
         <v>4</v>
       </c>
+      <c r="CK188">
+        <v>6</v>
+      </c>
+      <c r="CL188">
+        <v>4</v>
+      </c>
     </row>
-    <row r="189" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -32797,8 +33952,14 @@
       <c r="CJ189">
         <v>2</v>
       </c>
+      <c r="CK189">
+        <v>0</v>
+      </c>
+      <c r="CL189">
+        <v>2</v>
+      </c>
     </row>
-    <row r="190" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="190" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -32991,8 +34152,14 @@
       <c r="CI190">
         <v>5</v>
       </c>
+      <c r="CK190">
+        <v>0</v>
+      </c>
+      <c r="CL190">
+        <v>5</v>
+      </c>
     </row>
-    <row r="191" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="191" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -33188,8 +34355,14 @@
       <c r="CI191">
         <v>5</v>
       </c>
+      <c r="CK191">
+        <v>0</v>
+      </c>
+      <c r="CL191">
+        <v>5</v>
+      </c>
     </row>
-    <row r="192" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="192" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -33364,8 +34537,14 @@
       <c r="CI192">
         <v>3</v>
       </c>
+      <c r="CK192">
+        <v>0</v>
+      </c>
+      <c r="CL192">
+        <v>3</v>
+      </c>
     </row>
-    <row r="193" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="193" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -33561,8 +34740,17 @@
       <c r="CI193">
         <v>4</v>
       </c>
+      <c r="CK193">
+        <v>1</v>
+      </c>
+      <c r="CL193">
+        <v>4</v>
+      </c>
+      <c r="CM193">
+        <v>2</v>
+      </c>
     </row>
-    <row r="194" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="194" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B194" t="s">
         <v>4</v>
       </c>
@@ -33734,8 +34922,14 @@
       <c r="CI194">
         <v>1</v>
       </c>
+      <c r="CK194">
+        <v>6</v>
+      </c>
+      <c r="CL194">
+        <v>1</v>
+      </c>
     </row>
-    <row r="195" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="195" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -33922,8 +35116,17 @@
       <c r="CI195">
         <v>1</v>
       </c>
+      <c r="CK195">
+        <v>0</v>
+      </c>
+      <c r="CL195">
+        <v>1</v>
+      </c>
+      <c r="CM195">
+        <v>1</v>
+      </c>
     </row>
-    <row r="196" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="196" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -34146,8 +35349,14 @@
       <c r="CI196">
         <v>9</v>
       </c>
+      <c r="CK196">
+        <v>0</v>
+      </c>
+      <c r="CL196">
+        <v>9</v>
+      </c>
     </row>
-    <row r="197" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="197" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -34325,8 +35534,14 @@
       <c r="CI197">
         <v>4</v>
       </c>
+      <c r="CK197">
+        <v>0</v>
+      </c>
+      <c r="CL197">
+        <v>4</v>
+      </c>
     </row>
-    <row r="198" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="198" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -34486,8 +35701,14 @@
       <c r="CJ198">
         <v>1</v>
       </c>
+      <c r="CK198">
+        <v>0</v>
+      </c>
+      <c r="CL198">
+        <v>5</v>
+      </c>
     </row>
-    <row r="199" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="199" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -34659,8 +35880,14 @@
       <c r="CJ199">
         <v>1</v>
       </c>
+      <c r="CK199">
+        <v>5</v>
+      </c>
+      <c r="CL199">
+        <v>1</v>
+      </c>
     </row>
-    <row r="200" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="200" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
         <v>4</v>
       </c>
@@ -34826,8 +36053,14 @@
       <c r="CJ200">
         <v>1</v>
       </c>
+      <c r="CK200">
+        <v>1</v>
+      </c>
+      <c r="CL200">
+        <v>6</v>
+      </c>
     </row>
-    <row r="201" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="201" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -35032,8 +36265,14 @@
       <c r="CI201">
         <v>5</v>
       </c>
+      <c r="CK201">
+        <v>1</v>
+      </c>
+      <c r="CL201">
+        <v>5</v>
+      </c>
     </row>
-    <row r="202" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="202" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -35229,8 +36468,14 @@
       <c r="CI202">
         <v>1</v>
       </c>
+      <c r="CK202">
+        <v>0</v>
+      </c>
+      <c r="CL202">
+        <v>1</v>
+      </c>
     </row>
-    <row r="203" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="203" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -35420,8 +36665,14 @@
       <c r="CI203">
         <v>3</v>
       </c>
+      <c r="CK203">
+        <v>0</v>
+      </c>
+      <c r="CL203">
+        <v>3</v>
+      </c>
     </row>
-    <row r="204" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="204" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -35533,8 +36784,11 @@
       <c r="CH204">
         <v>6</v>
       </c>
+      <c r="CK204">
+        <v>6</v>
+      </c>
     </row>
-    <row r="205" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="205" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -35739,8 +36993,17 @@
       <c r="CJ205">
         <v>1</v>
       </c>
+      <c r="CK205">
+        <v>7</v>
+      </c>
+      <c r="CL205">
+        <v>1</v>
+      </c>
+      <c r="CM205">
+        <v>2</v>
+      </c>
     </row>
-    <row r="206" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="206" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B206" t="s">
         <v>4</v>
       </c>
@@ -35855,8 +37118,11 @@
       <c r="CI206">
         <v>6</v>
       </c>
+      <c r="CK206">
+        <v>6</v>
+      </c>
     </row>
-    <row r="207" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="207" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -36016,8 +37282,17 @@
       <c r="CJ207">
         <v>1</v>
       </c>
+      <c r="CK207">
+        <v>0</v>
+      </c>
+      <c r="CL207">
+        <v>3</v>
+      </c>
+      <c r="CM207">
+        <v>1</v>
+      </c>
     </row>
-    <row r="208" spans="2:88" x14ac:dyDescent="0.3">
+    <row r="208" spans="2:91" x14ac:dyDescent="0.3">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -36207,8 +37482,14 @@
       <c r="CI208">
         <v>3</v>
       </c>
+      <c r="CK208">
+        <v>0</v>
+      </c>
+      <c r="CL208">
+        <v>3</v>
+      </c>
     </row>
-    <row r="209" spans="2:87" x14ac:dyDescent="0.3">
+    <row r="209" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B209" t="s">
         <v>3</v>
       </c>
@@ -36383,8 +37664,14 @@
       <c r="CI209">
         <v>5</v>
       </c>
+      <c r="CK209">
+        <v>0</v>
+      </c>
+      <c r="CL209">
+        <v>5</v>
+      </c>
     </row>
-    <row r="210" spans="2:87" x14ac:dyDescent="0.3">
+    <row r="210" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B210" t="s">
         <v>1</v>
       </c>
@@ -36580,8 +37867,14 @@
       <c r="CI210">
         <v>1</v>
       </c>
+      <c r="CK210">
+        <v>4</v>
+      </c>
+      <c r="CL210">
+        <v>1</v>
+      </c>
     </row>
-    <row r="211" spans="2:87" x14ac:dyDescent="0.3">
+    <row r="211" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
         <v>4</v>
       </c>
@@ -36753,8 +38046,14 @@
       <c r="CI211">
         <v>2</v>
       </c>
+      <c r="CK211">
+        <v>3</v>
+      </c>
+      <c r="CL211">
+        <v>2</v>
+      </c>
     </row>
-    <row r="212" spans="2:87" x14ac:dyDescent="0.3">
+    <row r="212" spans="2:90" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
         <v>4</v>
       </c>
@@ -36920,8 +38219,13 @@
       <c r="CI212">
         <v>1</v>
       </c>
+      <c r="CK212">
+        <v>5</v>
+      </c>
+      <c r="CL212">
+        <v>1</v>
+      </c>
     </row>
-    <row r="213" spans="2:87" hidden="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
DOY 168 germinants data collection
</commit_message>
<xml_diff>
--- a/data/germination_data.xlsx
+++ b/data/germination_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temporal Ecology Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D7BFCE4-6EB9-4777-BFCA-89E73DC8D008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8CA7CFB-12E8-48CB-8A42-34B61559B563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="131">
   <si>
     <t>seed_species</t>
   </si>
@@ -456,6 +456,15 @@
   <si>
     <t>154_halfdead</t>
   </si>
+  <si>
+    <t>168_alive</t>
+  </si>
+  <si>
+    <t>168_dead</t>
+  </si>
+  <si>
+    <t>168_halfdead</t>
+  </si>
 </sst>
 </file>
 
@@ -559,9 +568,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CM213" totalsRowShown="0">
-  <autoFilter ref="B2:CM213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
-  <tableColumns count="90">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CP213" totalsRowShown="0">
+  <autoFilter ref="B2:CP213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
+  <tableColumns count="93">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
     <tableColumn id="3" xr3:uid="{B695F4B4-8561-9D48-9FF3-12A40CB2B7C7}" name="inoculated_%"/>
@@ -652,6 +661,9 @@
     <tableColumn id="88" xr3:uid="{5C77EBFE-EDC9-455C-A405-C2A7DA5D973E}" name="154_alive"/>
     <tableColumn id="89" xr3:uid="{1762B7C6-1B6C-4691-AC50-45E17B49E79D}" name="154_dead"/>
     <tableColumn id="90" xr3:uid="{E94F12E3-B02B-47BA-8281-4BD0C9F47EA5}" name="154_halfdead"/>
+    <tableColumn id="91" xr3:uid="{19796ADF-ED67-4616-A2F4-F5F6343D05C5}" name="168_alive"/>
+    <tableColumn id="92" xr3:uid="{7489BFD5-C58F-456E-A7EF-D0F7BF350167}" name="168_dead"/>
+    <tableColumn id="93" xr3:uid="{3DEB280A-450E-4E2A-8CF9-DAB35C6C1464}" name="168_halfdead"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -974,7 +986,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:CM212"/>
+  <dimension ref="B2:CP212"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -982,7 +994,7 @@
     <col min="4" max="4" width="17.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -1253,8 +1265,17 @@
       <c r="CM2" t="s">
         <v>127</v>
       </c>
+      <c r="CN2" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO2" t="s">
+        <v>129</v>
+      </c>
+      <c r="CP2" t="s">
+        <v>130</v>
+      </c>
     </row>
-    <row r="3" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1462,8 +1483,14 @@
       <c r="CL3">
         <v>3</v>
       </c>
+      <c r="CN3">
+        <v>1</v>
+      </c>
+      <c r="CO3">
+        <v>3</v>
+      </c>
     </row>
-    <row r="4" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1584,8 +1611,11 @@
       <c r="CK4">
         <v>9</v>
       </c>
+      <c r="CN4">
+        <v>9</v>
+      </c>
     </row>
-    <row r="5" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1793,8 +1823,14 @@
       <c r="CL5">
         <v>7</v>
       </c>
+      <c r="CN5">
+        <v>0</v>
+      </c>
+      <c r="CO5">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1912,8 +1948,14 @@
       <c r="CK6">
         <v>9</v>
       </c>
+      <c r="CN6">
+        <v>5</v>
+      </c>
+      <c r="CP6">
+        <v>4</v>
+      </c>
     </row>
-    <row r="7" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -2085,8 +2127,17 @@
       <c r="CL7">
         <v>5</v>
       </c>
+      <c r="CN7">
+        <v>0</v>
+      </c>
+      <c r="CO7">
+        <v>5</v>
+      </c>
+      <c r="CP7">
+        <v>1</v>
+      </c>
     </row>
-    <row r="8" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -2285,8 +2336,14 @@
       <c r="CL8">
         <v>1</v>
       </c>
+      <c r="CN8">
+        <v>6</v>
+      </c>
+      <c r="CO8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2491,8 +2548,17 @@
       <c r="CL9">
         <v>1</v>
       </c>
+      <c r="CN9">
+        <v>0</v>
+      </c>
+      <c r="CO9">
+        <v>6</v>
+      </c>
+      <c r="CP9">
+        <v>1</v>
+      </c>
     </row>
-    <row r="10" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -2631,8 +2697,14 @@
       <c r="CL10">
         <v>2</v>
       </c>
+      <c r="CN10">
+        <v>6</v>
+      </c>
+      <c r="CO10">
+        <v>2</v>
+      </c>
     </row>
-    <row r="11" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -2837,8 +2909,14 @@
       <c r="CL11">
         <v>8</v>
       </c>
+      <c r="CN11">
+        <v>0</v>
+      </c>
+      <c r="CO11">
+        <v>8</v>
+      </c>
     </row>
-    <row r="12" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -3046,8 +3124,14 @@
       <c r="CL12">
         <v>5</v>
       </c>
+      <c r="CN12">
+        <v>5</v>
+      </c>
+      <c r="CO12">
+        <v>5</v>
+      </c>
     </row>
-    <row r="13" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -3246,8 +3330,14 @@
       <c r="CL13">
         <v>7</v>
       </c>
+      <c r="CN13">
+        <v>0</v>
+      </c>
+      <c r="CO13">
+        <v>7</v>
+      </c>
     </row>
-    <row r="14" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -3404,8 +3494,14 @@
       <c r="CL14">
         <v>1</v>
       </c>
+      <c r="CN14">
+        <v>8</v>
+      </c>
+      <c r="CO14">
+        <v>1</v>
+      </c>
     </row>
-    <row r="15" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -3593,8 +3689,14 @@
       <c r="CL15">
         <v>8</v>
       </c>
+      <c r="CN15">
+        <v>0</v>
+      </c>
+      <c r="CO15">
+        <v>8</v>
+      </c>
     </row>
-    <row r="16" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -3764,8 +3866,17 @@
       <c r="CL16">
         <v>1</v>
       </c>
+      <c r="CN16">
+        <v>6</v>
+      </c>
+      <c r="CO16">
+        <v>2</v>
+      </c>
+      <c r="CP16">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -3956,8 +4067,14 @@
       <c r="CL17">
         <v>8</v>
       </c>
+      <c r="CN17">
+        <v>0</v>
+      </c>
+      <c r="CO17">
+        <v>8</v>
+      </c>
     </row>
-    <row r="18" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -4073,8 +4190,17 @@
       <c r="CK18">
         <v>10</v>
       </c>
+      <c r="CN18">
+        <v>2</v>
+      </c>
+      <c r="CO18">
+        <v>4</v>
+      </c>
+      <c r="CP18">
+        <v>4</v>
+      </c>
     </row>
-    <row r="19" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -4283,8 +4409,14 @@
       <c r="CL19">
         <v>7</v>
       </c>
+      <c r="CN19">
+        <v>0</v>
+      </c>
+      <c r="CO19">
+        <v>7</v>
+      </c>
     </row>
-    <row r="20" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -4454,8 +4586,14 @@
       <c r="CL20">
         <v>1</v>
       </c>
+      <c r="CN20">
+        <v>13</v>
+      </c>
+      <c r="CO20">
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -4630,8 +4768,14 @@
       <c r="CL21">
         <v>6</v>
       </c>
+      <c r="CN21">
+        <v>0</v>
+      </c>
+      <c r="CO21">
+        <v>6</v>
+      </c>
     </row>
-    <row r="22" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -4759,8 +4903,14 @@
       <c r="CM22">
         <v>1</v>
       </c>
+      <c r="CN22">
+        <v>6</v>
+      </c>
+      <c r="CO22">
+        <v>2</v>
+      </c>
     </row>
-    <row r="23" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -4963,8 +5113,14 @@
       <c r="CL23">
         <v>10</v>
       </c>
+      <c r="CN23">
+        <v>0</v>
+      </c>
+      <c r="CO23">
+        <v>10</v>
+      </c>
     </row>
-    <row r="24" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -5140,8 +5296,14 @@
       <c r="CL24">
         <v>4</v>
       </c>
+      <c r="CN24">
+        <v>8</v>
+      </c>
+      <c r="CO24">
+        <v>4</v>
+      </c>
     </row>
-    <row r="25" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -5266,8 +5428,14 @@
       <c r="CL25">
         <v>8</v>
       </c>
+      <c r="CN25">
+        <v>0</v>
+      </c>
+      <c r="CO25">
+        <v>8</v>
+      </c>
     </row>
-    <row r="26" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -5518,8 +5686,17 @@
       <c r="CM26">
         <v>1</v>
       </c>
+      <c r="CN26">
+        <v>1</v>
+      </c>
+      <c r="CO26">
+        <v>9</v>
+      </c>
+      <c r="CP26">
+        <v>1</v>
+      </c>
     </row>
-    <row r="27" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -5701,8 +5878,14 @@
       <c r="CL27">
         <v>4</v>
       </c>
+      <c r="CN27">
+        <v>2</v>
+      </c>
+      <c r="CO27">
+        <v>4</v>
+      </c>
     </row>
-    <row r="28" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -5923,8 +6106,14 @@
       <c r="CL28">
         <v>4</v>
       </c>
+      <c r="CN28">
+        <v>0</v>
+      </c>
+      <c r="CO28">
+        <v>10</v>
+      </c>
     </row>
-    <row r="29" spans="2:91" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:94" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>3</v>
       </c>
@@ -6115,8 +6304,14 @@
       <c r="CL29" s="3">
         <v>4</v>
       </c>
+      <c r="CN29" s="3">
+        <v>0</v>
+      </c>
+      <c r="CO29" s="3">
+        <v>4</v>
+      </c>
     </row>
-    <row r="30" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -6238,8 +6433,17 @@
       <c r="CK30">
         <v>8</v>
       </c>
+      <c r="CN30">
+        <v>1</v>
+      </c>
+      <c r="CO30">
+        <v>4</v>
+      </c>
+      <c r="CP30">
+        <v>3</v>
+      </c>
     </row>
-    <row r="31" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -6448,8 +6652,14 @@
       <c r="CL31">
         <v>5</v>
       </c>
+      <c r="CN31">
+        <v>0</v>
+      </c>
+      <c r="CO31">
+        <v>5</v>
+      </c>
     </row>
-    <row r="32" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -6616,8 +6826,17 @@
       <c r="CL32">
         <v>1</v>
       </c>
+      <c r="CN32">
+        <v>5</v>
+      </c>
+      <c r="CO32">
+        <v>1</v>
+      </c>
+      <c r="CP32">
+        <v>4</v>
+      </c>
     </row>
-    <row r="33" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -6781,8 +7000,14 @@
       <c r="CL33">
         <v>9</v>
       </c>
+      <c r="CN33">
+        <v>0</v>
+      </c>
+      <c r="CO33">
+        <v>9</v>
+      </c>
     </row>
-    <row r="34" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -6937,8 +7162,14 @@
       <c r="CL34">
         <v>5</v>
       </c>
+      <c r="CN34">
+        <v>1</v>
+      </c>
+      <c r="CO34">
+        <v>5</v>
+      </c>
     </row>
-    <row r="35" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -7126,8 +7357,14 @@
       <c r="CL35">
         <v>8</v>
       </c>
+      <c r="CN35">
+        <v>0</v>
+      </c>
+      <c r="CO35">
+        <v>8</v>
+      </c>
     </row>
-    <row r="36" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -7309,8 +7546,17 @@
       <c r="CL36">
         <v>2</v>
       </c>
+      <c r="CN36">
+        <v>4</v>
+      </c>
+      <c r="CO36">
+        <v>2</v>
+      </c>
+      <c r="CP36">
+        <v>4</v>
+      </c>
     </row>
-    <row r="37" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -7441,8 +7687,14 @@
       <c r="CL37">
         <v>5</v>
       </c>
+      <c r="CN37">
+        <v>0</v>
+      </c>
+      <c r="CO37">
+        <v>6</v>
+      </c>
     </row>
-    <row r="38" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -7666,8 +7918,14 @@
       <c r="CL38">
         <v>4</v>
       </c>
+      <c r="CN38">
+        <v>2</v>
+      </c>
+      <c r="CO38">
+        <v>4</v>
+      </c>
     </row>
-    <row r="39" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -7870,8 +8128,17 @@
       <c r="CL39">
         <v>4</v>
       </c>
+      <c r="CN39">
+        <v>1</v>
+      </c>
+      <c r="CO39">
+        <v>4</v>
+      </c>
+      <c r="CP39">
+        <v>1</v>
+      </c>
     </row>
-    <row r="40" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -8092,8 +8359,17 @@
       <c r="CL40">
         <v>8</v>
       </c>
+      <c r="CN40">
+        <v>1</v>
+      </c>
+      <c r="CO40">
+        <v>8</v>
+      </c>
+      <c r="CP40">
+        <v>1</v>
+      </c>
     </row>
-    <row r="41" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -8278,8 +8554,14 @@
       <c r="CL41">
         <v>6</v>
       </c>
+      <c r="CN41">
+        <v>0</v>
+      </c>
+      <c r="CO41">
+        <v>6</v>
+      </c>
     </row>
-    <row r="42" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -8410,8 +8692,17 @@
       <c r="CK42">
         <v>7</v>
       </c>
+      <c r="CN42">
+        <v>0</v>
+      </c>
+      <c r="CO42">
+        <v>5</v>
+      </c>
+      <c r="CP42">
+        <v>2</v>
+      </c>
     </row>
-    <row r="43" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -8623,8 +8914,14 @@
       <c r="CL43">
         <v>9</v>
       </c>
+      <c r="CN43">
+        <v>0</v>
+      </c>
+      <c r="CO43">
+        <v>9</v>
+      </c>
     </row>
-    <row r="44" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -8743,8 +9040,17 @@
       <c r="CM44">
         <v>4</v>
       </c>
+      <c r="CN44">
+        <v>0</v>
+      </c>
+      <c r="CO44">
+        <v>5</v>
+      </c>
+      <c r="CP44">
+        <v>1</v>
+      </c>
     </row>
-    <row r="45" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -8998,8 +9304,14 @@
       <c r="CL45">
         <v>9</v>
       </c>
+      <c r="CN45">
+        <v>0</v>
+      </c>
+      <c r="CO45">
+        <v>9</v>
+      </c>
     </row>
-    <row r="46" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -9127,8 +9439,14 @@
       <c r="CL46">
         <v>5</v>
       </c>
+      <c r="CN46">
+        <v>1</v>
+      </c>
+      <c r="CO46">
+        <v>5</v>
+      </c>
     </row>
-    <row r="47" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -9286,8 +9604,14 @@
       <c r="CL47">
         <v>9</v>
       </c>
+      <c r="CN47">
+        <v>0</v>
+      </c>
+      <c r="CO47">
+        <v>9</v>
+      </c>
     </row>
-    <row r="48" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -9514,8 +9838,14 @@
       <c r="CL48">
         <v>10</v>
       </c>
+      <c r="CN48">
+        <v>1</v>
+      </c>
+      <c r="CO48">
+        <v>10</v>
+      </c>
     </row>
-    <row r="49" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -9649,8 +9979,17 @@
       <c r="CL49">
         <v>6</v>
       </c>
+      <c r="CN49">
+        <v>0</v>
+      </c>
+      <c r="CO49">
+        <v>6</v>
+      </c>
+      <c r="CP49">
+        <v>1</v>
+      </c>
     </row>
-    <row r="50" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -9880,8 +10219,17 @@
       <c r="CM50">
         <v>1</v>
       </c>
+      <c r="CN50">
+        <v>4</v>
+      </c>
+      <c r="CO50">
+        <v>3</v>
+      </c>
+      <c r="CP50">
+        <v>1</v>
+      </c>
     </row>
-    <row r="51" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -10099,8 +10447,14 @@
       <c r="CL51">
         <v>5</v>
       </c>
+      <c r="CN51">
+        <v>1</v>
+      </c>
+      <c r="CO51">
+        <v>5</v>
+      </c>
     </row>
-    <row r="52" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -10219,8 +10573,14 @@
       <c r="CM52">
         <v>1</v>
       </c>
+      <c r="CN52">
+        <v>5</v>
+      </c>
+      <c r="CP52">
+        <v>1</v>
+      </c>
     </row>
-    <row r="53" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -10411,8 +10771,14 @@
       <c r="CL53">
         <v>4</v>
       </c>
+      <c r="CN53">
+        <v>0</v>
+      </c>
+      <c r="CO53">
+        <v>4</v>
+      </c>
     </row>
-    <row r="54" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -10534,8 +10900,14 @@
       <c r="CK54">
         <v>6</v>
       </c>
+      <c r="CN54">
+        <v>5</v>
+      </c>
+      <c r="CP54">
+        <v>1</v>
+      </c>
     </row>
-    <row r="55" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -10729,8 +11101,14 @@
       <c r="CM55">
         <v>2</v>
       </c>
+      <c r="CN55">
+        <v>0</v>
+      </c>
+      <c r="CO55">
+        <v>6</v>
+      </c>
     </row>
-    <row r="56" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -10852,8 +11230,11 @@
       <c r="CK56">
         <v>10</v>
       </c>
+      <c r="CN56">
+        <v>10</v>
+      </c>
     </row>
-    <row r="57" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -10993,8 +11374,17 @@
       <c r="CL57">
         <v>1</v>
       </c>
+      <c r="CN57">
+        <v>3</v>
+      </c>
+      <c r="CO57">
+        <v>3</v>
+      </c>
+      <c r="CP57">
+        <v>1</v>
+      </c>
     </row>
-    <row r="58" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -11125,8 +11515,14 @@
       <c r="CL58">
         <v>4</v>
       </c>
+      <c r="CN58">
+        <v>2</v>
+      </c>
+      <c r="CO58">
+        <v>4</v>
+      </c>
     </row>
-    <row r="59" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -11254,8 +11650,14 @@
       <c r="CL59">
         <v>7</v>
       </c>
+      <c r="CN59">
+        <v>0</v>
+      </c>
+      <c r="CO59">
+        <v>7</v>
+      </c>
     </row>
-    <row r="60" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -11440,8 +11842,14 @@
       <c r="CL60">
         <v>2</v>
       </c>
+      <c r="CN60">
+        <v>7</v>
+      </c>
+      <c r="CO60">
+        <v>2</v>
+      </c>
     </row>
-    <row r="61" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -11578,8 +11986,14 @@
       <c r="CL61">
         <v>4</v>
       </c>
+      <c r="CN61">
+        <v>0</v>
+      </c>
+      <c r="CO61">
+        <v>7</v>
+      </c>
     </row>
-    <row r="62" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -11794,8 +12208,17 @@
       <c r="CL62">
         <v>2</v>
       </c>
+      <c r="CN62">
+        <v>2</v>
+      </c>
+      <c r="CO62">
+        <v>2</v>
+      </c>
+      <c r="CP62">
+        <v>1</v>
+      </c>
     </row>
-    <row r="63" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -12010,8 +12433,14 @@
       <c r="CL63">
         <v>9</v>
       </c>
+      <c r="CN63">
+        <v>0</v>
+      </c>
+      <c r="CO63">
+        <v>9</v>
+      </c>
     </row>
-    <row r="64" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -12199,8 +12628,17 @@
       <c r="CM64">
         <v>1</v>
       </c>
+      <c r="CN64">
+        <v>4</v>
+      </c>
+      <c r="CO64">
+        <v>4</v>
+      </c>
+      <c r="CP64">
+        <v>2</v>
+      </c>
     </row>
-    <row r="65" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -12388,8 +12826,14 @@
       <c r="CL65">
         <v>6</v>
       </c>
+      <c r="CN65">
+        <v>0</v>
+      </c>
+      <c r="CO65">
+        <v>6</v>
+      </c>
     </row>
-    <row r="66" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -12517,8 +12961,14 @@
       <c r="CK66">
         <v>5</v>
       </c>
+      <c r="CN66">
+        <v>4</v>
+      </c>
+      <c r="CP66">
+        <v>1</v>
+      </c>
     </row>
-    <row r="67" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -12736,8 +13186,14 @@
       <c r="CM67">
         <v>1</v>
       </c>
+      <c r="CN67">
+        <v>0</v>
+      </c>
+      <c r="CO67">
+        <v>10</v>
+      </c>
     </row>
-    <row r="68" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -12850,8 +13306,14 @@
       <c r="CK68">
         <v>11</v>
       </c>
+      <c r="CN68">
+        <v>8</v>
+      </c>
+      <c r="CP68">
+        <v>3</v>
+      </c>
     </row>
-    <row r="69" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -12979,8 +13441,14 @@
       <c r="CM69">
         <v>1</v>
       </c>
+      <c r="CN69">
+        <v>0</v>
+      </c>
+      <c r="CO69">
+        <v>9</v>
+      </c>
     </row>
-    <row r="70" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -13111,8 +13579,14 @@
       <c r="CM70">
         <v>2</v>
       </c>
+      <c r="CN70">
+        <v>2</v>
+      </c>
+      <c r="CO70">
+        <v>6</v>
+      </c>
     </row>
-    <row r="71" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -13321,8 +13795,14 @@
       <c r="CL71">
         <v>10</v>
       </c>
+      <c r="CN71">
+        <v>0</v>
+      </c>
+      <c r="CO71">
+        <v>10</v>
+      </c>
     </row>
-    <row r="72" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -13516,8 +13996,17 @@
       <c r="CL72">
         <v>1</v>
       </c>
+      <c r="CN72">
+        <v>1</v>
+      </c>
+      <c r="CO72">
+        <v>2</v>
+      </c>
+      <c r="CP72">
+        <v>4</v>
+      </c>
     </row>
-    <row r="73" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -13642,8 +14131,14 @@
       <c r="CL73">
         <v>8</v>
       </c>
+      <c r="CN73">
+        <v>1</v>
+      </c>
+      <c r="CO73">
+        <v>9</v>
+      </c>
     </row>
-    <row r="74" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -13768,8 +14263,14 @@
       <c r="CK74">
         <v>9</v>
       </c>
+      <c r="CN74">
+        <v>7</v>
+      </c>
+      <c r="CP74">
+        <v>2</v>
+      </c>
     </row>
-    <row r="75" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -13963,8 +14464,14 @@
       <c r="CL75">
         <v>8</v>
       </c>
+      <c r="CN75">
+        <v>1</v>
+      </c>
+      <c r="CO75">
+        <v>8</v>
+      </c>
     </row>
-    <row r="76" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -14179,8 +14686,17 @@
       <c r="CM76">
         <v>1</v>
       </c>
+      <c r="CN76">
+        <v>2</v>
+      </c>
+      <c r="CO76">
+        <v>4</v>
+      </c>
+      <c r="CP76">
+        <v>2</v>
+      </c>
     </row>
-    <row r="77" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -14359,8 +14875,14 @@
       <c r="CL77">
         <v>7</v>
       </c>
+      <c r="CN77">
+        <v>0</v>
+      </c>
+      <c r="CO77">
+        <v>7</v>
+      </c>
     </row>
-    <row r="78" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -14485,8 +15007,17 @@
       <c r="CK78">
         <v>7</v>
       </c>
+      <c r="CN78">
+        <v>4</v>
+      </c>
+      <c r="CO78">
+        <v>1</v>
+      </c>
+      <c r="CP78">
+        <v>2</v>
+      </c>
     </row>
-    <row r="79" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -14698,8 +15229,17 @@
       <c r="CM79">
         <v>1</v>
       </c>
+      <c r="CN79">
+        <v>0</v>
+      </c>
+      <c r="CO79">
+        <v>8</v>
+      </c>
+      <c r="CP79">
+        <v>1</v>
+      </c>
     </row>
-    <row r="80" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -14878,8 +15418,17 @@
       <c r="CL80">
         <v>1</v>
       </c>
+      <c r="CN80">
+        <v>5</v>
+      </c>
+      <c r="CO80">
+        <v>1</v>
+      </c>
+      <c r="CP80">
+        <v>4</v>
+      </c>
     </row>
-    <row r="81" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -15070,8 +15619,14 @@
       <c r="CL81">
         <v>7</v>
       </c>
+      <c r="CN81">
+        <v>0</v>
+      </c>
+      <c r="CO81">
+        <v>7</v>
+      </c>
     </row>
-    <row r="82" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -15301,8 +15856,14 @@
       <c r="CL82">
         <v>10</v>
       </c>
+      <c r="CN82">
+        <v>0</v>
+      </c>
+      <c r="CO82">
+        <v>10</v>
+      </c>
     </row>
-    <row r="83" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -15514,8 +16075,14 @@
       <c r="CL83">
         <v>9</v>
       </c>
+      <c r="CN83">
+        <v>0</v>
+      </c>
+      <c r="CO83">
+        <v>9</v>
+      </c>
     </row>
-    <row r="84" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -15721,8 +16288,17 @@
       <c r="CL84">
         <v>2</v>
       </c>
+      <c r="CN84">
+        <v>2</v>
+      </c>
+      <c r="CO84">
+        <v>5</v>
+      </c>
+      <c r="CP84">
+        <v>2</v>
+      </c>
     </row>
-    <row r="85" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -15934,8 +16510,14 @@
       <c r="CL85">
         <v>6</v>
       </c>
+      <c r="CN85">
+        <v>0</v>
+      </c>
+      <c r="CO85">
+        <v>6</v>
+      </c>
     </row>
-    <row r="86" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -16126,8 +16708,17 @@
       <c r="CM86">
         <v>1</v>
       </c>
+      <c r="CN86">
+        <v>1</v>
+      </c>
+      <c r="CO86">
+        <v>7</v>
+      </c>
+      <c r="CP86">
+        <v>1</v>
+      </c>
     </row>
-    <row r="87" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -16342,8 +16933,17 @@
       <c r="CM87">
         <v>1</v>
       </c>
+      <c r="CN87">
+        <v>0</v>
+      </c>
+      <c r="CO87">
+        <v>6</v>
+      </c>
+      <c r="CP87">
+        <v>1</v>
+      </c>
     </row>
-    <row r="88" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -16540,8 +17140,17 @@
       <c r="CL88">
         <v>3</v>
       </c>
+      <c r="CN88">
+        <v>2</v>
+      </c>
+      <c r="CO88">
+        <v>6</v>
+      </c>
+      <c r="CP88">
+        <v>1</v>
+      </c>
     </row>
-    <row r="89" spans="2:91" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:94" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>3</v>
       </c>
@@ -16717,8 +17326,14 @@
       <c r="CL89" s="3">
         <v>5</v>
       </c>
+      <c r="CN89" s="3">
+        <v>0</v>
+      </c>
+      <c r="CO89" s="3">
+        <v>5</v>
+      </c>
     </row>
-    <row r="90" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -16843,8 +17458,17 @@
       <c r="CM90">
         <v>1</v>
       </c>
+      <c r="CN90">
+        <v>3</v>
+      </c>
+      <c r="CO90">
+        <v>1</v>
+      </c>
+      <c r="CP90">
+        <v>3</v>
+      </c>
     </row>
-    <row r="91" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -17065,8 +17689,17 @@
       <c r="CL91">
         <v>5</v>
       </c>
+      <c r="CN91">
+        <v>0</v>
+      </c>
+      <c r="CO91">
+        <v>5</v>
+      </c>
+      <c r="CP91">
+        <v>1</v>
+      </c>
     </row>
-    <row r="92" spans="2:91" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:94" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>1</v>
       </c>
@@ -17266,8 +17899,17 @@
       <c r="CL92" s="3">
         <v>3</v>
       </c>
+      <c r="CN92" s="3">
+        <v>1</v>
+      </c>
+      <c r="CO92" s="3">
+        <v>5</v>
+      </c>
+      <c r="CP92" s="3">
+        <v>2</v>
+      </c>
     </row>
-    <row r="93" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -17428,8 +18070,14 @@
       <c r="CL93">
         <v>9</v>
       </c>
+      <c r="CN93">
+        <v>0</v>
+      </c>
+      <c r="CO93">
+        <v>9</v>
+      </c>
     </row>
-    <row r="94" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -17560,8 +18208,14 @@
       <c r="CL94">
         <v>7</v>
       </c>
+      <c r="CN94">
+        <v>0</v>
+      </c>
+      <c r="CO94">
+        <v>7</v>
+      </c>
     </row>
-    <row r="95" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -17731,8 +18385,14 @@
       <c r="CL95">
         <v>8</v>
       </c>
+      <c r="CN95">
+        <v>0</v>
+      </c>
+      <c r="CO95">
+        <v>8</v>
+      </c>
     </row>
-    <row r="96" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -17926,8 +18586,14 @@
       <c r="CM96">
         <v>1</v>
       </c>
+      <c r="CN96">
+        <v>5</v>
+      </c>
+      <c r="CO96">
+        <v>5</v>
+      </c>
     </row>
-    <row r="97" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -18061,8 +18727,14 @@
       <c r="CL97">
         <v>7</v>
       </c>
+      <c r="CN97">
+        <v>0</v>
+      </c>
+      <c r="CO97">
+        <v>8</v>
+      </c>
     </row>
-    <row r="98" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -18253,8 +18925,14 @@
       <c r="CL98">
         <v>6</v>
       </c>
+      <c r="CN98">
+        <v>1</v>
+      </c>
+      <c r="CO98">
+        <v>6</v>
+      </c>
     </row>
-    <row r="99" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -18397,8 +19075,14 @@
       <c r="CL99">
         <v>1</v>
       </c>
+      <c r="CN99">
+        <v>2</v>
+      </c>
+      <c r="CO99">
+        <v>1</v>
+      </c>
     </row>
-    <row r="100" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -18520,8 +19204,11 @@
       <c r="CK100">
         <v>8</v>
       </c>
+      <c r="CN100">
+        <v>8</v>
+      </c>
     </row>
-    <row r="101" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -18697,8 +19384,14 @@
       <c r="CL101">
         <v>4</v>
       </c>
+      <c r="CN101">
+        <v>1</v>
+      </c>
+      <c r="CO101">
+        <v>4</v>
+      </c>
     </row>
-    <row r="102" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -18829,8 +19522,14 @@
       <c r="CM102">
         <v>1</v>
       </c>
+      <c r="CN102">
+        <v>3</v>
+      </c>
+      <c r="CO102">
+        <v>4</v>
+      </c>
     </row>
-    <row r="103" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -19027,8 +19726,14 @@
       <c r="CL103">
         <v>6</v>
       </c>
+      <c r="CN103">
+        <v>0</v>
+      </c>
+      <c r="CO103">
+        <v>6</v>
+      </c>
     </row>
-    <row r="104" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -19222,8 +19927,14 @@
       <c r="CL104">
         <v>8</v>
       </c>
+      <c r="CN104">
+        <v>2</v>
+      </c>
+      <c r="CO104">
+        <v>8</v>
+      </c>
     </row>
-    <row r="105" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -19411,8 +20122,14 @@
       <c r="CL105">
         <v>6</v>
       </c>
+      <c r="CN105">
+        <v>0</v>
+      </c>
+      <c r="CO105">
+        <v>6</v>
+      </c>
     </row>
-    <row r="106" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -19591,8 +20308,14 @@
       <c r="CM106">
         <v>1</v>
       </c>
+      <c r="CN106">
+        <v>0</v>
+      </c>
+      <c r="CO106">
+        <v>8</v>
+      </c>
     </row>
-    <row r="107" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -19792,8 +20515,14 @@
       <c r="CL107">
         <v>5</v>
       </c>
+      <c r="CN107">
+        <v>0</v>
+      </c>
+      <c r="CO107">
+        <v>5</v>
+      </c>
     </row>
-    <row r="108" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -19978,8 +20707,14 @@
       <c r="CL108">
         <v>10</v>
       </c>
+      <c r="CN108">
+        <v>0</v>
+      </c>
+      <c r="CO108">
+        <v>10</v>
+      </c>
     </row>
-    <row r="109" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -20179,8 +20914,14 @@
       <c r="CL109">
         <v>9</v>
       </c>
+      <c r="CN109">
+        <v>0</v>
+      </c>
+      <c r="CO109">
+        <v>9</v>
+      </c>
     </row>
-    <row r="110" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -20383,8 +21124,14 @@
       <c r="CL110">
         <v>3</v>
       </c>
+      <c r="CN110">
+        <v>6</v>
+      </c>
+      <c r="CO110">
+        <v>3</v>
+      </c>
     </row>
-    <row r="111" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -20572,8 +21319,17 @@
       <c r="CL111">
         <v>3</v>
       </c>
+      <c r="CN111">
+        <v>0</v>
+      </c>
+      <c r="CO111">
+        <v>4</v>
+      </c>
+      <c r="CP111">
+        <v>4</v>
+      </c>
     </row>
-    <row r="112" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -20770,8 +21526,14 @@
       <c r="CM112">
         <v>1</v>
       </c>
+      <c r="CN112">
+        <v>4</v>
+      </c>
+      <c r="CO112">
+        <v>4</v>
+      </c>
     </row>
-    <row r="113" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -20974,8 +21736,14 @@
       <c r="CL113">
         <v>2</v>
       </c>
+      <c r="CN113">
+        <v>4</v>
+      </c>
+      <c r="CO113">
+        <v>2</v>
+      </c>
     </row>
-    <row r="114" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -21103,8 +21871,14 @@
       <c r="CL114">
         <v>8</v>
       </c>
+      <c r="CN114">
+        <v>0</v>
+      </c>
+      <c r="CO114">
+        <v>8</v>
+      </c>
     </row>
-    <row r="115" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -21310,8 +22084,14 @@
       <c r="CL115">
         <v>4</v>
       </c>
+      <c r="CN115">
+        <v>0</v>
+      </c>
+      <c r="CO115">
+        <v>4</v>
+      </c>
     </row>
-    <row r="116" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -21502,8 +22282,14 @@
       <c r="CL116">
         <v>8</v>
       </c>
+      <c r="CN116">
+        <v>0</v>
+      </c>
+      <c r="CO116">
+        <v>8</v>
+      </c>
     </row>
-    <row r="117" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -21700,8 +22486,14 @@
       <c r="CL117">
         <v>5</v>
       </c>
+      <c r="CN117">
+        <v>0</v>
+      </c>
+      <c r="CO117">
+        <v>5</v>
+      </c>
     </row>
-    <row r="118" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -21839,8 +22631,14 @@
       <c r="CL118">
         <v>6</v>
       </c>
+      <c r="CN118">
+        <v>0</v>
+      </c>
+      <c r="CO118">
+        <v>6</v>
+      </c>
     </row>
-    <row r="119" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -21980,8 +22778,14 @@
       <c r="CL119">
         <v>7</v>
       </c>
+      <c r="CN119">
+        <v>0</v>
+      </c>
+      <c r="CO119">
+        <v>7</v>
+      </c>
     </row>
-    <row r="120" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -22112,8 +22916,14 @@
       <c r="CL120">
         <v>10</v>
       </c>
+      <c r="CN120">
+        <v>0</v>
+      </c>
+      <c r="CO120">
+        <v>10</v>
+      </c>
     </row>
-    <row r="121" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -22244,8 +23054,14 @@
       <c r="CM121">
         <v>2</v>
       </c>
+      <c r="CN121">
+        <v>0</v>
+      </c>
+      <c r="CO121">
+        <v>8</v>
+      </c>
     </row>
-    <row r="122" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -22379,8 +23195,14 @@
       <c r="CM122">
         <v>1</v>
       </c>
+      <c r="CN122">
+        <v>0</v>
+      </c>
+      <c r="CO122">
+        <v>6</v>
+      </c>
     </row>
-    <row r="123" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -22565,8 +23387,14 @@
       <c r="CL123">
         <v>3</v>
       </c>
+      <c r="CN123">
+        <v>3</v>
+      </c>
+      <c r="CO123">
+        <v>3</v>
+      </c>
     </row>
-    <row r="124" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -22790,8 +23618,17 @@
       <c r="CM124">
         <v>1</v>
       </c>
+      <c r="CN124">
+        <v>2</v>
+      </c>
+      <c r="CO124">
+        <v>6</v>
+      </c>
+      <c r="CP124">
+        <v>1</v>
+      </c>
     </row>
-    <row r="125" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -23003,8 +23840,14 @@
       <c r="CL125">
         <v>6</v>
       </c>
+      <c r="CN125">
+        <v>0</v>
+      </c>
+      <c r="CO125">
+        <v>6</v>
+      </c>
     </row>
-    <row r="126" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -23198,8 +24041,14 @@
       <c r="CL126">
         <v>6</v>
       </c>
+      <c r="CN126">
+        <v>0</v>
+      </c>
+      <c r="CO126">
+        <v>6</v>
+      </c>
     </row>
-    <row r="127" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -23387,8 +24236,14 @@
       <c r="CL127">
         <v>3</v>
       </c>
+      <c r="CN127">
+        <v>0</v>
+      </c>
+      <c r="CO127">
+        <v>3</v>
+      </c>
     </row>
-    <row r="128" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -23507,8 +24362,14 @@
       <c r="CL128">
         <v>7</v>
       </c>
+      <c r="CN128">
+        <v>0</v>
+      </c>
+      <c r="CO128">
+        <v>7</v>
+      </c>
     </row>
-    <row r="129" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -23711,8 +24572,14 @@
       <c r="CL129">
         <v>6</v>
       </c>
+      <c r="CN129">
+        <v>0</v>
+      </c>
+      <c r="CO129">
+        <v>6</v>
+      </c>
     </row>
-    <row r="130" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -23852,8 +24719,14 @@
       <c r="CL130">
         <v>10</v>
       </c>
+      <c r="CN130">
+        <v>0</v>
+      </c>
+      <c r="CO130">
+        <v>10</v>
+      </c>
     </row>
-    <row r="131" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -24059,8 +24932,14 @@
       <c r="CL131">
         <v>10</v>
       </c>
+      <c r="CN131">
+        <v>0</v>
+      </c>
+      <c r="CO131">
+        <v>10</v>
+      </c>
     </row>
-    <row r="132" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -24188,8 +25067,14 @@
       <c r="CL132">
         <v>6</v>
       </c>
+      <c r="CN132">
+        <v>0</v>
+      </c>
+      <c r="CO132">
+        <v>6</v>
+      </c>
     </row>
-    <row r="133" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -24350,8 +25235,14 @@
       <c r="CL133">
         <v>7</v>
       </c>
+      <c r="CN133">
+        <v>0</v>
+      </c>
+      <c r="CO133">
+        <v>7</v>
+      </c>
     </row>
-    <row r="134" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -24512,8 +25403,14 @@
       <c r="CL134">
         <v>8</v>
       </c>
+      <c r="CN134">
+        <v>0</v>
+      </c>
+      <c r="CO134">
+        <v>10</v>
+      </c>
     </row>
-    <row r="135" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -24695,8 +25592,14 @@
       <c r="CL135">
         <v>7</v>
       </c>
+      <c r="CN135">
+        <v>1</v>
+      </c>
+      <c r="CO135">
+        <v>7</v>
+      </c>
     </row>
-    <row r="136" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -24872,8 +25775,14 @@
       <c r="CL136">
         <v>7</v>
       </c>
+      <c r="CN136">
+        <v>0</v>
+      </c>
+      <c r="CO136">
+        <v>7</v>
+      </c>
     </row>
-    <row r="137" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -25052,8 +25961,17 @@
       <c r="CL137">
         <v>2</v>
       </c>
+      <c r="CN137">
+        <v>2</v>
+      </c>
+      <c r="CO137">
+        <v>2</v>
+      </c>
+      <c r="CP137">
+        <v>1</v>
+      </c>
     </row>
-    <row r="138" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -25250,8 +26168,14 @@
       <c r="CL138">
         <v>7</v>
       </c>
+      <c r="CN138">
+        <v>0</v>
+      </c>
+      <c r="CO138">
+        <v>7</v>
+      </c>
     </row>
-    <row r="139" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -25430,8 +26354,14 @@
       <c r="CL139">
         <v>5</v>
       </c>
+      <c r="CN139">
+        <v>0</v>
+      </c>
+      <c r="CO139">
+        <v>5</v>
+      </c>
     </row>
-    <row r="140" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -25565,8 +26495,14 @@
       <c r="CL140">
         <v>9</v>
       </c>
+      <c r="CN140">
+        <v>0</v>
+      </c>
+      <c r="CO140">
+        <v>9</v>
+      </c>
     </row>
-    <row r="141" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -25781,8 +26717,14 @@
       <c r="CL141">
         <v>8</v>
       </c>
+      <c r="CN141">
+        <v>0</v>
+      </c>
+      <c r="CO141">
+        <v>8</v>
+      </c>
     </row>
-    <row r="142" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -25997,8 +26939,14 @@
       <c r="CL142">
         <v>8</v>
       </c>
+      <c r="CN142">
+        <v>0</v>
+      </c>
+      <c r="CO142">
+        <v>8</v>
+      </c>
     </row>
-    <row r="143" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -26171,8 +27119,14 @@
       <c r="CL143">
         <v>11</v>
       </c>
+      <c r="CN143">
+        <v>0</v>
+      </c>
+      <c r="CO143">
+        <v>11</v>
+      </c>
     </row>
-    <row r="144" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -26297,8 +27251,14 @@
       <c r="CL144">
         <v>7</v>
       </c>
+      <c r="CN144">
+        <v>0</v>
+      </c>
+      <c r="CO144">
+        <v>7</v>
+      </c>
     </row>
-    <row r="145" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -26432,8 +27392,14 @@
       <c r="CL145">
         <v>5</v>
       </c>
+      <c r="CN145">
+        <v>0</v>
+      </c>
+      <c r="CO145">
+        <v>5</v>
+      </c>
     </row>
-    <row r="146" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -26657,8 +27623,17 @@
       <c r="CL146">
         <v>7</v>
       </c>
+      <c r="CN146">
+        <v>0</v>
+      </c>
+      <c r="CO146">
+        <v>9</v>
+      </c>
+      <c r="CP146">
+        <v>1</v>
+      </c>
     </row>
-    <row r="147" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -26873,8 +27848,14 @@
       <c r="CL147">
         <v>1</v>
       </c>
+      <c r="CN147">
+        <v>2</v>
+      </c>
+      <c r="CO147">
+        <v>1</v>
+      </c>
     </row>
-    <row r="148" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -26993,8 +27974,11 @@
       <c r="CK148">
         <v>9</v>
       </c>
+      <c r="CN148">
+        <v>9</v>
+      </c>
     </row>
-    <row r="149" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -27212,8 +28196,17 @@
       <c r="CM149">
         <v>2</v>
       </c>
+      <c r="CN149">
+        <v>1</v>
+      </c>
+      <c r="CO149">
+        <v>3</v>
+      </c>
+      <c r="CP149">
+        <v>1</v>
+      </c>
     </row>
-    <row r="150" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -27422,8 +28415,14 @@
       <c r="CL150">
         <v>1</v>
       </c>
+      <c r="CN150">
+        <v>0</v>
+      </c>
+      <c r="CO150">
+        <v>9</v>
+      </c>
     </row>
-    <row r="151" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -27608,8 +28607,14 @@
       <c r="CL151">
         <v>10</v>
       </c>
+      <c r="CN151">
+        <v>0</v>
+      </c>
+      <c r="CO151">
+        <v>10</v>
+      </c>
     </row>
-    <row r="152" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -27731,8 +28736,14 @@
       <c r="CM152">
         <v>4</v>
       </c>
+      <c r="CN152">
+        <v>0</v>
+      </c>
+      <c r="CO152">
+        <v>9</v>
+      </c>
     </row>
-    <row r="153" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -27908,8 +28919,14 @@
       <c r="CL153">
         <v>7</v>
       </c>
+      <c r="CN153">
+        <v>0</v>
+      </c>
+      <c r="CO153">
+        <v>7</v>
+      </c>
     </row>
-    <row r="154" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -28151,8 +29168,14 @@
       <c r="CL154">
         <v>8</v>
       </c>
+      <c r="CN154">
+        <v>0</v>
+      </c>
+      <c r="CO154">
+        <v>8</v>
+      </c>
     </row>
-    <row r="155" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -28343,8 +29366,14 @@
       <c r="CL155">
         <v>9</v>
       </c>
+      <c r="CN155">
+        <v>0</v>
+      </c>
+      <c r="CO155">
+        <v>9</v>
+      </c>
     </row>
-    <row r="156" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="156" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -28469,8 +29498,17 @@
       <c r="CL156">
         <v>5</v>
       </c>
+      <c r="CN156">
+        <v>0</v>
+      </c>
+      <c r="CO156">
+        <v>5</v>
+      </c>
+      <c r="CP156">
+        <v>1</v>
+      </c>
     </row>
-    <row r="157" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="157" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -28598,8 +29636,14 @@
       <c r="CL157">
         <v>6</v>
       </c>
+      <c r="CN157">
+        <v>0</v>
+      </c>
+      <c r="CO157">
+        <v>6</v>
+      </c>
     </row>
-    <row r="158" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="158" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -28757,8 +29801,17 @@
       <c r="CM158">
         <v>2</v>
       </c>
+      <c r="CN158">
+        <v>4</v>
+      </c>
+      <c r="CO158">
+        <v>2</v>
+      </c>
+      <c r="CP158">
+        <v>2</v>
+      </c>
     </row>
-    <row r="159" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -28964,8 +30017,14 @@
       <c r="CL159">
         <v>5</v>
       </c>
+      <c r="CN159">
+        <v>0</v>
+      </c>
+      <c r="CO159">
+        <v>5</v>
+      </c>
     </row>
-    <row r="160" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -29084,8 +30143,14 @@
       <c r="CK160">
         <v>9</v>
       </c>
+      <c r="CN160">
+        <v>8</v>
+      </c>
+      <c r="CP160">
+        <v>1</v>
+      </c>
     </row>
-    <row r="161" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -29309,8 +30374,14 @@
       <c r="CL161">
         <v>6</v>
       </c>
+      <c r="CN161">
+        <v>1</v>
+      </c>
+      <c r="CO161">
+        <v>6</v>
+      </c>
     </row>
-    <row r="162" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -29432,8 +30503,17 @@
       <c r="CM162">
         <v>1</v>
       </c>
+      <c r="CN162">
+        <v>0</v>
+      </c>
+      <c r="CO162">
+        <v>5</v>
+      </c>
+      <c r="CP162">
+        <v>3</v>
+      </c>
     </row>
-    <row r="163" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="163" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -29618,8 +30698,14 @@
       <c r="CL163">
         <v>8</v>
       </c>
+      <c r="CN163">
+        <v>0</v>
+      </c>
+      <c r="CO163">
+        <v>8</v>
+      </c>
     </row>
-    <row r="164" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="164" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -29747,8 +30833,14 @@
       <c r="CM164">
         <v>1</v>
       </c>
+      <c r="CN164">
+        <v>1</v>
+      </c>
+      <c r="CO164">
+        <v>8</v>
+      </c>
     </row>
-    <row r="165" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -29933,8 +31025,14 @@
       <c r="CL165">
         <v>6</v>
       </c>
+      <c r="CN165">
+        <v>0</v>
+      </c>
+      <c r="CO165">
+        <v>6</v>
+      </c>
     </row>
-    <row r="166" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="166" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -30104,8 +31202,14 @@
       <c r="CL166">
         <v>6</v>
       </c>
+      <c r="CN166">
+        <v>0</v>
+      </c>
+      <c r="CO166">
+        <v>6</v>
+      </c>
     </row>
-    <row r="167" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -30278,8 +31382,14 @@
       <c r="CL167">
         <v>8</v>
       </c>
+      <c r="CN167">
+        <v>0</v>
+      </c>
+      <c r="CO167">
+        <v>8</v>
+      </c>
     </row>
-    <row r="168" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -30485,8 +31595,14 @@
       <c r="CL168">
         <v>11</v>
       </c>
+      <c r="CN168">
+        <v>0</v>
+      </c>
+      <c r="CO168">
+        <v>11</v>
+      </c>
     </row>
-    <row r="169" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -30614,8 +31730,14 @@
       <c r="CL169">
         <v>6</v>
       </c>
+      <c r="CN169">
+        <v>0</v>
+      </c>
+      <c r="CO169">
+        <v>6</v>
+      </c>
     </row>
-    <row r="170" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -30764,8 +31886,14 @@
       <c r="CM170">
         <v>1</v>
       </c>
+      <c r="CN170">
+        <v>4</v>
+      </c>
+      <c r="CP170">
+        <v>4</v>
+      </c>
     </row>
-    <row r="171" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="171" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -30980,8 +32108,14 @@
       <c r="CL171">
         <v>8</v>
       </c>
+      <c r="CN171">
+        <v>2</v>
+      </c>
+      <c r="CO171">
+        <v>8</v>
+      </c>
     </row>
-    <row r="172" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -31112,8 +32246,14 @@
       <c r="CM172">
         <v>1</v>
       </c>
+      <c r="CN172">
+        <v>4</v>
+      </c>
+      <c r="CO172">
+        <v>4</v>
+      </c>
     </row>
-    <row r="173" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -31262,8 +32402,14 @@
       <c r="CL173">
         <v>2</v>
       </c>
+      <c r="CN173">
+        <v>6</v>
+      </c>
+      <c r="CO173">
+        <v>2</v>
+      </c>
     </row>
-    <row r="174" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -31394,8 +32540,17 @@
       <c r="CL174">
         <v>3</v>
       </c>
+      <c r="CN174">
+        <v>0</v>
+      </c>
+      <c r="CO174">
+        <v>7</v>
+      </c>
+      <c r="CP174">
+        <v>2</v>
+      </c>
     </row>
-    <row r="175" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -31586,8 +32741,14 @@
       <c r="CM175">
         <v>1</v>
       </c>
+      <c r="CN175">
+        <v>0</v>
+      </c>
+      <c r="CO175">
+        <v>9</v>
+      </c>
     </row>
-    <row r="176" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="176" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -31712,8 +32873,14 @@
       <c r="CL176">
         <v>8</v>
       </c>
+      <c r="CN176">
+        <v>0</v>
+      </c>
+      <c r="CO176">
+        <v>8</v>
+      </c>
     </row>
-    <row r="177" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -31847,8 +33014,14 @@
       <c r="CL177">
         <v>5</v>
       </c>
+      <c r="CN177">
+        <v>0</v>
+      </c>
+      <c r="CO177">
+        <v>5</v>
+      </c>
     </row>
-    <row r="178" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -31988,8 +33161,14 @@
       <c r="CL178">
         <v>8</v>
       </c>
+      <c r="CN178">
+        <v>0</v>
+      </c>
+      <c r="CO178">
+        <v>8</v>
+      </c>
     </row>
-    <row r="179" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -32180,8 +33359,14 @@
       <c r="CL179">
         <v>10</v>
       </c>
+      <c r="CN179">
+        <v>0</v>
+      </c>
+      <c r="CO179">
+        <v>10</v>
+      </c>
     </row>
-    <row r="180" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -32369,8 +33554,14 @@
       <c r="CL180">
         <v>9</v>
       </c>
+      <c r="CN180">
+        <v>0</v>
+      </c>
+      <c r="CO180">
+        <v>9</v>
+      </c>
     </row>
-    <row r="181" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -32558,8 +33749,14 @@
       <c r="CL181">
         <v>9</v>
       </c>
+      <c r="CN181">
+        <v>0</v>
+      </c>
+      <c r="CO181">
+        <v>9</v>
+      </c>
     </row>
-    <row r="182" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -32690,8 +33887,14 @@
       <c r="CL182">
         <v>4</v>
       </c>
+      <c r="CN182">
+        <v>1</v>
+      </c>
+      <c r="CO182">
+        <v>5</v>
+      </c>
     </row>
-    <row r="183" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -32911,8 +34114,14 @@
       <c r="CL183">
         <v>2</v>
       </c>
+      <c r="CN183">
+        <v>0</v>
+      </c>
+      <c r="CO183">
+        <v>5</v>
+      </c>
     </row>
-    <row r="184" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -33051,8 +34260,14 @@
       <c r="CL184">
         <v>6</v>
       </c>
+      <c r="CN184">
+        <v>0</v>
+      </c>
+      <c r="CO184">
+        <v>6</v>
+      </c>
     </row>
-    <row r="185" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -33242,8 +34457,14 @@
       <c r="CL185">
         <v>7</v>
       </c>
+      <c r="CN185">
+        <v>0</v>
+      </c>
+      <c r="CO185">
+        <v>7</v>
+      </c>
     </row>
-    <row r="186" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -33421,8 +34642,14 @@
       <c r="CL186">
         <v>1</v>
       </c>
+      <c r="CN186">
+        <v>6</v>
+      </c>
+      <c r="CO186">
+        <v>1</v>
+      </c>
     </row>
-    <row r="187" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -33567,8 +34794,14 @@
       <c r="CM187">
         <v>1</v>
       </c>
+      <c r="CN187">
+        <v>6</v>
+      </c>
+      <c r="CP187">
+        <v>1</v>
+      </c>
     </row>
-    <row r="188" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B188" t="s">
         <v>4</v>
       </c>
@@ -33761,8 +34994,17 @@
       <c r="CL188">
         <v>4</v>
       </c>
+      <c r="CN188">
+        <v>4</v>
+      </c>
+      <c r="CO188">
+        <v>4</v>
+      </c>
+      <c r="CP188">
+        <v>2</v>
+      </c>
     </row>
-    <row r="189" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -33958,8 +35200,14 @@
       <c r="CL189">
         <v>2</v>
       </c>
+      <c r="CN189">
+        <v>0</v>
+      </c>
+      <c r="CO189">
+        <v>2</v>
+      </c>
     </row>
-    <row r="190" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="190" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -34158,8 +35406,14 @@
       <c r="CL190">
         <v>5</v>
       </c>
+      <c r="CN190">
+        <v>0</v>
+      </c>
+      <c r="CO190">
+        <v>5</v>
+      </c>
     </row>
-    <row r="191" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="191" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -34361,8 +35615,14 @@
       <c r="CL191">
         <v>5</v>
       </c>
+      <c r="CN191">
+        <v>0</v>
+      </c>
+      <c r="CO191">
+        <v>5</v>
+      </c>
     </row>
-    <row r="192" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="192" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -34543,8 +35803,14 @@
       <c r="CL192">
         <v>3</v>
       </c>
+      <c r="CN192">
+        <v>0</v>
+      </c>
+      <c r="CO192">
+        <v>3</v>
+      </c>
     </row>
-    <row r="193" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="193" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -34749,8 +36015,14 @@
       <c r="CM193">
         <v>2</v>
       </c>
+      <c r="CN193">
+        <v>3</v>
+      </c>
+      <c r="CO193">
+        <v>4</v>
+      </c>
     </row>
-    <row r="194" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="194" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B194" t="s">
         <v>4</v>
       </c>
@@ -34928,8 +36200,17 @@
       <c r="CL194">
         <v>1</v>
       </c>
+      <c r="CN194">
+        <v>0</v>
+      </c>
+      <c r="CO194">
+        <v>6</v>
+      </c>
+      <c r="CP194">
+        <v>1</v>
+      </c>
     </row>
-    <row r="195" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="195" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -35125,8 +36406,14 @@
       <c r="CM195">
         <v>1</v>
       </c>
+      <c r="CN195">
+        <v>0</v>
+      </c>
+      <c r="CO195">
+        <v>2</v>
+      </c>
     </row>
-    <row r="196" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="196" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -35355,8 +36642,14 @@
       <c r="CL196">
         <v>9</v>
       </c>
+      <c r="CN196">
+        <v>0</v>
+      </c>
+      <c r="CO196">
+        <v>9</v>
+      </c>
     </row>
-    <row r="197" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="197" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -35540,8 +36833,14 @@
       <c r="CL197">
         <v>4</v>
       </c>
+      <c r="CN197">
+        <v>0</v>
+      </c>
+      <c r="CO197">
+        <v>4</v>
+      </c>
     </row>
-    <row r="198" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="198" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -35707,8 +37006,14 @@
       <c r="CL198">
         <v>5</v>
       </c>
+      <c r="CN198">
+        <v>0</v>
+      </c>
+      <c r="CO198">
+        <v>5</v>
+      </c>
     </row>
-    <row r="199" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="199" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -35883,11 +37188,17 @@
       <c r="CK199">
         <v>5</v>
       </c>
-      <c r="CL199">
-        <v>1</v>
+      <c r="CM199">
+        <v>1</v>
+      </c>
+      <c r="CN199">
+        <v>1</v>
+      </c>
+      <c r="CP199">
+        <v>5</v>
       </c>
     </row>
-    <row r="200" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="200" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
         <v>4</v>
       </c>
@@ -36059,8 +37370,17 @@
       <c r="CL200">
         <v>6</v>
       </c>
+      <c r="CN200">
+        <v>0</v>
+      </c>
+      <c r="CO200">
+        <v>6</v>
+      </c>
+      <c r="CP200">
+        <v>1</v>
+      </c>
     </row>
-    <row r="201" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="201" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -36271,8 +37591,14 @@
       <c r="CL201">
         <v>5</v>
       </c>
+      <c r="CN201">
+        <v>0</v>
+      </c>
+      <c r="CO201">
+        <v>6</v>
+      </c>
     </row>
-    <row r="202" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="202" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -36474,8 +37800,14 @@
       <c r="CL202">
         <v>1</v>
       </c>
+      <c r="CN202">
+        <v>0</v>
+      </c>
+      <c r="CO202">
+        <v>1</v>
+      </c>
     </row>
-    <row r="203" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="203" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -36671,8 +38003,14 @@
       <c r="CL203">
         <v>3</v>
       </c>
+      <c r="CN203">
+        <v>0</v>
+      </c>
+      <c r="CO203">
+        <v>3</v>
+      </c>
     </row>
-    <row r="204" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="204" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -36787,8 +38125,11 @@
       <c r="CK204">
         <v>6</v>
       </c>
+      <c r="CN204">
+        <v>6</v>
+      </c>
     </row>
-    <row r="205" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="205" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -37002,8 +38343,14 @@
       <c r="CM205">
         <v>2</v>
       </c>
+      <c r="CN205">
+        <v>8</v>
+      </c>
+      <c r="CO205">
+        <v>2</v>
+      </c>
     </row>
-    <row r="206" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="206" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B206" t="s">
         <v>4</v>
       </c>
@@ -37121,8 +38468,14 @@
       <c r="CK206">
         <v>6</v>
       </c>
+      <c r="CN206">
+        <v>1</v>
+      </c>
+      <c r="CP206">
+        <v>5</v>
+      </c>
     </row>
-    <row r="207" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="207" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -37291,8 +38644,14 @@
       <c r="CM207">
         <v>1</v>
       </c>
+      <c r="CN207">
+        <v>0</v>
+      </c>
+      <c r="CO207">
+        <v>4</v>
+      </c>
     </row>
-    <row r="208" spans="2:91" x14ac:dyDescent="0.3">
+    <row r="208" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -37488,8 +38847,14 @@
       <c r="CL208">
         <v>3</v>
       </c>
+      <c r="CN208">
+        <v>0</v>
+      </c>
+      <c r="CO208">
+        <v>3</v>
+      </c>
     </row>
-    <row r="209" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="209" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B209" t="s">
         <v>3</v>
       </c>
@@ -37670,8 +39035,14 @@
       <c r="CL209">
         <v>5</v>
       </c>
+      <c r="CN209">
+        <v>0</v>
+      </c>
+      <c r="CO209">
+        <v>5</v>
+      </c>
     </row>
-    <row r="210" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="210" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B210" t="s">
         <v>1</v>
       </c>
@@ -37873,8 +39244,14 @@
       <c r="CL210">
         <v>1</v>
       </c>
+      <c r="CN210">
+        <v>4</v>
+      </c>
+      <c r="CO210">
+        <v>1</v>
+      </c>
     </row>
-    <row r="211" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="211" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
         <v>4</v>
       </c>
@@ -38052,8 +39429,14 @@
       <c r="CL211">
         <v>2</v>
       </c>
+      <c r="CN211">
+        <v>3</v>
+      </c>
+      <c r="CO211">
+        <v>2</v>
+      </c>
     </row>
-    <row r="212" spans="2:90" x14ac:dyDescent="0.3">
+    <row r="212" spans="2:94" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
         <v>4</v>
       </c>
@@ -38224,6 +39607,15 @@
       </c>
       <c r="CL212">
         <v>1</v>
+      </c>
+      <c r="CN212">
+        <v>0</v>
+      </c>
+      <c r="CO212">
+        <v>4</v>
+      </c>
+      <c r="CP212">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DOY 182 germinants data collection
</commit_message>
<xml_diff>
--- a/data/germination_data.xlsx
+++ b/data/germination_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temporal Ecology Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8CA7CFB-12E8-48CB-8A42-34B61559B563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E758C45-0616-473D-BA12-4E9C32541A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="134">
   <si>
     <t>seed_species</t>
   </si>
@@ -465,6 +465,15 @@
   <si>
     <t>168_halfdead</t>
   </si>
+  <si>
+    <t>182_alive</t>
+  </si>
+  <si>
+    <t>182_dead</t>
+  </si>
+  <si>
+    <t>182_halfdead</t>
+  </si>
 </sst>
 </file>
 
@@ -568,9 +577,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CP213" totalsRowShown="0">
-  <autoFilter ref="B2:CP213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
-  <tableColumns count="93">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CS213" totalsRowShown="0">
+  <autoFilter ref="B2:CS213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
+  <tableColumns count="96">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
     <tableColumn id="3" xr3:uid="{B695F4B4-8561-9D48-9FF3-12A40CB2B7C7}" name="inoculated_%"/>
@@ -664,6 +673,9 @@
     <tableColumn id="91" xr3:uid="{19796ADF-ED67-4616-A2F4-F5F6343D05C5}" name="168_alive"/>
     <tableColumn id="92" xr3:uid="{7489BFD5-C58F-456E-A7EF-D0F7BF350167}" name="168_dead"/>
     <tableColumn id="93" xr3:uid="{3DEB280A-450E-4E2A-8CF9-DAB35C6C1464}" name="168_halfdead"/>
+    <tableColumn id="94" xr3:uid="{9578CF96-5AE8-4645-B28F-F07D512CF35B}" name="182_alive"/>
+    <tableColumn id="95" xr3:uid="{D47C9C3A-2489-4F83-963C-62C798893172}" name="182_dead"/>
+    <tableColumn id="96" xr3:uid="{AC274215-49C4-4F5F-8E83-C3C811642720}" name="182_halfdead"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -986,7 +998,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:CP212"/>
+  <dimension ref="B2:CS212"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -994,7 +1006,7 @@
     <col min="4" max="4" width="17.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -1274,8 +1286,17 @@
       <c r="CP2" t="s">
         <v>130</v>
       </c>
+      <c r="CQ2" t="s">
+        <v>131</v>
+      </c>
+      <c r="CR2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CS2" t="s">
+        <v>133</v>
+      </c>
     </row>
-    <row r="3" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1489,8 +1510,17 @@
       <c r="CO3">
         <v>3</v>
       </c>
+      <c r="CQ3">
+        <v>0</v>
+      </c>
+      <c r="CR3">
+        <v>3</v>
+      </c>
+      <c r="CS3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1614,8 +1644,11 @@
       <c r="CN4">
         <v>9</v>
       </c>
+      <c r="CQ4">
+        <v>9</v>
+      </c>
     </row>
-    <row r="5" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1829,8 +1862,14 @@
       <c r="CO5">
         <v>7</v>
       </c>
+      <c r="CQ5">
+        <v>0</v>
+      </c>
+      <c r="CR5">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1954,8 +1993,14 @@
       <c r="CP6">
         <v>4</v>
       </c>
+      <c r="CQ6">
+        <v>2</v>
+      </c>
+      <c r="CR6">
+        <v>7</v>
+      </c>
     </row>
-    <row r="7" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -2136,8 +2181,14 @@
       <c r="CP7">
         <v>1</v>
       </c>
+      <c r="CQ7">
+        <v>0</v>
+      </c>
+      <c r="CR7">
+        <v>6</v>
+      </c>
     </row>
-    <row r="8" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -2342,8 +2393,14 @@
       <c r="CO8">
         <v>1</v>
       </c>
+      <c r="CQ8">
+        <v>6</v>
+      </c>
+      <c r="CR8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2557,8 +2614,14 @@
       <c r="CP9">
         <v>1</v>
       </c>
+      <c r="CQ9">
+        <v>0</v>
+      </c>
+      <c r="CR9">
+        <v>7</v>
+      </c>
     </row>
-    <row r="10" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -2703,8 +2766,17 @@
       <c r="CO10">
         <v>2</v>
       </c>
+      <c r="CQ10">
+        <v>5</v>
+      </c>
+      <c r="CR10">
+        <v>2</v>
+      </c>
+      <c r="CS10">
+        <v>1</v>
+      </c>
     </row>
-    <row r="11" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -2915,8 +2987,14 @@
       <c r="CO11">
         <v>8</v>
       </c>
+      <c r="CQ11">
+        <v>0</v>
+      </c>
+      <c r="CR11">
+        <v>8</v>
+      </c>
     </row>
-    <row r="12" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -3130,8 +3208,14 @@
       <c r="CO12">
         <v>5</v>
       </c>
+      <c r="CQ12">
+        <v>5</v>
+      </c>
+      <c r="CR12">
+        <v>5</v>
+      </c>
     </row>
-    <row r="13" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -3336,8 +3420,14 @@
       <c r="CO13">
         <v>7</v>
       </c>
+      <c r="CQ13">
+        <v>0</v>
+      </c>
+      <c r="CR13">
+        <v>7</v>
+      </c>
     </row>
-    <row r="14" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -3500,8 +3590,17 @@
       <c r="CO14">
         <v>1</v>
       </c>
+      <c r="CQ14">
+        <v>4</v>
+      </c>
+      <c r="CR14">
+        <v>2</v>
+      </c>
+      <c r="CS14">
+        <v>3</v>
+      </c>
     </row>
-    <row r="15" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -3695,8 +3794,14 @@
       <c r="CO15">
         <v>8</v>
       </c>
+      <c r="CQ15">
+        <v>0</v>
+      </c>
+      <c r="CR15">
+        <v>8</v>
+      </c>
     </row>
-    <row r="16" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -3875,8 +3980,17 @@
       <c r="CP16">
         <v>1</v>
       </c>
+      <c r="CQ16">
+        <v>4</v>
+      </c>
+      <c r="CR16">
+        <v>3</v>
+      </c>
+      <c r="CS16">
+        <v>2</v>
+      </c>
     </row>
-    <row r="17" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -4073,8 +4187,14 @@
       <c r="CO17">
         <v>8</v>
       </c>
+      <c r="CQ17">
+        <v>0</v>
+      </c>
+      <c r="CR17">
+        <v>8</v>
+      </c>
     </row>
-    <row r="18" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -4199,8 +4319,14 @@
       <c r="CP18">
         <v>4</v>
       </c>
+      <c r="CQ18">
+        <v>2</v>
+      </c>
+      <c r="CR18">
+        <v>8</v>
+      </c>
     </row>
-    <row r="19" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -4415,8 +4541,14 @@
       <c r="CO19">
         <v>7</v>
       </c>
+      <c r="CQ19">
+        <v>0</v>
+      </c>
+      <c r="CR19">
+        <v>7</v>
+      </c>
     </row>
-    <row r="20" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -4592,8 +4724,17 @@
       <c r="CO20">
         <v>1</v>
       </c>
+      <c r="CQ20">
+        <v>9</v>
+      </c>
+      <c r="CR20">
+        <v>4</v>
+      </c>
+      <c r="CS20">
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -4774,8 +4915,14 @@
       <c r="CO21">
         <v>6</v>
       </c>
+      <c r="CQ21">
+        <v>0</v>
+      </c>
+      <c r="CR21">
+        <v>6</v>
+      </c>
     </row>
-    <row r="22" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -4909,8 +5056,17 @@
       <c r="CO22">
         <v>2</v>
       </c>
+      <c r="CQ22">
+        <v>2</v>
+      </c>
+      <c r="CR22">
+        <v>4</v>
+      </c>
+      <c r="CS22">
+        <v>2</v>
+      </c>
     </row>
-    <row r="23" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -5119,8 +5275,14 @@
       <c r="CO23">
         <v>10</v>
       </c>
+      <c r="CQ23">
+        <v>0</v>
+      </c>
+      <c r="CR23">
+        <v>10</v>
+      </c>
     </row>
-    <row r="24" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -5302,8 +5464,14 @@
       <c r="CO24">
         <v>4</v>
       </c>
+      <c r="CQ24">
+        <v>8</v>
+      </c>
+      <c r="CR24">
+        <v>4</v>
+      </c>
     </row>
-    <row r="25" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -5434,8 +5602,14 @@
       <c r="CO25">
         <v>8</v>
       </c>
+      <c r="CQ25">
+        <v>0</v>
+      </c>
+      <c r="CR25">
+        <v>8</v>
+      </c>
     </row>
-    <row r="26" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -5695,8 +5869,17 @@
       <c r="CP26">
         <v>1</v>
       </c>
+      <c r="CQ26">
+        <v>0</v>
+      </c>
+      <c r="CR26">
+        <v>10</v>
+      </c>
+      <c r="CS26">
+        <v>1</v>
+      </c>
     </row>
-    <row r="27" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -5884,8 +6067,14 @@
       <c r="CO27">
         <v>4</v>
       </c>
+      <c r="CQ27">
+        <v>1</v>
+      </c>
+      <c r="CR27">
+        <v>5</v>
+      </c>
     </row>
-    <row r="28" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -6112,8 +6301,14 @@
       <c r="CO28">
         <v>10</v>
       </c>
+      <c r="CQ28">
+        <v>0</v>
+      </c>
+      <c r="CR28">
+        <v>10</v>
+      </c>
     </row>
-    <row r="29" spans="2:94" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:97" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>3</v>
       </c>
@@ -6310,8 +6505,14 @@
       <c r="CO29" s="3">
         <v>4</v>
       </c>
+      <c r="CQ29" s="3">
+        <v>0</v>
+      </c>
+      <c r="CR29" s="3">
+        <v>4</v>
+      </c>
     </row>
-    <row r="30" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -6442,8 +6643,14 @@
       <c r="CP30">
         <v>3</v>
       </c>
+      <c r="CQ30">
+        <v>1</v>
+      </c>
+      <c r="CR30">
+        <v>7</v>
+      </c>
     </row>
-    <row r="31" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -6658,8 +6865,14 @@
       <c r="CO31">
         <v>5</v>
       </c>
+      <c r="CQ31">
+        <v>0</v>
+      </c>
+      <c r="CR31">
+        <v>5</v>
+      </c>
     </row>
-    <row r="32" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -6835,8 +7048,17 @@
       <c r="CP32">
         <v>4</v>
       </c>
+      <c r="CQ32">
+        <v>4</v>
+      </c>
+      <c r="CR32">
+        <v>4</v>
+      </c>
+      <c r="CS32">
+        <v>2</v>
+      </c>
     </row>
-    <row r="33" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -7006,8 +7228,14 @@
       <c r="CO33">
         <v>9</v>
       </c>
+      <c r="CQ33">
+        <v>0</v>
+      </c>
+      <c r="CR33">
+        <v>9</v>
+      </c>
     </row>
-    <row r="34" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -7168,8 +7396,14 @@
       <c r="CO34">
         <v>5</v>
       </c>
+      <c r="CQ34">
+        <v>1</v>
+      </c>
+      <c r="CR34">
+        <v>5</v>
+      </c>
     </row>
-    <row r="35" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -7363,8 +7597,14 @@
       <c r="CO35">
         <v>8</v>
       </c>
+      <c r="CQ35">
+        <v>0</v>
+      </c>
+      <c r="CR35">
+        <v>8</v>
+      </c>
     </row>
-    <row r="36" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -7555,8 +7795,14 @@
       <c r="CP36">
         <v>4</v>
       </c>
+      <c r="CQ36">
+        <v>3</v>
+      </c>
+      <c r="CR36">
+        <v>7</v>
+      </c>
     </row>
-    <row r="37" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -7693,8 +7939,14 @@
       <c r="CO37">
         <v>6</v>
       </c>
+      <c r="CQ37">
+        <v>0</v>
+      </c>
+      <c r="CR37">
+        <v>6</v>
+      </c>
     </row>
-    <row r="38" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -7924,8 +8176,14 @@
       <c r="CO38">
         <v>4</v>
       </c>
+      <c r="CQ38">
+        <v>2</v>
+      </c>
+      <c r="CR38">
+        <v>4</v>
+      </c>
     </row>
-    <row r="39" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -8137,8 +8395,14 @@
       <c r="CP39">
         <v>1</v>
       </c>
+      <c r="CQ39">
+        <v>1</v>
+      </c>
+      <c r="CR39">
+        <v>5</v>
+      </c>
     </row>
-    <row r="40" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -8368,8 +8632,14 @@
       <c r="CP40">
         <v>1</v>
       </c>
+      <c r="CQ40">
+        <v>1</v>
+      </c>
+      <c r="CR40">
+        <v>9</v>
+      </c>
     </row>
-    <row r="41" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -8560,8 +8830,14 @@
       <c r="CO41">
         <v>6</v>
       </c>
+      <c r="CQ41">
+        <v>0</v>
+      </c>
+      <c r="CR41">
+        <v>6</v>
+      </c>
     </row>
-    <row r="42" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -8701,8 +8977,14 @@
       <c r="CP42">
         <v>2</v>
       </c>
+      <c r="CQ42">
+        <v>0</v>
+      </c>
+      <c r="CR42">
+        <v>7</v>
+      </c>
     </row>
-    <row r="43" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -8920,8 +9202,14 @@
       <c r="CO43">
         <v>9</v>
       </c>
+      <c r="CQ43">
+        <v>0</v>
+      </c>
+      <c r="CR43">
+        <v>9</v>
+      </c>
     </row>
-    <row r="44" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -9049,8 +9337,14 @@
       <c r="CP44">
         <v>1</v>
       </c>
+      <c r="CQ44">
+        <v>0</v>
+      </c>
+      <c r="CR44">
+        <v>6</v>
+      </c>
     </row>
-    <row r="45" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -9310,8 +9604,14 @@
       <c r="CO45">
         <v>9</v>
       </c>
+      <c r="CQ45">
+        <v>0</v>
+      </c>
+      <c r="CR45">
+        <v>9</v>
+      </c>
     </row>
-    <row r="46" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -9445,8 +9745,14 @@
       <c r="CO46">
         <v>5</v>
       </c>
+      <c r="CQ46">
+        <v>1</v>
+      </c>
+      <c r="CR46">
+        <v>5</v>
+      </c>
     </row>
-    <row r="47" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -9610,8 +9916,14 @@
       <c r="CO47">
         <v>9</v>
       </c>
+      <c r="CQ47">
+        <v>0</v>
+      </c>
+      <c r="CR47">
+        <v>9</v>
+      </c>
     </row>
-    <row r="48" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:96" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -9844,8 +10156,14 @@
       <c r="CO48">
         <v>10</v>
       </c>
+      <c r="CQ48">
+        <v>1</v>
+      </c>
+      <c r="CR48">
+        <v>10</v>
+      </c>
     </row>
-    <row r="49" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -9988,8 +10306,14 @@
       <c r="CP49">
         <v>1</v>
       </c>
+      <c r="CQ49">
+        <v>0</v>
+      </c>
+      <c r="CR49">
+        <v>7</v>
+      </c>
     </row>
-    <row r="50" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -10228,8 +10552,14 @@
       <c r="CP50">
         <v>1</v>
       </c>
+      <c r="CQ50">
+        <v>4</v>
+      </c>
+      <c r="CR50">
+        <v>4</v>
+      </c>
     </row>
-    <row r="51" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -10453,8 +10783,14 @@
       <c r="CO51">
         <v>5</v>
       </c>
+      <c r="CQ51">
+        <v>1</v>
+      </c>
+      <c r="CR51">
+        <v>5</v>
+      </c>
     </row>
-    <row r="52" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -10579,8 +10915,14 @@
       <c r="CP52">
         <v>1</v>
       </c>
+      <c r="CQ52">
+        <v>5</v>
+      </c>
+      <c r="CS52">
+        <v>1</v>
+      </c>
     </row>
-    <row r="53" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -10777,8 +11119,14 @@
       <c r="CO53">
         <v>4</v>
       </c>
+      <c r="CQ53">
+        <v>0</v>
+      </c>
+      <c r="CR53">
+        <v>4</v>
+      </c>
     </row>
-    <row r="54" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -10906,8 +11254,14 @@
       <c r="CP54">
         <v>1</v>
       </c>
+      <c r="CQ54">
+        <v>4</v>
+      </c>
+      <c r="CR54">
+        <v>2</v>
+      </c>
     </row>
-    <row r="55" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -11107,8 +11461,14 @@
       <c r="CO55">
         <v>6</v>
       </c>
+      <c r="CQ55">
+        <v>0</v>
+      </c>
+      <c r="CR55">
+        <v>6</v>
+      </c>
     </row>
-    <row r="56" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -11233,8 +11593,11 @@
       <c r="CN56">
         <v>10</v>
       </c>
+      <c r="CQ56">
+        <v>10</v>
+      </c>
     </row>
-    <row r="57" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -11383,8 +11746,14 @@
       <c r="CP57">
         <v>1</v>
       </c>
+      <c r="CQ57">
+        <v>2</v>
+      </c>
+      <c r="CR57">
+        <v>5</v>
+      </c>
     </row>
-    <row r="58" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -11521,8 +11890,14 @@
       <c r="CO58">
         <v>4</v>
       </c>
+      <c r="CQ58">
+        <v>2</v>
+      </c>
+      <c r="CR58">
+        <v>4</v>
+      </c>
     </row>
-    <row r="59" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -11656,8 +12031,14 @@
       <c r="CO59">
         <v>7</v>
       </c>
+      <c r="CQ59">
+        <v>0</v>
+      </c>
+      <c r="CR59">
+        <v>7</v>
+      </c>
     </row>
-    <row r="60" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -11848,8 +12229,14 @@
       <c r="CO60">
         <v>2</v>
       </c>
+      <c r="CQ60">
+        <v>7</v>
+      </c>
+      <c r="CR60">
+        <v>2</v>
+      </c>
     </row>
-    <row r="61" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -11992,8 +12379,14 @@
       <c r="CO61">
         <v>7</v>
       </c>
+      <c r="CQ61">
+        <v>0</v>
+      </c>
+      <c r="CR61">
+        <v>7</v>
+      </c>
     </row>
-    <row r="62" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -12217,8 +12610,14 @@
       <c r="CP62">
         <v>1</v>
       </c>
+      <c r="CQ62">
+        <v>1</v>
+      </c>
+      <c r="CR62">
+        <v>4</v>
+      </c>
     </row>
-    <row r="63" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -12439,8 +12838,14 @@
       <c r="CO63">
         <v>9</v>
       </c>
+      <c r="CQ63">
+        <v>0</v>
+      </c>
+      <c r="CR63">
+        <v>9</v>
+      </c>
     </row>
-    <row r="64" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -12637,8 +13042,17 @@
       <c r="CP64">
         <v>2</v>
       </c>
+      <c r="CQ64">
+        <v>3</v>
+      </c>
+      <c r="CR64">
+        <v>6</v>
+      </c>
+      <c r="CS64">
+        <v>1</v>
+      </c>
     </row>
-    <row r="65" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -12832,8 +13246,14 @@
       <c r="CO65">
         <v>6</v>
       </c>
+      <c r="CQ65">
+        <v>0</v>
+      </c>
+      <c r="CR65">
+        <v>6</v>
+      </c>
     </row>
-    <row r="66" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -12967,8 +13387,14 @@
       <c r="CP66">
         <v>1</v>
       </c>
+      <c r="CQ66">
+        <v>4</v>
+      </c>
+      <c r="CR66">
+        <v>1</v>
+      </c>
     </row>
-    <row r="67" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -13192,8 +13618,14 @@
       <c r="CO67">
         <v>10</v>
       </c>
+      <c r="CQ67">
+        <v>0</v>
+      </c>
+      <c r="CR67">
+        <v>10</v>
+      </c>
     </row>
-    <row r="68" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -13312,8 +13744,17 @@
       <c r="CP68">
         <v>3</v>
       </c>
+      <c r="CQ68">
+        <v>6</v>
+      </c>
+      <c r="CR68">
+        <v>4</v>
+      </c>
+      <c r="CS68">
+        <v>1</v>
+      </c>
     </row>
-    <row r="69" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -13447,8 +13888,14 @@
       <c r="CO69">
         <v>9</v>
       </c>
+      <c r="CQ69">
+        <v>0</v>
+      </c>
+      <c r="CR69">
+        <v>9</v>
+      </c>
     </row>
-    <row r="70" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -13585,8 +14032,14 @@
       <c r="CO70">
         <v>6</v>
       </c>
+      <c r="CQ70">
+        <v>2</v>
+      </c>
+      <c r="CR70">
+        <v>6</v>
+      </c>
     </row>
-    <row r="71" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -13801,8 +14254,14 @@
       <c r="CO71">
         <v>10</v>
       </c>
+      <c r="CQ71">
+        <v>0</v>
+      </c>
+      <c r="CR71">
+        <v>10</v>
+      </c>
     </row>
-    <row r="72" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -14005,8 +14464,14 @@
       <c r="CP72">
         <v>4</v>
       </c>
+      <c r="CQ72">
+        <v>1</v>
+      </c>
+      <c r="CR72">
+        <v>6</v>
+      </c>
     </row>
-    <row r="73" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -14137,8 +14602,14 @@
       <c r="CO73">
         <v>9</v>
       </c>
+      <c r="CQ73">
+        <v>0</v>
+      </c>
+      <c r="CR73">
+        <v>10</v>
+      </c>
     </row>
-    <row r="74" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -14269,8 +14740,17 @@
       <c r="CP74">
         <v>2</v>
       </c>
+      <c r="CQ74">
+        <v>6</v>
+      </c>
+      <c r="CR74">
+        <v>2</v>
+      </c>
+      <c r="CS74">
+        <v>1</v>
+      </c>
     </row>
-    <row r="75" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -14470,8 +14950,14 @@
       <c r="CO75">
         <v>8</v>
       </c>
+      <c r="CQ75">
+        <v>1</v>
+      </c>
+      <c r="CR75">
+        <v>8</v>
+      </c>
     </row>
-    <row r="76" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -14695,8 +15181,14 @@
       <c r="CP76">
         <v>2</v>
       </c>
+      <c r="CQ76">
+        <v>2</v>
+      </c>
+      <c r="CR76">
+        <v>6</v>
+      </c>
     </row>
-    <row r="77" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -14881,8 +15373,14 @@
       <c r="CO77">
         <v>7</v>
       </c>
+      <c r="CQ77">
+        <v>0</v>
+      </c>
+      <c r="CR77">
+        <v>7</v>
+      </c>
     </row>
-    <row r="78" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -15016,8 +15514,17 @@
       <c r="CP78">
         <v>2</v>
       </c>
+      <c r="CQ78">
+        <v>4</v>
+      </c>
+      <c r="CR78">
+        <v>1</v>
+      </c>
+      <c r="CS78">
+        <v>2</v>
+      </c>
     </row>
-    <row r="79" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -15238,8 +15745,14 @@
       <c r="CP79">
         <v>1</v>
       </c>
+      <c r="CQ79">
+        <v>0</v>
+      </c>
+      <c r="CR79">
+        <v>9</v>
+      </c>
     </row>
-    <row r="80" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -15427,8 +15940,17 @@
       <c r="CP80">
         <v>4</v>
       </c>
+      <c r="CQ80">
+        <v>4</v>
+      </c>
+      <c r="CR80">
+        <v>5</v>
+      </c>
+      <c r="CS80">
+        <v>1</v>
+      </c>
     </row>
-    <row r="81" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -15625,8 +16147,14 @@
       <c r="CO81">
         <v>7</v>
       </c>
+      <c r="CQ81">
+        <v>0</v>
+      </c>
+      <c r="CR81">
+        <v>7</v>
+      </c>
     </row>
-    <row r="82" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -15862,8 +16390,14 @@
       <c r="CO82">
         <v>10</v>
       </c>
+      <c r="CQ82">
+        <v>0</v>
+      </c>
+      <c r="CR82">
+        <v>10</v>
+      </c>
     </row>
-    <row r="83" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -16081,8 +16615,14 @@
       <c r="CO83">
         <v>9</v>
       </c>
+      <c r="CQ83">
+        <v>0</v>
+      </c>
+      <c r="CR83">
+        <v>9</v>
+      </c>
     </row>
-    <row r="84" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -16297,8 +16837,14 @@
       <c r="CP84">
         <v>2</v>
       </c>
+      <c r="CQ84">
+        <v>2</v>
+      </c>
+      <c r="CR84">
+        <v>7</v>
+      </c>
     </row>
-    <row r="85" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -16516,8 +17062,14 @@
       <c r="CO85">
         <v>6</v>
       </c>
+      <c r="CQ85">
+        <v>0</v>
+      </c>
+      <c r="CR85">
+        <v>6</v>
+      </c>
     </row>
-    <row r="86" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -16717,8 +17269,14 @@
       <c r="CP86">
         <v>1</v>
       </c>
+      <c r="CQ86">
+        <v>1</v>
+      </c>
+      <c r="CR86">
+        <v>8</v>
+      </c>
     </row>
-    <row r="87" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -16942,8 +17500,14 @@
       <c r="CP87">
         <v>1</v>
       </c>
+      <c r="CQ87">
+        <v>0</v>
+      </c>
+      <c r="CR87">
+        <v>7</v>
+      </c>
     </row>
-    <row r="88" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -17149,8 +17713,14 @@
       <c r="CP88">
         <v>1</v>
       </c>
+      <c r="CQ88">
+        <v>2</v>
+      </c>
+      <c r="CR88">
+        <v>7</v>
+      </c>
     </row>
-    <row r="89" spans="2:94" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:97" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>3</v>
       </c>
@@ -17332,8 +17902,14 @@
       <c r="CO89" s="3">
         <v>5</v>
       </c>
+      <c r="CQ89" s="3">
+        <v>0</v>
+      </c>
+      <c r="CR89" s="3">
+        <v>5</v>
+      </c>
     </row>
-    <row r="90" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -17467,8 +18043,17 @@
       <c r="CP90">
         <v>3</v>
       </c>
+      <c r="CQ90">
+        <v>0</v>
+      </c>
+      <c r="CR90">
+        <v>5</v>
+      </c>
+      <c r="CS90">
+        <v>2</v>
+      </c>
     </row>
-    <row r="91" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -17698,8 +18283,14 @@
       <c r="CP91">
         <v>1</v>
       </c>
+      <c r="CQ91">
+        <v>0</v>
+      </c>
+      <c r="CR91">
+        <v>6</v>
+      </c>
     </row>
-    <row r="92" spans="2:94" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:97" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>1</v>
       </c>
@@ -17908,8 +18499,14 @@
       <c r="CP92" s="3">
         <v>2</v>
       </c>
+      <c r="CQ92" s="3">
+        <v>1</v>
+      </c>
+      <c r="CR92" s="3">
+        <v>7</v>
+      </c>
     </row>
-    <row r="93" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -18076,8 +18673,14 @@
       <c r="CO93">
         <v>9</v>
       </c>
+      <c r="CQ93">
+        <v>0</v>
+      </c>
+      <c r="CR93">
+        <v>9</v>
+      </c>
     </row>
-    <row r="94" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -18214,8 +18817,14 @@
       <c r="CO94">
         <v>7</v>
       </c>
+      <c r="CQ94">
+        <v>0</v>
+      </c>
+      <c r="CR94">
+        <v>7</v>
+      </c>
     </row>
-    <row r="95" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -18391,8 +19000,14 @@
       <c r="CO95">
         <v>8</v>
       </c>
+      <c r="CQ95">
+        <v>0</v>
+      </c>
+      <c r="CR95">
+        <v>8</v>
+      </c>
     </row>
-    <row r="96" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -18592,8 +19207,14 @@
       <c r="CO96">
         <v>5</v>
       </c>
+      <c r="CQ96">
+        <v>5</v>
+      </c>
+      <c r="CR96">
+        <v>5</v>
+      </c>
     </row>
-    <row r="97" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -18733,8 +19354,14 @@
       <c r="CO97">
         <v>8</v>
       </c>
+      <c r="CQ97">
+        <v>0</v>
+      </c>
+      <c r="CR97">
+        <v>8</v>
+      </c>
     </row>
-    <row r="98" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -18931,8 +19558,14 @@
       <c r="CO98">
         <v>6</v>
       </c>
+      <c r="CQ98">
+        <v>0</v>
+      </c>
+      <c r="CR98">
+        <v>7</v>
+      </c>
     </row>
-    <row r="99" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -19081,8 +19714,14 @@
       <c r="CO99">
         <v>1</v>
       </c>
+      <c r="CQ99">
+        <v>2</v>
+      </c>
+      <c r="CR99">
+        <v>1</v>
+      </c>
     </row>
-    <row r="100" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -19207,8 +19846,11 @@
       <c r="CN100">
         <v>8</v>
       </c>
+      <c r="CQ100">
+        <v>8</v>
+      </c>
     </row>
-    <row r="101" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -19390,8 +20032,14 @@
       <c r="CO101">
         <v>4</v>
       </c>
+      <c r="CQ101">
+        <v>1</v>
+      </c>
+      <c r="CR101">
+        <v>4</v>
+      </c>
     </row>
-    <row r="102" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -19528,8 +20176,14 @@
       <c r="CO102">
         <v>4</v>
       </c>
+      <c r="CQ102">
+        <v>1</v>
+      </c>
+      <c r="CR102">
+        <v>6</v>
+      </c>
     </row>
-    <row r="103" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -19732,8 +20386,14 @@
       <c r="CO103">
         <v>6</v>
       </c>
+      <c r="CQ103">
+        <v>0</v>
+      </c>
+      <c r="CR103">
+        <v>6</v>
+      </c>
     </row>
-    <row r="104" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -19933,8 +20593,14 @@
       <c r="CO104">
         <v>8</v>
       </c>
+      <c r="CQ104">
+        <v>2</v>
+      </c>
+      <c r="CR104">
+        <v>8</v>
+      </c>
     </row>
-    <row r="105" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -20128,8 +20794,14 @@
       <c r="CO105">
         <v>6</v>
       </c>
+      <c r="CQ105">
+        <v>0</v>
+      </c>
+      <c r="CR105">
+        <v>6</v>
+      </c>
     </row>
-    <row r="106" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -20314,8 +20986,14 @@
       <c r="CO106">
         <v>8</v>
       </c>
+      <c r="CQ106">
+        <v>0</v>
+      </c>
+      <c r="CR106">
+        <v>8</v>
+      </c>
     </row>
-    <row r="107" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -20521,8 +21199,14 @@
       <c r="CO107">
         <v>5</v>
       </c>
+      <c r="CQ107">
+        <v>0</v>
+      </c>
+      <c r="CR107">
+        <v>5</v>
+      </c>
     </row>
-    <row r="108" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -20713,8 +21397,14 @@
       <c r="CO108">
         <v>10</v>
       </c>
+      <c r="CQ108">
+        <v>0</v>
+      </c>
+      <c r="CR108">
+        <v>10</v>
+      </c>
     </row>
-    <row r="109" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -20920,8 +21610,14 @@
       <c r="CO109">
         <v>9</v>
       </c>
+      <c r="CQ109">
+        <v>0</v>
+      </c>
+      <c r="CR109">
+        <v>9</v>
+      </c>
     </row>
-    <row r="110" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -21130,8 +21826,17 @@
       <c r="CO110">
         <v>3</v>
       </c>
+      <c r="CQ110">
+        <v>4</v>
+      </c>
+      <c r="CR110">
+        <v>3</v>
+      </c>
+      <c r="CS110">
+        <v>2</v>
+      </c>
     </row>
-    <row r="111" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -21328,8 +22033,14 @@
       <c r="CP111">
         <v>4</v>
       </c>
+      <c r="CQ111">
+        <v>1</v>
+      </c>
+      <c r="CR111">
+        <v>7</v>
+      </c>
     </row>
-    <row r="112" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -21532,8 +22243,14 @@
       <c r="CO112">
         <v>4</v>
       </c>
+      <c r="CQ112">
+        <v>3</v>
+      </c>
+      <c r="CR112">
+        <v>5</v>
+      </c>
     </row>
-    <row r="113" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -21742,8 +22459,14 @@
       <c r="CO113">
         <v>2</v>
       </c>
+      <c r="CQ113">
+        <v>4</v>
+      </c>
+      <c r="CR113">
+        <v>2</v>
+      </c>
     </row>
-    <row r="114" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -21877,8 +22600,14 @@
       <c r="CO114">
         <v>8</v>
       </c>
+      <c r="CQ114">
+        <v>0</v>
+      </c>
+      <c r="CR114">
+        <v>8</v>
+      </c>
     </row>
-    <row r="115" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -22090,8 +22819,14 @@
       <c r="CO115">
         <v>4</v>
       </c>
+      <c r="CQ115">
+        <v>0</v>
+      </c>
+      <c r="CR115">
+        <v>4</v>
+      </c>
     </row>
-    <row r="116" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -22288,8 +23023,14 @@
       <c r="CO116">
         <v>8</v>
       </c>
+      <c r="CQ116">
+        <v>0</v>
+      </c>
+      <c r="CR116">
+        <v>8</v>
+      </c>
     </row>
-    <row r="117" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -22492,8 +23233,14 @@
       <c r="CO117">
         <v>5</v>
       </c>
+      <c r="CQ117">
+        <v>0</v>
+      </c>
+      <c r="CR117">
+        <v>5</v>
+      </c>
     </row>
-    <row r="118" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -22637,8 +23384,14 @@
       <c r="CO118">
         <v>6</v>
       </c>
+      <c r="CQ118">
+        <v>0</v>
+      </c>
+      <c r="CR118">
+        <v>6</v>
+      </c>
     </row>
-    <row r="119" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -22784,8 +23537,14 @@
       <c r="CO119">
         <v>7</v>
       </c>
+      <c r="CQ119">
+        <v>0</v>
+      </c>
+      <c r="CR119">
+        <v>7</v>
+      </c>
     </row>
-    <row r="120" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -22922,8 +23681,14 @@
       <c r="CO120">
         <v>10</v>
       </c>
+      <c r="CQ120">
+        <v>0</v>
+      </c>
+      <c r="CR120">
+        <v>10</v>
+      </c>
     </row>
-    <row r="121" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -23060,8 +23825,14 @@
       <c r="CO121">
         <v>8</v>
       </c>
+      <c r="CQ121">
+        <v>0</v>
+      </c>
+      <c r="CR121">
+        <v>8</v>
+      </c>
     </row>
-    <row r="122" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -23201,8 +23972,14 @@
       <c r="CO122">
         <v>6</v>
       </c>
+      <c r="CQ122">
+        <v>0</v>
+      </c>
+      <c r="CR122">
+        <v>6</v>
+      </c>
     </row>
-    <row r="123" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -23393,8 +24170,14 @@
       <c r="CO123">
         <v>3</v>
       </c>
+      <c r="CQ123">
+        <v>3</v>
+      </c>
+      <c r="CR123">
+        <v>3</v>
+      </c>
     </row>
-    <row r="124" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -23627,8 +24410,17 @@
       <c r="CP124">
         <v>1</v>
       </c>
+      <c r="CQ124">
+        <v>2</v>
+      </c>
+      <c r="CR124">
+        <v>6</v>
+      </c>
+      <c r="CS124">
+        <v>1</v>
+      </c>
     </row>
-    <row r="125" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -23846,8 +24638,14 @@
       <c r="CO125">
         <v>6</v>
       </c>
+      <c r="CQ125">
+        <v>0</v>
+      </c>
+      <c r="CR125">
+        <v>6</v>
+      </c>
     </row>
-    <row r="126" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -24047,8 +24845,14 @@
       <c r="CO126">
         <v>6</v>
       </c>
+      <c r="CQ126">
+        <v>0</v>
+      </c>
+      <c r="CR126">
+        <v>6</v>
+      </c>
     </row>
-    <row r="127" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -24242,8 +25046,14 @@
       <c r="CO127">
         <v>3</v>
       </c>
+      <c r="CQ127">
+        <v>0</v>
+      </c>
+      <c r="CR127">
+        <v>3</v>
+      </c>
     </row>
-    <row r="128" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -24368,8 +25178,14 @@
       <c r="CO128">
         <v>7</v>
       </c>
+      <c r="CQ128">
+        <v>0</v>
+      </c>
+      <c r="CR128">
+        <v>7</v>
+      </c>
     </row>
-    <row r="129" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -24578,8 +25394,14 @@
       <c r="CO129">
         <v>6</v>
       </c>
+      <c r="CQ129">
+        <v>0</v>
+      </c>
+      <c r="CR129">
+        <v>6</v>
+      </c>
     </row>
-    <row r="130" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -24725,8 +25547,14 @@
       <c r="CO130">
         <v>10</v>
       </c>
+      <c r="CQ130">
+        <v>0</v>
+      </c>
+      <c r="CR130">
+        <v>10</v>
+      </c>
     </row>
-    <row r="131" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -24938,8 +25766,14 @@
       <c r="CO131">
         <v>10</v>
       </c>
+      <c r="CQ131">
+        <v>0</v>
+      </c>
+      <c r="CR131">
+        <v>10</v>
+      </c>
     </row>
-    <row r="132" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -25073,8 +25907,14 @@
       <c r="CO132">
         <v>6</v>
       </c>
+      <c r="CQ132">
+        <v>0</v>
+      </c>
+      <c r="CR132">
+        <v>6</v>
+      </c>
     </row>
-    <row r="133" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -25241,8 +26081,14 @@
       <c r="CO133">
         <v>7</v>
       </c>
+      <c r="CQ133">
+        <v>0</v>
+      </c>
+      <c r="CR133">
+        <v>7</v>
+      </c>
     </row>
-    <row r="134" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -25409,8 +26255,14 @@
       <c r="CO134">
         <v>10</v>
       </c>
+      <c r="CQ134">
+        <v>0</v>
+      </c>
+      <c r="CR134">
+        <v>10</v>
+      </c>
     </row>
-    <row r="135" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -25598,8 +26450,14 @@
       <c r="CO135">
         <v>7</v>
       </c>
+      <c r="CQ135">
+        <v>1</v>
+      </c>
+      <c r="CR135">
+        <v>7</v>
+      </c>
     </row>
-    <row r="136" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -25781,8 +26639,14 @@
       <c r="CO136">
         <v>7</v>
       </c>
+      <c r="CQ136">
+        <v>0</v>
+      </c>
+      <c r="CR136">
+        <v>7</v>
+      </c>
     </row>
-    <row r="137" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -25970,8 +26834,17 @@
       <c r="CP137">
         <v>1</v>
       </c>
+      <c r="CQ137">
+        <v>1</v>
+      </c>
+      <c r="CR137">
+        <v>3</v>
+      </c>
+      <c r="CS137">
+        <v>1</v>
+      </c>
     </row>
-    <row r="138" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -26174,8 +27047,14 @@
       <c r="CO138">
         <v>7</v>
       </c>
+      <c r="CQ138">
+        <v>0</v>
+      </c>
+      <c r="CR138">
+        <v>7</v>
+      </c>
     </row>
-    <row r="139" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -26360,8 +27239,14 @@
       <c r="CO139">
         <v>5</v>
       </c>
+      <c r="CQ139">
+        <v>0</v>
+      </c>
+      <c r="CR139">
+        <v>5</v>
+      </c>
     </row>
-    <row r="140" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -26501,8 +27386,14 @@
       <c r="CO140">
         <v>9</v>
       </c>
+      <c r="CQ140">
+        <v>0</v>
+      </c>
+      <c r="CR140">
+        <v>9</v>
+      </c>
     </row>
-    <row r="141" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -26723,8 +27614,14 @@
       <c r="CO141">
         <v>8</v>
       </c>
+      <c r="CQ141">
+        <v>0</v>
+      </c>
+      <c r="CR141">
+        <v>8</v>
+      </c>
     </row>
-    <row r="142" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -26945,8 +27842,14 @@
       <c r="CO142">
         <v>8</v>
       </c>
+      <c r="CQ142">
+        <v>0</v>
+      </c>
+      <c r="CR142">
+        <v>8</v>
+      </c>
     </row>
-    <row r="143" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -27125,8 +28028,14 @@
       <c r="CO143">
         <v>11</v>
       </c>
+      <c r="CQ143">
+        <v>0</v>
+      </c>
+      <c r="CR143">
+        <v>11</v>
+      </c>
     </row>
-    <row r="144" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -27257,8 +28166,14 @@
       <c r="CO144">
         <v>7</v>
       </c>
+      <c r="CQ144">
+        <v>0</v>
+      </c>
+      <c r="CR144">
+        <v>7</v>
+      </c>
     </row>
-    <row r="145" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -27398,8 +28313,14 @@
       <c r="CO145">
         <v>5</v>
       </c>
+      <c r="CQ145">
+        <v>0</v>
+      </c>
+      <c r="CR145">
+        <v>5</v>
+      </c>
     </row>
-    <row r="146" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -27632,8 +28553,14 @@
       <c r="CP146">
         <v>1</v>
       </c>
+      <c r="CQ146">
+        <v>0</v>
+      </c>
+      <c r="CR146">
+        <v>10</v>
+      </c>
     </row>
-    <row r="147" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -27854,8 +28781,14 @@
       <c r="CO147">
         <v>1</v>
       </c>
+      <c r="CQ147">
+        <v>2</v>
+      </c>
+      <c r="CR147">
+        <v>1</v>
+      </c>
     </row>
-    <row r="148" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -27977,8 +28910,11 @@
       <c r="CN148">
         <v>9</v>
       </c>
+      <c r="CQ148">
+        <v>9</v>
+      </c>
     </row>
-    <row r="149" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -28205,8 +29141,17 @@
       <c r="CP149">
         <v>1</v>
       </c>
+      <c r="CQ149">
+        <v>1</v>
+      </c>
+      <c r="CR149">
+        <v>3</v>
+      </c>
+      <c r="CS149">
+        <v>1</v>
+      </c>
     </row>
-    <row r="150" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -28421,8 +29366,14 @@
       <c r="CO150">
         <v>9</v>
       </c>
+      <c r="CQ150">
+        <v>0</v>
+      </c>
+      <c r="CR150">
+        <v>9</v>
+      </c>
     </row>
-    <row r="151" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -28613,8 +29564,14 @@
       <c r="CO151">
         <v>10</v>
       </c>
+      <c r="CQ151">
+        <v>0</v>
+      </c>
+      <c r="CR151">
+        <v>10</v>
+      </c>
     </row>
-    <row r="152" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -28742,8 +29699,14 @@
       <c r="CO152">
         <v>9</v>
       </c>
+      <c r="CQ152">
+        <v>0</v>
+      </c>
+      <c r="CR152">
+        <v>9</v>
+      </c>
     </row>
-    <row r="153" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -28925,8 +29888,14 @@
       <c r="CO153">
         <v>7</v>
       </c>
+      <c r="CQ153">
+        <v>0</v>
+      </c>
+      <c r="CR153">
+        <v>7</v>
+      </c>
     </row>
-    <row r="154" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -29174,8 +30143,14 @@
       <c r="CO154">
         <v>8</v>
       </c>
+      <c r="CQ154">
+        <v>0</v>
+      </c>
+      <c r="CR154">
+        <v>8</v>
+      </c>
     </row>
-    <row r="155" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -29372,8 +30347,14 @@
       <c r="CO155">
         <v>9</v>
       </c>
+      <c r="CQ155">
+        <v>0</v>
+      </c>
+      <c r="CR155">
+        <v>9</v>
+      </c>
     </row>
-    <row r="156" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="156" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -29507,8 +30488,14 @@
       <c r="CP156">
         <v>1</v>
       </c>
+      <c r="CQ156">
+        <v>0</v>
+      </c>
+      <c r="CR156">
+        <v>6</v>
+      </c>
     </row>
-    <row r="157" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="157" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -29642,8 +30629,14 @@
       <c r="CO157">
         <v>6</v>
       </c>
+      <c r="CQ157">
+        <v>0</v>
+      </c>
+      <c r="CR157">
+        <v>6</v>
+      </c>
     </row>
-    <row r="158" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="158" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -29810,8 +30803,17 @@
       <c r="CP158">
         <v>2</v>
       </c>
+      <c r="CQ158">
+        <v>4</v>
+      </c>
+      <c r="CR158">
+        <v>2</v>
+      </c>
+      <c r="CS158">
+        <v>2</v>
+      </c>
     </row>
-    <row r="159" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -30023,8 +31025,14 @@
       <c r="CO159">
         <v>5</v>
       </c>
+      <c r="CQ159">
+        <v>0</v>
+      </c>
+      <c r="CR159">
+        <v>5</v>
+      </c>
     </row>
-    <row r="160" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -30149,8 +31157,11 @@
       <c r="CP160">
         <v>1</v>
       </c>
+      <c r="CQ160">
+        <v>9</v>
+      </c>
     </row>
-    <row r="161" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -30380,8 +31391,14 @@
       <c r="CO161">
         <v>6</v>
       </c>
+      <c r="CQ161">
+        <v>1</v>
+      </c>
+      <c r="CR161">
+        <v>6</v>
+      </c>
     </row>
-    <row r="162" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -30512,8 +31529,14 @@
       <c r="CP162">
         <v>3</v>
       </c>
+      <c r="CQ162">
+        <v>0</v>
+      </c>
+      <c r="CR162">
+        <v>8</v>
+      </c>
     </row>
-    <row r="163" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="163" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -30704,8 +31727,14 @@
       <c r="CO163">
         <v>8</v>
       </c>
+      <c r="CQ163">
+        <v>0</v>
+      </c>
+      <c r="CR163">
+        <v>8</v>
+      </c>
     </row>
-    <row r="164" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="164" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -30839,8 +31868,14 @@
       <c r="CO164">
         <v>8</v>
       </c>
+      <c r="CQ164">
+        <v>1</v>
+      </c>
+      <c r="CR164">
+        <v>8</v>
+      </c>
     </row>
-    <row r="165" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -31031,8 +32066,14 @@
       <c r="CO165">
         <v>6</v>
       </c>
+      <c r="CQ165">
+        <v>0</v>
+      </c>
+      <c r="CR165">
+        <v>6</v>
+      </c>
     </row>
-    <row r="166" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="166" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -31208,8 +32249,14 @@
       <c r="CO166">
         <v>6</v>
       </c>
+      <c r="CQ166">
+        <v>0</v>
+      </c>
+      <c r="CR166">
+        <v>6</v>
+      </c>
     </row>
-    <row r="167" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -31388,8 +32435,14 @@
       <c r="CO167">
         <v>8</v>
       </c>
+      <c r="CQ167">
+        <v>0</v>
+      </c>
+      <c r="CR167">
+        <v>8</v>
+      </c>
     </row>
-    <row r="168" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -31601,8 +32654,14 @@
       <c r="CO168">
         <v>11</v>
       </c>
+      <c r="CQ168">
+        <v>0</v>
+      </c>
+      <c r="CR168">
+        <v>11</v>
+      </c>
     </row>
-    <row r="169" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -31736,8 +32795,14 @@
       <c r="CO169">
         <v>6</v>
       </c>
+      <c r="CQ169">
+        <v>0</v>
+      </c>
+      <c r="CR169">
+        <v>6</v>
+      </c>
     </row>
-    <row r="170" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -31892,8 +32957,17 @@
       <c r="CP170">
         <v>4</v>
       </c>
+      <c r="CQ170">
+        <v>2</v>
+      </c>
+      <c r="CR170">
+        <v>4</v>
+      </c>
+      <c r="CS170">
+        <v>2</v>
+      </c>
     </row>
-    <row r="171" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="171" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -32114,8 +33188,14 @@
       <c r="CO171">
         <v>8</v>
       </c>
+      <c r="CQ171">
+        <v>0</v>
+      </c>
+      <c r="CR171">
+        <v>10</v>
+      </c>
     </row>
-    <row r="172" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -32252,8 +33332,17 @@
       <c r="CO172">
         <v>4</v>
       </c>
+      <c r="CQ172">
+        <v>3</v>
+      </c>
+      <c r="CR172">
+        <v>4</v>
+      </c>
+      <c r="CS172">
+        <v>1</v>
+      </c>
     </row>
-    <row r="173" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -32408,8 +33497,14 @@
       <c r="CO173">
         <v>2</v>
       </c>
+      <c r="CQ173">
+        <v>5</v>
+      </c>
+      <c r="CR173">
+        <v>3</v>
+      </c>
     </row>
-    <row r="174" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -32549,8 +33644,14 @@
       <c r="CP174">
         <v>2</v>
       </c>
+      <c r="CQ174">
+        <v>0</v>
+      </c>
+      <c r="CR174">
+        <v>9</v>
+      </c>
     </row>
-    <row r="175" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -32747,8 +33848,14 @@
       <c r="CO175">
         <v>9</v>
       </c>
+      <c r="CQ175">
+        <v>0</v>
+      </c>
+      <c r="CR175">
+        <v>9</v>
+      </c>
     </row>
-    <row r="176" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="176" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -32879,8 +33986,14 @@
       <c r="CO176">
         <v>8</v>
       </c>
+      <c r="CQ176">
+        <v>0</v>
+      </c>
+      <c r="CR176">
+        <v>8</v>
+      </c>
     </row>
-    <row r="177" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -33020,8 +34133,14 @@
       <c r="CO177">
         <v>5</v>
       </c>
+      <c r="CQ177">
+        <v>0</v>
+      </c>
+      <c r="CR177">
+        <v>5</v>
+      </c>
     </row>
-    <row r="178" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -33167,8 +34286,14 @@
       <c r="CO178">
         <v>8</v>
       </c>
+      <c r="CQ178">
+        <v>0</v>
+      </c>
+      <c r="CR178">
+        <v>8</v>
+      </c>
     </row>
-    <row r="179" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -33365,8 +34490,14 @@
       <c r="CO179">
         <v>10</v>
       </c>
+      <c r="CQ179">
+        <v>0</v>
+      </c>
+      <c r="CR179">
+        <v>10</v>
+      </c>
     </row>
-    <row r="180" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -33560,8 +34691,14 @@
       <c r="CO180">
         <v>9</v>
       </c>
+      <c r="CQ180">
+        <v>0</v>
+      </c>
+      <c r="CR180">
+        <v>9</v>
+      </c>
     </row>
-    <row r="181" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -33755,8 +34892,14 @@
       <c r="CO181">
         <v>9</v>
       </c>
+      <c r="CQ181">
+        <v>0</v>
+      </c>
+      <c r="CR181">
+        <v>9</v>
+      </c>
     </row>
-    <row r="182" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -33893,8 +35036,14 @@
       <c r="CO182">
         <v>5</v>
       </c>
+      <c r="CQ182">
+        <v>1</v>
+      </c>
+      <c r="CR182">
+        <v>5</v>
+      </c>
     </row>
-    <row r="183" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -34120,8 +35269,14 @@
       <c r="CO183">
         <v>5</v>
       </c>
+      <c r="CQ183">
+        <v>0</v>
+      </c>
+      <c r="CR183">
+        <v>5</v>
+      </c>
     </row>
-    <row r="184" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -34266,8 +35421,14 @@
       <c r="CO184">
         <v>6</v>
       </c>
+      <c r="CQ184">
+        <v>0</v>
+      </c>
+      <c r="CR184">
+        <v>6</v>
+      </c>
     </row>
-    <row r="185" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -34463,8 +35624,14 @@
       <c r="CO185">
         <v>7</v>
       </c>
+      <c r="CQ185">
+        <v>0</v>
+      </c>
+      <c r="CR185">
+        <v>7</v>
+      </c>
     </row>
-    <row r="186" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -34648,8 +35815,14 @@
       <c r="CO186">
         <v>1</v>
       </c>
+      <c r="CQ186">
+        <v>6</v>
+      </c>
+      <c r="CR186">
+        <v>1</v>
+      </c>
     </row>
-    <row r="187" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -34800,8 +35973,17 @@
       <c r="CP187">
         <v>1</v>
       </c>
+      <c r="CQ187">
+        <v>1</v>
+      </c>
+      <c r="CR187">
+        <v>3</v>
+      </c>
+      <c r="CS187">
+        <v>4</v>
+      </c>
     </row>
-    <row r="188" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B188" t="s">
         <v>4</v>
       </c>
@@ -35003,8 +36185,17 @@
       <c r="CP188">
         <v>2</v>
       </c>
+      <c r="CQ188">
+        <v>1</v>
+      </c>
+      <c r="CR188">
+        <v>8</v>
+      </c>
+      <c r="CS188">
+        <v>1</v>
+      </c>
     </row>
-    <row r="189" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -35206,8 +36397,14 @@
       <c r="CO189">
         <v>2</v>
       </c>
+      <c r="CQ189">
+        <v>0</v>
+      </c>
+      <c r="CR189">
+        <v>2</v>
+      </c>
     </row>
-    <row r="190" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="190" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -35412,8 +36609,14 @@
       <c r="CO190">
         <v>5</v>
       </c>
+      <c r="CQ190">
+        <v>0</v>
+      </c>
+      <c r="CR190">
+        <v>5</v>
+      </c>
     </row>
-    <row r="191" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="191" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -35621,8 +36824,14 @@
       <c r="CO191">
         <v>5</v>
       </c>
+      <c r="CQ191">
+        <v>0</v>
+      </c>
+      <c r="CR191">
+        <v>5</v>
+      </c>
     </row>
-    <row r="192" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="192" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -35809,8 +37018,14 @@
       <c r="CO192">
         <v>3</v>
       </c>
+      <c r="CQ192">
+        <v>0</v>
+      </c>
+      <c r="CR192">
+        <v>3</v>
+      </c>
     </row>
-    <row r="193" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="193" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -36021,8 +37236,14 @@
       <c r="CO193">
         <v>4</v>
       </c>
+      <c r="CQ193">
+        <v>1</v>
+      </c>
+      <c r="CR193">
+        <v>6</v>
+      </c>
     </row>
-    <row r="194" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="194" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B194" t="s">
         <v>4</v>
       </c>
@@ -36209,8 +37430,14 @@
       <c r="CP194">
         <v>1</v>
       </c>
+      <c r="CQ194">
+        <v>0</v>
+      </c>
+      <c r="CR194">
+        <v>7</v>
+      </c>
     </row>
-    <row r="195" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="195" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -36412,8 +37639,14 @@
       <c r="CO195">
         <v>2</v>
       </c>
+      <c r="CQ195">
+        <v>0</v>
+      </c>
+      <c r="CR195">
+        <v>2</v>
+      </c>
     </row>
-    <row r="196" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="196" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -36648,8 +37881,14 @@
       <c r="CO196">
         <v>9</v>
       </c>
+      <c r="CQ196">
+        <v>0</v>
+      </c>
+      <c r="CR196">
+        <v>9</v>
+      </c>
     </row>
-    <row r="197" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="197" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -36839,8 +38078,14 @@
       <c r="CO197">
         <v>4</v>
       </c>
+      <c r="CQ197">
+        <v>0</v>
+      </c>
+      <c r="CR197">
+        <v>4</v>
+      </c>
     </row>
-    <row r="198" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="198" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -37012,8 +38257,14 @@
       <c r="CO198">
         <v>5</v>
       </c>
+      <c r="CQ198">
+        <v>0</v>
+      </c>
+      <c r="CR198">
+        <v>5</v>
+      </c>
     </row>
-    <row r="199" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="199" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -37197,8 +38448,14 @@
       <c r="CP199">
         <v>5</v>
       </c>
+      <c r="CQ199">
+        <v>0</v>
+      </c>
+      <c r="CR199">
+        <v>6</v>
+      </c>
     </row>
-    <row r="200" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="200" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
         <v>4</v>
       </c>
@@ -37379,8 +38636,14 @@
       <c r="CP200">
         <v>1</v>
       </c>
+      <c r="CQ200">
+        <v>0</v>
+      </c>
+      <c r="CR200">
+        <v>7</v>
+      </c>
     </row>
-    <row r="201" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="201" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -37597,8 +38860,14 @@
       <c r="CO201">
         <v>6</v>
       </c>
+      <c r="CQ201">
+        <v>0</v>
+      </c>
+      <c r="CR201">
+        <v>6</v>
+      </c>
     </row>
-    <row r="202" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="202" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -37806,8 +39075,14 @@
       <c r="CO202">
         <v>1</v>
       </c>
+      <c r="CQ202">
+        <v>0</v>
+      </c>
+      <c r="CR202">
+        <v>1</v>
+      </c>
     </row>
-    <row r="203" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="203" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -38009,8 +39284,14 @@
       <c r="CO203">
         <v>3</v>
       </c>
+      <c r="CQ203">
+        <v>0</v>
+      </c>
+      <c r="CR203">
+        <v>3</v>
+      </c>
     </row>
-    <row r="204" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="204" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -38128,8 +39409,11 @@
       <c r="CN204">
         <v>6</v>
       </c>
+      <c r="CQ204">
+        <v>6</v>
+      </c>
     </row>
-    <row r="205" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="205" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -38349,8 +39633,17 @@
       <c r="CO205">
         <v>2</v>
       </c>
+      <c r="CQ205">
+        <v>6</v>
+      </c>
+      <c r="CR205">
+        <v>3</v>
+      </c>
+      <c r="CS205">
+        <v>1</v>
+      </c>
     </row>
-    <row r="206" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="206" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B206" t="s">
         <v>4</v>
       </c>
@@ -38474,8 +39767,14 @@
       <c r="CP206">
         <v>5</v>
       </c>
+      <c r="CQ206">
+        <v>1</v>
+      </c>
+      <c r="CR206">
+        <v>5</v>
+      </c>
     </row>
-    <row r="207" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="207" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -38650,8 +39949,14 @@
       <c r="CO207">
         <v>4</v>
       </c>
+      <c r="CQ207">
+        <v>0</v>
+      </c>
+      <c r="CR207">
+        <v>4</v>
+      </c>
     </row>
-    <row r="208" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="208" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -38853,8 +40158,14 @@
       <c r="CO208">
         <v>3</v>
       </c>
+      <c r="CQ208">
+        <v>0</v>
+      </c>
+      <c r="CR208">
+        <v>3</v>
+      </c>
     </row>
-    <row r="209" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="209" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B209" t="s">
         <v>3</v>
       </c>
@@ -39041,8 +40352,14 @@
       <c r="CO209">
         <v>5</v>
       </c>
+      <c r="CQ209">
+        <v>0</v>
+      </c>
+      <c r="CR209">
+        <v>5</v>
+      </c>
     </row>
-    <row r="210" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="210" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B210" t="s">
         <v>1</v>
       </c>
@@ -39250,8 +40567,14 @@
       <c r="CO210">
         <v>1</v>
       </c>
+      <c r="CQ210">
+        <v>4</v>
+      </c>
+      <c r="CR210">
+        <v>1</v>
+      </c>
     </row>
-    <row r="211" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="211" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
         <v>4</v>
       </c>
@@ -39435,8 +40758,17 @@
       <c r="CO211">
         <v>2</v>
       </c>
+      <c r="CQ211">
+        <v>1</v>
+      </c>
+      <c r="CR211">
+        <v>2</v>
+      </c>
+      <c r="CS211">
+        <v>2</v>
+      </c>
     </row>
-    <row r="212" spans="2:94" x14ac:dyDescent="0.3">
+    <row r="212" spans="2:97" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
         <v>4</v>
       </c>
@@ -39616,6 +40948,12 @@
       </c>
       <c r="CP212">
         <v>2</v>
+      </c>
+      <c r="CQ212">
+        <v>0</v>
+      </c>
+      <c r="CR212">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DOY 196 germinants data collection
</commit_message>
<xml_diff>
--- a/data/germination_data.xlsx
+++ b/data/germination_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temporal Ecology Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E758C45-0616-473D-BA12-4E9C32541A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2B1612-41B2-44F7-9947-19787E6B8ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="137">
   <si>
     <t>seed_species</t>
   </si>
@@ -474,6 +474,15 @@
   <si>
     <t>182_halfdead</t>
   </si>
+  <si>
+    <t>196_alive</t>
+  </si>
+  <si>
+    <t>196_dead</t>
+  </si>
+  <si>
+    <t>196_halfdead</t>
+  </si>
 </sst>
 </file>
 
@@ -577,9 +586,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CS213" totalsRowShown="0">
-  <autoFilter ref="B2:CS213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
-  <tableColumns count="96">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CV213" totalsRowShown="0">
+  <autoFilter ref="B2:CV213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
+  <tableColumns count="99">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
     <tableColumn id="3" xr3:uid="{B695F4B4-8561-9D48-9FF3-12A40CB2B7C7}" name="inoculated_%"/>
@@ -676,6 +685,9 @@
     <tableColumn id="94" xr3:uid="{9578CF96-5AE8-4645-B28F-F07D512CF35B}" name="182_alive"/>
     <tableColumn id="95" xr3:uid="{D47C9C3A-2489-4F83-963C-62C798893172}" name="182_dead"/>
     <tableColumn id="96" xr3:uid="{AC274215-49C4-4F5F-8E83-C3C811642720}" name="182_halfdead"/>
+    <tableColumn id="97" xr3:uid="{C0EE2BE8-9A00-4918-B7BC-CECE73317595}" name="196_alive"/>
+    <tableColumn id="98" xr3:uid="{757C4777-32C3-4210-A085-69139B19933D}" name="196_dead"/>
+    <tableColumn id="99" xr3:uid="{50FC3B28-770A-4906-B9B0-60C7F64F10FB}" name="196_halfdead"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -998,7 +1010,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:CS212"/>
+  <dimension ref="B2:CV212"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -1006,7 +1018,7 @@
     <col min="4" max="4" width="17.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -1295,8 +1307,17 @@
       <c r="CS2" t="s">
         <v>133</v>
       </c>
+      <c r="CT2" t="s">
+        <v>134</v>
+      </c>
+      <c r="CU2" t="s">
+        <v>135</v>
+      </c>
+      <c r="CV2" t="s">
+        <v>136</v>
+      </c>
     </row>
-    <row r="3" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1519,8 +1540,14 @@
       <c r="CS3">
         <v>1</v>
       </c>
+      <c r="CT3">
+        <v>0</v>
+      </c>
+      <c r="CU3">
+        <v>4</v>
+      </c>
     </row>
-    <row r="4" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1647,8 +1674,11 @@
       <c r="CQ4">
         <v>9</v>
       </c>
+      <c r="CT4">
+        <v>9</v>
+      </c>
     </row>
-    <row r="5" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1868,8 +1898,14 @@
       <c r="CR5">
         <v>7</v>
       </c>
+      <c r="CT5">
+        <v>0</v>
+      </c>
+      <c r="CU5">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1999,8 +2035,17 @@
       <c r="CR6">
         <v>7</v>
       </c>
+      <c r="CT6">
+        <v>0</v>
+      </c>
+      <c r="CU6">
+        <v>7</v>
+      </c>
+      <c r="CV6">
+        <v>2</v>
+      </c>
     </row>
-    <row r="7" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -2187,8 +2232,14 @@
       <c r="CR7">
         <v>6</v>
       </c>
+      <c r="CT7">
+        <v>0</v>
+      </c>
+      <c r="CU7">
+        <v>6</v>
+      </c>
     </row>
-    <row r="8" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -2399,8 +2450,14 @@
       <c r="CR8">
         <v>1</v>
       </c>
+      <c r="CT8">
+        <v>6</v>
+      </c>
+      <c r="CU8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2620,8 +2677,14 @@
       <c r="CR9">
         <v>7</v>
       </c>
+      <c r="CT9">
+        <v>0</v>
+      </c>
+      <c r="CU9">
+        <v>7</v>
+      </c>
     </row>
-    <row r="10" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -2775,8 +2838,17 @@
       <c r="CS10">
         <v>1</v>
       </c>
+      <c r="CT10">
+        <v>3</v>
+      </c>
+      <c r="CU10">
+        <v>3</v>
+      </c>
+      <c r="CV10">
+        <v>2</v>
+      </c>
     </row>
-    <row r="11" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -2993,8 +3065,14 @@
       <c r="CR11">
         <v>8</v>
       </c>
+      <c r="CT11">
+        <v>0</v>
+      </c>
+      <c r="CU11">
+        <v>8</v>
+      </c>
     </row>
-    <row r="12" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -3214,8 +3292,14 @@
       <c r="CR12">
         <v>5</v>
       </c>
+      <c r="CT12">
+        <v>5</v>
+      </c>
+      <c r="CU12">
+        <v>5</v>
+      </c>
     </row>
-    <row r="13" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -3426,8 +3510,14 @@
       <c r="CR13">
         <v>7</v>
       </c>
+      <c r="CT13">
+        <v>0</v>
+      </c>
+      <c r="CU13">
+        <v>7</v>
+      </c>
     </row>
-    <row r="14" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -3599,8 +3689,17 @@
       <c r="CS14">
         <v>3</v>
       </c>
+      <c r="CT14">
+        <v>4</v>
+      </c>
+      <c r="CU14">
+        <v>4</v>
+      </c>
+      <c r="CV14">
+        <v>1</v>
+      </c>
     </row>
-    <row r="15" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -3800,8 +3899,14 @@
       <c r="CR15">
         <v>8</v>
       </c>
+      <c r="CT15">
+        <v>0</v>
+      </c>
+      <c r="CU15">
+        <v>8</v>
+      </c>
     </row>
-    <row r="16" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -3989,8 +4094,17 @@
       <c r="CS16">
         <v>2</v>
       </c>
+      <c r="CT16">
+        <v>4</v>
+      </c>
+      <c r="CU16">
+        <v>4</v>
+      </c>
+      <c r="CV16">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -4193,8 +4307,14 @@
       <c r="CR17">
         <v>8</v>
       </c>
+      <c r="CT17">
+        <v>0</v>
+      </c>
+      <c r="CU17">
+        <v>8</v>
+      </c>
     </row>
-    <row r="18" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -4325,8 +4445,17 @@
       <c r="CR18">
         <v>8</v>
       </c>
+      <c r="CT18">
+        <v>1</v>
+      </c>
+      <c r="CU18">
+        <v>8</v>
+      </c>
+      <c r="CV18">
+        <v>1</v>
+      </c>
     </row>
-    <row r="19" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -4547,8 +4676,14 @@
       <c r="CR19">
         <v>7</v>
       </c>
+      <c r="CT19">
+        <v>0</v>
+      </c>
+      <c r="CU19">
+        <v>7</v>
+      </c>
     </row>
-    <row r="20" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -4733,8 +4868,17 @@
       <c r="CS20">
         <v>1</v>
       </c>
+      <c r="CT20">
+        <v>5</v>
+      </c>
+      <c r="CU20">
+        <v>5</v>
+      </c>
+      <c r="CV20">
+        <v>4</v>
+      </c>
     </row>
-    <row r="21" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -4921,8 +5065,14 @@
       <c r="CR21">
         <v>6</v>
       </c>
+      <c r="CT21">
+        <v>0</v>
+      </c>
+      <c r="CU21">
+        <v>6</v>
+      </c>
     </row>
-    <row r="22" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -5065,8 +5215,14 @@
       <c r="CS22">
         <v>2</v>
       </c>
+      <c r="CT22">
+        <v>2</v>
+      </c>
+      <c r="CU22">
+        <v>6</v>
+      </c>
     </row>
-    <row r="23" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -5281,8 +5437,14 @@
       <c r="CR23">
         <v>10</v>
       </c>
+      <c r="CT23">
+        <v>0</v>
+      </c>
+      <c r="CU23">
+        <v>10</v>
+      </c>
     </row>
-    <row r="24" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -5470,8 +5632,14 @@
       <c r="CR24">
         <v>4</v>
       </c>
+      <c r="CT24">
+        <v>8</v>
+      </c>
+      <c r="CU24">
+        <v>4</v>
+      </c>
     </row>
-    <row r="25" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -5608,8 +5776,14 @@
       <c r="CR25">
         <v>8</v>
       </c>
+      <c r="CT25">
+        <v>0</v>
+      </c>
+      <c r="CU25">
+        <v>8</v>
+      </c>
     </row>
-    <row r="26" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -5878,8 +6052,14 @@
       <c r="CS26">
         <v>1</v>
       </c>
+      <c r="CT26">
+        <v>0</v>
+      </c>
+      <c r="CU26">
+        <v>11</v>
+      </c>
     </row>
-    <row r="27" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -6073,8 +6253,14 @@
       <c r="CR27">
         <v>5</v>
       </c>
+      <c r="CT27">
+        <v>0</v>
+      </c>
+      <c r="CU27">
+        <v>6</v>
+      </c>
     </row>
-    <row r="28" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -6307,8 +6493,14 @@
       <c r="CR28">
         <v>10</v>
       </c>
+      <c r="CT28">
+        <v>0</v>
+      </c>
+      <c r="CU28">
+        <v>10</v>
+      </c>
     </row>
-    <row r="29" spans="2:97" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:100" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>3</v>
       </c>
@@ -6511,8 +6703,14 @@
       <c r="CR29" s="3">
         <v>4</v>
       </c>
+      <c r="CT29" s="3">
+        <v>0</v>
+      </c>
+      <c r="CU29" s="3">
+        <v>4</v>
+      </c>
     </row>
-    <row r="30" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -6649,8 +6847,14 @@
       <c r="CR30">
         <v>7</v>
       </c>
+      <c r="CT30">
+        <v>1</v>
+      </c>
+      <c r="CU30">
+        <v>7</v>
+      </c>
     </row>
-    <row r="31" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -6871,8 +7075,14 @@
       <c r="CR31">
         <v>5</v>
       </c>
+      <c r="CT31">
+        <v>0</v>
+      </c>
+      <c r="CU31">
+        <v>5</v>
+      </c>
     </row>
-    <row r="32" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -7057,8 +7267,14 @@
       <c r="CS32">
         <v>2</v>
       </c>
+      <c r="CT32">
+        <v>4</v>
+      </c>
+      <c r="CU32">
+        <v>6</v>
+      </c>
     </row>
-    <row r="33" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -7234,8 +7450,14 @@
       <c r="CR33">
         <v>9</v>
       </c>
+      <c r="CT33">
+        <v>0</v>
+      </c>
+      <c r="CU33">
+        <v>9</v>
+      </c>
     </row>
-    <row r="34" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -7402,8 +7624,14 @@
       <c r="CR34">
         <v>5</v>
       </c>
+      <c r="CT34">
+        <v>1</v>
+      </c>
+      <c r="CU34">
+        <v>5</v>
+      </c>
     </row>
-    <row r="35" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -7603,8 +7831,14 @@
       <c r="CR35">
         <v>8</v>
       </c>
+      <c r="CT35">
+        <v>0</v>
+      </c>
+      <c r="CU35">
+        <v>8</v>
+      </c>
     </row>
-    <row r="36" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -7801,8 +8035,17 @@
       <c r="CR36">
         <v>7</v>
       </c>
+      <c r="CT36">
+        <v>1</v>
+      </c>
+      <c r="CU36">
+        <v>7</v>
+      </c>
+      <c r="CV36">
+        <v>2</v>
+      </c>
     </row>
-    <row r="37" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -7945,8 +8188,14 @@
       <c r="CR37">
         <v>6</v>
       </c>
+      <c r="CT37">
+        <v>0</v>
+      </c>
+      <c r="CU37">
+        <v>6</v>
+      </c>
     </row>
-    <row r="38" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -8182,8 +8431,14 @@
       <c r="CR38">
         <v>4</v>
       </c>
+      <c r="CT38">
+        <v>2</v>
+      </c>
+      <c r="CU38">
+        <v>4</v>
+      </c>
     </row>
-    <row r="39" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -8401,8 +8656,17 @@
       <c r="CR39">
         <v>5</v>
       </c>
+      <c r="CT39">
+        <v>0</v>
+      </c>
+      <c r="CU39">
+        <v>5</v>
+      </c>
+      <c r="CV39">
+        <v>1</v>
+      </c>
     </row>
-    <row r="40" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -8638,8 +8902,14 @@
       <c r="CR40">
         <v>9</v>
       </c>
+      <c r="CT40">
+        <v>1</v>
+      </c>
+      <c r="CU40">
+        <v>9</v>
+      </c>
     </row>
-    <row r="41" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -8836,8 +9106,14 @@
       <c r="CR41">
         <v>6</v>
       </c>
+      <c r="CT41">
+        <v>0</v>
+      </c>
+      <c r="CU41">
+        <v>6</v>
+      </c>
     </row>
-    <row r="42" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -8983,8 +9259,14 @@
       <c r="CR42">
         <v>7</v>
       </c>
+      <c r="CT42">
+        <v>0</v>
+      </c>
+      <c r="CU42">
+        <v>7</v>
+      </c>
     </row>
-    <row r="43" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -9208,8 +9490,14 @@
       <c r="CR43">
         <v>9</v>
       </c>
+      <c r="CT43">
+        <v>0</v>
+      </c>
+      <c r="CU43">
+        <v>9</v>
+      </c>
     </row>
-    <row r="44" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -9343,8 +9631,14 @@
       <c r="CR44">
         <v>6</v>
       </c>
+      <c r="CT44">
+        <v>0</v>
+      </c>
+      <c r="CU44">
+        <v>6</v>
+      </c>
     </row>
-    <row r="45" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -9610,8 +9904,14 @@
       <c r="CR45">
         <v>9</v>
       </c>
+      <c r="CT45">
+        <v>0</v>
+      </c>
+      <c r="CU45">
+        <v>9</v>
+      </c>
     </row>
-    <row r="46" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -9751,8 +10051,14 @@
       <c r="CR46">
         <v>5</v>
       </c>
+      <c r="CT46">
+        <v>0</v>
+      </c>
+      <c r="CU46">
+        <v>6</v>
+      </c>
     </row>
-    <row r="47" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -9922,8 +10228,14 @@
       <c r="CR47">
         <v>9</v>
       </c>
+      <c r="CT47">
+        <v>0</v>
+      </c>
+      <c r="CU47">
+        <v>9</v>
+      </c>
     </row>
-    <row r="48" spans="2:96" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -10162,8 +10474,17 @@
       <c r="CR48">
         <v>10</v>
       </c>
+      <c r="CT48">
+        <v>0</v>
+      </c>
+      <c r="CU48">
+        <v>10</v>
+      </c>
+      <c r="CV48">
+        <v>1</v>
+      </c>
     </row>
-    <row r="49" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -10312,8 +10633,14 @@
       <c r="CR49">
         <v>7</v>
       </c>
+      <c r="CT49">
+        <v>0</v>
+      </c>
+      <c r="CU49">
+        <v>7</v>
+      </c>
     </row>
-    <row r="50" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -10558,8 +10885,14 @@
       <c r="CR50">
         <v>4</v>
       </c>
+      <c r="CT50">
+        <v>4</v>
+      </c>
+      <c r="CU50">
+        <v>4</v>
+      </c>
     </row>
-    <row r="51" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -10789,8 +11122,14 @@
       <c r="CR51">
         <v>5</v>
       </c>
+      <c r="CT51">
+        <v>1</v>
+      </c>
+      <c r="CU51">
+        <v>5</v>
+      </c>
     </row>
-    <row r="52" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -10921,8 +11260,14 @@
       <c r="CS52">
         <v>1</v>
       </c>
+      <c r="CT52">
+        <v>4</v>
+      </c>
+      <c r="CV52">
+        <v>2</v>
+      </c>
     </row>
-    <row r="53" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -11125,8 +11470,14 @@
       <c r="CR53">
         <v>4</v>
       </c>
+      <c r="CT53">
+        <v>0</v>
+      </c>
+      <c r="CU53">
+        <v>4</v>
+      </c>
     </row>
-    <row r="54" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -11260,8 +11611,17 @@
       <c r="CR54">
         <v>2</v>
       </c>
+      <c r="CT54">
+        <v>2</v>
+      </c>
+      <c r="CU54">
+        <v>2</v>
+      </c>
+      <c r="CV54">
+        <v>2</v>
+      </c>
     </row>
-    <row r="55" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -11467,8 +11827,14 @@
       <c r="CR55">
         <v>6</v>
       </c>
+      <c r="CT55">
+        <v>0</v>
+      </c>
+      <c r="CU55">
+        <v>6</v>
+      </c>
     </row>
-    <row r="56" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -11596,8 +11962,11 @@
       <c r="CQ56">
         <v>10</v>
       </c>
+      <c r="CT56">
+        <v>10</v>
+      </c>
     </row>
-    <row r="57" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -11752,8 +12121,17 @@
       <c r="CR57">
         <v>5</v>
       </c>
+      <c r="CT57">
+        <v>0</v>
+      </c>
+      <c r="CU57">
+        <v>6</v>
+      </c>
+      <c r="CV57">
+        <v>1</v>
+      </c>
     </row>
-    <row r="58" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -11896,8 +12274,17 @@
       <c r="CR58">
         <v>4</v>
       </c>
+      <c r="CT58">
+        <v>1</v>
+      </c>
+      <c r="CU58">
+        <v>4</v>
+      </c>
+      <c r="CV58">
+        <v>1</v>
+      </c>
     </row>
-    <row r="59" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -12037,8 +12424,14 @@
       <c r="CR59">
         <v>7</v>
       </c>
+      <c r="CT59">
+        <v>0</v>
+      </c>
+      <c r="CU59">
+        <v>7</v>
+      </c>
     </row>
-    <row r="60" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -12235,8 +12628,14 @@
       <c r="CR60">
         <v>2</v>
       </c>
+      <c r="CT60">
+        <v>7</v>
+      </c>
+      <c r="CU60">
+        <v>2</v>
+      </c>
     </row>
-    <row r="61" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -12385,8 +12784,14 @@
       <c r="CR61">
         <v>7</v>
       </c>
+      <c r="CT61">
+        <v>0</v>
+      </c>
+      <c r="CU61">
+        <v>7</v>
+      </c>
     </row>
-    <row r="62" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -12616,8 +13021,14 @@
       <c r="CR62">
         <v>4</v>
       </c>
+      <c r="CT62">
+        <v>1</v>
+      </c>
+      <c r="CU62">
+        <v>4</v>
+      </c>
     </row>
-    <row r="63" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -12844,8 +13255,14 @@
       <c r="CR63">
         <v>9</v>
       </c>
+      <c r="CT63">
+        <v>0</v>
+      </c>
+      <c r="CU63">
+        <v>9</v>
+      </c>
     </row>
-    <row r="64" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -13051,8 +13468,17 @@
       <c r="CS64">
         <v>1</v>
       </c>
+      <c r="CT64">
+        <v>3</v>
+      </c>
+      <c r="CU64">
+        <v>6</v>
+      </c>
+      <c r="CV64">
+        <v>1</v>
+      </c>
     </row>
-    <row r="65" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -13252,8 +13678,14 @@
       <c r="CR65">
         <v>6</v>
       </c>
+      <c r="CT65">
+        <v>0</v>
+      </c>
+      <c r="CU65">
+        <v>6</v>
+      </c>
     </row>
-    <row r="66" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -13393,8 +13825,17 @@
       <c r="CR66">
         <v>1</v>
       </c>
+      <c r="CT66">
+        <v>3</v>
+      </c>
+      <c r="CU66">
+        <v>1</v>
+      </c>
+      <c r="CV66">
+        <v>1</v>
+      </c>
     </row>
-    <row r="67" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -13624,8 +14065,14 @@
       <c r="CR67">
         <v>10</v>
       </c>
+      <c r="CT67">
+        <v>0</v>
+      </c>
+      <c r="CU67">
+        <v>10</v>
+      </c>
     </row>
-    <row r="68" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -13753,8 +14200,17 @@
       <c r="CS68">
         <v>1</v>
       </c>
+      <c r="CT68">
+        <v>4</v>
+      </c>
+      <c r="CU68">
+        <v>5</v>
+      </c>
+      <c r="CV68">
+        <v>2</v>
+      </c>
     </row>
-    <row r="69" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -13894,8 +14350,14 @@
       <c r="CR69">
         <v>9</v>
       </c>
+      <c r="CT69">
+        <v>0</v>
+      </c>
+      <c r="CU69">
+        <v>9</v>
+      </c>
     </row>
-    <row r="70" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -14038,8 +14500,14 @@
       <c r="CR70">
         <v>6</v>
       </c>
+      <c r="CT70">
+        <v>2</v>
+      </c>
+      <c r="CU70">
+        <v>6</v>
+      </c>
     </row>
-    <row r="71" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -14260,8 +14728,14 @@
       <c r="CR71">
         <v>10</v>
       </c>
+      <c r="CT71">
+        <v>0</v>
+      </c>
+      <c r="CU71">
+        <v>10</v>
+      </c>
     </row>
-    <row r="72" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -14470,8 +14944,14 @@
       <c r="CR72">
         <v>6</v>
       </c>
+      <c r="CT72">
+        <v>1</v>
+      </c>
+      <c r="CU72">
+        <v>6</v>
+      </c>
     </row>
-    <row r="73" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -14608,8 +15088,14 @@
       <c r="CR73">
         <v>10</v>
       </c>
+      <c r="CT73">
+        <v>0</v>
+      </c>
+      <c r="CU73">
+        <v>10</v>
+      </c>
     </row>
-    <row r="74" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -14749,8 +15235,17 @@
       <c r="CS74">
         <v>1</v>
       </c>
+      <c r="CT74">
+        <v>5</v>
+      </c>
+      <c r="CU74">
+        <v>3</v>
+      </c>
+      <c r="CV74">
+        <v>1</v>
+      </c>
     </row>
-    <row r="75" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -14956,8 +15451,17 @@
       <c r="CR75">
         <v>8</v>
       </c>
+      <c r="CT75">
+        <v>0</v>
+      </c>
+      <c r="CU75">
+        <v>8</v>
+      </c>
+      <c r="CV75">
+        <v>1</v>
+      </c>
     </row>
-    <row r="76" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -15187,8 +15691,17 @@
       <c r="CR76">
         <v>6</v>
       </c>
+      <c r="CT76">
+        <v>1</v>
+      </c>
+      <c r="CU76">
+        <v>6</v>
+      </c>
+      <c r="CV76">
+        <v>1</v>
+      </c>
     </row>
-    <row r="77" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -15379,8 +15892,14 @@
       <c r="CR77">
         <v>7</v>
       </c>
+      <c r="CT77">
+        <v>0</v>
+      </c>
+      <c r="CU77">
+        <v>7</v>
+      </c>
     </row>
-    <row r="78" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -15523,8 +16042,17 @@
       <c r="CS78">
         <v>2</v>
       </c>
+      <c r="CT78">
+        <v>2</v>
+      </c>
+      <c r="CU78">
+        <v>3</v>
+      </c>
+      <c r="CV78">
+        <v>2</v>
+      </c>
     </row>
-    <row r="79" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -15751,8 +16279,14 @@
       <c r="CR79">
         <v>9</v>
       </c>
+      <c r="CT79">
+        <v>0</v>
+      </c>
+      <c r="CU79">
+        <v>9</v>
+      </c>
     </row>
-    <row r="80" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -15949,8 +16483,14 @@
       <c r="CS80">
         <v>1</v>
       </c>
+      <c r="CT80">
+        <v>4</v>
+      </c>
+      <c r="CU80">
+        <v>6</v>
+      </c>
     </row>
-    <row r="81" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -16153,8 +16693,14 @@
       <c r="CR81">
         <v>7</v>
       </c>
+      <c r="CT81">
+        <v>0</v>
+      </c>
+      <c r="CU81">
+        <v>7</v>
+      </c>
     </row>
-    <row r="82" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -16396,8 +16942,14 @@
       <c r="CR82">
         <v>10</v>
       </c>
+      <c r="CT82">
+        <v>0</v>
+      </c>
+      <c r="CU82">
+        <v>10</v>
+      </c>
     </row>
-    <row r="83" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -16621,8 +17173,14 @@
       <c r="CR83">
         <v>9</v>
       </c>
+      <c r="CT83">
+        <v>0</v>
+      </c>
+      <c r="CU83">
+        <v>9</v>
+      </c>
     </row>
-    <row r="84" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -16843,8 +17401,17 @@
       <c r="CR84">
         <v>7</v>
       </c>
+      <c r="CT84">
+        <v>0</v>
+      </c>
+      <c r="CU84">
+        <v>7</v>
+      </c>
+      <c r="CV84">
+        <v>2</v>
+      </c>
     </row>
-    <row r="85" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -17068,8 +17635,14 @@
       <c r="CR85">
         <v>6</v>
       </c>
+      <c r="CT85">
+        <v>0</v>
+      </c>
+      <c r="CU85">
+        <v>6</v>
+      </c>
     </row>
-    <row r="86" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -17275,8 +17848,14 @@
       <c r="CR86">
         <v>8</v>
       </c>
+      <c r="CT86">
+        <v>1</v>
+      </c>
+      <c r="CU86">
+        <v>8</v>
+      </c>
     </row>
-    <row r="87" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -17506,8 +18085,14 @@
       <c r="CR87">
         <v>7</v>
       </c>
+      <c r="CT87">
+        <v>0</v>
+      </c>
+      <c r="CU87">
+        <v>7</v>
+      </c>
     </row>
-    <row r="88" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -17719,8 +18304,14 @@
       <c r="CR88">
         <v>7</v>
       </c>
+      <c r="CT88">
+        <v>2</v>
+      </c>
+      <c r="CU88">
+        <v>7</v>
+      </c>
     </row>
-    <row r="89" spans="2:97" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:100" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>3</v>
       </c>
@@ -17908,8 +18499,14 @@
       <c r="CR89" s="3">
         <v>5</v>
       </c>
+      <c r="CT89" s="3">
+        <v>0</v>
+      </c>
+      <c r="CU89" s="3">
+        <v>5</v>
+      </c>
     </row>
-    <row r="90" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -18052,8 +18649,17 @@
       <c r="CS90">
         <v>2</v>
       </c>
+      <c r="CT90">
+        <v>0</v>
+      </c>
+      <c r="CU90">
+        <v>5</v>
+      </c>
+      <c r="CV90">
+        <v>2</v>
+      </c>
     </row>
-    <row r="91" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -18289,8 +18895,14 @@
       <c r="CR91">
         <v>6</v>
       </c>
+      <c r="CT91">
+        <v>0</v>
+      </c>
+      <c r="CU91">
+        <v>6</v>
+      </c>
     </row>
-    <row r="92" spans="2:97" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:100" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>1</v>
       </c>
@@ -18505,8 +19117,17 @@
       <c r="CR92" s="3">
         <v>7</v>
       </c>
+      <c r="CT92" s="3">
+        <v>0</v>
+      </c>
+      <c r="CU92" s="3">
+        <v>7</v>
+      </c>
+      <c r="CV92" s="3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="93" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -18679,8 +19300,14 @@
       <c r="CR93">
         <v>9</v>
       </c>
+      <c r="CT93">
+        <v>0</v>
+      </c>
+      <c r="CU93">
+        <v>9</v>
+      </c>
     </row>
-    <row r="94" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -18823,8 +19450,14 @@
       <c r="CR94">
         <v>7</v>
       </c>
+      <c r="CT94">
+        <v>0</v>
+      </c>
+      <c r="CU94">
+        <v>7</v>
+      </c>
     </row>
-    <row r="95" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -19006,8 +19639,14 @@
       <c r="CR95">
         <v>8</v>
       </c>
+      <c r="CT95">
+        <v>0</v>
+      </c>
+      <c r="CU95">
+        <v>8</v>
+      </c>
     </row>
-    <row r="96" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -19213,8 +19852,17 @@
       <c r="CR96">
         <v>5</v>
       </c>
+      <c r="CT96">
+        <v>0</v>
+      </c>
+      <c r="CU96">
+        <v>6</v>
+      </c>
+      <c r="CV96">
+        <v>4</v>
+      </c>
     </row>
-    <row r="97" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -19360,8 +20008,14 @@
       <c r="CR97">
         <v>8</v>
       </c>
+      <c r="CT97">
+        <v>0</v>
+      </c>
+      <c r="CU97">
+        <v>8</v>
+      </c>
     </row>
-    <row r="98" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -19564,8 +20218,14 @@
       <c r="CR98">
         <v>7</v>
       </c>
+      <c r="CT98">
+        <v>0</v>
+      </c>
+      <c r="CU98">
+        <v>7</v>
+      </c>
     </row>
-    <row r="99" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -19720,8 +20380,17 @@
       <c r="CR99">
         <v>1</v>
       </c>
+      <c r="CT99">
+        <v>0</v>
+      </c>
+      <c r="CU99">
+        <v>1</v>
+      </c>
+      <c r="CV99">
+        <v>2</v>
+      </c>
     </row>
-    <row r="100" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -19849,8 +20518,14 @@
       <c r="CQ100">
         <v>8</v>
       </c>
+      <c r="CT100">
+        <v>7</v>
+      </c>
+      <c r="CU100">
+        <v>1</v>
+      </c>
     </row>
-    <row r="101" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -20038,8 +20713,14 @@
       <c r="CR101">
         <v>4</v>
       </c>
+      <c r="CT101">
+        <v>0</v>
+      </c>
+      <c r="CU101">
+        <v>5</v>
+      </c>
     </row>
-    <row r="102" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -20182,8 +20863,14 @@
       <c r="CR102">
         <v>6</v>
       </c>
+      <c r="CT102">
+        <v>1</v>
+      </c>
+      <c r="CU102">
+        <v>6</v>
+      </c>
     </row>
-    <row r="103" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -20392,8 +21079,14 @@
       <c r="CR103">
         <v>6</v>
       </c>
+      <c r="CT103">
+        <v>0</v>
+      </c>
+      <c r="CU103">
+        <v>6</v>
+      </c>
     </row>
-    <row r="104" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -20599,8 +21292,14 @@
       <c r="CR104">
         <v>8</v>
       </c>
+      <c r="CT104">
+        <v>2</v>
+      </c>
+      <c r="CU104">
+        <v>8</v>
+      </c>
     </row>
-    <row r="105" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -20800,8 +21499,14 @@
       <c r="CR105">
         <v>6</v>
       </c>
+      <c r="CT105">
+        <v>0</v>
+      </c>
+      <c r="CU105">
+        <v>6</v>
+      </c>
     </row>
-    <row r="106" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -20992,8 +21697,14 @@
       <c r="CR106">
         <v>8</v>
       </c>
+      <c r="CT106">
+        <v>0</v>
+      </c>
+      <c r="CU106">
+        <v>8</v>
+      </c>
     </row>
-    <row r="107" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -21205,8 +21916,14 @@
       <c r="CR107">
         <v>5</v>
       </c>
+      <c r="CT107">
+        <v>0</v>
+      </c>
+      <c r="CU107">
+        <v>5</v>
+      </c>
     </row>
-    <row r="108" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -21403,8 +22120,14 @@
       <c r="CR108">
         <v>10</v>
       </c>
+      <c r="CT108">
+        <v>0</v>
+      </c>
+      <c r="CU108">
+        <v>10</v>
+      </c>
     </row>
-    <row r="109" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -21616,8 +22339,14 @@
       <c r="CR109">
         <v>9</v>
       </c>
+      <c r="CT109">
+        <v>0</v>
+      </c>
+      <c r="CU109">
+        <v>9</v>
+      </c>
     </row>
-    <row r="110" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -21835,8 +22564,17 @@
       <c r="CS110">
         <v>2</v>
       </c>
+      <c r="CT110">
+        <v>0</v>
+      </c>
+      <c r="CU110">
+        <v>7</v>
+      </c>
+      <c r="CV110">
+        <v>2</v>
+      </c>
     </row>
-    <row r="111" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -22039,8 +22777,14 @@
       <c r="CR111">
         <v>7</v>
       </c>
+      <c r="CT111">
+        <v>0</v>
+      </c>
+      <c r="CU111">
+        <v>8</v>
+      </c>
     </row>
-    <row r="112" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -22249,8 +22993,14 @@
       <c r="CR112">
         <v>5</v>
       </c>
+      <c r="CT112">
+        <v>1</v>
+      </c>
+      <c r="CU112">
+        <v>7</v>
+      </c>
     </row>
-    <row r="113" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -22465,8 +23215,17 @@
       <c r="CR113">
         <v>2</v>
       </c>
+      <c r="CT113">
+        <v>0</v>
+      </c>
+      <c r="CU113">
+        <v>4</v>
+      </c>
+      <c r="CV113">
+        <v>2</v>
+      </c>
     </row>
-    <row r="114" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -22606,8 +23365,14 @@
       <c r="CR114">
         <v>8</v>
       </c>
+      <c r="CT114">
+        <v>0</v>
+      </c>
+      <c r="CU114">
+        <v>8</v>
+      </c>
     </row>
-    <row r="115" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -22825,8 +23590,14 @@
       <c r="CR115">
         <v>4</v>
       </c>
+      <c r="CT115">
+        <v>0</v>
+      </c>
+      <c r="CU115">
+        <v>4</v>
+      </c>
     </row>
-    <row r="116" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -23029,8 +23800,14 @@
       <c r="CR116">
         <v>8</v>
       </c>
+      <c r="CT116">
+        <v>0</v>
+      </c>
+      <c r="CU116">
+        <v>8</v>
+      </c>
     </row>
-    <row r="117" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -23239,8 +24016,14 @@
       <c r="CR117">
         <v>5</v>
       </c>
+      <c r="CT117">
+        <v>0</v>
+      </c>
+      <c r="CU117">
+        <v>5</v>
+      </c>
     </row>
-    <row r="118" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -23390,8 +24173,14 @@
       <c r="CR118">
         <v>6</v>
       </c>
+      <c r="CT118">
+        <v>0</v>
+      </c>
+      <c r="CU118">
+        <v>6</v>
+      </c>
     </row>
-    <row r="119" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -23543,8 +24332,14 @@
       <c r="CR119">
         <v>7</v>
       </c>
+      <c r="CT119">
+        <v>0</v>
+      </c>
+      <c r="CU119">
+        <v>7</v>
+      </c>
     </row>
-    <row r="120" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -23687,8 +24482,14 @@
       <c r="CR120">
         <v>10</v>
       </c>
+      <c r="CT120">
+        <v>0</v>
+      </c>
+      <c r="CU120">
+        <v>10</v>
+      </c>
     </row>
-    <row r="121" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -23831,8 +24632,14 @@
       <c r="CR121">
         <v>8</v>
       </c>
+      <c r="CT121">
+        <v>0</v>
+      </c>
+      <c r="CU121">
+        <v>8</v>
+      </c>
     </row>
-    <row r="122" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -23978,8 +24785,14 @@
       <c r="CR122">
         <v>6</v>
       </c>
+      <c r="CT122">
+        <v>0</v>
+      </c>
+      <c r="CU122">
+        <v>6</v>
+      </c>
     </row>
-    <row r="123" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -24176,8 +24989,17 @@
       <c r="CR123">
         <v>3</v>
       </c>
+      <c r="CT123">
+        <v>0</v>
+      </c>
+      <c r="CU123">
+        <v>3</v>
+      </c>
+      <c r="CV123">
+        <v>3</v>
+      </c>
     </row>
-    <row r="124" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -24419,8 +25241,14 @@
       <c r="CS124">
         <v>1</v>
       </c>
+      <c r="CT124">
+        <v>1</v>
+      </c>
+      <c r="CU124">
+        <v>8</v>
+      </c>
     </row>
-    <row r="125" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -24644,8 +25472,14 @@
       <c r="CR125">
         <v>6</v>
       </c>
+      <c r="CT125">
+        <v>0</v>
+      </c>
+      <c r="CU125">
+        <v>6</v>
+      </c>
     </row>
-    <row r="126" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -24851,8 +25685,14 @@
       <c r="CR126">
         <v>6</v>
       </c>
+      <c r="CT126">
+        <v>0</v>
+      </c>
+      <c r="CU126">
+        <v>6</v>
+      </c>
     </row>
-    <row r="127" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -25052,8 +25892,14 @@
       <c r="CR127">
         <v>3</v>
       </c>
+      <c r="CT127">
+        <v>0</v>
+      </c>
+      <c r="CU127">
+        <v>3</v>
+      </c>
     </row>
-    <row r="128" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -25184,8 +26030,14 @@
       <c r="CR128">
         <v>7</v>
       </c>
+      <c r="CT128">
+        <v>0</v>
+      </c>
+      <c r="CU128">
+        <v>7</v>
+      </c>
     </row>
-    <row r="129" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -25400,8 +26252,14 @@
       <c r="CR129">
         <v>6</v>
       </c>
+      <c r="CT129">
+        <v>0</v>
+      </c>
+      <c r="CU129">
+        <v>6</v>
+      </c>
     </row>
-    <row r="130" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -25553,8 +26411,14 @@
       <c r="CR130">
         <v>10</v>
       </c>
+      <c r="CT130">
+        <v>0</v>
+      </c>
+      <c r="CU130">
+        <v>10</v>
+      </c>
     </row>
-    <row r="131" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -25772,8 +26636,14 @@
       <c r="CR131">
         <v>10</v>
       </c>
+      <c r="CT131">
+        <v>0</v>
+      </c>
+      <c r="CU131">
+        <v>10</v>
+      </c>
     </row>
-    <row r="132" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -25913,8 +26783,14 @@
       <c r="CR132">
         <v>6</v>
       </c>
+      <c r="CT132">
+        <v>0</v>
+      </c>
+      <c r="CU132">
+        <v>6</v>
+      </c>
     </row>
-    <row r="133" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -26087,8 +26963,14 @@
       <c r="CR133">
         <v>7</v>
       </c>
+      <c r="CT133">
+        <v>0</v>
+      </c>
+      <c r="CU133">
+        <v>7</v>
+      </c>
     </row>
-    <row r="134" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -26261,8 +27143,14 @@
       <c r="CR134">
         <v>10</v>
       </c>
+      <c r="CT134">
+        <v>0</v>
+      </c>
+      <c r="CU134">
+        <v>10</v>
+      </c>
     </row>
-    <row r="135" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -26456,8 +27344,14 @@
       <c r="CR135">
         <v>7</v>
       </c>
+      <c r="CT135">
+        <v>0</v>
+      </c>
+      <c r="CU135">
+        <v>8</v>
+      </c>
     </row>
-    <row r="136" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -26645,8 +27539,14 @@
       <c r="CR136">
         <v>7</v>
       </c>
+      <c r="CT136">
+        <v>0</v>
+      </c>
+      <c r="CU136">
+        <v>7</v>
+      </c>
     </row>
-    <row r="137" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -26843,8 +27743,14 @@
       <c r="CS137">
         <v>1</v>
       </c>
+      <c r="CT137">
+        <v>0</v>
+      </c>
+      <c r="CU137">
+        <v>5</v>
+      </c>
     </row>
-    <row r="138" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -27053,8 +27959,14 @@
       <c r="CR138">
         <v>7</v>
       </c>
+      <c r="CT138">
+        <v>0</v>
+      </c>
+      <c r="CU138">
+        <v>7</v>
+      </c>
     </row>
-    <row r="139" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -27245,8 +28157,14 @@
       <c r="CR139">
         <v>5</v>
       </c>
+      <c r="CT139">
+        <v>0</v>
+      </c>
+      <c r="CU139">
+        <v>5</v>
+      </c>
     </row>
-    <row r="140" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -27392,8 +28310,14 @@
       <c r="CR140">
         <v>9</v>
       </c>
+      <c r="CT140">
+        <v>0</v>
+      </c>
+      <c r="CU140">
+        <v>9</v>
+      </c>
     </row>
-    <row r="141" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -27620,8 +28544,14 @@
       <c r="CR141">
         <v>8</v>
       </c>
+      <c r="CT141">
+        <v>0</v>
+      </c>
+      <c r="CU141">
+        <v>8</v>
+      </c>
     </row>
-    <row r="142" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -27848,8 +28778,14 @@
       <c r="CR142">
         <v>8</v>
       </c>
+      <c r="CT142">
+        <v>0</v>
+      </c>
+      <c r="CU142">
+        <v>8</v>
+      </c>
     </row>
-    <row r="143" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -28034,8 +28970,14 @@
       <c r="CR143">
         <v>11</v>
       </c>
+      <c r="CT143">
+        <v>0</v>
+      </c>
+      <c r="CU143">
+        <v>11</v>
+      </c>
     </row>
-    <row r="144" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -28172,8 +29114,14 @@
       <c r="CR144">
         <v>7</v>
       </c>
+      <c r="CT144">
+        <v>0</v>
+      </c>
+      <c r="CU144">
+        <v>7</v>
+      </c>
     </row>
-    <row r="145" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -28319,8 +29267,14 @@
       <c r="CR145">
         <v>5</v>
       </c>
+      <c r="CT145">
+        <v>0</v>
+      </c>
+      <c r="CU145">
+        <v>5</v>
+      </c>
     </row>
-    <row r="146" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -28559,8 +29513,14 @@
       <c r="CR146">
         <v>10</v>
       </c>
+      <c r="CT146">
+        <v>0</v>
+      </c>
+      <c r="CU146">
+        <v>10</v>
+      </c>
     </row>
-    <row r="147" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -28787,8 +29747,17 @@
       <c r="CR147">
         <v>1</v>
       </c>
+      <c r="CT147">
+        <v>0</v>
+      </c>
+      <c r="CU147">
+        <v>2</v>
+      </c>
+      <c r="CV147">
+        <v>1</v>
+      </c>
     </row>
-    <row r="148" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -28913,8 +29882,11 @@
       <c r="CQ148">
         <v>9</v>
       </c>
+      <c r="CT148">
+        <v>9</v>
+      </c>
     </row>
-    <row r="149" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -29150,8 +30122,17 @@
       <c r="CS149">
         <v>1</v>
       </c>
+      <c r="CT149">
+        <v>0</v>
+      </c>
+      <c r="CU149">
+        <v>4</v>
+      </c>
+      <c r="CV149">
+        <v>1</v>
+      </c>
     </row>
-    <row r="150" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -29372,8 +30353,14 @@
       <c r="CR150">
         <v>9</v>
       </c>
+      <c r="CT150">
+        <v>0</v>
+      </c>
+      <c r="CU150">
+        <v>9</v>
+      </c>
     </row>
-    <row r="151" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -29570,8 +30557,14 @@
       <c r="CR151">
         <v>10</v>
       </c>
+      <c r="CT151">
+        <v>0</v>
+      </c>
+      <c r="CU151">
+        <v>10</v>
+      </c>
     </row>
-    <row r="152" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -29705,8 +30698,14 @@
       <c r="CR152">
         <v>9</v>
       </c>
+      <c r="CT152">
+        <v>0</v>
+      </c>
+      <c r="CU152">
+        <v>9</v>
+      </c>
     </row>
-    <row r="153" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -29894,8 +30893,14 @@
       <c r="CR153">
         <v>7</v>
       </c>
+      <c r="CT153">
+        <v>0</v>
+      </c>
+      <c r="CU153">
+        <v>7</v>
+      </c>
     </row>
-    <row r="154" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -30149,8 +31154,14 @@
       <c r="CR154">
         <v>8</v>
       </c>
+      <c r="CT154">
+        <v>0</v>
+      </c>
+      <c r="CU154">
+        <v>8</v>
+      </c>
     </row>
-    <row r="155" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -30353,8 +31364,14 @@
       <c r="CR155">
         <v>9</v>
       </c>
+      <c r="CT155">
+        <v>0</v>
+      </c>
+      <c r="CU155">
+        <v>9</v>
+      </c>
     </row>
-    <row r="156" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="156" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -30494,8 +31511,14 @@
       <c r="CR156">
         <v>6</v>
       </c>
+      <c r="CT156">
+        <v>0</v>
+      </c>
+      <c r="CU156">
+        <v>6</v>
+      </c>
     </row>
-    <row r="157" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="157" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -30635,8 +31658,14 @@
       <c r="CR157">
         <v>6</v>
       </c>
+      <c r="CT157">
+        <v>0</v>
+      </c>
+      <c r="CU157">
+        <v>6</v>
+      </c>
     </row>
-    <row r="158" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="158" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -30812,8 +31841,14 @@
       <c r="CS158">
         <v>2</v>
       </c>
+      <c r="CT158">
+        <v>1</v>
+      </c>
+      <c r="CU158">
+        <v>7</v>
+      </c>
     </row>
-    <row r="159" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -31031,8 +32066,14 @@
       <c r="CR159">
         <v>5</v>
       </c>
+      <c r="CT159">
+        <v>0</v>
+      </c>
+      <c r="CU159">
+        <v>5</v>
+      </c>
     </row>
-    <row r="160" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -31160,8 +32201,17 @@
       <c r="CQ160">
         <v>9</v>
       </c>
+      <c r="CT160">
+        <v>3</v>
+      </c>
+      <c r="CU160">
+        <v>3</v>
+      </c>
+      <c r="CV160">
+        <v>3</v>
+      </c>
     </row>
-    <row r="161" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -31397,8 +32447,17 @@
       <c r="CR161">
         <v>6</v>
       </c>
+      <c r="CT161">
+        <v>0</v>
+      </c>
+      <c r="CU161">
+        <v>6</v>
+      </c>
+      <c r="CV161">
+        <v>1</v>
+      </c>
     </row>
-    <row r="162" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -31535,8 +32594,14 @@
       <c r="CR162">
         <v>8</v>
       </c>
+      <c r="CT162">
+        <v>0</v>
+      </c>
+      <c r="CU162">
+        <v>8</v>
+      </c>
     </row>
-    <row r="163" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="163" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -31733,8 +32798,14 @@
       <c r="CR163">
         <v>8</v>
       </c>
+      <c r="CT163">
+        <v>0</v>
+      </c>
+      <c r="CU163">
+        <v>8</v>
+      </c>
     </row>
-    <row r="164" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="164" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -31874,8 +32945,14 @@
       <c r="CR164">
         <v>8</v>
       </c>
+      <c r="CT164">
+        <v>1</v>
+      </c>
+      <c r="CU164">
+        <v>8</v>
+      </c>
     </row>
-    <row r="165" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -32072,8 +33149,14 @@
       <c r="CR165">
         <v>6</v>
       </c>
+      <c r="CT165">
+        <v>0</v>
+      </c>
+      <c r="CU165">
+        <v>6</v>
+      </c>
     </row>
-    <row r="166" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="166" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -32255,8 +33338,14 @@
       <c r="CR166">
         <v>6</v>
       </c>
+      <c r="CT166">
+        <v>0</v>
+      </c>
+      <c r="CU166">
+        <v>6</v>
+      </c>
     </row>
-    <row r="167" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -32441,8 +33530,14 @@
       <c r="CR167">
         <v>8</v>
       </c>
+      <c r="CT167">
+        <v>0</v>
+      </c>
+      <c r="CU167">
+        <v>8</v>
+      </c>
     </row>
-    <row r="168" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -32660,8 +33755,14 @@
       <c r="CR168">
         <v>11</v>
       </c>
+      <c r="CT168">
+        <v>0</v>
+      </c>
+      <c r="CU168">
+        <v>11</v>
+      </c>
     </row>
-    <row r="169" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -32801,8 +33902,14 @@
       <c r="CR169">
         <v>6</v>
       </c>
+      <c r="CT169">
+        <v>0</v>
+      </c>
+      <c r="CU169">
+        <v>6</v>
+      </c>
     </row>
-    <row r="170" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -32966,8 +34073,14 @@
       <c r="CS170">
         <v>2</v>
       </c>
+      <c r="CT170">
+        <v>0</v>
+      </c>
+      <c r="CU170">
+        <v>8</v>
+      </c>
     </row>
-    <row r="171" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="171" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -33194,8 +34307,14 @@
       <c r="CR171">
         <v>10</v>
       </c>
+      <c r="CT171">
+        <v>0</v>
+      </c>
+      <c r="CU171">
+        <v>10</v>
+      </c>
     </row>
-    <row r="172" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -33341,8 +34460,14 @@
       <c r="CS172">
         <v>1</v>
       </c>
+      <c r="CT172">
+        <v>1</v>
+      </c>
+      <c r="CU172">
+        <v>7</v>
+      </c>
     </row>
-    <row r="173" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -33503,8 +34628,14 @@
       <c r="CR173">
         <v>3</v>
       </c>
+      <c r="CT173">
+        <v>0</v>
+      </c>
+      <c r="CU173">
+        <v>8</v>
+      </c>
     </row>
-    <row r="174" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -33650,8 +34781,14 @@
       <c r="CR174">
         <v>9</v>
       </c>
+      <c r="CT174">
+        <v>0</v>
+      </c>
+      <c r="CU174">
+        <v>9</v>
+      </c>
     </row>
-    <row r="175" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -33854,8 +34991,14 @@
       <c r="CR175">
         <v>9</v>
       </c>
+      <c r="CT175">
+        <v>0</v>
+      </c>
+      <c r="CU175">
+        <v>9</v>
+      </c>
     </row>
-    <row r="176" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="176" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -33992,8 +35135,14 @@
       <c r="CR176">
         <v>8</v>
       </c>
+      <c r="CT176">
+        <v>0</v>
+      </c>
+      <c r="CU176">
+        <v>8</v>
+      </c>
     </row>
-    <row r="177" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -34139,8 +35288,14 @@
       <c r="CR177">
         <v>5</v>
       </c>
+      <c r="CT177">
+        <v>0</v>
+      </c>
+      <c r="CU177">
+        <v>5</v>
+      </c>
     </row>
-    <row r="178" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -34292,8 +35447,14 @@
       <c r="CR178">
         <v>8</v>
       </c>
+      <c r="CT178">
+        <v>0</v>
+      </c>
+      <c r="CU178">
+        <v>8</v>
+      </c>
     </row>
-    <row r="179" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -34496,8 +35657,14 @@
       <c r="CR179">
         <v>10</v>
       </c>
+      <c r="CT179">
+        <v>0</v>
+      </c>
+      <c r="CU179">
+        <v>10</v>
+      </c>
     </row>
-    <row r="180" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -34697,8 +35864,14 @@
       <c r="CR180">
         <v>9</v>
       </c>
+      <c r="CT180">
+        <v>0</v>
+      </c>
+      <c r="CU180">
+        <v>9</v>
+      </c>
     </row>
-    <row r="181" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -34898,8 +36071,14 @@
       <c r="CR181">
         <v>9</v>
       </c>
+      <c r="CT181">
+        <v>0</v>
+      </c>
+      <c r="CU181">
+        <v>9</v>
+      </c>
     </row>
-    <row r="182" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -35042,8 +36221,14 @@
       <c r="CR182">
         <v>5</v>
       </c>
+      <c r="CT182">
+        <v>0</v>
+      </c>
+      <c r="CU182">
+        <v>6</v>
+      </c>
     </row>
-    <row r="183" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -35275,8 +36460,14 @@
       <c r="CR183">
         <v>5</v>
       </c>
+      <c r="CT183">
+        <v>0</v>
+      </c>
+      <c r="CU183">
+        <v>5</v>
+      </c>
     </row>
-    <row r="184" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -35427,8 +36618,14 @@
       <c r="CR184">
         <v>6</v>
       </c>
+      <c r="CT184">
+        <v>0</v>
+      </c>
+      <c r="CU184">
+        <v>6</v>
+      </c>
     </row>
-    <row r="185" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -35630,8 +36827,14 @@
       <c r="CR185">
         <v>7</v>
       </c>
+      <c r="CT185">
+        <v>0</v>
+      </c>
+      <c r="CU185">
+        <v>7</v>
+      </c>
     </row>
-    <row r="186" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -35821,8 +37024,14 @@
       <c r="CR186">
         <v>1</v>
       </c>
+      <c r="CT186">
+        <v>6</v>
+      </c>
+      <c r="CU186">
+        <v>1</v>
+      </c>
     </row>
-    <row r="187" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -35982,8 +37191,14 @@
       <c r="CS187">
         <v>4</v>
       </c>
+      <c r="CT187">
+        <v>0</v>
+      </c>
+      <c r="CU187">
+        <v>8</v>
+      </c>
     </row>
-    <row r="188" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B188" t="s">
         <v>4</v>
       </c>
@@ -36194,8 +37409,17 @@
       <c r="CS188">
         <v>1</v>
       </c>
+      <c r="CT188">
+        <v>0</v>
+      </c>
+      <c r="CU188">
+        <v>9</v>
+      </c>
+      <c r="CV188">
+        <v>1</v>
+      </c>
     </row>
-    <row r="189" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -36403,8 +37627,14 @@
       <c r="CR189">
         <v>2</v>
       </c>
+      <c r="CT189">
+        <v>0</v>
+      </c>
+      <c r="CU189">
+        <v>2</v>
+      </c>
     </row>
-    <row r="190" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="190" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -36615,8 +37845,14 @@
       <c r="CR190">
         <v>5</v>
       </c>
+      <c r="CT190">
+        <v>0</v>
+      </c>
+      <c r="CU190">
+        <v>5</v>
+      </c>
     </row>
-    <row r="191" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="191" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -36830,8 +38066,14 @@
       <c r="CR191">
         <v>5</v>
       </c>
+      <c r="CT191">
+        <v>0</v>
+      </c>
+      <c r="CU191">
+        <v>5</v>
+      </c>
     </row>
-    <row r="192" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="192" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -37024,8 +38266,14 @@
       <c r="CR192">
         <v>3</v>
       </c>
+      <c r="CT192">
+        <v>0</v>
+      </c>
+      <c r="CU192">
+        <v>3</v>
+      </c>
     </row>
-    <row r="193" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="193" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -37242,8 +38490,14 @@
       <c r="CR193">
         <v>6</v>
       </c>
+      <c r="CT193">
+        <v>0</v>
+      </c>
+      <c r="CU193">
+        <v>7</v>
+      </c>
     </row>
-    <row r="194" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="194" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B194" t="s">
         <v>4</v>
       </c>
@@ -37436,8 +38690,14 @@
       <c r="CR194">
         <v>7</v>
       </c>
+      <c r="CT194">
+        <v>0</v>
+      </c>
+      <c r="CU194">
+        <v>7</v>
+      </c>
     </row>
-    <row r="195" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="195" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -37645,8 +38905,14 @@
       <c r="CR195">
         <v>2</v>
       </c>
+      <c r="CT195">
+        <v>0</v>
+      </c>
+      <c r="CU195">
+        <v>2</v>
+      </c>
     </row>
-    <row r="196" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="196" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -37887,8 +39153,14 @@
       <c r="CR196">
         <v>9</v>
       </c>
+      <c r="CT196">
+        <v>0</v>
+      </c>
+      <c r="CU196">
+        <v>9</v>
+      </c>
     </row>
-    <row r="197" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="197" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -38084,8 +39356,14 @@
       <c r="CR197">
         <v>4</v>
       </c>
+      <c r="CT197">
+        <v>0</v>
+      </c>
+      <c r="CU197">
+        <v>4</v>
+      </c>
     </row>
-    <row r="198" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="198" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -38263,8 +39541,14 @@
       <c r="CR198">
         <v>5</v>
       </c>
+      <c r="CT198">
+        <v>0</v>
+      </c>
+      <c r="CU198">
+        <v>5</v>
+      </c>
     </row>
-    <row r="199" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="199" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -38454,8 +39738,14 @@
       <c r="CR199">
         <v>6</v>
       </c>
+      <c r="CT199">
+        <v>0</v>
+      </c>
+      <c r="CU199">
+        <v>6</v>
+      </c>
     </row>
-    <row r="200" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="200" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
         <v>4</v>
       </c>
@@ -38642,8 +39932,14 @@
       <c r="CR200">
         <v>7</v>
       </c>
+      <c r="CT200">
+        <v>0</v>
+      </c>
+      <c r="CU200">
+        <v>7</v>
+      </c>
     </row>
-    <row r="201" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="201" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -38866,8 +40162,14 @@
       <c r="CR201">
         <v>6</v>
       </c>
+      <c r="CT201">
+        <v>0</v>
+      </c>
+      <c r="CU201">
+        <v>6</v>
+      </c>
     </row>
-    <row r="202" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="202" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -39081,8 +40383,14 @@
       <c r="CR202">
         <v>1</v>
       </c>
+      <c r="CT202">
+        <v>0</v>
+      </c>
+      <c r="CU202">
+        <v>1</v>
+      </c>
     </row>
-    <row r="203" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="203" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -39290,8 +40598,14 @@
       <c r="CR203">
         <v>3</v>
       </c>
+      <c r="CT203">
+        <v>0</v>
+      </c>
+      <c r="CU203">
+        <v>3</v>
+      </c>
     </row>
-    <row r="204" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="204" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -39412,8 +40726,11 @@
       <c r="CQ204">
         <v>6</v>
       </c>
+      <c r="CT204">
+        <v>6</v>
+      </c>
     </row>
-    <row r="205" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="205" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -39642,8 +40959,14 @@
       <c r="CS205">
         <v>1</v>
       </c>
+      <c r="CT205">
+        <v>2</v>
+      </c>
+      <c r="CU205">
+        <v>8</v>
+      </c>
     </row>
-    <row r="206" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="206" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B206" t="s">
         <v>4</v>
       </c>
@@ -39773,8 +41096,17 @@
       <c r="CR206">
         <v>5</v>
       </c>
+      <c r="CT206">
+        <v>0</v>
+      </c>
+      <c r="CU206">
+        <v>5</v>
+      </c>
+      <c r="CV206">
+        <v>1</v>
+      </c>
     </row>
-    <row r="207" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="207" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -39955,8 +41287,14 @@
       <c r="CR207">
         <v>4</v>
       </c>
+      <c r="CT207">
+        <v>0</v>
+      </c>
+      <c r="CU207">
+        <v>4</v>
+      </c>
     </row>
-    <row r="208" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="208" spans="2:100" x14ac:dyDescent="0.3">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -40164,8 +41502,14 @@
       <c r="CR208">
         <v>3</v>
       </c>
+      <c r="CT208">
+        <v>0</v>
+      </c>
+      <c r="CU208">
+        <v>3</v>
+      </c>
     </row>
-    <row r="209" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="209" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B209" t="s">
         <v>3</v>
       </c>
@@ -40358,8 +41702,14 @@
       <c r="CR209">
         <v>5</v>
       </c>
+      <c r="CT209">
+        <v>0</v>
+      </c>
+      <c r="CU209">
+        <v>5</v>
+      </c>
     </row>
-    <row r="210" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="210" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B210" t="s">
         <v>1</v>
       </c>
@@ -40573,8 +41923,14 @@
       <c r="CR210">
         <v>1</v>
       </c>
+      <c r="CT210">
+        <v>4</v>
+      </c>
+      <c r="CU210">
+        <v>1</v>
+      </c>
     </row>
-    <row r="211" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="211" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
         <v>4</v>
       </c>
@@ -40767,8 +42123,14 @@
       <c r="CS211">
         <v>2</v>
       </c>
+      <c r="CT211">
+        <v>1</v>
+      </c>
+      <c r="CU211">
+        <v>4</v>
+      </c>
     </row>
-    <row r="212" spans="2:97" x14ac:dyDescent="0.3">
+    <row r="212" spans="2:99" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
         <v>4</v>
       </c>
@@ -40953,6 +42315,12 @@
         <v>0</v>
       </c>
       <c r="CR212">
+        <v>6</v>
+      </c>
+      <c r="CT212">
+        <v>0</v>
+      </c>
+      <c r="CU212">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
DOY 210 germinants data collection
</commit_message>
<xml_diff>
--- a/data/germination_data.xlsx
+++ b/data/germination_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temporal Ecology Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2B1612-41B2-44F7-9947-19787E6B8ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4CF0AA-D2AC-4DD6-B312-DC3AFB560E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="141">
   <si>
     <t>seed_species</t>
   </si>
@@ -483,6 +483,18 @@
   <si>
     <t>196_halfdead</t>
   </si>
+  <si>
+    <t>210_alive</t>
+  </si>
+  <si>
+    <t>210_dead</t>
+  </si>
+  <si>
+    <t>210_halfdead</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
 </sst>
 </file>
 
@@ -586,9 +598,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CV213" totalsRowShown="0">
-  <autoFilter ref="B2:CV213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
-  <tableColumns count="99">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CY213" totalsRowShown="0">
+  <autoFilter ref="B2:CY213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
+  <tableColumns count="102">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
     <tableColumn id="3" xr3:uid="{B695F4B4-8561-9D48-9FF3-12A40CB2B7C7}" name="inoculated_%"/>
@@ -688,6 +700,9 @@
     <tableColumn id="97" xr3:uid="{C0EE2BE8-9A00-4918-B7BC-CECE73317595}" name="196_alive"/>
     <tableColumn id="98" xr3:uid="{757C4777-32C3-4210-A085-69139B19933D}" name="196_dead"/>
     <tableColumn id="99" xr3:uid="{50FC3B28-770A-4906-B9B0-60C7F64F10FB}" name="196_halfdead"/>
+    <tableColumn id="100" xr3:uid="{3B2AF124-4421-47CA-8DE0-0702AB08EBA4}" name="210_alive"/>
+    <tableColumn id="101" xr3:uid="{89EA52E1-8A22-4896-9795-5647630F196D}" name="210_dead"/>
+    <tableColumn id="102" xr3:uid="{590F0C34-0381-42D4-A386-55EA13C347CD}" name="210_halfdead"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1010,7 +1025,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:CV212"/>
+  <dimension ref="B2:DA214"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -1018,7 +1033,7 @@
     <col min="4" max="4" width="17.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -1316,8 +1331,17 @@
       <c r="CV2" t="s">
         <v>136</v>
       </c>
+      <c r="CW2" t="s">
+        <v>137</v>
+      </c>
+      <c r="CX2" t="s">
+        <v>138</v>
+      </c>
+      <c r="CY2" t="s">
+        <v>139</v>
+      </c>
     </row>
-    <row r="3" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1546,8 +1570,14 @@
       <c r="CU3">
         <v>4</v>
       </c>
+      <c r="CW3">
+        <v>0</v>
+      </c>
+      <c r="CX3">
+        <v>4</v>
+      </c>
     </row>
-    <row r="4" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1677,8 +1707,14 @@
       <c r="CT4">
         <v>9</v>
       </c>
+      <c r="CW4">
+        <v>8</v>
+      </c>
+      <c r="CY4">
+        <v>1</v>
+      </c>
     </row>
-    <row r="5" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1904,8 +1940,14 @@
       <c r="CU5">
         <v>7</v>
       </c>
+      <c r="CW5">
+        <v>0</v>
+      </c>
+      <c r="CX5">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -2044,8 +2086,17 @@
       <c r="CV6">
         <v>2</v>
       </c>
+      <c r="CW6">
+        <v>0</v>
+      </c>
+      <c r="CX6">
+        <v>8</v>
+      </c>
+      <c r="CY6">
+        <v>1</v>
+      </c>
     </row>
-    <row r="7" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -2238,8 +2289,14 @@
       <c r="CU7">
         <v>6</v>
       </c>
+      <c r="CW7">
+        <v>0</v>
+      </c>
+      <c r="CX7">
+        <v>6</v>
+      </c>
     </row>
-    <row r="8" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -2456,8 +2513,17 @@
       <c r="CU8">
         <v>1</v>
       </c>
+      <c r="CW8">
+        <v>4</v>
+      </c>
+      <c r="CX8">
+        <v>1</v>
+      </c>
+      <c r="CY8">
+        <v>2</v>
+      </c>
     </row>
-    <row r="9" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2683,8 +2749,14 @@
       <c r="CU9">
         <v>7</v>
       </c>
+      <c r="CW9">
+        <v>0</v>
+      </c>
+      <c r="CX9">
+        <v>7</v>
+      </c>
     </row>
-    <row r="10" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -2847,8 +2919,14 @@
       <c r="CV10">
         <v>2</v>
       </c>
+      <c r="CW10">
+        <v>2</v>
+      </c>
+      <c r="CX10">
+        <v>6</v>
+      </c>
     </row>
-    <row r="11" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -3071,8 +3149,14 @@
       <c r="CU11">
         <v>8</v>
       </c>
+      <c r="CW11">
+        <v>0</v>
+      </c>
+      <c r="CX11">
+        <v>8</v>
+      </c>
     </row>
-    <row r="12" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -3298,8 +3382,17 @@
       <c r="CU12">
         <v>5</v>
       </c>
+      <c r="CW12">
+        <v>4</v>
+      </c>
+      <c r="CX12">
+        <v>5</v>
+      </c>
+      <c r="CY12">
+        <v>1</v>
+      </c>
     </row>
-    <row r="13" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -3516,8 +3609,14 @@
       <c r="CU13">
         <v>7</v>
       </c>
+      <c r="CW13">
+        <v>0</v>
+      </c>
+      <c r="CX13">
+        <v>7</v>
+      </c>
     </row>
-    <row r="14" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -3698,8 +3797,14 @@
       <c r="CV14">
         <v>1</v>
       </c>
+      <c r="CW14">
+        <v>1</v>
+      </c>
+      <c r="CX14">
+        <v>8</v>
+      </c>
     </row>
-    <row r="15" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -3905,8 +4010,14 @@
       <c r="CU15">
         <v>8</v>
       </c>
+      <c r="CW15">
+        <v>0</v>
+      </c>
+      <c r="CX15">
+        <v>8</v>
+      </c>
     </row>
-    <row r="16" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -4103,8 +4214,17 @@
       <c r="CV16">
         <v>1</v>
       </c>
+      <c r="CW16">
+        <v>3</v>
+      </c>
+      <c r="CX16">
+        <v>5</v>
+      </c>
+      <c r="CY16">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -4313,8 +4433,14 @@
       <c r="CU17">
         <v>8</v>
       </c>
+      <c r="CW17">
+        <v>0</v>
+      </c>
+      <c r="CX17">
+        <v>8</v>
+      </c>
     </row>
-    <row r="18" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -4454,8 +4580,14 @@
       <c r="CV18">
         <v>1</v>
       </c>
+      <c r="CW18">
+        <v>0</v>
+      </c>
+      <c r="CX18">
+        <v>10</v>
+      </c>
     </row>
-    <row r="19" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -4682,8 +4814,14 @@
       <c r="CU19">
         <v>7</v>
       </c>
+      <c r="CW19">
+        <v>0</v>
+      </c>
+      <c r="CX19">
+        <v>7</v>
+      </c>
     </row>
-    <row r="20" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -4877,8 +5015,17 @@
       <c r="CV20">
         <v>4</v>
       </c>
+      <c r="CW20">
+        <v>2</v>
+      </c>
+      <c r="CX20">
+        <v>10</v>
+      </c>
+      <c r="CY20">
+        <v>2</v>
+      </c>
     </row>
-    <row r="21" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -5071,8 +5218,14 @@
       <c r="CU21">
         <v>6</v>
       </c>
+      <c r="CW21">
+        <v>0</v>
+      </c>
+      <c r="CX21">
+        <v>6</v>
+      </c>
     </row>
-    <row r="22" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -5221,8 +5374,14 @@
       <c r="CU22">
         <v>6</v>
       </c>
+      <c r="CW22">
+        <v>0</v>
+      </c>
+      <c r="CX22">
+        <v>8</v>
+      </c>
     </row>
-    <row r="23" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -5443,8 +5602,14 @@
       <c r="CU23">
         <v>10</v>
       </c>
+      <c r="CW23">
+        <v>0</v>
+      </c>
+      <c r="CX23">
+        <v>10</v>
+      </c>
     </row>
-    <row r="24" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -5638,8 +5803,17 @@
       <c r="CU24">
         <v>4</v>
       </c>
+      <c r="CW24">
+        <v>5</v>
+      </c>
+      <c r="CX24">
+        <v>5</v>
+      </c>
+      <c r="CY24">
+        <v>2</v>
+      </c>
     </row>
-    <row r="25" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -5782,8 +5956,14 @@
       <c r="CU25">
         <v>8</v>
       </c>
+      <c r="CW25">
+        <v>0</v>
+      </c>
+      <c r="CX25">
+        <v>8</v>
+      </c>
     </row>
-    <row r="26" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -6058,8 +6238,14 @@
       <c r="CU26">
         <v>11</v>
       </c>
+      <c r="CW26">
+        <v>0</v>
+      </c>
+      <c r="CX26">
+        <v>11</v>
+      </c>
     </row>
-    <row r="27" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -6259,8 +6445,14 @@
       <c r="CU27">
         <v>6</v>
       </c>
+      <c r="CW27">
+        <v>0</v>
+      </c>
+      <c r="CX27">
+        <v>6</v>
+      </c>
     </row>
-    <row r="28" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -6499,8 +6691,14 @@
       <c r="CU28">
         <v>10</v>
       </c>
+      <c r="CW28">
+        <v>0</v>
+      </c>
+      <c r="CX28">
+        <v>10</v>
+      </c>
     </row>
-    <row r="29" spans="2:100" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:103" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>3</v>
       </c>
@@ -6709,8 +6907,14 @@
       <c r="CU29" s="3">
         <v>4</v>
       </c>
+      <c r="CW29" s="3">
+        <v>0</v>
+      </c>
+      <c r="CX29" s="3">
+        <v>4</v>
+      </c>
     </row>
-    <row r="30" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -6853,8 +7057,14 @@
       <c r="CU30">
         <v>7</v>
       </c>
+      <c r="CW30">
+        <v>0</v>
+      </c>
+      <c r="CX30">
+        <v>8</v>
+      </c>
     </row>
-    <row r="31" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -7081,8 +7291,14 @@
       <c r="CU31">
         <v>5</v>
       </c>
+      <c r="CW31">
+        <v>0</v>
+      </c>
+      <c r="CX31">
+        <v>5</v>
+      </c>
     </row>
-    <row r="32" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -7273,8 +7489,17 @@
       <c r="CU32">
         <v>6</v>
       </c>
+      <c r="CW32">
+        <v>0</v>
+      </c>
+      <c r="CX32">
+        <v>6</v>
+      </c>
+      <c r="CY32">
+        <v>4</v>
+      </c>
     </row>
-    <row r="33" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -7456,8 +7681,14 @@
       <c r="CU33">
         <v>9</v>
       </c>
+      <c r="CW33">
+        <v>0</v>
+      </c>
+      <c r="CX33">
+        <v>9</v>
+      </c>
     </row>
-    <row r="34" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -7630,8 +7861,14 @@
       <c r="CU34">
         <v>5</v>
       </c>
+      <c r="CW34">
+        <v>0</v>
+      </c>
+      <c r="CX34">
+        <v>6</v>
+      </c>
     </row>
-    <row r="35" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -7837,8 +8074,14 @@
       <c r="CU35">
         <v>8</v>
       </c>
+      <c r="CW35">
+        <v>0</v>
+      </c>
+      <c r="CX35">
+        <v>8</v>
+      </c>
     </row>
-    <row r="36" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -8044,8 +8287,14 @@
       <c r="CV36">
         <v>2</v>
       </c>
+      <c r="CW36">
+        <v>0</v>
+      </c>
+      <c r="CX36">
+        <v>10</v>
+      </c>
     </row>
-    <row r="37" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -8194,8 +8443,14 @@
       <c r="CU37">
         <v>6</v>
       </c>
+      <c r="CW37">
+        <v>0</v>
+      </c>
+      <c r="CX37">
+        <v>6</v>
+      </c>
     </row>
-    <row r="38" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -8437,8 +8692,17 @@
       <c r="CU38">
         <v>4</v>
       </c>
+      <c r="CW38">
+        <v>0</v>
+      </c>
+      <c r="CX38">
+        <v>5</v>
+      </c>
+      <c r="CY38">
+        <v>1</v>
+      </c>
     </row>
-    <row r="39" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -8665,8 +8929,14 @@
       <c r="CV39">
         <v>1</v>
       </c>
+      <c r="CW39">
+        <v>0</v>
+      </c>
+      <c r="CX39">
+        <v>6</v>
+      </c>
     </row>
-    <row r="40" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -8908,8 +9178,17 @@
       <c r="CU40">
         <v>9</v>
       </c>
+      <c r="CW40">
+        <v>0</v>
+      </c>
+      <c r="CX40">
+        <v>9</v>
+      </c>
+      <c r="CY40">
+        <v>1</v>
+      </c>
     </row>
-    <row r="41" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -9112,8 +9391,14 @@
       <c r="CU41">
         <v>6</v>
       </c>
+      <c r="CW41">
+        <v>0</v>
+      </c>
+      <c r="CX41">
+        <v>6</v>
+      </c>
     </row>
-    <row r="42" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -9265,8 +9550,14 @@
       <c r="CU42">
         <v>7</v>
       </c>
+      <c r="CW42">
+        <v>0</v>
+      </c>
+      <c r="CX42">
+        <v>7</v>
+      </c>
     </row>
-    <row r="43" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -9496,8 +9787,14 @@
       <c r="CU43">
         <v>9</v>
       </c>
+      <c r="CW43">
+        <v>0</v>
+      </c>
+      <c r="CX43">
+        <v>9</v>
+      </c>
     </row>
-    <row r="44" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -9637,8 +9934,14 @@
       <c r="CU44">
         <v>6</v>
       </c>
+      <c r="CW44">
+        <v>0</v>
+      </c>
+      <c r="CX44">
+        <v>6</v>
+      </c>
     </row>
-    <row r="45" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -9910,8 +10213,14 @@
       <c r="CU45">
         <v>9</v>
       </c>
+      <c r="CW45">
+        <v>0</v>
+      </c>
+      <c r="CX45">
+        <v>9</v>
+      </c>
     </row>
-    <row r="46" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -10057,8 +10366,14 @@
       <c r="CU46">
         <v>6</v>
       </c>
+      <c r="CW46">
+        <v>0</v>
+      </c>
+      <c r="CX46">
+        <v>6</v>
+      </c>
     </row>
-    <row r="47" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -10234,8 +10549,14 @@
       <c r="CU47">
         <v>9</v>
       </c>
+      <c r="CW47">
+        <v>0</v>
+      </c>
+      <c r="CX47">
+        <v>9</v>
+      </c>
     </row>
-    <row r="48" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -10483,8 +10804,14 @@
       <c r="CV48">
         <v>1</v>
       </c>
+      <c r="CW48">
+        <v>0</v>
+      </c>
+      <c r="CX48">
+        <v>11</v>
+      </c>
     </row>
-    <row r="49" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -10639,8 +10966,14 @@
       <c r="CU49">
         <v>7</v>
       </c>
+      <c r="CW49">
+        <v>0</v>
+      </c>
+      <c r="CX49">
+        <v>7</v>
+      </c>
     </row>
-    <row r="50" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -10891,8 +11224,17 @@
       <c r="CU50">
         <v>4</v>
       </c>
+      <c r="CW50">
+        <v>0</v>
+      </c>
+      <c r="CX50">
+        <v>6</v>
+      </c>
+      <c r="CY50">
+        <v>2</v>
+      </c>
     </row>
-    <row r="51" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -11128,8 +11470,14 @@
       <c r="CU51">
         <v>5</v>
       </c>
+      <c r="CW51">
+        <v>0</v>
+      </c>
+      <c r="CX51">
+        <v>6</v>
+      </c>
     </row>
-    <row r="52" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -11266,8 +11614,14 @@
       <c r="CV52">
         <v>2</v>
       </c>
+      <c r="CW52">
+        <v>4</v>
+      </c>
+      <c r="CY52">
+        <v>2</v>
+      </c>
     </row>
-    <row r="53" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -11476,8 +11830,14 @@
       <c r="CU53">
         <v>4</v>
       </c>
+      <c r="CW53">
+        <v>0</v>
+      </c>
+      <c r="CX53">
+        <v>4</v>
+      </c>
     </row>
-    <row r="54" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -11620,8 +11980,14 @@
       <c r="CV54">
         <v>2</v>
       </c>
+      <c r="CW54">
+        <v>0</v>
+      </c>
+      <c r="CX54">
+        <v>6</v>
+      </c>
     </row>
-    <row r="55" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -11833,8 +12199,14 @@
       <c r="CU55">
         <v>6</v>
       </c>
+      <c r="CW55">
+        <v>0</v>
+      </c>
+      <c r="CX55">
+        <v>6</v>
+      </c>
     </row>
-    <row r="56" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -11965,8 +12337,17 @@
       <c r="CT56">
         <v>10</v>
       </c>
+      <c r="CW56">
+        <v>6</v>
+      </c>
+      <c r="CX56">
+        <v>2</v>
+      </c>
+      <c r="CY56">
+        <v>2</v>
+      </c>
     </row>
-    <row r="57" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -12130,8 +12511,17 @@
       <c r="CV57">
         <v>1</v>
       </c>
+      <c r="CW57">
+        <v>0</v>
+      </c>
+      <c r="CX57">
+        <v>6</v>
+      </c>
+      <c r="CY57">
+        <v>1</v>
+      </c>
     </row>
-    <row r="58" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -12283,8 +12673,14 @@
       <c r="CV58">
         <v>1</v>
       </c>
+      <c r="CW58">
+        <v>1</v>
+      </c>
+      <c r="CX58">
+        <v>5</v>
+      </c>
     </row>
-    <row r="59" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -12430,8 +12826,14 @@
       <c r="CU59">
         <v>7</v>
       </c>
+      <c r="CW59">
+        <v>0</v>
+      </c>
+      <c r="CX59">
+        <v>7</v>
+      </c>
     </row>
-    <row r="60" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -12634,8 +13036,17 @@
       <c r="CU60">
         <v>2</v>
       </c>
+      <c r="CW60">
+        <v>6</v>
+      </c>
+      <c r="CX60">
+        <v>2</v>
+      </c>
+      <c r="CY60">
+        <v>1</v>
+      </c>
     </row>
-    <row r="61" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -12790,8 +13201,14 @@
       <c r="CU61">
         <v>7</v>
       </c>
+      <c r="CW61">
+        <v>0</v>
+      </c>
+      <c r="CX61">
+        <v>7</v>
+      </c>
     </row>
-    <row r="62" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -13027,8 +13444,14 @@
       <c r="CU62">
         <v>4</v>
       </c>
+      <c r="CW62">
+        <v>1</v>
+      </c>
+      <c r="CX62">
+        <v>4</v>
+      </c>
     </row>
-    <row r="63" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -13261,8 +13684,14 @@
       <c r="CU63">
         <v>9</v>
       </c>
+      <c r="CW63">
+        <v>0</v>
+      </c>
+      <c r="CX63">
+        <v>9</v>
+      </c>
     </row>
-    <row r="64" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -13477,8 +13906,14 @@
       <c r="CV64">
         <v>1</v>
       </c>
+      <c r="CW64">
+        <v>3</v>
+      </c>
+      <c r="CX64">
+        <v>7</v>
+      </c>
     </row>
-    <row r="65" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -13684,8 +14119,14 @@
       <c r="CU65">
         <v>6</v>
       </c>
+      <c r="CW65">
+        <v>0</v>
+      </c>
+      <c r="CX65">
+        <v>6</v>
+      </c>
     </row>
-    <row r="66" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -13834,8 +14275,14 @@
       <c r="CV66">
         <v>1</v>
       </c>
+      <c r="CW66">
+        <v>0</v>
+      </c>
+      <c r="CX66">
+        <v>5</v>
+      </c>
     </row>
-    <row r="67" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -14071,8 +14518,14 @@
       <c r="CU67">
         <v>10</v>
       </c>
+      <c r="CW67">
+        <v>0</v>
+      </c>
+      <c r="CX67">
+        <v>10</v>
+      </c>
     </row>
-    <row r="68" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -14209,8 +14662,17 @@
       <c r="CV68">
         <v>2</v>
       </c>
+      <c r="CW68">
+        <v>3</v>
+      </c>
+      <c r="CX68">
+        <v>7</v>
+      </c>
+      <c r="CY68">
+        <v>1</v>
+      </c>
     </row>
-    <row r="69" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -14356,8 +14818,14 @@
       <c r="CU69">
         <v>9</v>
       </c>
+      <c r="CW69">
+        <v>0</v>
+      </c>
+      <c r="CX69">
+        <v>9</v>
+      </c>
     </row>
-    <row r="70" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -14506,8 +14974,17 @@
       <c r="CU70">
         <v>6</v>
       </c>
+      <c r="CW70">
+        <v>0</v>
+      </c>
+      <c r="CX70">
+        <v>6</v>
+      </c>
+      <c r="CY70">
+        <v>2</v>
+      </c>
     </row>
-    <row r="71" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -14734,8 +15211,14 @@
       <c r="CU71">
         <v>10</v>
       </c>
+      <c r="CW71">
+        <v>0</v>
+      </c>
+      <c r="CX71">
+        <v>10</v>
+      </c>
     </row>
-    <row r="72" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -14950,8 +15433,14 @@
       <c r="CU72">
         <v>6</v>
       </c>
+      <c r="CW72">
+        <v>0</v>
+      </c>
+      <c r="CX72">
+        <v>7</v>
+      </c>
     </row>
-    <row r="73" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -15094,8 +15583,14 @@
       <c r="CU73">
         <v>10</v>
       </c>
+      <c r="CW73">
+        <v>0</v>
+      </c>
+      <c r="CX73">
+        <v>10</v>
+      </c>
     </row>
-    <row r="74" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -15244,8 +15739,14 @@
       <c r="CV74">
         <v>1</v>
       </c>
+      <c r="CW74">
+        <v>2</v>
+      </c>
+      <c r="CX74">
+        <v>7</v>
+      </c>
     </row>
-    <row r="75" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -15460,8 +15961,14 @@
       <c r="CV75">
         <v>1</v>
       </c>
+      <c r="CW75">
+        <v>0</v>
+      </c>
+      <c r="CX75">
+        <v>9</v>
+      </c>
     </row>
-    <row r="76" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -15700,8 +16207,14 @@
       <c r="CV76">
         <v>1</v>
       </c>
+      <c r="CW76">
+        <v>1</v>
+      </c>
+      <c r="CX76">
+        <v>7</v>
+      </c>
     </row>
-    <row r="77" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -15898,8 +16411,14 @@
       <c r="CU77">
         <v>7</v>
       </c>
+      <c r="CW77">
+        <v>0</v>
+      </c>
+      <c r="CX77">
+        <v>7</v>
+      </c>
     </row>
-    <row r="78" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -16051,8 +16570,14 @@
       <c r="CV78">
         <v>2</v>
       </c>
+      <c r="CW78">
+        <v>1</v>
+      </c>
+      <c r="CX78">
+        <v>6</v>
+      </c>
     </row>
-    <row r="79" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -16285,8 +16810,14 @@
       <c r="CU79">
         <v>9</v>
       </c>
+      <c r="CW79">
+        <v>0</v>
+      </c>
+      <c r="CX79">
+        <v>9</v>
+      </c>
     </row>
-    <row r="80" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -16489,8 +17020,17 @@
       <c r="CU80">
         <v>6</v>
       </c>
+      <c r="CW80">
+        <v>0</v>
+      </c>
+      <c r="CX80">
+        <v>6</v>
+      </c>
+      <c r="CY80">
+        <v>4</v>
+      </c>
     </row>
-    <row r="81" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -16699,8 +17239,14 @@
       <c r="CU81">
         <v>7</v>
       </c>
+      <c r="CW81">
+        <v>0</v>
+      </c>
+      <c r="CX81">
+        <v>7</v>
+      </c>
     </row>
-    <row r="82" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -16948,8 +17494,14 @@
       <c r="CU82">
         <v>10</v>
       </c>
+      <c r="CW82">
+        <v>0</v>
+      </c>
+      <c r="CX82">
+        <v>10</v>
+      </c>
     </row>
-    <row r="83" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -17179,8 +17731,14 @@
       <c r="CU83">
         <v>9</v>
       </c>
+      <c r="CW83">
+        <v>0</v>
+      </c>
+      <c r="CX83">
+        <v>9</v>
+      </c>
     </row>
-    <row r="84" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -17410,8 +17968,14 @@
       <c r="CV84">
         <v>2</v>
       </c>
+      <c r="CW84">
+        <v>0</v>
+      </c>
+      <c r="CX84">
+        <v>9</v>
+      </c>
     </row>
-    <row r="85" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -17641,8 +18205,14 @@
       <c r="CU85">
         <v>6</v>
       </c>
+      <c r="CW85">
+        <v>0</v>
+      </c>
+      <c r="CX85">
+        <v>6</v>
+      </c>
     </row>
-    <row r="86" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -17854,8 +18424,14 @@
       <c r="CU86">
         <v>8</v>
       </c>
+      <c r="CW86">
+        <v>0</v>
+      </c>
+      <c r="CX86">
+        <v>9</v>
+      </c>
     </row>
-    <row r="87" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -18091,8 +18667,14 @@
       <c r="CU87">
         <v>7</v>
       </c>
+      <c r="CW87">
+        <v>0</v>
+      </c>
+      <c r="CX87">
+        <v>7</v>
+      </c>
     </row>
-    <row r="88" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -18310,8 +18892,14 @@
       <c r="CU88">
         <v>7</v>
       </c>
+      <c r="CW88">
+        <v>0</v>
+      </c>
+      <c r="CX88">
+        <v>9</v>
+      </c>
     </row>
-    <row r="89" spans="2:100" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:102" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>3</v>
       </c>
@@ -18505,8 +19093,14 @@
       <c r="CU89" s="3">
         <v>5</v>
       </c>
+      <c r="CW89" s="3">
+        <v>0</v>
+      </c>
+      <c r="CX89" s="3">
+        <v>5</v>
+      </c>
     </row>
-    <row r="90" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -18658,8 +19252,14 @@
       <c r="CV90">
         <v>2</v>
       </c>
+      <c r="CW90">
+        <v>0</v>
+      </c>
+      <c r="CX90">
+        <v>7</v>
+      </c>
     </row>
-    <row r="91" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -18901,8 +19501,14 @@
       <c r="CU91">
         <v>6</v>
       </c>
+      <c r="CW91">
+        <v>0</v>
+      </c>
+      <c r="CX91">
+        <v>6</v>
+      </c>
     </row>
-    <row r="92" spans="2:100" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:102" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>1</v>
       </c>
@@ -19126,8 +19732,14 @@
       <c r="CV92" s="3">
         <v>1</v>
       </c>
+      <c r="CW92" s="3">
+        <v>0</v>
+      </c>
+      <c r="CX92" s="3">
+        <v>8</v>
+      </c>
     </row>
-    <row r="93" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -19306,8 +19918,14 @@
       <c r="CU93">
         <v>9</v>
       </c>
+      <c r="CW93">
+        <v>0</v>
+      </c>
+      <c r="CX93">
+        <v>9</v>
+      </c>
     </row>
-    <row r="94" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -19456,8 +20074,14 @@
       <c r="CU94">
         <v>7</v>
       </c>
+      <c r="CW94">
+        <v>0</v>
+      </c>
+      <c r="CX94">
+        <v>7</v>
+      </c>
     </row>
-    <row r="95" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -19645,8 +20269,14 @@
       <c r="CU95">
         <v>8</v>
       </c>
+      <c r="CW95">
+        <v>0</v>
+      </c>
+      <c r="CX95">
+        <v>8</v>
+      </c>
     </row>
-    <row r="96" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -19861,8 +20491,14 @@
       <c r="CV96">
         <v>4</v>
       </c>
+      <c r="CW96">
+        <v>0</v>
+      </c>
+      <c r="CX96">
+        <v>10</v>
+      </c>
     </row>
-    <row r="97" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -20014,8 +20650,14 @@
       <c r="CU97">
         <v>8</v>
       </c>
+      <c r="CW97">
+        <v>0</v>
+      </c>
+      <c r="CX97">
+        <v>8</v>
+      </c>
     </row>
-    <row r="98" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -20224,8 +20866,14 @@
       <c r="CU98">
         <v>7</v>
       </c>
+      <c r="CW98">
+        <v>0</v>
+      </c>
+      <c r="CX98">
+        <v>7</v>
+      </c>
     </row>
-    <row r="99" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -20389,8 +21037,14 @@
       <c r="CV99">
         <v>2</v>
       </c>
+      <c r="CW99">
+        <v>0</v>
+      </c>
+      <c r="CX99">
+        <v>3</v>
+      </c>
     </row>
-    <row r="100" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -20524,8 +21178,17 @@
       <c r="CU100">
         <v>1</v>
       </c>
+      <c r="CW100">
+        <v>6</v>
+      </c>
+      <c r="CX100">
+        <v>1</v>
+      </c>
+      <c r="CY100">
+        <v>1</v>
+      </c>
     </row>
-    <row r="101" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -20719,8 +21382,14 @@
       <c r="CU101">
         <v>5</v>
       </c>
+      <c r="CW101">
+        <v>0</v>
+      </c>
+      <c r="CX101">
+        <v>5</v>
+      </c>
     </row>
-    <row r="102" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -20869,8 +21538,14 @@
       <c r="CU102">
         <v>6</v>
       </c>
+      <c r="CW102">
+        <v>0</v>
+      </c>
+      <c r="CX102">
+        <v>7</v>
+      </c>
     </row>
-    <row r="103" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -21085,8 +21760,14 @@
       <c r="CU103">
         <v>6</v>
       </c>
+      <c r="CW103">
+        <v>0</v>
+      </c>
+      <c r="CX103">
+        <v>6</v>
+      </c>
     </row>
-    <row r="104" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -21298,8 +21979,14 @@
       <c r="CU104">
         <v>8</v>
       </c>
+      <c r="CW104">
+        <v>1</v>
+      </c>
+      <c r="CX104">
+        <v>9</v>
+      </c>
     </row>
-    <row r="105" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -21505,8 +22192,14 @@
       <c r="CU105">
         <v>6</v>
       </c>
+      <c r="CW105">
+        <v>0</v>
+      </c>
+      <c r="CX105">
+        <v>6</v>
+      </c>
     </row>
-    <row r="106" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -21703,8 +22396,14 @@
       <c r="CU106">
         <v>8</v>
       </c>
+      <c r="CW106">
+        <v>0</v>
+      </c>
+      <c r="CX106">
+        <v>8</v>
+      </c>
     </row>
-    <row r="107" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -21922,8 +22621,14 @@
       <c r="CU107">
         <v>5</v>
       </c>
+      <c r="CW107">
+        <v>0</v>
+      </c>
+      <c r="CX107">
+        <v>5</v>
+      </c>
     </row>
-    <row r="108" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -22126,8 +22831,14 @@
       <c r="CU108">
         <v>10</v>
       </c>
+      <c r="CW108">
+        <v>0</v>
+      </c>
+      <c r="CX108">
+        <v>10</v>
+      </c>
     </row>
-    <row r="109" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -22345,8 +23056,14 @@
       <c r="CU109">
         <v>9</v>
       </c>
+      <c r="CW109">
+        <v>0</v>
+      </c>
+      <c r="CX109">
+        <v>9</v>
+      </c>
     </row>
-    <row r="110" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -22573,8 +23290,14 @@
       <c r="CV110">
         <v>2</v>
       </c>
+      <c r="CW110">
+        <v>0</v>
+      </c>
+      <c r="CX110">
+        <v>9</v>
+      </c>
     </row>
-    <row r="111" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -22783,8 +23506,14 @@
       <c r="CU111">
         <v>8</v>
       </c>
+      <c r="CW111">
+        <v>0</v>
+      </c>
+      <c r="CX111">
+        <v>8</v>
+      </c>
     </row>
-    <row r="112" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -22999,8 +23728,14 @@
       <c r="CU112">
         <v>7</v>
       </c>
+      <c r="CW112">
+        <v>0</v>
+      </c>
+      <c r="CX112">
+        <v>8</v>
+      </c>
     </row>
-    <row r="113" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -23224,8 +23959,14 @@
       <c r="CV113">
         <v>2</v>
       </c>
+      <c r="CW113">
+        <v>0</v>
+      </c>
+      <c r="CX113">
+        <v>6</v>
+      </c>
     </row>
-    <row r="114" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -23371,8 +24112,14 @@
       <c r="CU114">
         <v>8</v>
       </c>
+      <c r="CW114">
+        <v>0</v>
+      </c>
+      <c r="CX114">
+        <v>8</v>
+      </c>
     </row>
-    <row r="115" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -23596,8 +24343,14 @@
       <c r="CU115">
         <v>4</v>
       </c>
+      <c r="CW115">
+        <v>0</v>
+      </c>
+      <c r="CX115">
+        <v>4</v>
+      </c>
     </row>
-    <row r="116" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -23806,8 +24559,14 @@
       <c r="CU116">
         <v>8</v>
       </c>
+      <c r="CW116">
+        <v>0</v>
+      </c>
+      <c r="CX116">
+        <v>8</v>
+      </c>
     </row>
-    <row r="117" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -24022,8 +24781,14 @@
       <c r="CU117">
         <v>5</v>
       </c>
+      <c r="CW117">
+        <v>0</v>
+      </c>
+      <c r="CX117">
+        <v>5</v>
+      </c>
     </row>
-    <row r="118" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -24179,8 +24944,14 @@
       <c r="CU118">
         <v>6</v>
       </c>
+      <c r="CW118">
+        <v>0</v>
+      </c>
+      <c r="CX118">
+        <v>6</v>
+      </c>
     </row>
-    <row r="119" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -24338,8 +25109,14 @@
       <c r="CU119">
         <v>7</v>
       </c>
+      <c r="CW119">
+        <v>0</v>
+      </c>
+      <c r="CX119">
+        <v>7</v>
+      </c>
     </row>
-    <row r="120" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -24488,8 +25265,14 @@
       <c r="CU120">
         <v>10</v>
       </c>
+      <c r="CW120">
+        <v>0</v>
+      </c>
+      <c r="CX120">
+        <v>10</v>
+      </c>
     </row>
-    <row r="121" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -24638,8 +25421,14 @@
       <c r="CU121">
         <v>8</v>
       </c>
+      <c r="CW121">
+        <v>0</v>
+      </c>
+      <c r="CX121">
+        <v>8</v>
+      </c>
     </row>
-    <row r="122" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -24791,8 +25580,14 @@
       <c r="CU122">
         <v>6</v>
       </c>
+      <c r="CW122">
+        <v>0</v>
+      </c>
+      <c r="CX122">
+        <v>6</v>
+      </c>
     </row>
-    <row r="123" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -24998,8 +25793,14 @@
       <c r="CV123">
         <v>3</v>
       </c>
+      <c r="CW123">
+        <v>0</v>
+      </c>
+      <c r="CX123">
+        <v>6</v>
+      </c>
     </row>
-    <row r="124" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -25247,8 +26048,14 @@
       <c r="CU124">
         <v>8</v>
       </c>
+      <c r="CW124">
+        <v>0</v>
+      </c>
+      <c r="CX124">
+        <v>8</v>
+      </c>
     </row>
-    <row r="125" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -25478,8 +26285,14 @@
       <c r="CU125">
         <v>6</v>
       </c>
+      <c r="CW125">
+        <v>0</v>
+      </c>
+      <c r="CX125">
+        <v>6</v>
+      </c>
     </row>
-    <row r="126" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -25691,8 +26504,14 @@
       <c r="CU126">
         <v>6</v>
       </c>
+      <c r="CW126">
+        <v>0</v>
+      </c>
+      <c r="CX126">
+        <v>6</v>
+      </c>
     </row>
-    <row r="127" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -25898,8 +26717,14 @@
       <c r="CU127">
         <v>3</v>
       </c>
+      <c r="CW127">
+        <v>0</v>
+      </c>
+      <c r="CX127">
+        <v>3</v>
+      </c>
     </row>
-    <row r="128" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -26036,8 +26861,14 @@
       <c r="CU128">
         <v>7</v>
       </c>
+      <c r="CW128">
+        <v>0</v>
+      </c>
+      <c r="CX128">
+        <v>7</v>
+      </c>
     </row>
-    <row r="129" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -26258,8 +27089,14 @@
       <c r="CU129">
         <v>6</v>
       </c>
+      <c r="CW129">
+        <v>0</v>
+      </c>
+      <c r="CX129">
+        <v>6</v>
+      </c>
     </row>
-    <row r="130" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -26417,8 +27254,14 @@
       <c r="CU130">
         <v>10</v>
       </c>
+      <c r="CW130">
+        <v>0</v>
+      </c>
+      <c r="CX130">
+        <v>10</v>
+      </c>
     </row>
-    <row r="131" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -26642,8 +27485,14 @@
       <c r="CU131">
         <v>10</v>
       </c>
+      <c r="CW131">
+        <v>0</v>
+      </c>
+      <c r="CX131">
+        <v>10</v>
+      </c>
     </row>
-    <row r="132" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -26789,8 +27638,14 @@
       <c r="CU132">
         <v>6</v>
       </c>
+      <c r="CW132">
+        <v>0</v>
+      </c>
+      <c r="CX132">
+        <v>6</v>
+      </c>
     </row>
-    <row r="133" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -26969,8 +27824,14 @@
       <c r="CU133">
         <v>7</v>
       </c>
+      <c r="CW133">
+        <v>0</v>
+      </c>
+      <c r="CX133">
+        <v>7</v>
+      </c>
     </row>
-    <row r="134" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -27149,8 +28010,14 @@
       <c r="CU134">
         <v>10</v>
       </c>
+      <c r="CW134">
+        <v>0</v>
+      </c>
+      <c r="CX134">
+        <v>10</v>
+      </c>
     </row>
-    <row r="135" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -27350,8 +28217,14 @@
       <c r="CU135">
         <v>8</v>
       </c>
+      <c r="CW135">
+        <v>0</v>
+      </c>
+      <c r="CX135">
+        <v>8</v>
+      </c>
     </row>
-    <row r="136" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -27545,8 +28418,14 @@
       <c r="CU136">
         <v>7</v>
       </c>
+      <c r="CW136">
+        <v>0</v>
+      </c>
+      <c r="CX136">
+        <v>7</v>
+      </c>
     </row>
-    <row r="137" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -27749,8 +28628,14 @@
       <c r="CU137">
         <v>5</v>
       </c>
+      <c r="CW137">
+        <v>0</v>
+      </c>
+      <c r="CX137">
+        <v>5</v>
+      </c>
     </row>
-    <row r="138" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -27965,8 +28850,14 @@
       <c r="CU138">
         <v>7</v>
       </c>
+      <c r="CW138">
+        <v>0</v>
+      </c>
+      <c r="CX138">
+        <v>7</v>
+      </c>
     </row>
-    <row r="139" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -28163,8 +29054,14 @@
       <c r="CU139">
         <v>5</v>
       </c>
+      <c r="CW139">
+        <v>0</v>
+      </c>
+      <c r="CX139">
+        <v>5</v>
+      </c>
     </row>
-    <row r="140" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -28316,8 +29213,14 @@
       <c r="CU140">
         <v>9</v>
       </c>
+      <c r="CW140">
+        <v>0</v>
+      </c>
+      <c r="CX140">
+        <v>9</v>
+      </c>
     </row>
-    <row r="141" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -28550,8 +29453,14 @@
       <c r="CU141">
         <v>8</v>
       </c>
+      <c r="CW141">
+        <v>0</v>
+      </c>
+      <c r="CX141">
+        <v>8</v>
+      </c>
     </row>
-    <row r="142" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -28784,8 +29693,14 @@
       <c r="CU142">
         <v>8</v>
       </c>
+      <c r="CW142">
+        <v>0</v>
+      </c>
+      <c r="CX142">
+        <v>8</v>
+      </c>
     </row>
-    <row r="143" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -28976,8 +29891,14 @@
       <c r="CU143">
         <v>11</v>
       </c>
+      <c r="CW143">
+        <v>0</v>
+      </c>
+      <c r="CX143">
+        <v>11</v>
+      </c>
     </row>
-    <row r="144" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -29120,8 +30041,14 @@
       <c r="CU144">
         <v>7</v>
       </c>
+      <c r="CW144">
+        <v>0</v>
+      </c>
+      <c r="CX144">
+        <v>7</v>
+      </c>
     </row>
-    <row r="145" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -29273,8 +30200,14 @@
       <c r="CU145">
         <v>5</v>
       </c>
+      <c r="CW145">
+        <v>0</v>
+      </c>
+      <c r="CX145">
+        <v>5</v>
+      </c>
     </row>
-    <row r="146" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -29519,8 +30452,14 @@
       <c r="CU146">
         <v>10</v>
       </c>
+      <c r="CW146">
+        <v>0</v>
+      </c>
+      <c r="CX146">
+        <v>10</v>
+      </c>
     </row>
-    <row r="147" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -29756,8 +30695,14 @@
       <c r="CV147">
         <v>1</v>
       </c>
+      <c r="CW147">
+        <v>0</v>
+      </c>
+      <c r="CX147">
+        <v>3</v>
+      </c>
     </row>
-    <row r="148" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -29885,8 +30830,14 @@
       <c r="CT148">
         <v>9</v>
       </c>
+      <c r="CW148">
+        <v>8</v>
+      </c>
+      <c r="CY148">
+        <v>1</v>
+      </c>
     </row>
-    <row r="149" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -30131,8 +31082,14 @@
       <c r="CV149">
         <v>1</v>
       </c>
+      <c r="CW149">
+        <v>0</v>
+      </c>
+      <c r="CX149">
+        <v>5</v>
+      </c>
     </row>
-    <row r="150" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -30359,8 +31316,14 @@
       <c r="CU150">
         <v>9</v>
       </c>
+      <c r="CW150">
+        <v>0</v>
+      </c>
+      <c r="CX150">
+        <v>9</v>
+      </c>
     </row>
-    <row r="151" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -30563,8 +31526,14 @@
       <c r="CU151">
         <v>10</v>
       </c>
+      <c r="CW151">
+        <v>0</v>
+      </c>
+      <c r="CX151">
+        <v>10</v>
+      </c>
     </row>
-    <row r="152" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -30704,8 +31673,14 @@
       <c r="CU152">
         <v>9</v>
       </c>
+      <c r="CW152">
+        <v>0</v>
+      </c>
+      <c r="CX152">
+        <v>9</v>
+      </c>
     </row>
-    <row r="153" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -30899,8 +31874,14 @@
       <c r="CU153">
         <v>7</v>
       </c>
+      <c r="CW153">
+        <v>0</v>
+      </c>
+      <c r="CX153">
+        <v>7</v>
+      </c>
     </row>
-    <row r="154" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -31160,8 +32141,14 @@
       <c r="CU154">
         <v>8</v>
       </c>
+      <c r="CW154">
+        <v>0</v>
+      </c>
+      <c r="CX154">
+        <v>8</v>
+      </c>
     </row>
-    <row r="155" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -31370,8 +32357,14 @@
       <c r="CU155">
         <v>9</v>
       </c>
+      <c r="CW155">
+        <v>0</v>
+      </c>
+      <c r="CX155">
+        <v>9</v>
+      </c>
     </row>
-    <row r="156" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="156" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -31517,8 +32510,14 @@
       <c r="CU156">
         <v>6</v>
       </c>
+      <c r="CW156">
+        <v>0</v>
+      </c>
+      <c r="CX156">
+        <v>6</v>
+      </c>
     </row>
-    <row r="157" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="157" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -31664,8 +32663,14 @@
       <c r="CU157">
         <v>6</v>
       </c>
+      <c r="CW157">
+        <v>0</v>
+      </c>
+      <c r="CX157">
+        <v>6</v>
+      </c>
     </row>
-    <row r="158" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="158" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -31847,8 +32852,14 @@
       <c r="CU158">
         <v>7</v>
       </c>
+      <c r="CW158">
+        <v>0</v>
+      </c>
+      <c r="CX158">
+        <v>8</v>
+      </c>
     </row>
-    <row r="159" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -32072,8 +33083,14 @@
       <c r="CU159">
         <v>5</v>
       </c>
+      <c r="CW159">
+        <v>0</v>
+      </c>
+      <c r="CX159">
+        <v>5</v>
+      </c>
     </row>
-    <row r="160" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -32210,8 +33227,17 @@
       <c r="CV160">
         <v>3</v>
       </c>
+      <c r="CW160">
+        <v>1</v>
+      </c>
+      <c r="CX160">
+        <v>7</v>
+      </c>
+      <c r="CY160">
+        <v>1</v>
+      </c>
     </row>
-    <row r="161" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -32456,8 +33482,14 @@
       <c r="CV161">
         <v>1</v>
       </c>
+      <c r="CW161">
+        <v>0</v>
+      </c>
+      <c r="CX161">
+        <v>7</v>
+      </c>
     </row>
-    <row r="162" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -32600,8 +33632,14 @@
       <c r="CU162">
         <v>8</v>
       </c>
+      <c r="CW162">
+        <v>0</v>
+      </c>
+      <c r="CX162">
+        <v>8</v>
+      </c>
     </row>
-    <row r="163" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="163" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -32804,8 +33842,14 @@
       <c r="CU163">
         <v>8</v>
       </c>
+      <c r="CW163">
+        <v>0</v>
+      </c>
+      <c r="CX163">
+        <v>8</v>
+      </c>
     </row>
-    <row r="164" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="164" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -32951,8 +33995,17 @@
       <c r="CU164">
         <v>8</v>
       </c>
+      <c r="CW164">
+        <v>0</v>
+      </c>
+      <c r="CX164">
+        <v>8</v>
+      </c>
+      <c r="CY164">
+        <v>1</v>
+      </c>
     </row>
-    <row r="165" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -33155,8 +34208,14 @@
       <c r="CU165">
         <v>6</v>
       </c>
+      <c r="CW165">
+        <v>0</v>
+      </c>
+      <c r="CX165">
+        <v>6</v>
+      </c>
     </row>
-    <row r="166" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="166" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -33344,8 +34403,14 @@
       <c r="CU166">
         <v>6</v>
       </c>
+      <c r="CW166">
+        <v>0</v>
+      </c>
+      <c r="CX166">
+        <v>6</v>
+      </c>
     </row>
-    <row r="167" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -33536,8 +34601,14 @@
       <c r="CU167">
         <v>8</v>
       </c>
+      <c r="CW167">
+        <v>0</v>
+      </c>
+      <c r="CX167">
+        <v>8</v>
+      </c>
     </row>
-    <row r="168" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -33761,8 +34832,14 @@
       <c r="CU168">
         <v>11</v>
       </c>
+      <c r="CW168">
+        <v>0</v>
+      </c>
+      <c r="CX168">
+        <v>11</v>
+      </c>
     </row>
-    <row r="169" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -33908,8 +34985,14 @@
       <c r="CU169">
         <v>6</v>
       </c>
+      <c r="CW169">
+        <v>0</v>
+      </c>
+      <c r="CX169">
+        <v>6</v>
+      </c>
     </row>
-    <row r="170" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -34079,8 +35162,14 @@
       <c r="CU170">
         <v>8</v>
       </c>
+      <c r="CW170">
+        <v>0</v>
+      </c>
+      <c r="CX170">
+        <v>8</v>
+      </c>
     </row>
-    <row r="171" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="171" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -34313,8 +35402,14 @@
       <c r="CU171">
         <v>10</v>
       </c>
+      <c r="CW171">
+        <v>0</v>
+      </c>
+      <c r="CX171">
+        <v>10</v>
+      </c>
     </row>
-    <row r="172" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -34466,8 +35561,14 @@
       <c r="CU172">
         <v>7</v>
       </c>
+      <c r="CW172">
+        <v>0</v>
+      </c>
+      <c r="CX172">
+        <v>8</v>
+      </c>
     </row>
-    <row r="173" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -34634,8 +35735,14 @@
       <c r="CU173">
         <v>8</v>
       </c>
+      <c r="CW173">
+        <v>0</v>
+      </c>
+      <c r="CX173">
+        <v>8</v>
+      </c>
     </row>
-    <row r="174" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -34787,8 +35894,14 @@
       <c r="CU174">
         <v>9</v>
       </c>
+      <c r="CW174">
+        <v>0</v>
+      </c>
+      <c r="CX174">
+        <v>9</v>
+      </c>
     </row>
-    <row r="175" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -34997,8 +36110,14 @@
       <c r="CU175">
         <v>9</v>
       </c>
+      <c r="CW175">
+        <v>0</v>
+      </c>
+      <c r="CX175">
+        <v>9</v>
+      </c>
     </row>
-    <row r="176" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="176" spans="2:103" x14ac:dyDescent="0.3">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -35141,8 +36260,14 @@
       <c r="CU176">
         <v>8</v>
       </c>
+      <c r="CW176">
+        <v>0</v>
+      </c>
+      <c r="CX176">
+        <v>8</v>
+      </c>
     </row>
-    <row r="177" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -35294,8 +36419,14 @@
       <c r="CU177">
         <v>5</v>
       </c>
+      <c r="CW177">
+        <v>0</v>
+      </c>
+      <c r="CX177">
+        <v>5</v>
+      </c>
     </row>
-    <row r="178" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -35453,8 +36584,14 @@
       <c r="CU178">
         <v>8</v>
       </c>
+      <c r="CW178">
+        <v>0</v>
+      </c>
+      <c r="CX178">
+        <v>8</v>
+      </c>
     </row>
-    <row r="179" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -35663,8 +36800,14 @@
       <c r="CU179">
         <v>10</v>
       </c>
+      <c r="CW179">
+        <v>0</v>
+      </c>
+      <c r="CX179">
+        <v>10</v>
+      </c>
     </row>
-    <row r="180" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -35870,8 +37013,14 @@
       <c r="CU180">
         <v>9</v>
       </c>
+      <c r="CW180">
+        <v>0</v>
+      </c>
+      <c r="CX180">
+        <v>9</v>
+      </c>
     </row>
-    <row r="181" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -36077,8 +37226,14 @@
       <c r="CU181">
         <v>9</v>
       </c>
+      <c r="CW181">
+        <v>0</v>
+      </c>
+      <c r="CX181">
+        <v>9</v>
+      </c>
     </row>
-    <row r="182" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -36227,8 +37382,14 @@
       <c r="CU182">
         <v>6</v>
       </c>
+      <c r="CW182">
+        <v>0</v>
+      </c>
+      <c r="CX182">
+        <v>6</v>
+      </c>
     </row>
-    <row r="183" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -36466,8 +37627,14 @@
       <c r="CU183">
         <v>5</v>
       </c>
+      <c r="CW183">
+        <v>0</v>
+      </c>
+      <c r="CX183">
+        <v>5</v>
+      </c>
     </row>
-    <row r="184" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -36624,8 +37791,14 @@
       <c r="CU184">
         <v>6</v>
       </c>
+      <c r="CW184">
+        <v>0</v>
+      </c>
+      <c r="CX184">
+        <v>6</v>
+      </c>
     </row>
-    <row r="185" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -36833,8 +38006,14 @@
       <c r="CU185">
         <v>7</v>
       </c>
+      <c r="CW185">
+        <v>0</v>
+      </c>
+      <c r="CX185">
+        <v>7</v>
+      </c>
     </row>
-    <row r="186" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -37030,8 +38209,14 @@
       <c r="CU186">
         <v>1</v>
       </c>
+      <c r="CW186">
+        <v>6</v>
+      </c>
+      <c r="CX186">
+        <v>1</v>
+      </c>
     </row>
-    <row r="187" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -37197,8 +38382,14 @@
       <c r="CU187">
         <v>8</v>
       </c>
+      <c r="CW187">
+        <v>0</v>
+      </c>
+      <c r="CX187">
+        <v>8</v>
+      </c>
     </row>
-    <row r="188" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B188" t="s">
         <v>4</v>
       </c>
@@ -37418,8 +38609,14 @@
       <c r="CV188">
         <v>1</v>
       </c>
+      <c r="CW188">
+        <v>0</v>
+      </c>
+      <c r="CX188">
+        <v>10</v>
+      </c>
     </row>
-    <row r="189" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -37633,8 +38830,14 @@
       <c r="CU189">
         <v>2</v>
       </c>
+      <c r="CW189">
+        <v>0</v>
+      </c>
+      <c r="CX189">
+        <v>2</v>
+      </c>
     </row>
-    <row r="190" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="190" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -37851,8 +39054,14 @@
       <c r="CU190">
         <v>5</v>
       </c>
+      <c r="CW190">
+        <v>0</v>
+      </c>
+      <c r="CX190">
+        <v>5</v>
+      </c>
     </row>
-    <row r="191" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="191" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -38072,8 +39281,14 @@
       <c r="CU191">
         <v>5</v>
       </c>
+      <c r="CW191">
+        <v>0</v>
+      </c>
+      <c r="CX191">
+        <v>5</v>
+      </c>
     </row>
-    <row r="192" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="192" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -38272,8 +39487,14 @@
       <c r="CU192">
         <v>3</v>
       </c>
+      <c r="CW192">
+        <v>0</v>
+      </c>
+      <c r="CX192">
+        <v>3</v>
+      </c>
     </row>
-    <row r="193" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="193" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -38496,8 +39717,14 @@
       <c r="CU193">
         <v>7</v>
       </c>
+      <c r="CW193">
+        <v>0</v>
+      </c>
+      <c r="CX193">
+        <v>7</v>
+      </c>
     </row>
-    <row r="194" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="194" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B194" t="s">
         <v>4</v>
       </c>
@@ -38696,8 +39923,14 @@
       <c r="CU194">
         <v>7</v>
       </c>
+      <c r="CW194">
+        <v>0</v>
+      </c>
+      <c r="CX194">
+        <v>7</v>
+      </c>
     </row>
-    <row r="195" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="195" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -38911,8 +40144,14 @@
       <c r="CU195">
         <v>2</v>
       </c>
+      <c r="CW195">
+        <v>0</v>
+      </c>
+      <c r="CX195">
+        <v>2</v>
+      </c>
     </row>
-    <row r="196" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="196" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -39159,8 +40398,14 @@
       <c r="CU196">
         <v>9</v>
       </c>
+      <c r="CW196">
+        <v>0</v>
+      </c>
+      <c r="CX196">
+        <v>9</v>
+      </c>
     </row>
-    <row r="197" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="197" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -39362,8 +40607,14 @@
       <c r="CU197">
         <v>4</v>
       </c>
+      <c r="CW197">
+        <v>0</v>
+      </c>
+      <c r="CX197">
+        <v>4</v>
+      </c>
     </row>
-    <row r="198" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="198" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -39547,8 +40798,14 @@
       <c r="CU198">
         <v>5</v>
       </c>
+      <c r="CW198">
+        <v>0</v>
+      </c>
+      <c r="CX198">
+        <v>5</v>
+      </c>
     </row>
-    <row r="199" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="199" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -39744,8 +41001,14 @@
       <c r="CU199">
         <v>6</v>
       </c>
+      <c r="CW199">
+        <v>0</v>
+      </c>
+      <c r="CX199">
+        <v>6</v>
+      </c>
     </row>
-    <row r="200" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="200" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
         <v>4</v>
       </c>
@@ -39938,8 +41201,14 @@
       <c r="CU200">
         <v>7</v>
       </c>
+      <c r="CW200">
+        <v>0</v>
+      </c>
+      <c r="CX200">
+        <v>7</v>
+      </c>
     </row>
-    <row r="201" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="201" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -40168,8 +41437,14 @@
       <c r="CU201">
         <v>6</v>
       </c>
+      <c r="CW201">
+        <v>0</v>
+      </c>
+      <c r="CX201">
+        <v>6</v>
+      </c>
     </row>
-    <row r="202" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="202" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -40389,8 +41664,14 @@
       <c r="CU202">
         <v>1</v>
       </c>
+      <c r="CW202">
+        <v>0</v>
+      </c>
+      <c r="CX202">
+        <v>1</v>
+      </c>
     </row>
-    <row r="203" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="203" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -40604,8 +41885,14 @@
       <c r="CU203">
         <v>3</v>
       </c>
+      <c r="CW203">
+        <v>0</v>
+      </c>
+      <c r="CX203">
+        <v>3</v>
+      </c>
     </row>
-    <row r="204" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="204" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -40729,8 +42016,11 @@
       <c r="CT204">
         <v>6</v>
       </c>
+      <c r="CW204">
+        <v>6</v>
+      </c>
     </row>
-    <row r="205" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="205" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -40965,8 +42255,14 @@
       <c r="CU205">
         <v>8</v>
       </c>
+      <c r="CW205">
+        <v>2</v>
+      </c>
+      <c r="CX205">
+        <v>8</v>
+      </c>
     </row>
-    <row r="206" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="206" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B206" t="s">
         <v>4</v>
       </c>
@@ -41105,8 +42401,14 @@
       <c r="CV206">
         <v>1</v>
       </c>
+      <c r="CW206">
+        <v>0</v>
+      </c>
+      <c r="CX206">
+        <v>6</v>
+      </c>
     </row>
-    <row r="207" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="207" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -41293,8 +42595,14 @@
       <c r="CU207">
         <v>4</v>
       </c>
+      <c r="CW207">
+        <v>0</v>
+      </c>
+      <c r="CX207">
+        <v>4</v>
+      </c>
     </row>
-    <row r="208" spans="2:100" x14ac:dyDescent="0.3">
+    <row r="208" spans="2:102" x14ac:dyDescent="0.3">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -41508,8 +42816,14 @@
       <c r="CU208">
         <v>3</v>
       </c>
+      <c r="CW208">
+        <v>0</v>
+      </c>
+      <c r="CX208">
+        <v>3</v>
+      </c>
     </row>
-    <row r="209" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="209" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B209" t="s">
         <v>3</v>
       </c>
@@ -41708,8 +43022,14 @@
       <c r="CU209">
         <v>5</v>
       </c>
+      <c r="CW209">
+        <v>0</v>
+      </c>
+      <c r="CX209">
+        <v>5</v>
+      </c>
     </row>
-    <row r="210" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="210" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B210" t="s">
         <v>1</v>
       </c>
@@ -41929,8 +43249,17 @@
       <c r="CU210">
         <v>1</v>
       </c>
+      <c r="CW210">
+        <v>0</v>
+      </c>
+      <c r="CX210">
+        <v>4</v>
+      </c>
+      <c r="CY210">
+        <v>1</v>
+      </c>
     </row>
-    <row r="211" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="211" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
         <v>4</v>
       </c>
@@ -42129,8 +43458,14 @@
       <c r="CU211">
         <v>4</v>
       </c>
+      <c r="CW211">
+        <v>1</v>
+      </c>
+      <c r="CX211">
+        <v>4</v>
+      </c>
     </row>
-    <row r="212" spans="2:99" x14ac:dyDescent="0.3">
+    <row r="212" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
         <v>4</v>
       </c>
@@ -42322,6 +43657,17 @@
       </c>
       <c r="CU212">
         <v>6</v>
+      </c>
+      <c r="CW212">
+        <v>0</v>
+      </c>
+      <c r="CX212">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="214" spans="2:105" x14ac:dyDescent="0.3">
+      <c r="DA214" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DOY 224 germinants data collection
</commit_message>
<xml_diff>
--- a/data/germination_data.xlsx
+++ b/data/germination_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temporal Ecology Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4CF0AA-D2AC-4DD6-B312-DC3AFB560E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{628D6490-0E04-4D95-8F67-7D1AFA84E6E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="144">
   <si>
     <t>seed_species</t>
   </si>
@@ -495,6 +495,15 @@
   <si>
     <t xml:space="preserve"> </t>
   </si>
+  <si>
+    <t>224_alive</t>
+  </si>
+  <si>
+    <t>224_halfdead2</t>
+  </si>
+  <si>
+    <t>224_dead</t>
+  </si>
 </sst>
 </file>
 
@@ -598,9 +607,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:CY213" totalsRowShown="0">
-  <autoFilter ref="B2:CY213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
-  <tableColumns count="102">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:DB213" totalsRowShown="0">
+  <autoFilter ref="B2:DB213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
+  <tableColumns count="105">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
     <tableColumn id="3" xr3:uid="{B695F4B4-8561-9D48-9FF3-12A40CB2B7C7}" name="inoculated_%"/>
@@ -703,6 +712,9 @@
     <tableColumn id="100" xr3:uid="{3B2AF124-4421-47CA-8DE0-0702AB08EBA4}" name="210_alive"/>
     <tableColumn id="101" xr3:uid="{89EA52E1-8A22-4896-9795-5647630F196D}" name="210_dead"/>
     <tableColumn id="102" xr3:uid="{590F0C34-0381-42D4-A386-55EA13C347CD}" name="210_halfdead"/>
+    <tableColumn id="103" xr3:uid="{CE80CE81-DB3D-432B-8E99-37C858ECEC0B}" name="224_alive"/>
+    <tableColumn id="104" xr3:uid="{796333B4-43FF-4338-B0FA-638B1B0DF92E}" name="224_dead"/>
+    <tableColumn id="105" xr3:uid="{652C9F16-4173-4432-AABD-63C40291A31C}" name="224_halfdead2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1025,7 +1037,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:DA214"/>
+  <dimension ref="B2:DB214"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -1033,7 +1045,7 @@
     <col min="4" max="4" width="17.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -1340,8 +1352,17 @@
       <c r="CY2" t="s">
         <v>139</v>
       </c>
+      <c r="CZ2" t="s">
+        <v>141</v>
+      </c>
+      <c r="DA2" t="s">
+        <v>143</v>
+      </c>
+      <c r="DB2" t="s">
+        <v>142</v>
+      </c>
     </row>
-    <row r="3" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1576,8 +1597,14 @@
       <c r="CX3">
         <v>4</v>
       </c>
+      <c r="CZ3">
+        <v>0</v>
+      </c>
+      <c r="DA3">
+        <v>4</v>
+      </c>
     </row>
-    <row r="4" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1713,8 +1740,11 @@
       <c r="CY4">
         <v>1</v>
       </c>
+      <c r="CZ4">
+        <v>9</v>
+      </c>
     </row>
-    <row r="5" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1946,8 +1976,14 @@
       <c r="CX5">
         <v>7</v>
       </c>
+      <c r="CZ5">
+        <v>0</v>
+      </c>
+      <c r="DA5">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -2095,8 +2131,14 @@
       <c r="CY6">
         <v>1</v>
       </c>
+      <c r="CZ6">
+        <v>0</v>
+      </c>
+      <c r="DA6">
+        <v>9</v>
+      </c>
     </row>
-    <row r="7" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -2295,8 +2337,14 @@
       <c r="CX7">
         <v>6</v>
       </c>
+      <c r="CZ7">
+        <v>0</v>
+      </c>
+      <c r="DA7">
+        <v>6</v>
+      </c>
     </row>
-    <row r="8" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -2522,8 +2570,14 @@
       <c r="CY8">
         <v>2</v>
       </c>
+      <c r="CZ8">
+        <v>1</v>
+      </c>
+      <c r="DA8">
+        <v>6</v>
+      </c>
     </row>
-    <row r="9" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2755,8 +2809,14 @@
       <c r="CX9">
         <v>7</v>
       </c>
+      <c r="CZ9">
+        <v>0</v>
+      </c>
+      <c r="DA9">
+        <v>7</v>
+      </c>
     </row>
-    <row r="10" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -2925,8 +2985,14 @@
       <c r="CX10">
         <v>6</v>
       </c>
+      <c r="CZ10">
+        <v>2</v>
+      </c>
+      <c r="DA10">
+        <v>6</v>
+      </c>
     </row>
-    <row r="11" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -3155,8 +3221,14 @@
       <c r="CX11">
         <v>8</v>
       </c>
+      <c r="CZ11">
+        <v>0</v>
+      </c>
+      <c r="DA11">
+        <v>8</v>
+      </c>
     </row>
-    <row r="12" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -3391,8 +3463,17 @@
       <c r="CY12">
         <v>1</v>
       </c>
+      <c r="CZ12">
+        <v>4</v>
+      </c>
+      <c r="DA12">
+        <v>5</v>
+      </c>
+      <c r="DB12">
+        <v>1</v>
+      </c>
     </row>
-    <row r="13" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -3615,8 +3696,14 @@
       <c r="CX13">
         <v>7</v>
       </c>
+      <c r="CZ13">
+        <v>0</v>
+      </c>
+      <c r="DA13">
+        <v>7</v>
+      </c>
     </row>
-    <row r="14" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -3803,8 +3890,17 @@
       <c r="CX14">
         <v>8</v>
       </c>
+      <c r="CZ14">
+        <v>0</v>
+      </c>
+      <c r="DA14">
+        <v>8</v>
+      </c>
+      <c r="DB14">
+        <v>1</v>
+      </c>
     </row>
-    <row r="15" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -4016,8 +4112,14 @@
       <c r="CX15">
         <v>8</v>
       </c>
+      <c r="CZ15">
+        <v>0</v>
+      </c>
+      <c r="DA15">
+        <v>8</v>
+      </c>
     </row>
-    <row r="16" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -4223,8 +4325,14 @@
       <c r="CY16">
         <v>1</v>
       </c>
+      <c r="CZ16">
+        <v>3</v>
+      </c>
+      <c r="DA16">
+        <v>6</v>
+      </c>
     </row>
-    <row r="17" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -4439,8 +4547,14 @@
       <c r="CX17">
         <v>8</v>
       </c>
+      <c r="CZ17">
+        <v>0</v>
+      </c>
+      <c r="DA17">
+        <v>8</v>
+      </c>
     </row>
-    <row r="18" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -4586,8 +4700,14 @@
       <c r="CX18">
         <v>10</v>
       </c>
+      <c r="CZ18">
+        <v>0</v>
+      </c>
+      <c r="DA18">
+        <v>10</v>
+      </c>
     </row>
-    <row r="19" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -4820,8 +4940,14 @@
       <c r="CX19">
         <v>7</v>
       </c>
+      <c r="CZ19">
+        <v>0</v>
+      </c>
+      <c r="DA19">
+        <v>7</v>
+      </c>
     </row>
-    <row r="20" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -5024,8 +5150,17 @@
       <c r="CY20">
         <v>2</v>
       </c>
+      <c r="CZ20">
+        <v>0</v>
+      </c>
+      <c r="DA20">
+        <v>13</v>
+      </c>
+      <c r="DB20">
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -5224,8 +5359,14 @@
       <c r="CX21">
         <v>6</v>
       </c>
+      <c r="CZ21">
+        <v>0</v>
+      </c>
+      <c r="DA21">
+        <v>6</v>
+      </c>
     </row>
-    <row r="22" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -5380,8 +5521,14 @@
       <c r="CX22">
         <v>8</v>
       </c>
+      <c r="CZ22">
+        <v>0</v>
+      </c>
+      <c r="DA22">
+        <v>8</v>
+      </c>
     </row>
-    <row r="23" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -5608,8 +5755,14 @@
       <c r="CX23">
         <v>10</v>
       </c>
+      <c r="CZ23">
+        <v>0</v>
+      </c>
+      <c r="DA23">
+        <v>10</v>
+      </c>
     </row>
-    <row r="24" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -5812,8 +5965,17 @@
       <c r="CY24">
         <v>2</v>
       </c>
+      <c r="CZ24">
+        <v>1</v>
+      </c>
+      <c r="DA24">
+        <v>9</v>
+      </c>
+      <c r="DB24">
+        <v>2</v>
+      </c>
     </row>
-    <row r="25" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -5962,8 +6124,14 @@
       <c r="CX25">
         <v>8</v>
       </c>
+      <c r="CZ25">
+        <v>0</v>
+      </c>
+      <c r="DA25">
+        <v>8</v>
+      </c>
     </row>
-    <row r="26" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -6244,8 +6412,14 @@
       <c r="CX26">
         <v>11</v>
       </c>
+      <c r="CZ26">
+        <v>0</v>
+      </c>
+      <c r="DA26">
+        <v>11</v>
+      </c>
     </row>
-    <row r="27" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -6451,8 +6625,14 @@
       <c r="CX27">
         <v>6</v>
       </c>
+      <c r="CZ27">
+        <v>0</v>
+      </c>
+      <c r="DA27">
+        <v>6</v>
+      </c>
     </row>
-    <row r="28" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -6697,8 +6877,14 @@
       <c r="CX28">
         <v>10</v>
       </c>
+      <c r="CZ28">
+        <v>0</v>
+      </c>
+      <c r="DA28">
+        <v>10</v>
+      </c>
     </row>
-    <row r="29" spans="2:103" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:106" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>3</v>
       </c>
@@ -6913,8 +7099,14 @@
       <c r="CX29" s="3">
         <v>4</v>
       </c>
+      <c r="CZ29" s="3">
+        <v>0</v>
+      </c>
+      <c r="DA29" s="3">
+        <v>4</v>
+      </c>
     </row>
-    <row r="30" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -7063,8 +7255,14 @@
       <c r="CX30">
         <v>8</v>
       </c>
+      <c r="CZ30">
+        <v>0</v>
+      </c>
+      <c r="DA30">
+        <v>8</v>
+      </c>
     </row>
-    <row r="31" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -7297,8 +7495,14 @@
       <c r="CX31">
         <v>5</v>
       </c>
+      <c r="CZ31">
+        <v>0</v>
+      </c>
+      <c r="DA31">
+        <v>5</v>
+      </c>
     </row>
-    <row r="32" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -7498,8 +7702,14 @@
       <c r="CY32">
         <v>4</v>
       </c>
+      <c r="CZ32">
+        <v>0</v>
+      </c>
+      <c r="DA32">
+        <v>10</v>
+      </c>
     </row>
-    <row r="33" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -7687,8 +7897,14 @@
       <c r="CX33">
         <v>9</v>
       </c>
+      <c r="CZ33">
+        <v>0</v>
+      </c>
+      <c r="DA33">
+        <v>9</v>
+      </c>
     </row>
-    <row r="34" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -7867,8 +8083,14 @@
       <c r="CX34">
         <v>6</v>
       </c>
+      <c r="CZ34">
+        <v>0</v>
+      </c>
+      <c r="DA34">
+        <v>6</v>
+      </c>
     </row>
-    <row r="35" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -8080,8 +8302,14 @@
       <c r="CX35">
         <v>8</v>
       </c>
+      <c r="CZ35">
+        <v>0</v>
+      </c>
+      <c r="DA35">
+        <v>8</v>
+      </c>
     </row>
-    <row r="36" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -8293,8 +8521,14 @@
       <c r="CX36">
         <v>10</v>
       </c>
+      <c r="CZ36">
+        <v>0</v>
+      </c>
+      <c r="DA36">
+        <v>10</v>
+      </c>
     </row>
-    <row r="37" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -8449,8 +8683,14 @@
       <c r="CX37">
         <v>6</v>
       </c>
+      <c r="CZ37">
+        <v>0</v>
+      </c>
+      <c r="DA37">
+        <v>6</v>
+      </c>
     </row>
-    <row r="38" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -8701,8 +8941,14 @@
       <c r="CY38">
         <v>1</v>
       </c>
+      <c r="CZ38">
+        <v>0</v>
+      </c>
+      <c r="DA38">
+        <v>6</v>
+      </c>
     </row>
-    <row r="39" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -8935,8 +9181,14 @@
       <c r="CX39">
         <v>6</v>
       </c>
+      <c r="CZ39">
+        <v>0</v>
+      </c>
+      <c r="DA39">
+        <v>6</v>
+      </c>
     </row>
-    <row r="40" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -9187,8 +9439,14 @@
       <c r="CY40">
         <v>1</v>
       </c>
+      <c r="CZ40">
+        <v>0</v>
+      </c>
+      <c r="DA40">
+        <v>10</v>
+      </c>
     </row>
-    <row r="41" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -9397,8 +9655,14 @@
       <c r="CX41">
         <v>6</v>
       </c>
+      <c r="CZ41">
+        <v>0</v>
+      </c>
+      <c r="DA41">
+        <v>6</v>
+      </c>
     </row>
-    <row r="42" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -9556,8 +9820,14 @@
       <c r="CX42">
         <v>7</v>
       </c>
+      <c r="CZ42">
+        <v>0</v>
+      </c>
+      <c r="DA42">
+        <v>7</v>
+      </c>
     </row>
-    <row r="43" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -9793,8 +10063,14 @@
       <c r="CX43">
         <v>9</v>
       </c>
+      <c r="CZ43">
+        <v>0</v>
+      </c>
+      <c r="DA43">
+        <v>9</v>
+      </c>
     </row>
-    <row r="44" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -9940,8 +10216,14 @@
       <c r="CX44">
         <v>6</v>
       </c>
+      <c r="CZ44">
+        <v>0</v>
+      </c>
+      <c r="DA44">
+        <v>6</v>
+      </c>
     </row>
-    <row r="45" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -10219,8 +10501,14 @@
       <c r="CX45">
         <v>9</v>
       </c>
+      <c r="CZ45">
+        <v>0</v>
+      </c>
+      <c r="DA45">
+        <v>9</v>
+      </c>
     </row>
-    <row r="46" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -10372,8 +10660,14 @@
       <c r="CX46">
         <v>6</v>
       </c>
+      <c r="CZ46">
+        <v>0</v>
+      </c>
+      <c r="DA46">
+        <v>6</v>
+      </c>
     </row>
-    <row r="47" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -10555,8 +10849,14 @@
       <c r="CX47">
         <v>9</v>
       </c>
+      <c r="CZ47">
+        <v>0</v>
+      </c>
+      <c r="DA47">
+        <v>9</v>
+      </c>
     </row>
-    <row r="48" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -10810,8 +11110,14 @@
       <c r="CX48">
         <v>11</v>
       </c>
+      <c r="CZ48">
+        <v>0</v>
+      </c>
+      <c r="DA48">
+        <v>11</v>
+      </c>
     </row>
-    <row r="49" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -10972,8 +11278,14 @@
       <c r="CX49">
         <v>7</v>
       </c>
+      <c r="CZ49">
+        <v>0</v>
+      </c>
+      <c r="DA49">
+        <v>7</v>
+      </c>
     </row>
-    <row r="50" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -11233,8 +11545,14 @@
       <c r="CY50">
         <v>2</v>
       </c>
+      <c r="CZ50">
+        <v>0</v>
+      </c>
+      <c r="DA50">
+        <v>8</v>
+      </c>
     </row>
-    <row r="51" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -11476,8 +11794,14 @@
       <c r="CX51">
         <v>6</v>
       </c>
+      <c r="CZ51">
+        <v>0</v>
+      </c>
+      <c r="DA51">
+        <v>6</v>
+      </c>
     </row>
-    <row r="52" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -11620,8 +11944,11 @@
       <c r="CY52">
         <v>2</v>
       </c>
+      <c r="CZ52">
+        <v>6</v>
+      </c>
     </row>
-    <row r="53" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -11836,8 +12163,14 @@
       <c r="CX53">
         <v>4</v>
       </c>
+      <c r="CZ53">
+        <v>0</v>
+      </c>
+      <c r="DA53">
+        <v>4</v>
+      </c>
     </row>
-    <row r="54" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -11986,8 +12319,14 @@
       <c r="CX54">
         <v>6</v>
       </c>
+      <c r="CZ54">
+        <v>0</v>
+      </c>
+      <c r="DA54">
+        <v>6</v>
+      </c>
     </row>
-    <row r="55" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -12205,8 +12544,14 @@
       <c r="CX55">
         <v>6</v>
       </c>
+      <c r="CZ55">
+        <v>0</v>
+      </c>
+      <c r="DA55">
+        <v>6</v>
+      </c>
     </row>
-    <row r="56" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -12346,8 +12691,17 @@
       <c r="CY56">
         <v>2</v>
       </c>
+      <c r="CZ56">
+        <v>2</v>
+      </c>
+      <c r="DA56">
+        <v>5</v>
+      </c>
+      <c r="DB56">
+        <v>3</v>
+      </c>
     </row>
-    <row r="57" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -12520,8 +12874,14 @@
       <c r="CY57">
         <v>1</v>
       </c>
+      <c r="CZ57">
+        <v>0</v>
+      </c>
+      <c r="DA57">
+        <v>7</v>
+      </c>
     </row>
-    <row r="58" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -12679,8 +13039,14 @@
       <c r="CX58">
         <v>5</v>
       </c>
+      <c r="CZ58">
+        <v>1</v>
+      </c>
+      <c r="DA58">
+        <v>5</v>
+      </c>
     </row>
-    <row r="59" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -12832,8 +13198,14 @@
       <c r="CX59">
         <v>7</v>
       </c>
+      <c r="CZ59">
+        <v>0</v>
+      </c>
+      <c r="DA59">
+        <v>7</v>
+      </c>
     </row>
-    <row r="60" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -13045,8 +13417,17 @@
       <c r="CY60">
         <v>1</v>
       </c>
+      <c r="CZ60">
+        <v>1</v>
+      </c>
+      <c r="DA60">
+        <v>6</v>
+      </c>
+      <c r="DB60">
+        <v>2</v>
+      </c>
     </row>
-    <row r="61" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -13207,8 +13588,14 @@
       <c r="CX61">
         <v>7</v>
       </c>
+      <c r="CZ61">
+        <v>0</v>
+      </c>
+      <c r="DA61">
+        <v>7</v>
+      </c>
     </row>
-    <row r="62" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -13450,8 +13837,14 @@
       <c r="CX62">
         <v>4</v>
       </c>
+      <c r="CZ62">
+        <v>1</v>
+      </c>
+      <c r="DA62">
+        <v>4</v>
+      </c>
     </row>
-    <row r="63" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -13690,8 +14083,14 @@
       <c r="CX63">
         <v>9</v>
       </c>
+      <c r="CZ63">
+        <v>0</v>
+      </c>
+      <c r="DA63">
+        <v>9</v>
+      </c>
     </row>
-    <row r="64" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -13912,8 +14311,14 @@
       <c r="CX64">
         <v>7</v>
       </c>
+      <c r="CZ64">
+        <v>3</v>
+      </c>
+      <c r="DA64">
+        <v>7</v>
+      </c>
     </row>
-    <row r="65" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -14125,8 +14530,14 @@
       <c r="CX65">
         <v>6</v>
       </c>
+      <c r="CZ65">
+        <v>0</v>
+      </c>
+      <c r="DA65">
+        <v>6</v>
+      </c>
     </row>
-    <row r="66" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -14281,8 +14692,14 @@
       <c r="CX66">
         <v>5</v>
       </c>
+      <c r="CZ66">
+        <v>0</v>
+      </c>
+      <c r="DA66">
+        <v>5</v>
+      </c>
     </row>
-    <row r="67" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -14524,8 +14941,14 @@
       <c r="CX67">
         <v>10</v>
       </c>
+      <c r="CZ67">
+        <v>0</v>
+      </c>
+      <c r="DA67">
+        <v>10</v>
+      </c>
     </row>
-    <row r="68" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -14671,8 +15094,17 @@
       <c r="CY68">
         <v>1</v>
       </c>
+      <c r="CZ68">
+        <v>0</v>
+      </c>
+      <c r="DA68">
+        <v>10</v>
+      </c>
+      <c r="DB68">
+        <v>1</v>
+      </c>
     </row>
-    <row r="69" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -14824,8 +15256,14 @@
       <c r="CX69">
         <v>9</v>
       </c>
+      <c r="CZ69">
+        <v>0</v>
+      </c>
+      <c r="DA69">
+        <v>9</v>
+      </c>
     </row>
-    <row r="70" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -14983,8 +15421,17 @@
       <c r="CY70">
         <v>2</v>
       </c>
+      <c r="CZ70">
+        <v>0</v>
+      </c>
+      <c r="DA70">
+        <v>7</v>
+      </c>
+      <c r="DB70">
+        <v>1</v>
+      </c>
     </row>
-    <row r="71" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -15217,8 +15664,14 @@
       <c r="CX71">
         <v>10</v>
       </c>
+      <c r="CZ71">
+        <v>0</v>
+      </c>
+      <c r="DA71">
+        <v>10</v>
+      </c>
     </row>
-    <row r="72" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -15439,8 +15892,14 @@
       <c r="CX72">
         <v>7</v>
       </c>
+      <c r="CZ72">
+        <v>0</v>
+      </c>
+      <c r="DA72">
+        <v>7</v>
+      </c>
     </row>
-    <row r="73" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -15589,8 +16048,14 @@
       <c r="CX73">
         <v>10</v>
       </c>
+      <c r="CZ73">
+        <v>0</v>
+      </c>
+      <c r="DA73">
+        <v>10</v>
+      </c>
     </row>
-    <row r="74" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -15745,8 +16210,14 @@
       <c r="CX74">
         <v>7</v>
       </c>
+      <c r="CZ74">
+        <v>0</v>
+      </c>
+      <c r="DA74">
+        <v>9</v>
+      </c>
     </row>
-    <row r="75" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -15967,8 +16438,14 @@
       <c r="CX75">
         <v>9</v>
       </c>
+      <c r="CZ75">
+        <v>0</v>
+      </c>
+      <c r="DA75">
+        <v>9</v>
+      </c>
     </row>
-    <row r="76" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -16213,8 +16690,14 @@
       <c r="CX76">
         <v>7</v>
       </c>
+      <c r="CZ76">
+        <v>1</v>
+      </c>
+      <c r="DA76">
+        <v>7</v>
+      </c>
     </row>
-    <row r="77" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -16417,8 +16900,14 @@
       <c r="CX77">
         <v>7</v>
       </c>
+      <c r="CZ77">
+        <v>0</v>
+      </c>
+      <c r="DA77">
+        <v>7</v>
+      </c>
     </row>
-    <row r="78" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -16576,8 +17065,14 @@
       <c r="CX78">
         <v>6</v>
       </c>
+      <c r="CZ78">
+        <v>0</v>
+      </c>
+      <c r="DA78">
+        <v>7</v>
+      </c>
     </row>
-    <row r="79" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -16816,8 +17311,14 @@
       <c r="CX79">
         <v>9</v>
       </c>
+      <c r="CZ79">
+        <v>0</v>
+      </c>
+      <c r="DA79">
+        <v>9</v>
+      </c>
     </row>
-    <row r="80" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -17029,8 +17530,14 @@
       <c r="CY80">
         <v>4</v>
       </c>
+      <c r="CZ80">
+        <v>0</v>
+      </c>
+      <c r="DA80">
+        <v>10</v>
+      </c>
     </row>
-    <row r="81" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -17245,8 +17752,14 @@
       <c r="CX81">
         <v>7</v>
       </c>
+      <c r="CZ81">
+        <v>0</v>
+      </c>
+      <c r="DA81">
+        <v>7</v>
+      </c>
     </row>
-    <row r="82" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -17500,8 +18013,14 @@
       <c r="CX82">
         <v>10</v>
       </c>
+      <c r="CZ82">
+        <v>0</v>
+      </c>
+      <c r="DA82">
+        <v>10</v>
+      </c>
     </row>
-    <row r="83" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -17737,8 +18256,14 @@
       <c r="CX83">
         <v>9</v>
       </c>
+      <c r="CZ83">
+        <v>0</v>
+      </c>
+      <c r="DA83">
+        <v>9</v>
+      </c>
     </row>
-    <row r="84" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -17974,8 +18499,14 @@
       <c r="CX84">
         <v>9</v>
       </c>
+      <c r="CZ84">
+        <v>0</v>
+      </c>
+      <c r="DA84">
+        <v>9</v>
+      </c>
     </row>
-    <row r="85" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -18211,8 +18742,14 @@
       <c r="CX85">
         <v>6</v>
       </c>
+      <c r="CZ85">
+        <v>0</v>
+      </c>
+      <c r="DA85">
+        <v>6</v>
+      </c>
     </row>
-    <row r="86" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -18430,8 +18967,14 @@
       <c r="CX86">
         <v>9</v>
       </c>
+      <c r="CZ86">
+        <v>0</v>
+      </c>
+      <c r="DA86">
+        <v>9</v>
+      </c>
     </row>
-    <row r="87" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -18673,8 +19216,14 @@
       <c r="CX87">
         <v>7</v>
       </c>
+      <c r="CZ87">
+        <v>0</v>
+      </c>
+      <c r="DA87">
+        <v>7</v>
+      </c>
     </row>
-    <row r="88" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -18898,8 +19447,14 @@
       <c r="CX88">
         <v>9</v>
       </c>
+      <c r="CZ88">
+        <v>0</v>
+      </c>
+      <c r="DA88">
+        <v>9</v>
+      </c>
     </row>
-    <row r="89" spans="2:102" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:105" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>3</v>
       </c>
@@ -19099,8 +19654,14 @@
       <c r="CX89" s="3">
         <v>5</v>
       </c>
+      <c r="CZ89" s="3">
+        <v>0</v>
+      </c>
+      <c r="DA89" s="3">
+        <v>5</v>
+      </c>
     </row>
-    <row r="90" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -19258,8 +19819,14 @@
       <c r="CX90">
         <v>7</v>
       </c>
+      <c r="CZ90">
+        <v>0</v>
+      </c>
+      <c r="DA90">
+        <v>7</v>
+      </c>
     </row>
-    <row r="91" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -19507,8 +20074,14 @@
       <c r="CX91">
         <v>6</v>
       </c>
+      <c r="CZ91">
+        <v>0</v>
+      </c>
+      <c r="DA91">
+        <v>6</v>
+      </c>
     </row>
-    <row r="92" spans="2:102" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:105" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>1</v>
       </c>
@@ -19738,8 +20311,14 @@
       <c r="CX92" s="3">
         <v>8</v>
       </c>
+      <c r="CZ92" s="3">
+        <v>0</v>
+      </c>
+      <c r="DA92" s="3">
+        <v>8</v>
+      </c>
     </row>
-    <row r="93" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -19924,8 +20503,14 @@
       <c r="CX93">
         <v>9</v>
       </c>
+      <c r="CZ93">
+        <v>0</v>
+      </c>
+      <c r="DA93">
+        <v>9</v>
+      </c>
     </row>
-    <row r="94" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -20080,8 +20665,14 @@
       <c r="CX94">
         <v>7</v>
       </c>
+      <c r="CZ94">
+        <v>0</v>
+      </c>
+      <c r="DA94">
+        <v>7</v>
+      </c>
     </row>
-    <row r="95" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -20275,8 +20866,14 @@
       <c r="CX95">
         <v>8</v>
       </c>
+      <c r="CZ95">
+        <v>0</v>
+      </c>
+      <c r="DA95">
+        <v>8</v>
+      </c>
     </row>
-    <row r="96" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -20497,8 +21094,14 @@
       <c r="CX96">
         <v>10</v>
       </c>
+      <c r="CZ96">
+        <v>0</v>
+      </c>
+      <c r="DA96">
+        <v>10</v>
+      </c>
     </row>
-    <row r="97" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -20656,8 +21259,14 @@
       <c r="CX97">
         <v>8</v>
       </c>
+      <c r="CZ97">
+        <v>0</v>
+      </c>
+      <c r="DA97">
+        <v>8</v>
+      </c>
     </row>
-    <row r="98" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -20872,8 +21481,14 @@
       <c r="CX98">
         <v>7</v>
       </c>
+      <c r="CZ98">
+        <v>0</v>
+      </c>
+      <c r="DA98">
+        <v>7</v>
+      </c>
     </row>
-    <row r="99" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -21043,8 +21658,14 @@
       <c r="CX99">
         <v>3</v>
       </c>
+      <c r="CZ99">
+        <v>0</v>
+      </c>
+      <c r="DA99">
+        <v>3</v>
+      </c>
     </row>
-    <row r="100" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -21187,8 +21808,14 @@
       <c r="CY100">
         <v>1</v>
       </c>
+      <c r="CZ100">
+        <v>3</v>
+      </c>
+      <c r="DA100">
+        <v>5</v>
+      </c>
     </row>
-    <row r="101" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -21388,8 +22015,14 @@
       <c r="CX101">
         <v>5</v>
       </c>
+      <c r="CZ101">
+        <v>0</v>
+      </c>
+      <c r="DA101">
+        <v>5</v>
+      </c>
     </row>
-    <row r="102" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -21544,8 +22177,14 @@
       <c r="CX102">
         <v>7</v>
       </c>
+      <c r="CZ102">
+        <v>0</v>
+      </c>
+      <c r="DA102">
+        <v>7</v>
+      </c>
     </row>
-    <row r="103" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -21766,8 +22405,14 @@
       <c r="CX103">
         <v>6</v>
       </c>
+      <c r="CZ103">
+        <v>0</v>
+      </c>
+      <c r="DA103">
+        <v>6</v>
+      </c>
     </row>
-    <row r="104" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -21985,8 +22630,14 @@
       <c r="CX104">
         <v>9</v>
       </c>
+      <c r="CZ104">
+        <v>0</v>
+      </c>
+      <c r="DA104">
+        <v>10</v>
+      </c>
     </row>
-    <row r="105" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -22198,8 +22849,14 @@
       <c r="CX105">
         <v>6</v>
       </c>
+      <c r="CZ105">
+        <v>0</v>
+      </c>
+      <c r="DA105">
+        <v>6</v>
+      </c>
     </row>
-    <row r="106" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -22402,8 +23059,14 @@
       <c r="CX106">
         <v>8</v>
       </c>
+      <c r="CZ106">
+        <v>0</v>
+      </c>
+      <c r="DA106">
+        <v>8</v>
+      </c>
     </row>
-    <row r="107" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -22627,8 +23290,14 @@
       <c r="CX107">
         <v>5</v>
       </c>
+      <c r="CZ107">
+        <v>0</v>
+      </c>
+      <c r="DA107">
+        <v>5</v>
+      </c>
     </row>
-    <row r="108" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -22837,8 +23506,14 @@
       <c r="CX108">
         <v>10</v>
       </c>
+      <c r="CZ108">
+        <v>0</v>
+      </c>
+      <c r="DA108">
+        <v>10</v>
+      </c>
     </row>
-    <row r="109" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -23062,8 +23737,14 @@
       <c r="CX109">
         <v>9</v>
       </c>
+      <c r="CZ109">
+        <v>0</v>
+      </c>
+      <c r="DA109">
+        <v>9</v>
+      </c>
     </row>
-    <row r="110" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -23296,8 +23977,14 @@
       <c r="CX110">
         <v>9</v>
       </c>
+      <c r="CZ110">
+        <v>0</v>
+      </c>
+      <c r="DA110">
+        <v>9</v>
+      </c>
     </row>
-    <row r="111" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -23512,8 +24199,14 @@
       <c r="CX111">
         <v>8</v>
       </c>
+      <c r="CZ111">
+        <v>0</v>
+      </c>
+      <c r="DA111">
+        <v>8</v>
+      </c>
     </row>
-    <row r="112" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -23734,8 +24427,14 @@
       <c r="CX112">
         <v>8</v>
       </c>
+      <c r="CZ112">
+        <v>0</v>
+      </c>
+      <c r="DA112">
+        <v>8</v>
+      </c>
     </row>
-    <row r="113" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -23965,8 +24664,14 @@
       <c r="CX113">
         <v>6</v>
       </c>
+      <c r="CZ113">
+        <v>0</v>
+      </c>
+      <c r="DA113">
+        <v>6</v>
+      </c>
     </row>
-    <row r="114" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -24118,8 +24823,14 @@
       <c r="CX114">
         <v>8</v>
       </c>
+      <c r="CZ114">
+        <v>0</v>
+      </c>
+      <c r="DA114">
+        <v>8</v>
+      </c>
     </row>
-    <row r="115" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -24349,8 +25060,14 @@
       <c r="CX115">
         <v>4</v>
       </c>
+      <c r="CZ115">
+        <v>0</v>
+      </c>
+      <c r="DA115">
+        <v>4</v>
+      </c>
     </row>
-    <row r="116" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -24565,8 +25282,14 @@
       <c r="CX116">
         <v>8</v>
       </c>
+      <c r="CZ116">
+        <v>0</v>
+      </c>
+      <c r="DA116">
+        <v>8</v>
+      </c>
     </row>
-    <row r="117" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -24787,8 +25510,14 @@
       <c r="CX117">
         <v>5</v>
       </c>
+      <c r="CZ117">
+        <v>0</v>
+      </c>
+      <c r="DA117">
+        <v>5</v>
+      </c>
     </row>
-    <row r="118" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -24950,8 +25679,14 @@
       <c r="CX118">
         <v>6</v>
       </c>
+      <c r="CZ118">
+        <v>0</v>
+      </c>
+      <c r="DA118">
+        <v>6</v>
+      </c>
     </row>
-    <row r="119" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -25115,8 +25850,14 @@
       <c r="CX119">
         <v>7</v>
       </c>
+      <c r="CZ119">
+        <v>0</v>
+      </c>
+      <c r="DA119">
+        <v>7</v>
+      </c>
     </row>
-    <row r="120" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -25271,8 +26012,14 @@
       <c r="CX120">
         <v>10</v>
       </c>
+      <c r="CZ120">
+        <v>0</v>
+      </c>
+      <c r="DA120">
+        <v>10</v>
+      </c>
     </row>
-    <row r="121" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -25427,8 +26174,14 @@
       <c r="CX121">
         <v>8</v>
       </c>
+      <c r="CZ121">
+        <v>0</v>
+      </c>
+      <c r="DA121">
+        <v>8</v>
+      </c>
     </row>
-    <row r="122" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -25586,8 +26339,14 @@
       <c r="CX122">
         <v>6</v>
       </c>
+      <c r="CZ122">
+        <v>0</v>
+      </c>
+      <c r="DA122">
+        <v>6</v>
+      </c>
     </row>
-    <row r="123" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -25799,8 +26558,14 @@
       <c r="CX123">
         <v>6</v>
       </c>
+      <c r="CZ123">
+        <v>0</v>
+      </c>
+      <c r="DA123">
+        <v>6</v>
+      </c>
     </row>
-    <row r="124" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -26054,8 +26819,14 @@
       <c r="CX124">
         <v>8</v>
       </c>
+      <c r="CZ124">
+        <v>0</v>
+      </c>
+      <c r="DA124">
+        <v>8</v>
+      </c>
     </row>
-    <row r="125" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -26291,8 +27062,14 @@
       <c r="CX125">
         <v>6</v>
       </c>
+      <c r="CZ125">
+        <v>0</v>
+      </c>
+      <c r="DA125">
+        <v>6</v>
+      </c>
     </row>
-    <row r="126" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -26510,8 +27287,14 @@
       <c r="CX126">
         <v>6</v>
       </c>
+      <c r="CZ126">
+        <v>0</v>
+      </c>
+      <c r="DA126">
+        <v>6</v>
+      </c>
     </row>
-    <row r="127" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -26723,8 +27506,14 @@
       <c r="CX127">
         <v>3</v>
       </c>
+      <c r="CZ127">
+        <v>0</v>
+      </c>
+      <c r="DA127">
+        <v>3</v>
+      </c>
     </row>
-    <row r="128" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -26867,8 +27656,14 @@
       <c r="CX128">
         <v>7</v>
       </c>
+      <c r="CZ128">
+        <v>0</v>
+      </c>
+      <c r="DA128">
+        <v>7</v>
+      </c>
     </row>
-    <row r="129" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -27095,8 +27890,14 @@
       <c r="CX129">
         <v>6</v>
       </c>
+      <c r="CZ129">
+        <v>0</v>
+      </c>
+      <c r="DA129">
+        <v>6</v>
+      </c>
     </row>
-    <row r="130" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -27260,8 +28061,14 @@
       <c r="CX130">
         <v>10</v>
       </c>
+      <c r="CZ130">
+        <v>0</v>
+      </c>
+      <c r="DA130">
+        <v>10</v>
+      </c>
     </row>
-    <row r="131" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -27491,8 +28298,14 @@
       <c r="CX131">
         <v>10</v>
       </c>
+      <c r="CZ131">
+        <v>0</v>
+      </c>
+      <c r="DA131">
+        <v>10</v>
+      </c>
     </row>
-    <row r="132" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -27644,8 +28457,14 @@
       <c r="CX132">
         <v>6</v>
       </c>
+      <c r="CZ132">
+        <v>0</v>
+      </c>
+      <c r="DA132">
+        <v>6</v>
+      </c>
     </row>
-    <row r="133" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -27830,8 +28649,14 @@
       <c r="CX133">
         <v>7</v>
       </c>
+      <c r="CZ133">
+        <v>0</v>
+      </c>
+      <c r="DA133">
+        <v>7</v>
+      </c>
     </row>
-    <row r="134" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -28016,8 +28841,14 @@
       <c r="CX134">
         <v>10</v>
       </c>
+      <c r="CZ134">
+        <v>0</v>
+      </c>
+      <c r="DA134">
+        <v>10</v>
+      </c>
     </row>
-    <row r="135" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -28223,8 +29054,14 @@
       <c r="CX135">
         <v>8</v>
       </c>
+      <c r="CZ135">
+        <v>0</v>
+      </c>
+      <c r="DA135">
+        <v>8</v>
+      </c>
     </row>
-    <row r="136" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -28424,8 +29261,14 @@
       <c r="CX136">
         <v>7</v>
       </c>
+      <c r="CZ136">
+        <v>0</v>
+      </c>
+      <c r="DA136">
+        <v>7</v>
+      </c>
     </row>
-    <row r="137" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -28634,8 +29477,14 @@
       <c r="CX137">
         <v>5</v>
       </c>
+      <c r="CZ137">
+        <v>0</v>
+      </c>
+      <c r="DA137">
+        <v>5</v>
+      </c>
     </row>
-    <row r="138" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -28856,8 +29705,14 @@
       <c r="CX138">
         <v>7</v>
       </c>
+      <c r="CZ138">
+        <v>0</v>
+      </c>
+      <c r="DA138">
+        <v>7</v>
+      </c>
     </row>
-    <row r="139" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -29060,8 +29915,14 @@
       <c r="CX139">
         <v>5</v>
       </c>
+      <c r="CZ139">
+        <v>0</v>
+      </c>
+      <c r="DA139">
+        <v>5</v>
+      </c>
     </row>
-    <row r="140" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -29219,8 +30080,14 @@
       <c r="CX140">
         <v>9</v>
       </c>
+      <c r="CZ140">
+        <v>0</v>
+      </c>
+      <c r="DA140">
+        <v>9</v>
+      </c>
     </row>
-    <row r="141" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -29459,8 +30326,14 @@
       <c r="CX141">
         <v>8</v>
       </c>
+      <c r="CZ141">
+        <v>0</v>
+      </c>
+      <c r="DA141">
+        <v>8</v>
+      </c>
     </row>
-    <row r="142" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -29699,8 +30572,14 @@
       <c r="CX142">
         <v>8</v>
       </c>
+      <c r="CZ142">
+        <v>0</v>
+      </c>
+      <c r="DA142">
+        <v>8</v>
+      </c>
     </row>
-    <row r="143" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -29897,8 +30776,14 @@
       <c r="CX143">
         <v>11</v>
       </c>
+      <c r="CZ143">
+        <v>0</v>
+      </c>
+      <c r="DA143">
+        <v>11</v>
+      </c>
     </row>
-    <row r="144" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -30047,8 +30932,14 @@
       <c r="CX144">
         <v>7</v>
       </c>
+      <c r="CZ144">
+        <v>0</v>
+      </c>
+      <c r="DA144">
+        <v>7</v>
+      </c>
     </row>
-    <row r="145" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -30206,8 +31097,14 @@
       <c r="CX145">
         <v>5</v>
       </c>
+      <c r="CZ145">
+        <v>0</v>
+      </c>
+      <c r="DA145">
+        <v>5</v>
+      </c>
     </row>
-    <row r="146" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -30458,8 +31355,14 @@
       <c r="CX146">
         <v>10</v>
       </c>
+      <c r="CZ146">
+        <v>0</v>
+      </c>
+      <c r="DA146">
+        <v>10</v>
+      </c>
     </row>
-    <row r="147" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -30701,8 +31604,14 @@
       <c r="CX147">
         <v>3</v>
       </c>
+      <c r="CZ147">
+        <v>0</v>
+      </c>
+      <c r="DA147">
+        <v>3</v>
+      </c>
     </row>
-    <row r="148" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -30836,8 +31745,17 @@
       <c r="CY148">
         <v>1</v>
       </c>
+      <c r="CZ148">
+        <v>6</v>
+      </c>
+      <c r="DA148">
+        <v>2</v>
+      </c>
+      <c r="DB148">
+        <v>1</v>
+      </c>
     </row>
-    <row r="149" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -31088,8 +32006,14 @@
       <c r="CX149">
         <v>5</v>
       </c>
+      <c r="CZ149">
+        <v>0</v>
+      </c>
+      <c r="DA149">
+        <v>5</v>
+      </c>
     </row>
-    <row r="150" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -31322,8 +32246,14 @@
       <c r="CX150">
         <v>9</v>
       </c>
+      <c r="CZ150">
+        <v>0</v>
+      </c>
+      <c r="DA150">
+        <v>9</v>
+      </c>
     </row>
-    <row r="151" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -31532,8 +32462,14 @@
       <c r="CX151">
         <v>10</v>
       </c>
+      <c r="CZ151">
+        <v>0</v>
+      </c>
+      <c r="DA151">
+        <v>10</v>
+      </c>
     </row>
-    <row r="152" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -31679,8 +32615,14 @@
       <c r="CX152">
         <v>9</v>
       </c>
+      <c r="CZ152">
+        <v>0</v>
+      </c>
+      <c r="DA152">
+        <v>9</v>
+      </c>
     </row>
-    <row r="153" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -31880,8 +32822,14 @@
       <c r="CX153">
         <v>7</v>
       </c>
+      <c r="CZ153">
+        <v>0</v>
+      </c>
+      <c r="DA153">
+        <v>7</v>
+      </c>
     </row>
-    <row r="154" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -32147,8 +33095,14 @@
       <c r="CX154">
         <v>8</v>
       </c>
+      <c r="CZ154">
+        <v>0</v>
+      </c>
+      <c r="DA154">
+        <v>8</v>
+      </c>
     </row>
-    <row r="155" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -32363,8 +33317,14 @@
       <c r="CX155">
         <v>9</v>
       </c>
+      <c r="CZ155">
+        <v>0</v>
+      </c>
+      <c r="DA155">
+        <v>9</v>
+      </c>
     </row>
-    <row r="156" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="156" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -32516,8 +33476,14 @@
       <c r="CX156">
         <v>6</v>
       </c>
+      <c r="CZ156">
+        <v>0</v>
+      </c>
+      <c r="DA156">
+        <v>6</v>
+      </c>
     </row>
-    <row r="157" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="157" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -32669,8 +33635,14 @@
       <c r="CX157">
         <v>6</v>
       </c>
+      <c r="CZ157">
+        <v>0</v>
+      </c>
+      <c r="DA157">
+        <v>6</v>
+      </c>
     </row>
-    <row r="158" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="158" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -32858,8 +33830,14 @@
       <c r="CX158">
         <v>8</v>
       </c>
+      <c r="CZ158">
+        <v>0</v>
+      </c>
+      <c r="DA158">
+        <v>8</v>
+      </c>
     </row>
-    <row r="159" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -33089,8 +34067,14 @@
       <c r="CX159">
         <v>5</v>
       </c>
+      <c r="CZ159">
+        <v>0</v>
+      </c>
+      <c r="DA159">
+        <v>5</v>
+      </c>
     </row>
-    <row r="160" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:106" x14ac:dyDescent="0.3">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -33236,8 +34220,14 @@
       <c r="CY160">
         <v>1</v>
       </c>
+      <c r="CZ160">
+        <v>1</v>
+      </c>
+      <c r="DA160">
+        <v>8</v>
+      </c>
     </row>
-    <row r="161" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -33488,8 +34478,14 @@
       <c r="CX161">
         <v>7</v>
       </c>
+      <c r="CZ161">
+        <v>0</v>
+      </c>
+      <c r="DA161">
+        <v>7</v>
+      </c>
     </row>
-    <row r="162" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -33638,8 +34634,14 @@
       <c r="CX162">
         <v>8</v>
       </c>
+      <c r="CZ162">
+        <v>0</v>
+      </c>
+      <c r="DA162">
+        <v>8</v>
+      </c>
     </row>
-    <row r="163" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="163" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -33848,8 +34850,14 @@
       <c r="CX163">
         <v>8</v>
       </c>
+      <c r="CZ163">
+        <v>0</v>
+      </c>
+      <c r="DA163">
+        <v>8</v>
+      </c>
     </row>
-    <row r="164" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="164" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -34004,8 +35012,14 @@
       <c r="CY164">
         <v>1</v>
       </c>
+      <c r="CZ164">
+        <v>0</v>
+      </c>
+      <c r="DA164">
+        <v>9</v>
+      </c>
     </row>
-    <row r="165" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -34214,8 +35228,14 @@
       <c r="CX165">
         <v>6</v>
       </c>
+      <c r="CZ165">
+        <v>0</v>
+      </c>
+      <c r="DA165">
+        <v>6</v>
+      </c>
     </row>
-    <row r="166" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="166" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -34409,8 +35429,14 @@
       <c r="CX166">
         <v>6</v>
       </c>
+      <c r="CZ166">
+        <v>0</v>
+      </c>
+      <c r="DA166">
+        <v>6</v>
+      </c>
     </row>
-    <row r="167" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -34607,8 +35633,14 @@
       <c r="CX167">
         <v>8</v>
       </c>
+      <c r="CZ167">
+        <v>0</v>
+      </c>
+      <c r="DA167">
+        <v>8</v>
+      </c>
     </row>
-    <row r="168" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -34838,8 +35870,14 @@
       <c r="CX168">
         <v>11</v>
       </c>
+      <c r="CZ168">
+        <v>0</v>
+      </c>
+      <c r="DA168">
+        <v>11</v>
+      </c>
     </row>
-    <row r="169" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -34991,8 +36029,14 @@
       <c r="CX169">
         <v>6</v>
       </c>
+      <c r="CZ169">
+        <v>0</v>
+      </c>
+      <c r="DA169">
+        <v>6</v>
+      </c>
     </row>
-    <row r="170" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -35168,8 +36212,14 @@
       <c r="CX170">
         <v>8</v>
       </c>
+      <c r="CZ170">
+        <v>0</v>
+      </c>
+      <c r="DA170">
+        <v>8</v>
+      </c>
     </row>
-    <row r="171" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="171" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -35408,8 +36458,14 @@
       <c r="CX171">
         <v>10</v>
       </c>
+      <c r="CZ171">
+        <v>0</v>
+      </c>
+      <c r="DA171">
+        <v>10</v>
+      </c>
     </row>
-    <row r="172" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -35567,8 +36623,14 @@
       <c r="CX172">
         <v>8</v>
       </c>
+      <c r="CZ172">
+        <v>0</v>
+      </c>
+      <c r="DA172">
+        <v>8</v>
+      </c>
     </row>
-    <row r="173" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -35741,8 +36803,14 @@
       <c r="CX173">
         <v>8</v>
       </c>
+      <c r="CZ173">
+        <v>0</v>
+      </c>
+      <c r="DA173">
+        <v>8</v>
+      </c>
     </row>
-    <row r="174" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -35900,8 +36968,14 @@
       <c r="CX174">
         <v>9</v>
       </c>
+      <c r="CZ174">
+        <v>0</v>
+      </c>
+      <c r="DA174">
+        <v>9</v>
+      </c>
     </row>
-    <row r="175" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -36116,8 +37190,14 @@
       <c r="CX175">
         <v>9</v>
       </c>
+      <c r="CZ175">
+        <v>0</v>
+      </c>
+      <c r="DA175">
+        <v>9</v>
+      </c>
     </row>
-    <row r="176" spans="2:103" x14ac:dyDescent="0.3">
+    <row r="176" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -36266,8 +37346,14 @@
       <c r="CX176">
         <v>8</v>
       </c>
+      <c r="CZ176">
+        <v>0</v>
+      </c>
+      <c r="DA176">
+        <v>8</v>
+      </c>
     </row>
-    <row r="177" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -36425,8 +37511,14 @@
       <c r="CX177">
         <v>5</v>
       </c>
+      <c r="CZ177">
+        <v>0</v>
+      </c>
+      <c r="DA177">
+        <v>5</v>
+      </c>
     </row>
-    <row r="178" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -36590,8 +37682,14 @@
       <c r="CX178">
         <v>8</v>
       </c>
+      <c r="CZ178">
+        <v>0</v>
+      </c>
+      <c r="DA178">
+        <v>8</v>
+      </c>
     </row>
-    <row r="179" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -36806,8 +37904,14 @@
       <c r="CX179">
         <v>10</v>
       </c>
+      <c r="CZ179">
+        <v>0</v>
+      </c>
+      <c r="DA179">
+        <v>10</v>
+      </c>
     </row>
-    <row r="180" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -37019,8 +38123,14 @@
       <c r="CX180">
         <v>9</v>
       </c>
+      <c r="CZ180">
+        <v>0</v>
+      </c>
+      <c r="DA180">
+        <v>9</v>
+      </c>
     </row>
-    <row r="181" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -37232,8 +38342,14 @@
       <c r="CX181">
         <v>9</v>
       </c>
+      <c r="CZ181">
+        <v>0</v>
+      </c>
+      <c r="DA181">
+        <v>9</v>
+      </c>
     </row>
-    <row r="182" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -37388,8 +38504,14 @@
       <c r="CX182">
         <v>6</v>
       </c>
+      <c r="CZ182">
+        <v>0</v>
+      </c>
+      <c r="DA182">
+        <v>6</v>
+      </c>
     </row>
-    <row r="183" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -37633,8 +38755,14 @@
       <c r="CX183">
         <v>5</v>
       </c>
+      <c r="CZ183">
+        <v>0</v>
+      </c>
+      <c r="DA183">
+        <v>5</v>
+      </c>
     </row>
-    <row r="184" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -37797,8 +38925,14 @@
       <c r="CX184">
         <v>6</v>
       </c>
+      <c r="CZ184">
+        <v>0</v>
+      </c>
+      <c r="DA184">
+        <v>6</v>
+      </c>
     </row>
-    <row r="185" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -38012,8 +39146,14 @@
       <c r="CX185">
         <v>7</v>
       </c>
+      <c r="CZ185">
+        <v>0</v>
+      </c>
+      <c r="DA185">
+        <v>7</v>
+      </c>
     </row>
-    <row r="186" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -38215,8 +39355,14 @@
       <c r="CX186">
         <v>1</v>
       </c>
+      <c r="CZ186">
+        <v>5</v>
+      </c>
+      <c r="DA186">
+        <v>2</v>
+      </c>
     </row>
-    <row r="187" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -38388,8 +39534,14 @@
       <c r="CX187">
         <v>8</v>
       </c>
+      <c r="CZ187">
+        <v>0</v>
+      </c>
+      <c r="DA187">
+        <v>8</v>
+      </c>
     </row>
-    <row r="188" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B188" t="s">
         <v>4</v>
       </c>
@@ -38615,8 +39767,14 @@
       <c r="CX188">
         <v>10</v>
       </c>
+      <c r="CZ188">
+        <v>0</v>
+      </c>
+      <c r="DA188">
+        <v>10</v>
+      </c>
     </row>
-    <row r="189" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -38836,8 +39994,14 @@
       <c r="CX189">
         <v>2</v>
       </c>
+      <c r="CZ189">
+        <v>0</v>
+      </c>
+      <c r="DA189">
+        <v>2</v>
+      </c>
     </row>
-    <row r="190" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="190" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -39060,8 +40224,14 @@
       <c r="CX190">
         <v>5</v>
       </c>
+      <c r="CZ190">
+        <v>0</v>
+      </c>
+      <c r="DA190">
+        <v>5</v>
+      </c>
     </row>
-    <row r="191" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="191" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -39287,8 +40457,14 @@
       <c r="CX191">
         <v>5</v>
       </c>
+      <c r="CZ191">
+        <v>0</v>
+      </c>
+      <c r="DA191">
+        <v>5</v>
+      </c>
     </row>
-    <row r="192" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="192" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -39493,8 +40669,14 @@
       <c r="CX192">
         <v>3</v>
       </c>
+      <c r="CZ192">
+        <v>0</v>
+      </c>
+      <c r="DA192">
+        <v>3</v>
+      </c>
     </row>
-    <row r="193" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="193" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -39723,8 +40905,14 @@
       <c r="CX193">
         <v>7</v>
       </c>
+      <c r="CZ193">
+        <v>0</v>
+      </c>
+      <c r="DA193">
+        <v>7</v>
+      </c>
     </row>
-    <row r="194" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="194" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B194" t="s">
         <v>4</v>
       </c>
@@ -39929,8 +41117,14 @@
       <c r="CX194">
         <v>7</v>
       </c>
+      <c r="CZ194">
+        <v>0</v>
+      </c>
+      <c r="DA194">
+        <v>7</v>
+      </c>
     </row>
-    <row r="195" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="195" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -40150,8 +41344,14 @@
       <c r="CX195">
         <v>2</v>
       </c>
+      <c r="CZ195">
+        <v>0</v>
+      </c>
+      <c r="DA195">
+        <v>2</v>
+      </c>
     </row>
-    <row r="196" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="196" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -40404,8 +41604,14 @@
       <c r="CX196">
         <v>9</v>
       </c>
+      <c r="CZ196">
+        <v>0</v>
+      </c>
+      <c r="DA196">
+        <v>9</v>
+      </c>
     </row>
-    <row r="197" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="197" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -40613,8 +41819,14 @@
       <c r="CX197">
         <v>4</v>
       </c>
+      <c r="CZ197">
+        <v>0</v>
+      </c>
+      <c r="DA197">
+        <v>4</v>
+      </c>
     </row>
-    <row r="198" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="198" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -40804,8 +42016,14 @@
       <c r="CX198">
         <v>5</v>
       </c>
+      <c r="CZ198">
+        <v>0</v>
+      </c>
+      <c r="DA198">
+        <v>5</v>
+      </c>
     </row>
-    <row r="199" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="199" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -41007,8 +42225,14 @@
       <c r="CX199">
         <v>6</v>
       </c>
+      <c r="CZ199">
+        <v>0</v>
+      </c>
+      <c r="DA199">
+        <v>6</v>
+      </c>
     </row>
-    <row r="200" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="200" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
         <v>4</v>
       </c>
@@ -41207,8 +42431,14 @@
       <c r="CX200">
         <v>7</v>
       </c>
+      <c r="CZ200">
+        <v>0</v>
+      </c>
+      <c r="DA200">
+        <v>7</v>
+      </c>
     </row>
-    <row r="201" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="201" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -41443,8 +42673,14 @@
       <c r="CX201">
         <v>6</v>
       </c>
+      <c r="CZ201">
+        <v>0</v>
+      </c>
+      <c r="DA201">
+        <v>6</v>
+      </c>
     </row>
-    <row r="202" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="202" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -41670,8 +42906,14 @@
       <c r="CX202">
         <v>1</v>
       </c>
+      <c r="CZ202">
+        <v>0</v>
+      </c>
+      <c r="DA202">
+        <v>1</v>
+      </c>
     </row>
-    <row r="203" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="203" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -41891,8 +43133,14 @@
       <c r="CX203">
         <v>3</v>
       </c>
+      <c r="CZ203">
+        <v>0</v>
+      </c>
+      <c r="DA203">
+        <v>3</v>
+      </c>
     </row>
-    <row r="204" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="204" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -42019,8 +43267,11 @@
       <c r="CW204">
         <v>6</v>
       </c>
+      <c r="CZ204">
+        <v>6</v>
+      </c>
     </row>
-    <row r="205" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="205" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -42261,8 +43512,14 @@
       <c r="CX205">
         <v>8</v>
       </c>
+      <c r="CZ205">
+        <v>2</v>
+      </c>
+      <c r="DA205">
+        <v>8</v>
+      </c>
     </row>
-    <row r="206" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="206" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B206" t="s">
         <v>4</v>
       </c>
@@ -42407,8 +43664,14 @@
       <c r="CX206">
         <v>6</v>
       </c>
+      <c r="CZ206">
+        <v>0</v>
+      </c>
+      <c r="DA206">
+        <v>6</v>
+      </c>
     </row>
-    <row r="207" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="207" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -42601,8 +43864,14 @@
       <c r="CX207">
         <v>4</v>
       </c>
+      <c r="CZ207">
+        <v>0</v>
+      </c>
+      <c r="DA207">
+        <v>4</v>
+      </c>
     </row>
-    <row r="208" spans="2:102" x14ac:dyDescent="0.3">
+    <row r="208" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -42820,6 +44089,12 @@
         <v>0</v>
       </c>
       <c r="CX208">
+        <v>3</v>
+      </c>
+      <c r="CZ208">
+        <v>0</v>
+      </c>
+      <c r="DA208">
         <v>3</v>
       </c>
     </row>
@@ -43028,6 +44303,12 @@
       <c r="CX209">
         <v>5</v>
       </c>
+      <c r="CZ209">
+        <v>0</v>
+      </c>
+      <c r="DA209">
+        <v>5</v>
+      </c>
     </row>
     <row r="210" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B210" t="s">
@@ -43258,6 +44539,12 @@
       <c r="CY210">
         <v>1</v>
       </c>
+      <c r="CZ210">
+        <v>0</v>
+      </c>
+      <c r="DA210">
+        <v>5</v>
+      </c>
     </row>
     <row r="211" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
@@ -43464,6 +44751,12 @@
       <c r="CX211">
         <v>4</v>
       </c>
+      <c r="CZ211">
+        <v>1</v>
+      </c>
+      <c r="DA211">
+        <v>4</v>
+      </c>
     </row>
     <row r="212" spans="2:105" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
@@ -43662,6 +44955,12 @@
         <v>0</v>
       </c>
       <c r="CX212">
+        <v>6</v>
+      </c>
+      <c r="CZ212">
+        <v>0</v>
+      </c>
+      <c r="DA212">
         <v>6</v>
       </c>
     </row>

</xml_diff>